<commit_message>
Expand concrete company dataset
</commit_message>
<xml_diff>
--- a/data/companies.xlsx
+++ b/data/companies.xlsx
@@ -12,7 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Importo žurnalas" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Įmonės'!$A$1:$AB$27</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Įmonės'!$A$1:$AB$46</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -169,8 +169,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ImonesTable" displayName="ImonesTable" ref="A1:AB27" headerRowCount="1">
-  <autoFilter ref="A1:AB27"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ImonesTable" displayName="ImonesTable" ref="A1:AB46" headerRowCount="1">
+  <autoFilter ref="A1:AB46"/>
   <tableColumns count="28">
     <tableColumn id="1" name="Įrašo ID"/>
     <tableColumn id="2" name="Įmonės kodas"/>
@@ -494,14 +494,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AB27"/>
+  <dimension ref="A1:AB46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="38" customWidth="1" min="1" max="1"/>
+    <col width="39" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
     <col width="42" customWidth="1" min="3" max="3"/>
-    <col width="29" customWidth="1" min="4" max="4"/>
-    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="33" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
     <col width="16" customWidth="1" min="6" max="6"/>
     <col width="19" customWidth="1" min="7" max="7"/>
     <col width="42" customWidth="1" min="8" max="8"/>
@@ -509,7 +509,7 @@
     <col width="12" customWidth="1" min="10" max="10"/>
     <col width="20" customWidth="1" min="11" max="11"/>
     <col width="24" customWidth="1" min="12" max="12"/>
-    <col width="38" customWidth="1" min="13" max="13"/>
+    <col width="40" customWidth="1" min="13" max="13"/>
     <col width="30" customWidth="1" min="14" max="14"/>
     <col width="42" customWidth="1" min="15" max="15"/>
     <col width="29" customWidth="1" min="16" max="16"/>
@@ -3173,8 +3173,1888 @@
         </is>
       </c>
     </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>sodbeta-siauliai</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr"/>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>UAB Sodbeta</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>Sodbeta</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="inlineStr">
+        <is>
+          <t>Papildomai rasta</t>
+        </is>
+      </c>
+      <c r="F28" s="2" t="inlineStr">
+        <is>
+          <t>Šiauliai</t>
+        </is>
+      </c>
+      <c r="G28" s="2" t="inlineStr">
+        <is>
+          <t>Šiaulių m. sav.</t>
+        </is>
+      </c>
+      <c r="H28" s="2" t="inlineStr">
+        <is>
+          <t>Sodo g. 20, Šiauliai</t>
+        </is>
+      </c>
+      <c r="I28" s="3" t="n">
+        <v>55.94918</v>
+      </c>
+      <c r="J28" s="3" t="n">
+        <v>23.3127083</v>
+      </c>
+      <c r="K28" s="2" t="inlineStr">
+        <is>
+          <t>precast_concrete</t>
+        </is>
+      </c>
+      <c r="L28" s="2" t="inlineStr">
+        <is>
+          <t>Betono gaminiai</t>
+        </is>
+      </c>
+      <c r="M28" s="2" t="inlineStr">
+        <is>
+          <t>Sodbeta betono gaminių gamykla</t>
+        </is>
+      </c>
+      <c r="N28" s="2" t="inlineStr"/>
+      <c r="O28" s="2" t="inlineStr">
+        <is>
+          <t>Viešai skelbiama gelžbetonio ir betono gaminių gamyba Šiauliuose.</t>
+        </is>
+      </c>
+      <c r="P28" s="4" t="n">
+        <v>0.82</v>
+      </c>
+      <c r="Q28" s="5" t="n"/>
+      <c r="R28" s="5" t="n"/>
+      <c r="S28" s="5" t="n"/>
+      <c r="T28" s="5" t="n"/>
+      <c r="U28" s="2" t="inlineStr">
+        <is>
+          <t>https://sodbeta.lt/</t>
+        </is>
+      </c>
+      <c r="V28" s="2" t="inlineStr">
+        <is>
+          <t>https://sodbeta.lt/</t>
+        </is>
+      </c>
+      <c r="W28" s="2" t="inlineStr"/>
+      <c r="X28" s="2" t="inlineStr"/>
+      <c r="Y28" s="2" t="inlineStr"/>
+      <c r="Z28" s="2" t="inlineStr">
+        <is>
+          <t>https://sodbeta.lt/</t>
+        </is>
+      </c>
+      <c r="AA28" s="2" t="inlineStr">
+        <is>
+          <t>Papildomai rasta pagal požymį betono gaminiai.</t>
+        </is>
+      </c>
+      <c r="AB28" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>alytaus-gelzbetonis-alytus</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="inlineStr"/>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>AB Alytaus gelžbetonis</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="inlineStr">
+        <is>
+          <t>Alytaus gelžbetonis</t>
+        </is>
+      </c>
+      <c r="E29" s="2" t="inlineStr">
+        <is>
+          <t>Papildomai rasta</t>
+        </is>
+      </c>
+      <c r="F29" s="2" t="inlineStr">
+        <is>
+          <t>Alytus</t>
+        </is>
+      </c>
+      <c r="G29" s="2" t="inlineStr">
+        <is>
+          <t>Alytaus m. sav.</t>
+        </is>
+      </c>
+      <c r="H29" s="2" t="inlineStr">
+        <is>
+          <t>Pramonės g. 15, Alytus</t>
+        </is>
+      </c>
+      <c r="I29" s="3" t="n">
+        <v>54.4259854</v>
+      </c>
+      <c r="J29" s="3" t="n">
+        <v>24.0150611</v>
+      </c>
+      <c r="K29" s="2" t="inlineStr">
+        <is>
+          <t>precast_concrete</t>
+        </is>
+      </c>
+      <c r="L29" s="2" t="inlineStr">
+        <is>
+          <t>Betono gaminiai</t>
+        </is>
+      </c>
+      <c r="M29" s="2" t="inlineStr">
+        <is>
+          <t>Alytaus gelžbetonio gamykla</t>
+        </is>
+      </c>
+      <c r="N29" s="2" t="inlineStr"/>
+      <c r="O29" s="2" t="inlineStr">
+        <is>
+          <t>Viešai skelbiami betono ir gelžbetonio gaminiai Alytuje.</t>
+        </is>
+      </c>
+      <c r="P29" s="4" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="Q29" s="5" t="n"/>
+      <c r="R29" s="5" t="n"/>
+      <c r="S29" s="5" t="n"/>
+      <c r="T29" s="5" t="n"/>
+      <c r="U29" s="2" t="inlineStr">
+        <is>
+          <t>https://alytausgelzbetonis.lt/</t>
+        </is>
+      </c>
+      <c r="V29" s="2" t="inlineStr">
+        <is>
+          <t>https://alytausgelzbetonis.lt/kontaktai/</t>
+        </is>
+      </c>
+      <c r="W29" s="2" t="inlineStr"/>
+      <c r="X29" s="2" t="inlineStr"/>
+      <c r="Y29" s="2" t="inlineStr"/>
+      <c r="Z29" s="2" t="inlineStr">
+        <is>
+          <t>https://alytausgelzbetonis.lt/kontaktai/</t>
+        </is>
+      </c>
+      <c r="AA29" s="2" t="inlineStr">
+        <is>
+          <t>Anksčiau ieškota pagal Presbetonas / Alytaus gelžbetonis požymius.</t>
+        </is>
+      </c>
+      <c r="AB29" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>gernora-marijampole</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="inlineStr"/>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t>UAB Gernora</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t>Gernora</t>
+        </is>
+      </c>
+      <c r="E30" s="2" t="inlineStr">
+        <is>
+          <t>Papildomai rasta</t>
+        </is>
+      </c>
+      <c r="F30" s="2" t="inlineStr">
+        <is>
+          <t>Marijampolė</t>
+        </is>
+      </c>
+      <c r="G30" s="2" t="inlineStr">
+        <is>
+          <t>Marijampolės sav.</t>
+        </is>
+      </c>
+      <c r="H30" s="2" t="inlineStr">
+        <is>
+          <t>Vingio g. 2M, Marijampolė</t>
+        </is>
+      </c>
+      <c r="I30" s="3" t="n">
+        <v>54.5358398</v>
+      </c>
+      <c r="J30" s="3" t="n">
+        <v>23.3344441</v>
+      </c>
+      <c r="K30" s="2" t="inlineStr">
+        <is>
+          <t>ready_mix_concrete</t>
+        </is>
+      </c>
+      <c r="L30" s="2" t="inlineStr">
+        <is>
+          <t>Betono mišiniai</t>
+        </is>
+      </c>
+      <c r="M30" s="2" t="inlineStr">
+        <is>
+          <t>Gernora betono mazgas</t>
+        </is>
+      </c>
+      <c r="N30" s="2" t="inlineStr"/>
+      <c r="O30" s="2" t="inlineStr">
+        <is>
+          <t>Viešai skelbiamas betono mišinių tiekėjas Marijampolėje.</t>
+        </is>
+      </c>
+      <c r="P30" s="4" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="Q30" s="5" t="n"/>
+      <c r="R30" s="5" t="n"/>
+      <c r="S30" s="5" t="n"/>
+      <c r="T30" s="5" t="n"/>
+      <c r="U30" s="2" t="inlineStr">
+        <is>
+          <t>https://gernora.lt/</t>
+        </is>
+      </c>
+      <c r="V30" s="2" t="inlineStr">
+        <is>
+          <t>https://gernora.lt/</t>
+        </is>
+      </c>
+      <c r="W30" s="2" t="inlineStr"/>
+      <c r="X30" s="2" t="inlineStr"/>
+      <c r="Y30" s="2" t="inlineStr"/>
+      <c r="Z30" s="2" t="inlineStr">
+        <is>
+          <t>https://gernora.lt/</t>
+        </is>
+      </c>
+      <c r="AA30" s="2" t="inlineStr">
+        <is>
+          <t>Reikia patikslinti našumą.</t>
+        </is>
+      </c>
+      <c r="AB30" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>re-betono-konstrukcijos-kretinga</t>
+        </is>
+      </c>
+      <c r="B31" s="2" t="inlineStr"/>
+      <c r="C31" s="2" t="inlineStr">
+        <is>
+          <t>UAB RE Betono konstrukcijos</t>
+        </is>
+      </c>
+      <c r="D31" s="2" t="inlineStr">
+        <is>
+          <t>RE Betono konstrukcijos</t>
+        </is>
+      </c>
+      <c r="E31" s="2" t="inlineStr">
+        <is>
+          <t>Papildomai rasta</t>
+        </is>
+      </c>
+      <c r="F31" s="2" t="inlineStr">
+        <is>
+          <t>Kretinga</t>
+        </is>
+      </c>
+      <c r="G31" s="2" t="inlineStr">
+        <is>
+          <t>Kretingos r. sav.</t>
+        </is>
+      </c>
+      <c r="H31" s="2" t="inlineStr">
+        <is>
+          <t>Tiek?j? g. 27B, Kretinga</t>
+        </is>
+      </c>
+      <c r="I31" s="3" t="n">
+        <v>55.8796284</v>
+      </c>
+      <c r="J31" s="3" t="n">
+        <v>21.2209417</v>
+      </c>
+      <c r="K31" s="2" t="inlineStr">
+        <is>
+          <t>precast_concrete</t>
+        </is>
+      </c>
+      <c r="L31" s="2" t="inlineStr">
+        <is>
+          <t>Betono gaminiai</t>
+        </is>
+      </c>
+      <c r="M31" s="2" t="inlineStr">
+        <is>
+          <t>RE Betono konstrukcij? gamyba</t>
+        </is>
+      </c>
+      <c r="N31" s="2" t="inlineStr"/>
+      <c r="O31" s="2" t="inlineStr">
+        <is>
+          <t>Viešame kataloge nurodomi betonas, cemento gaminiai, betono siurblys ir pamatų blokai Kretingoje.</t>
+        </is>
+      </c>
+      <c r="P31" s="4" t="n">
+        <v>0.78</v>
+      </c>
+      <c r="Q31" s="5" t="n"/>
+      <c r="R31" s="5" t="n"/>
+      <c r="S31" s="5" t="n"/>
+      <c r="T31" s="5" t="n"/>
+      <c r="U31" s="2" t="inlineStr"/>
+      <c r="V31" s="2" t="inlineStr">
+        <is>
+          <t>https://www.1551.lt/re-betono-konstrukcijos-uab-betonas-cementas-betono-siurblys-pamatu-blokai-kretingoje-104253/</t>
+        </is>
+      </c>
+      <c r="W31" s="2" t="inlineStr"/>
+      <c r="X31" s="2" t="inlineStr"/>
+      <c r="Y31" s="2" t="inlineStr"/>
+      <c r="Z31" s="2" t="inlineStr">
+        <is>
+          <t>https://www.1551.lt/re-betono-konstrukcijos-uab-betonas-cementas-betono-siurblys-pamatu-blokai-kretingoje-104253/</t>
+        </is>
+      </c>
+      <c r="AA31" s="2" t="inlineStr">
+        <is>
+          <t>Katalogo šaltinis, reikia patikslinti gamybos apimtį.</t>
+        </is>
+      </c>
+      <c r="AB31" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>silales-statyba-vingininkai</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="inlineStr"/>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>UAB Šilalės statyba</t>
+        </is>
+      </c>
+      <c r="D32" s="2" t="inlineStr">
+        <is>
+          <t>Šilalės statyba</t>
+        </is>
+      </c>
+      <c r="E32" s="2" t="inlineStr">
+        <is>
+          <t>Papildomai rasta</t>
+        </is>
+      </c>
+      <c r="F32" s="2" t="inlineStr">
+        <is>
+          <t>Vingininkai</t>
+        </is>
+      </c>
+      <c r="G32" s="2" t="inlineStr">
+        <is>
+          <t>Šilalės r. sav.</t>
+        </is>
+      </c>
+      <c r="H32" s="2" t="inlineStr">
+        <is>
+          <t>Lauryno Ivinskio g. 7, Vingininkai, Šilalės r.</t>
+        </is>
+      </c>
+      <c r="I32" s="3" t="n">
+        <v>55.4808288</v>
+      </c>
+      <c r="J32" s="3" t="n">
+        <v>22.1937625</v>
+      </c>
+      <c r="K32" s="2" t="inlineStr">
+        <is>
+          <t>precast_concrete</t>
+        </is>
+      </c>
+      <c r="L32" s="2" t="inlineStr">
+        <is>
+          <t>Betono gaminiai</t>
+        </is>
+      </c>
+      <c r="M32" s="2" t="inlineStr">
+        <is>
+          <t>Šilalės statybos betono gaminių gamyba</t>
+        </is>
+      </c>
+      <c r="N32" s="2" t="inlineStr"/>
+      <c r="O32" s="2" t="inlineStr">
+        <is>
+          <t>Viešai skelbiama betono gaminių ir statybinių konstrukcijų veikla Šilalės rajone.</t>
+        </is>
+      </c>
+      <c r="P32" s="4" t="n">
+        <v>0.72</v>
+      </c>
+      <c r="Q32" s="5" t="n"/>
+      <c r="R32" s="5" t="n"/>
+      <c r="S32" s="5" t="n"/>
+      <c r="T32" s="5" t="n"/>
+      <c r="U32" s="2" t="inlineStr">
+        <is>
+          <t>https://www.silalesstatyba.lt/</t>
+        </is>
+      </c>
+      <c r="V32" s="2" t="inlineStr">
+        <is>
+          <t>https://www.silalesstatyba.lt/</t>
+        </is>
+      </c>
+      <c r="W32" s="2" t="inlineStr"/>
+      <c r="X32" s="2" t="inlineStr"/>
+      <c r="Y32" s="2" t="inlineStr"/>
+      <c r="Z32" s="2" t="inlineStr">
+        <is>
+          <t>https://www.silalesstatyba.lt/</t>
+        </is>
+      </c>
+      <c r="AA32" s="2" t="inlineStr">
+        <is>
+          <t>Reikia patikslinti tikslų gaminių asortimentą.</t>
+        </is>
+      </c>
+      <c r="AB32" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>panevezio-gelzbetonis-panevezys</t>
+        </is>
+      </c>
+      <c r="B33" s="2" t="inlineStr"/>
+      <c r="C33" s="2" t="inlineStr">
+        <is>
+          <t>UAB Panevėžio gelžbetonis</t>
+        </is>
+      </c>
+      <c r="D33" s="2" t="inlineStr">
+        <is>
+          <t>Panevėžio gelžbetonis</t>
+        </is>
+      </c>
+      <c r="E33" s="2" t="inlineStr">
+        <is>
+          <t>Papildomai rasta</t>
+        </is>
+      </c>
+      <c r="F33" s="2" t="inlineStr">
+        <is>
+          <t>Panevėžys</t>
+        </is>
+      </c>
+      <c r="G33" s="2" t="inlineStr">
+        <is>
+          <t>Panevėžio m. sav.</t>
+        </is>
+      </c>
+      <c r="H33" s="2" t="inlineStr">
+        <is>
+          <t>S. Kerbedžio g. 52, Panevėžys</t>
+        </is>
+      </c>
+      <c r="I33" s="3" t="n">
+        <v>55.7409599</v>
+      </c>
+      <c r="J33" s="3" t="n">
+        <v>24.3802782</v>
+      </c>
+      <c r="K33" s="2" t="inlineStr">
+        <is>
+          <t>precast_concrete</t>
+        </is>
+      </c>
+      <c r="L33" s="2" t="inlineStr">
+        <is>
+          <t>Gelžbetonis</t>
+        </is>
+      </c>
+      <c r="M33" s="2" t="inlineStr">
+        <is>
+          <t>Panevėžio gelžbetonio gamykla</t>
+        </is>
+      </c>
+      <c r="N33" s="2" t="inlineStr"/>
+      <c r="O33" s="2" t="inlineStr">
+        <is>
+          <t>Viešame įmonių kataloge nurodomas gelžbetonio gaminių profilis Panevėžyje.</t>
+        </is>
+      </c>
+      <c r="P33" s="4" t="n">
+        <v>0.78</v>
+      </c>
+      <c r="Q33" s="5" t="n"/>
+      <c r="R33" s="5" t="n"/>
+      <c r="S33" s="5" t="n"/>
+      <c r="T33" s="5" t="n"/>
+      <c r="U33" s="2" t="inlineStr"/>
+      <c r="V33" s="2" t="inlineStr">
+        <is>
+          <t>https://www.spec.lt/imone/panevezio-gelzbetonis-uab</t>
+        </is>
+      </c>
+      <c r="W33" s="2" t="inlineStr"/>
+      <c r="X33" s="2" t="inlineStr"/>
+      <c r="Y33" s="2" t="inlineStr"/>
+      <c r="Z33" s="2" t="inlineStr">
+        <is>
+          <t>https://www.spec.lt/imone/panevezio-gelzbetonis-uab</t>
+        </is>
+      </c>
+      <c r="AA33" s="2" t="inlineStr">
+        <is>
+          <t>Reikia patikrinti veiklos aktyvumą ir produkcijos apimtį.</t>
+        </is>
+      </c>
+      <c r="AB33" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>pamatas-telsiai</t>
+        </is>
+      </c>
+      <c r="B34" s="2" t="inlineStr"/>
+      <c r="C34" s="2" t="inlineStr">
+        <is>
+          <t>UAB Pamatas</t>
+        </is>
+      </c>
+      <c r="D34" s="2" t="inlineStr">
+        <is>
+          <t>Pamatas</t>
+        </is>
+      </c>
+      <c r="E34" s="2" t="inlineStr">
+        <is>
+          <t>Papildomai rasta</t>
+        </is>
+      </c>
+      <c r="F34" s="2" t="inlineStr">
+        <is>
+          <t>Telšiai</t>
+        </is>
+      </c>
+      <c r="G34" s="2" t="inlineStr">
+        <is>
+          <t>Telšių r. sav.</t>
+        </is>
+      </c>
+      <c r="H34" s="2" t="inlineStr">
+        <is>
+          <t>Dimaičių k., Degaičių sen., Telšių r.</t>
+        </is>
+      </c>
+      <c r="I34" s="3" t="n">
+        <v>55.9838213</v>
+      </c>
+      <c r="J34" s="3" t="n">
+        <v>22.2664049</v>
+      </c>
+      <c r="K34" s="2" t="inlineStr">
+        <is>
+          <t>precast_concrete</t>
+        </is>
+      </c>
+      <c r="L34" s="2" t="inlineStr">
+        <is>
+          <t>Betono gaminiai</t>
+        </is>
+      </c>
+      <c r="M34" s="2" t="inlineStr">
+        <is>
+          <t>Pamatas betono gamini? gamyba</t>
+        </is>
+      </c>
+      <c r="N34" s="2" t="inlineStr"/>
+      <c r="O34" s="2" t="inlineStr">
+        <is>
+          <t>Viešai skelbiami pamatų ir kiti betono gaminiai Telšių rajone.</t>
+        </is>
+      </c>
+      <c r="P34" s="4" t="n">
+        <v>0.72</v>
+      </c>
+      <c r="Q34" s="5" t="n"/>
+      <c r="R34" s="5" t="n"/>
+      <c r="S34" s="5" t="n"/>
+      <c r="T34" s="5" t="n"/>
+      <c r="U34" s="2" t="inlineStr">
+        <is>
+          <t>https://pamatas.lt/</t>
+        </is>
+      </c>
+      <c r="V34" s="2" t="inlineStr">
+        <is>
+          <t>https://pamatas.lt/</t>
+        </is>
+      </c>
+      <c r="W34" s="2" t="inlineStr"/>
+      <c r="X34" s="2" t="inlineStr"/>
+      <c r="Y34" s="2" t="inlineStr"/>
+      <c r="Z34" s="2" t="inlineStr">
+        <is>
+          <t>https://pamatas.lt/</t>
+        </is>
+      </c>
+      <c r="AA34" s="2" t="inlineStr">
+        <is>
+          <t>Koordinatė nustatyta pagal vietovę; reikia patikslinti tikslų gamybos tašką.</t>
+        </is>
+      </c>
+      <c r="AB34" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>vilniaus-betono-gaminiai-vilnius</t>
+        </is>
+      </c>
+      <c r="B35" s="2" t="inlineStr"/>
+      <c r="C35" s="2" t="inlineStr">
+        <is>
+          <t>UAB Vilniaus betono gaminiai</t>
+        </is>
+      </c>
+      <c r="D35" s="2" t="inlineStr">
+        <is>
+          <t>HAUS / Vilniaus betono gaminiai</t>
+        </is>
+      </c>
+      <c r="E35" s="2" t="inlineStr">
+        <is>
+          <t>Papildomai rasta</t>
+        </is>
+      </c>
+      <c r="F35" s="2" t="inlineStr">
+        <is>
+          <t>Vilnius</t>
+        </is>
+      </c>
+      <c r="G35" s="2" t="inlineStr">
+        <is>
+          <t>Vilniaus m. sav.</t>
+        </is>
+      </c>
+      <c r="H35" s="2" t="inlineStr">
+        <is>
+          <t>A. Jakšto g. 5, Vilnius</t>
+        </is>
+      </c>
+      <c r="I35" s="3" t="n">
+        <v>54.6898036</v>
+      </c>
+      <c r="J35" s="3" t="n">
+        <v>25.2794289</v>
+      </c>
+      <c r="K35" s="2" t="inlineStr">
+        <is>
+          <t>precast_concrete</t>
+        </is>
+      </c>
+      <c r="L35" s="2" t="inlineStr">
+        <is>
+          <t>Betono gaminiai</t>
+        </is>
+      </c>
+      <c r="M35" s="2" t="inlineStr">
+        <is>
+          <t>Vilniaus betono gaminiai</t>
+        </is>
+      </c>
+      <c r="N35" s="2" t="inlineStr"/>
+      <c r="O35" s="2" t="inlineStr">
+        <is>
+          <t>Viešai skelbiamas HAUS blokelių ir betono gaminių gamintojas.</t>
+        </is>
+      </c>
+      <c r="P35" s="4" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="Q35" s="5" t="n"/>
+      <c r="R35" s="5" t="n"/>
+      <c r="S35" s="5" t="n"/>
+      <c r="T35" s="5" t="n"/>
+      <c r="U35" s="2" t="inlineStr">
+        <is>
+          <t>https://www.vbg.lt/</t>
+        </is>
+      </c>
+      <c r="V35" s="2" t="inlineStr">
+        <is>
+          <t>https://www.vbg.lt/</t>
+        </is>
+      </c>
+      <c r="W35" s="2" t="inlineStr"/>
+      <c r="X35" s="2" t="inlineStr"/>
+      <c r="Y35" s="2" t="inlineStr"/>
+      <c r="Z35" s="2" t="inlineStr">
+        <is>
+          <t>https://www.vbg.lt/</t>
+        </is>
+      </c>
+      <c r="AA35" s="2" t="inlineStr">
+        <is>
+          <t>Žemėlapyje naudotas viešai skelbiamas įmonės adresas; gamybos vietą reikia patikslinti.</t>
+        </is>
+      </c>
+      <c r="AB35" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>pamario-grupe-kalnuvenai</t>
+        </is>
+      </c>
+      <c r="B36" s="2" t="inlineStr"/>
+      <c r="C36" s="2" t="inlineStr">
+        <is>
+          <t>UAB Pamario grupė</t>
+        </is>
+      </c>
+      <c r="D36" s="2" t="inlineStr">
+        <is>
+          <t>Pamario grupė</t>
+        </is>
+      </c>
+      <c r="E36" s="2" t="inlineStr">
+        <is>
+          <t>Papildomai rasta</t>
+        </is>
+      </c>
+      <c r="F36" s="2" t="inlineStr">
+        <is>
+          <t>Kalnuvėnai</t>
+        </is>
+      </c>
+      <c r="G36" s="2" t="inlineStr">
+        <is>
+          <t>Klaipėdos r. sav.</t>
+        </is>
+      </c>
+      <c r="H36" s="2" t="inlineStr">
+        <is>
+          <t>Kaukėnų g. 12, Kalnuvėnai, Klaipėdos r.</t>
+        </is>
+      </c>
+      <c r="I36" s="3" t="n">
+        <v>55.7959735</v>
+      </c>
+      <c r="J36" s="3" t="n">
+        <v>21.1602296</v>
+      </c>
+      <c r="K36" s="2" t="inlineStr">
+        <is>
+          <t>ready_mix_concrete</t>
+        </is>
+      </c>
+      <c r="L36" s="2" t="inlineStr">
+        <is>
+          <t>Betono mišiniai</t>
+        </is>
+      </c>
+      <c r="M36" s="2" t="inlineStr">
+        <is>
+          <t>Pamario grupės betono mazgas</t>
+        </is>
+      </c>
+      <c r="N36" s="2" t="inlineStr"/>
+      <c r="O36" s="2" t="inlineStr">
+        <is>
+          <t>Viešai skelbiama betono mišinių veikla Klaipėdos rajone.</t>
+        </is>
+      </c>
+      <c r="P36" s="4" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="Q36" s="5" t="n"/>
+      <c r="R36" s="5" t="n"/>
+      <c r="S36" s="5" t="n"/>
+      <c r="T36" s="5" t="n"/>
+      <c r="U36" s="2" t="inlineStr">
+        <is>
+          <t>https://pamariogrupe.lt/</t>
+        </is>
+      </c>
+      <c r="V36" s="2" t="inlineStr">
+        <is>
+          <t>https://pamariogrupe.lt/</t>
+        </is>
+      </c>
+      <c r="W36" s="2" t="inlineStr"/>
+      <c r="X36" s="2" t="inlineStr"/>
+      <c r="Y36" s="2" t="inlineStr"/>
+      <c r="Z36" s="2" t="inlineStr">
+        <is>
+          <t>https://pamariogrupe.lt/</t>
+        </is>
+      </c>
+      <c r="AA36" s="2" t="inlineStr">
+        <is>
+          <t>Reikia patikslinti našumą ir gamybos režimą.</t>
+        </is>
+      </c>
+      <c r="AB36" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="inlineStr">
+        <is>
+          <t>betono-zona-klaipeda</t>
+        </is>
+      </c>
+      <c r="B37" s="2" t="inlineStr"/>
+      <c r="C37" s="2" t="inlineStr">
+        <is>
+          <t>UAB Betono zona</t>
+        </is>
+      </c>
+      <c r="D37" s="2" t="inlineStr">
+        <is>
+          <t>Betono zona</t>
+        </is>
+      </c>
+      <c r="E37" s="2" t="inlineStr">
+        <is>
+          <t>Papildomai rasta</t>
+        </is>
+      </c>
+      <c r="F37" s="2" t="inlineStr">
+        <is>
+          <t>Klaipėda</t>
+        </is>
+      </c>
+      <c r="G37" s="2" t="inlineStr">
+        <is>
+          <t>Klaipėdos m. sav.</t>
+        </is>
+      </c>
+      <c r="H37" s="2" t="inlineStr">
+        <is>
+          <t>Dvaro g. 6, Klaipėda</t>
+        </is>
+      </c>
+      <c r="I37" s="3" t="n">
+        <v>55.7550013</v>
+      </c>
+      <c r="J37" s="3" t="n">
+        <v>21.150534</v>
+      </c>
+      <c r="K37" s="2" t="inlineStr">
+        <is>
+          <t>precast_concrete</t>
+        </is>
+      </c>
+      <c r="L37" s="2" t="inlineStr">
+        <is>
+          <t>Betono gaminiai</t>
+        </is>
+      </c>
+      <c r="M37" s="2" t="inlineStr">
+        <is>
+          <t>Betono zona</t>
+        </is>
+      </c>
+      <c r="N37" s="2" t="inlineStr"/>
+      <c r="O37" s="2" t="inlineStr">
+        <is>
+          <t>Viešai skelbiama betono gaminių veikla Klaipėdoje.</t>
+        </is>
+      </c>
+      <c r="P37" s="4" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="Q37" s="5" t="n"/>
+      <c r="R37" s="5" t="n"/>
+      <c r="S37" s="5" t="n"/>
+      <c r="T37" s="5" t="n"/>
+      <c r="U37" s="2" t="inlineStr">
+        <is>
+          <t>https://betonozona.lt/</t>
+        </is>
+      </c>
+      <c r="V37" s="2" t="inlineStr">
+        <is>
+          <t>https://betonozona.lt/</t>
+        </is>
+      </c>
+      <c r="W37" s="2" t="inlineStr"/>
+      <c r="X37" s="2" t="inlineStr"/>
+      <c r="Y37" s="2" t="inlineStr"/>
+      <c r="Z37" s="2" t="inlineStr">
+        <is>
+          <t>https://betonozona.lt/</t>
+        </is>
+      </c>
+      <c r="AA37" s="2" t="inlineStr">
+        <is>
+          <t>Patikrinti, ar įmonė pati gamina, ar tik prekiauja betono gaminiais.</t>
+        </is>
+      </c>
+      <c r="AB37" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t>topbeton-panevezys</t>
+        </is>
+      </c>
+      <c r="B38" s="2" t="inlineStr"/>
+      <c r="C38" s="2" t="inlineStr">
+        <is>
+          <t>UAB Topbeton</t>
+        </is>
+      </c>
+      <c r="D38" s="2" t="inlineStr">
+        <is>
+          <t>Topbeton</t>
+        </is>
+      </c>
+      <c r="E38" s="2" t="inlineStr">
+        <is>
+          <t>Papildomai rasta</t>
+        </is>
+      </c>
+      <c r="F38" s="2" t="inlineStr">
+        <is>
+          <t>Panevėžys</t>
+        </is>
+      </c>
+      <c r="G38" s="2" t="inlineStr">
+        <is>
+          <t>Panevėžio m. sav.</t>
+        </is>
+      </c>
+      <c r="H38" s="2" t="inlineStr">
+        <is>
+          <t>Beržų g. 5C, Panevėžys</t>
+        </is>
+      </c>
+      <c r="I38" s="3" t="n">
+        <v>55.7168558</v>
+      </c>
+      <c r="J38" s="3" t="n">
+        <v>24.3617729</v>
+      </c>
+      <c r="K38" s="2" t="inlineStr">
+        <is>
+          <t>ready_mix_concrete</t>
+        </is>
+      </c>
+      <c r="L38" s="2" t="inlineStr">
+        <is>
+          <t>Betono mišiniai</t>
+        </is>
+      </c>
+      <c r="M38" s="2" t="inlineStr">
+        <is>
+          <t>Topbeton betono mazgas</t>
+        </is>
+      </c>
+      <c r="N38" s="2" t="inlineStr"/>
+      <c r="O38" s="2" t="inlineStr">
+        <is>
+          <t>Viešai skelbiama betono mišinių gamyba Panevėžyje.</t>
+        </is>
+      </c>
+      <c r="P38" s="4" t="n">
+        <v>0.78</v>
+      </c>
+      <c r="Q38" s="5" t="n"/>
+      <c r="R38" s="5" t="n"/>
+      <c r="S38" s="5" t="n"/>
+      <c r="T38" s="5" t="n"/>
+      <c r="U38" s="2" t="inlineStr">
+        <is>
+          <t>https://topbeton.lt/</t>
+        </is>
+      </c>
+      <c r="V38" s="2" t="inlineStr">
+        <is>
+          <t>https://topbeton.lt/</t>
+        </is>
+      </c>
+      <c r="W38" s="2" t="inlineStr"/>
+      <c r="X38" s="2" t="inlineStr"/>
+      <c r="Y38" s="2" t="inlineStr"/>
+      <c r="Z38" s="2" t="inlineStr">
+        <is>
+          <t>https://topbeton.lt/</t>
+        </is>
+      </c>
+      <c r="AA38" s="2" t="inlineStr">
+        <is>
+          <t>Papildomai rasta pagal prekinio betono požymį.</t>
+        </is>
+      </c>
+      <c r="AB38" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="inlineStr">
+        <is>
+          <t>gelzbetonio-gamyba-panevezys</t>
+        </is>
+      </c>
+      <c r="B39" s="2" t="inlineStr"/>
+      <c r="C39" s="2" t="inlineStr">
+        <is>
+          <t>MB Gelžbetonio gamyba</t>
+        </is>
+      </c>
+      <c r="D39" s="2" t="inlineStr">
+        <is>
+          <t>Gelžbetonio gamyba</t>
+        </is>
+      </c>
+      <c r="E39" s="2" t="inlineStr">
+        <is>
+          <t>Papildomai rasta</t>
+        </is>
+      </c>
+      <c r="F39" s="2" t="inlineStr">
+        <is>
+          <t>Panevėžys</t>
+        </is>
+      </c>
+      <c r="G39" s="2" t="inlineStr">
+        <is>
+          <t>Panevėžio m. sav.</t>
+        </is>
+      </c>
+      <c r="H39" s="2" t="inlineStr">
+        <is>
+          <t>S. Kerbedžio g. 52, Panevėžys</t>
+        </is>
+      </c>
+      <c r="I39" s="3" t="n">
+        <v>55.7409599</v>
+      </c>
+      <c r="J39" s="3" t="n">
+        <v>24.3802782</v>
+      </c>
+      <c r="K39" s="2" t="inlineStr">
+        <is>
+          <t>precast_concrete</t>
+        </is>
+      </c>
+      <c r="L39" s="2" t="inlineStr">
+        <is>
+          <t>Gelžbetonis</t>
+        </is>
+      </c>
+      <c r="M39" s="2" t="inlineStr">
+        <is>
+          <t>Gelžbetonio gamyba Panevėžyje</t>
+        </is>
+      </c>
+      <c r="N39" s="2" t="inlineStr"/>
+      <c r="O39" s="2" t="inlineStr">
+        <is>
+          <t>Viešai skelbiama gelžbetonio gaminių gamyba Panevėžyje.</t>
+        </is>
+      </c>
+      <c r="P39" s="4" t="n">
+        <v>0.72</v>
+      </c>
+      <c r="Q39" s="5" t="n"/>
+      <c r="R39" s="5" t="n"/>
+      <c r="S39" s="5" t="n"/>
+      <c r="T39" s="5" t="n"/>
+      <c r="U39" s="2" t="inlineStr">
+        <is>
+          <t>https://gelzbetoniogamyba.lt/</t>
+        </is>
+      </c>
+      <c r="V39" s="2" t="inlineStr">
+        <is>
+          <t>https://gelzbetoniogamyba.lt/</t>
+        </is>
+      </c>
+      <c r="W39" s="2" t="inlineStr"/>
+      <c r="X39" s="2" t="inlineStr"/>
+      <c r="Y39" s="2" t="inlineStr"/>
+      <c r="Z39" s="2" t="inlineStr">
+        <is>
+          <t>https://gelzbetoniogamyba.lt/</t>
+        </is>
+      </c>
+      <c r="AA39" s="2" t="inlineStr">
+        <is>
+          <t>Reikia patikslinti ryšį su kitomis S. Kerbedžio g. 52 įmonėmis.</t>
+        </is>
+      </c>
+      <c r="AB39" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="inlineStr">
+        <is>
+          <t>inroma-pakruojis</t>
+        </is>
+      </c>
+      <c r="B40" s="2" t="inlineStr"/>
+      <c r="C40" s="2" t="inlineStr">
+        <is>
+          <t>UAB Inroma</t>
+        </is>
+      </c>
+      <c r="D40" s="2" t="inlineStr">
+        <is>
+          <t>Inroma</t>
+        </is>
+      </c>
+      <c r="E40" s="2" t="inlineStr">
+        <is>
+          <t>Papildomai rasta</t>
+        </is>
+      </c>
+      <c r="F40" s="2" t="inlineStr">
+        <is>
+          <t>Pakruojis</t>
+        </is>
+      </c>
+      <c r="G40" s="2" t="inlineStr">
+        <is>
+          <t>Pakruojo r. sav.</t>
+        </is>
+      </c>
+      <c r="H40" s="2" t="inlineStr">
+        <is>
+          <t>Pramonės g. 5B, Pakruojis</t>
+        </is>
+      </c>
+      <c r="I40" s="3" t="n">
+        <v>55.9763263</v>
+      </c>
+      <c r="J40" s="3" t="n">
+        <v>23.8584712</v>
+      </c>
+      <c r="K40" s="2" t="inlineStr">
+        <is>
+          <t>ready_mix_concrete</t>
+        </is>
+      </c>
+      <c r="L40" s="2" t="inlineStr">
+        <is>
+          <t>Betono mišiniai</t>
+        </is>
+      </c>
+      <c r="M40" s="2" t="inlineStr">
+        <is>
+          <t>Inroma betono mazgas</t>
+        </is>
+      </c>
+      <c r="N40" s="2" t="inlineStr"/>
+      <c r="O40" s="2" t="inlineStr">
+        <is>
+          <t>Viešai skelbiama betono mišinių veikla Pakruojyje.</t>
+        </is>
+      </c>
+      <c r="P40" s="4" t="n">
+        <v>0.72</v>
+      </c>
+      <c r="Q40" s="5" t="n"/>
+      <c r="R40" s="5" t="n"/>
+      <c r="S40" s="5" t="n"/>
+      <c r="T40" s="5" t="n"/>
+      <c r="U40" s="2" t="inlineStr">
+        <is>
+          <t>https://inroma.lt/</t>
+        </is>
+      </c>
+      <c r="V40" s="2" t="inlineStr">
+        <is>
+          <t>https://inroma.lt/</t>
+        </is>
+      </c>
+      <c r="W40" s="2" t="inlineStr"/>
+      <c r="X40" s="2" t="inlineStr"/>
+      <c r="Y40" s="2" t="inlineStr"/>
+      <c r="Z40" s="2" t="inlineStr">
+        <is>
+          <t>https://inroma.lt/</t>
+        </is>
+      </c>
+      <c r="AA40" s="2" t="inlineStr">
+        <is>
+          <t>Reikia patikslinti našumą.</t>
+        </is>
+      </c>
+      <c r="AB40" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="2" t="inlineStr">
+        <is>
+          <t>seldra-vilnius</t>
+        </is>
+      </c>
+      <c r="B41" s="2" t="inlineStr"/>
+      <c r="C41" s="2" t="inlineStr">
+        <is>
+          <t>UAB Seldra</t>
+        </is>
+      </c>
+      <c r="D41" s="2" t="inlineStr">
+        <is>
+          <t>Seldra</t>
+        </is>
+      </c>
+      <c r="E41" s="2" t="inlineStr">
+        <is>
+          <t>Papildomai rasta</t>
+        </is>
+      </c>
+      <c r="F41" s="2" t="inlineStr">
+        <is>
+          <t>Vilnius</t>
+        </is>
+      </c>
+      <c r="G41" s="2" t="inlineStr">
+        <is>
+          <t>Vilniaus m. sav.</t>
+        </is>
+      </c>
+      <c r="H41" s="2" t="inlineStr">
+        <is>
+          <t>O. Miciūtės g. 7, Vilnius</t>
+        </is>
+      </c>
+      <c r="I41" s="3" t="n">
+        <v>54.7373</v>
+      </c>
+      <c r="J41" s="3" t="n">
+        <v>25.2277</v>
+      </c>
+      <c r="K41" s="2" t="inlineStr">
+        <is>
+          <t>ready_mix_concrete</t>
+        </is>
+      </c>
+      <c r="L41" s="2" t="inlineStr">
+        <is>
+          <t>Betono mišiniai</t>
+        </is>
+      </c>
+      <c r="M41" s="2" t="inlineStr">
+        <is>
+          <t>Seldra prekinio betono gamyba</t>
+        </is>
+      </c>
+      <c r="N41" s="2" t="inlineStr"/>
+      <c r="O41" s="2" t="inlineStr">
+        <is>
+          <t>Viešame kataloge nurodoma prekinio betono gamyba ir prekyba Vilniuje.</t>
+        </is>
+      </c>
+      <c r="P41" s="4" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="Q41" s="5" t="n"/>
+      <c r="R41" s="5" t="n"/>
+      <c r="S41" s="5" t="n"/>
+      <c r="T41" s="5" t="n"/>
+      <c r="U41" s="2" t="inlineStr"/>
+      <c r="V41" s="2" t="inlineStr">
+        <is>
+          <t>https://www.1551.lt/seldra-uab-prekinio-betono-gamyba-ir-prekyba-vilniuje-219193/</t>
+        </is>
+      </c>
+      <c r="W41" s="2" t="inlineStr"/>
+      <c r="X41" s="2" t="inlineStr"/>
+      <c r="Y41" s="2" t="inlineStr"/>
+      <c r="Z41" s="2" t="inlineStr">
+        <is>
+          <t>https://www.1551.lt/seldra-uab-prekinio-betono-gamyba-ir-prekyba-vilniuje-219193/</t>
+        </is>
+      </c>
+      <c r="AA41" s="2" t="inlineStr">
+        <is>
+          <t>Koordinatė apytikslė pagal adresą; reikia patikslinti gamybos tašką.</t>
+        </is>
+      </c>
+      <c r="AB41" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="2" t="inlineStr">
+        <is>
+          <t>utenos-betonas-utena</t>
+        </is>
+      </c>
+      <c r="B42" s="2" t="inlineStr"/>
+      <c r="C42" s="2" t="inlineStr">
+        <is>
+          <t>UAB Utenos betonas</t>
+        </is>
+      </c>
+      <c r="D42" s="2" t="inlineStr">
+        <is>
+          <t>Utenos betonas</t>
+        </is>
+      </c>
+      <c r="E42" s="2" t="inlineStr">
+        <is>
+          <t>Papildomai rasta</t>
+        </is>
+      </c>
+      <c r="F42" s="2" t="inlineStr">
+        <is>
+          <t>Utena</t>
+        </is>
+      </c>
+      <c r="G42" s="2" t="inlineStr">
+        <is>
+          <t>Utenos r. sav.</t>
+        </is>
+      </c>
+      <c r="H42" s="2" t="inlineStr">
+        <is>
+          <t>Metalo g. 9B, Utena</t>
+        </is>
+      </c>
+      <c r="I42" s="3" t="n">
+        <v>55.4947626</v>
+      </c>
+      <c r="J42" s="3" t="n">
+        <v>25.6225137</v>
+      </c>
+      <c r="K42" s="2" t="inlineStr">
+        <is>
+          <t>ready_mix_concrete</t>
+        </is>
+      </c>
+      <c r="L42" s="2" t="inlineStr">
+        <is>
+          <t>Betono mišiniai</t>
+        </is>
+      </c>
+      <c r="M42" s="2" t="inlineStr">
+        <is>
+          <t>Utenos betono mazgas</t>
+        </is>
+      </c>
+      <c r="N42" s="2" t="inlineStr"/>
+      <c r="O42" s="2" t="inlineStr">
+        <is>
+          <t>Viešai skelbiama betono mišinių veikla Utenoje.</t>
+        </is>
+      </c>
+      <c r="P42" s="4" t="n">
+        <v>0.78</v>
+      </c>
+      <c r="Q42" s="5" t="n"/>
+      <c r="R42" s="5" t="n"/>
+      <c r="S42" s="5" t="n"/>
+      <c r="T42" s="5" t="n"/>
+      <c r="U42" s="2" t="inlineStr">
+        <is>
+          <t>https://utenosbetonas.lt/</t>
+        </is>
+      </c>
+      <c r="V42" s="2" t="inlineStr">
+        <is>
+          <t>https://utenosbetonas.lt/</t>
+        </is>
+      </c>
+      <c r="W42" s="2" t="inlineStr"/>
+      <c r="X42" s="2" t="inlineStr"/>
+      <c r="Y42" s="2" t="inlineStr"/>
+      <c r="Z42" s="2" t="inlineStr">
+        <is>
+          <t>https://utenosbetonas.lt/</t>
+        </is>
+      </c>
+      <c r="AA42" s="2" t="inlineStr">
+        <is>
+          <t>Reikia patikslinti našumą.</t>
+        </is>
+      </c>
+      <c r="AB42" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="2" t="inlineStr">
+        <is>
+          <t>sbetonas-jonava</t>
+        </is>
+      </c>
+      <c r="B43" s="2" t="inlineStr"/>
+      <c r="C43" s="2" t="inlineStr">
+        <is>
+          <t>UAB Sbetonas</t>
+        </is>
+      </c>
+      <c r="D43" s="2" t="inlineStr">
+        <is>
+          <t>Sbetonas</t>
+        </is>
+      </c>
+      <c r="E43" s="2" t="inlineStr">
+        <is>
+          <t>Papildomai rasta</t>
+        </is>
+      </c>
+      <c r="F43" s="2" t="inlineStr">
+        <is>
+          <t>Jonava</t>
+        </is>
+      </c>
+      <c r="G43" s="2" t="inlineStr">
+        <is>
+          <t>Jonavos r. sav.</t>
+        </is>
+      </c>
+      <c r="H43" s="2" t="inlineStr">
+        <is>
+          <t>Skarulių g. 58, Jonava</t>
+        </is>
+      </c>
+      <c r="I43" s="3" t="n">
+        <v>55.0781771</v>
+      </c>
+      <c r="J43" s="3" t="n">
+        <v>24.3203017</v>
+      </c>
+      <c r="K43" s="2" t="inlineStr">
+        <is>
+          <t>ready_mix_concrete</t>
+        </is>
+      </c>
+      <c r="L43" s="2" t="inlineStr">
+        <is>
+          <t>Betono mišiniai</t>
+        </is>
+      </c>
+      <c r="M43" s="2" t="inlineStr">
+        <is>
+          <t>Sbetonas betono mazgas</t>
+        </is>
+      </c>
+      <c r="N43" s="2" t="inlineStr"/>
+      <c r="O43" s="2" t="inlineStr">
+        <is>
+          <t>Viešai skelbiama prekinio betono gamyba Jonavoje.</t>
+        </is>
+      </c>
+      <c r="P43" s="4" t="n">
+        <v>0.78</v>
+      </c>
+      <c r="Q43" s="5" t="n"/>
+      <c r="R43" s="5" t="n"/>
+      <c r="S43" s="5" t="n"/>
+      <c r="T43" s="5" t="n"/>
+      <c r="U43" s="2" t="inlineStr">
+        <is>
+          <t>https://sbetonas.lt/</t>
+        </is>
+      </c>
+      <c r="V43" s="2" t="inlineStr">
+        <is>
+          <t>https://sbetonas.lt/</t>
+        </is>
+      </c>
+      <c r="W43" s="2" t="inlineStr"/>
+      <c r="X43" s="2" t="inlineStr"/>
+      <c r="Y43" s="2" t="inlineStr"/>
+      <c r="Z43" s="2" t="inlineStr">
+        <is>
+          <t>https://sbetonas.lt/</t>
+        </is>
+      </c>
+      <c r="AA43" s="2" t="inlineStr">
+        <is>
+          <t>Papildomai rasta pagal prekinio betono požymį.</t>
+        </is>
+      </c>
+      <c r="AB43" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="inlineStr">
+        <is>
+          <t>kalcitas-naujoji-akmene</t>
+        </is>
+      </c>
+      <c r="B44" s="2" t="inlineStr"/>
+      <c r="C44" s="2" t="inlineStr">
+        <is>
+          <t>AB Kalcitas</t>
+        </is>
+      </c>
+      <c r="D44" s="2" t="inlineStr">
+        <is>
+          <t>Kalcitas</t>
+        </is>
+      </c>
+      <c r="E44" s="2" t="inlineStr">
+        <is>
+          <t>Papildomai rasta</t>
+        </is>
+      </c>
+      <c r="F44" s="2" t="inlineStr">
+        <is>
+          <t>Naujoji Akmenė</t>
+        </is>
+      </c>
+      <c r="G44" s="2" t="inlineStr">
+        <is>
+          <t>Akmenės r. sav.</t>
+        </is>
+      </c>
+      <c r="H44" s="2" t="inlineStr">
+        <is>
+          <t>J. Dalinkevičiaus g. 2, Naujoji Akmenė</t>
+        </is>
+      </c>
+      <c r="I44" s="3" t="n">
+        <v>56.3155328</v>
+      </c>
+      <c r="J44" s="3" t="n">
+        <v>22.9143308</v>
+      </c>
+      <c r="K44" s="2" t="inlineStr">
+        <is>
+          <t>ready_mix_concrete</t>
+        </is>
+      </c>
+      <c r="L44" s="2" t="inlineStr">
+        <is>
+          <t>Betono mišiniai</t>
+        </is>
+      </c>
+      <c r="M44" s="2" t="inlineStr">
+        <is>
+          <t>Kalcitas betono mišinių gamybos linija</t>
+        </is>
+      </c>
+      <c r="N44" s="2" t="inlineStr"/>
+      <c r="O44" s="2" t="inlineStr">
+        <is>
+          <t>Viešame kataloge nurodomi betonas, betono mišiniai ir betono gamybos linija Naujojoje Akmenėje.</t>
+        </is>
+      </c>
+      <c r="P44" s="4" t="n">
+        <v>0.78</v>
+      </c>
+      <c r="Q44" s="5" t="n"/>
+      <c r="R44" s="5" t="n"/>
+      <c r="S44" s="5" t="n"/>
+      <c r="T44" s="5" t="n"/>
+      <c r="U44" s="2" t="inlineStr"/>
+      <c r="V44" s="2" t="inlineStr">
+        <is>
+          <t>https://www.1551.lt/kalcitas-ab-betonas-betono-misiniai-betono-gamybos-linija-technikos-nuoma-naujojoje-akmeneje-59982/</t>
+        </is>
+      </c>
+      <c r="W44" s="2" t="inlineStr"/>
+      <c r="X44" s="2" t="inlineStr"/>
+      <c r="Y44" s="2" t="inlineStr"/>
+      <c r="Z44" s="2" t="inlineStr">
+        <is>
+          <t>https://www.1551.lt/kalcitas-ab-betonas-betono-misiniai-betono-gamybos-linija-technikos-nuoma-naujojoje-akmeneje-59982/</t>
+        </is>
+      </c>
+      <c r="AA44" s="2" t="inlineStr">
+        <is>
+          <t>Reikia patikslinti, ar veikla yra nuolat aktyvi.</t>
+        </is>
+      </c>
+      <c r="AB44" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="2" t="inlineStr">
+        <is>
+          <t>gelgaudiskio-gelzbetonis-gelgaudiskis</t>
+        </is>
+      </c>
+      <c r="B45" s="2" t="inlineStr"/>
+      <c r="C45" s="2" t="inlineStr">
+        <is>
+          <t>UAB Gelgaudiškio gelžbetonis</t>
+        </is>
+      </c>
+      <c r="D45" s="2" t="inlineStr">
+        <is>
+          <t>Gelgaudiškio gelžbetonis</t>
+        </is>
+      </c>
+      <c r="E45" s="2" t="inlineStr">
+        <is>
+          <t>Papildomai rasta</t>
+        </is>
+      </c>
+      <c r="F45" s="2" t="inlineStr">
+        <is>
+          <t>Gelgaudiškis</t>
+        </is>
+      </c>
+      <c r="G45" s="2" t="inlineStr">
+        <is>
+          <t>Šakių r. sav.</t>
+        </is>
+      </c>
+      <c r="H45" s="2" t="inlineStr">
+        <is>
+          <t>Gelgaudi?kis, ?aki? r.</t>
+        </is>
+      </c>
+      <c r="I45" s="3" t="n">
+        <v>55.0786004</v>
+      </c>
+      <c r="J45" s="3" t="n">
+        <v>22.9754331</v>
+      </c>
+      <c r="K45" s="2" t="inlineStr">
+        <is>
+          <t>precast_concrete</t>
+        </is>
+      </c>
+      <c r="L45" s="2" t="inlineStr">
+        <is>
+          <t>Gelžbetonis</t>
+        </is>
+      </c>
+      <c r="M45" s="2" t="inlineStr">
+        <is>
+          <t>Gelgaudiškio gelžbetonio gamykla</t>
+        </is>
+      </c>
+      <c r="N45" s="2" t="inlineStr"/>
+      <c r="O45" s="2" t="inlineStr">
+        <is>
+          <t>Viešai skelbiami gelžbetonio gaminiai.</t>
+        </is>
+      </c>
+      <c r="P45" s="4" t="n">
+        <v>0.78</v>
+      </c>
+      <c r="Q45" s="5" t="n"/>
+      <c r="R45" s="5" t="n"/>
+      <c r="S45" s="5" t="n"/>
+      <c r="T45" s="5" t="n"/>
+      <c r="U45" s="2" t="inlineStr">
+        <is>
+          <t>https://glg.lt/</t>
+        </is>
+      </c>
+      <c r="V45" s="2" t="inlineStr">
+        <is>
+          <t>https://glg.lt/kontaktai/</t>
+        </is>
+      </c>
+      <c r="W45" s="2" t="inlineStr"/>
+      <c r="X45" s="2" t="inlineStr"/>
+      <c r="Y45" s="2" t="inlineStr"/>
+      <c r="Z45" s="2" t="inlineStr">
+        <is>
+          <t>https://glg.lt/kontaktai/</t>
+        </is>
+      </c>
+      <c r="AA45" s="2" t="inlineStr">
+        <is>
+          <t>Reikia patikslinti tikslų gamyklos adresą.</t>
+        </is>
+      </c>
+      <c r="AB45" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="2" t="inlineStr">
+        <is>
+          <t>sausta-trakai</t>
+        </is>
+      </c>
+      <c r="B46" s="2" t="inlineStr"/>
+      <c r="C46" s="2" t="inlineStr">
+        <is>
+          <t>UAB Sausta</t>
+        </is>
+      </c>
+      <c r="D46" s="2" t="inlineStr">
+        <is>
+          <t>Sausta</t>
+        </is>
+      </c>
+      <c r="E46" s="2" t="inlineStr">
+        <is>
+          <t>Papildomai rasta</t>
+        </is>
+      </c>
+      <c r="F46" s="2" t="inlineStr">
+        <is>
+          <t>Trakai</t>
+        </is>
+      </c>
+      <c r="G46" s="2" t="inlineStr">
+        <is>
+          <t>Trakų r. sav.</t>
+        </is>
+      </c>
+      <c r="H46" s="2" t="inlineStr">
+        <is>
+          <t>Karaimų g. 73, Trakai</t>
+        </is>
+      </c>
+      <c r="I46" s="3" t="n">
+        <v>54.6524792</v>
+      </c>
+      <c r="J46" s="3" t="n">
+        <v>24.9225479</v>
+      </c>
+      <c r="K46" s="2" t="inlineStr">
+        <is>
+          <t>ready_mix_concrete</t>
+        </is>
+      </c>
+      <c r="L46" s="2" t="inlineStr">
+        <is>
+          <t>Betono mišiniai</t>
+        </is>
+      </c>
+      <c r="M46" s="2" t="inlineStr">
+        <is>
+          <t>Sausta betono mišinių veikla</t>
+        </is>
+      </c>
+      <c r="N46" s="2" t="inlineStr"/>
+      <c r="O46" s="2" t="inlineStr">
+        <is>
+          <t>Viešame kataloge įmonė siejama su betono mišinių veikla.</t>
+        </is>
+      </c>
+      <c r="P46" s="4" t="n">
+        <v>0.62</v>
+      </c>
+      <c r="Q46" s="5" t="n"/>
+      <c r="R46" s="5" t="n"/>
+      <c r="S46" s="5" t="n"/>
+      <c r="T46" s="5" t="n"/>
+      <c r="U46" s="2" t="inlineStr"/>
+      <c r="V46" s="2" t="inlineStr">
+        <is>
+          <t>https://www.1551.lt/sausta-uab-240915/</t>
+        </is>
+      </c>
+      <c r="W46" s="2" t="inlineStr"/>
+      <c r="X46" s="2" t="inlineStr"/>
+      <c r="Y46" s="2" t="inlineStr"/>
+      <c r="Z46" s="2" t="inlineStr">
+        <is>
+          <t>https://www.1551.lt/sausta-uab-240915/</t>
+        </is>
+      </c>
+      <c r="AA46" s="2" t="inlineStr">
+        <is>
+          <t>Žemos pasitikėjimo įrašas; reikia patikslinti, ar gamyba vykdoma šiame taške.</t>
+        </is>
+      </c>
+      <c r="AB46" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:AB27"/>
+  <autoFilter ref="A1:AB46"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -3263,7 +5143,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-06-29T19:52:46.971317+00:00</t>
+          <t>2026-06-30T04:05:06.791114+00:00</t>
         </is>
       </c>
     </row>
@@ -3318,7 +5198,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-06-29T19:52:46.971317+00:00</t>
+          <t>2026-06-30T04:05:06.791114+00:00</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -3332,7 +5212,7 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>26</v>
+        <v>45</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Correct Betono centras Klaipeda location
</commit_message>
<xml_diff>
--- a/data/companies.xlsx
+++ b/data/companies.xlsx
@@ -895,14 +895,14 @@
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>Liepų g. 85, Klaipėda</t>
+          <t>Liepų g. 87N, Klaipėda</t>
         </is>
       </c>
       <c r="I4" s="3" t="n">
-        <v>55.7255212</v>
+        <v>55.7292816</v>
       </c>
       <c r="J4" s="3" t="n">
-        <v>21.159293</v>
+        <v>21.1540759</v>
       </c>
       <c r="K4" s="2" t="inlineStr">
         <is>
@@ -939,7 +939,7 @@
       </c>
       <c r="V4" s="2" t="inlineStr">
         <is>
-          <t>https://betonocentras.lt/kontaktai/</t>
+          <t>https://spsc.lt/registrai/regsapp/ser_produktai_view.php?editid1=13020</t>
         </is>
       </c>
       <c r="W4" s="2" t="inlineStr"/>
@@ -947,13 +947,17 @@
       <c r="Y4" s="2" t="inlineStr"/>
       <c r="Z4" s="2" t="inlineStr">
         <is>
-          <t>https://betonocentras.lt/kontaktai/</t>
-        </is>
-      </c>
-      <c r="AA4" s="2" t="inlineStr"/>
+          <t>https://spsc.lt/registrai/regsapp/ser_produktai_view.php?editid1=13020</t>
+        </is>
+      </c>
+      <c r="AA4" s="2" t="inlineStr">
+        <is>
+          <t>Adresas ir koordinatės patikslinti pagal Google Maps ir SPSC registro įrašą.</t>
+        </is>
+      </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
     </row>
@@ -5143,7 +5147,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-06-30T04:05:06.791114+00:00</t>
+          <t>2026-06-30T04:22:16.649112+00:00</t>
         </is>
       </c>
     </row>
@@ -5198,7 +5202,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-06-30T04:05:06.791114+00:00</t>
+          <t>2026-06-30T04:22:16.650112+00:00</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">

</xml_diff>

<commit_message>
Add EVRK 236300 concrete producers
</commit_message>
<xml_diff>
--- a/data/companies.xlsx
+++ b/data/companies.xlsx
@@ -12,7 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Importo žurnalas" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Įmonės'!$A$1:$AB$46</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Įmonės'!$A$1:$AB$59</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -169,8 +169,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ImonesTable" displayName="ImonesTable" ref="A1:AB46" headerRowCount="1">
-  <autoFilter ref="A1:AB46"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ImonesTable" displayName="ImonesTable" ref="A1:AB59" headerRowCount="1">
+  <autoFilter ref="A1:AB59"/>
   <tableColumns count="28">
     <tableColumn id="1" name="Įrašo ID"/>
     <tableColumn id="2" name="Įmonės kodas"/>
@@ -494,16 +494,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AB46"/>
+  <dimension ref="A1:AB59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="39" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
     <col width="42" customWidth="1" min="3" max="3"/>
     <col width="33" customWidth="1" min="4" max="4"/>
-    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="29" customWidth="1" min="5" max="5"/>
     <col width="16" customWidth="1" min="6" max="6"/>
-    <col width="19" customWidth="1" min="7" max="7"/>
+    <col width="21" customWidth="1" min="7" max="7"/>
     <col width="42" customWidth="1" min="8" max="8"/>
     <col width="12" customWidth="1" min="9" max="9"/>
     <col width="12" customWidth="1" min="10" max="10"/>
@@ -675,7 +675,11 @@
           <t>betono-centras-vilnius</t>
         </is>
       </c>
-      <c r="B2" s="2" t="inlineStr"/>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>123018186</t>
+        </is>
+      </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
           <t>UAB Betono centras</t>
@@ -771,7 +775,11 @@
           <t>betono-centras-kaunas</t>
         </is>
       </c>
-      <c r="B3" s="2" t="inlineStr"/>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>123018186</t>
+        </is>
+      </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
           <t>UAB Betono centras</t>
@@ -867,7 +875,11 @@
           <t>betono-centras-klaipeda</t>
         </is>
       </c>
-      <c r="B4" s="2" t="inlineStr"/>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>123018186</t>
+        </is>
+      </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
           <t>UAB Betono centras</t>
@@ -967,7 +979,11 @@
           <t>betono-centras-siauliai</t>
         </is>
       </c>
-      <c r="B5" s="2" t="inlineStr"/>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>123018186</t>
+        </is>
+      </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
           <t>UAB Betono centras</t>
@@ -1063,7 +1079,11 @@
           <t>betono-centras-mazeikiai</t>
         </is>
       </c>
-      <c r="B6" s="2" t="inlineStr"/>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>123018186</t>
+        </is>
+      </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
           <t>UAB Betono centras</t>
@@ -1159,7 +1179,11 @@
           <t>betono-centras-panevezys</t>
         </is>
       </c>
-      <c r="B7" s="2" t="inlineStr"/>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>123018186</t>
+        </is>
+      </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
           <t>UAB Betono centras</t>
@@ -1255,7 +1279,11 @@
           <t>heidelberg-vilnius-siaures</t>
         </is>
       </c>
-      <c r="B8" s="2" t="inlineStr"/>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>304102190</t>
+        </is>
+      </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
           <t>UAB Heidelberg Materials Lietuva Betonas</t>
@@ -1351,7 +1379,11 @@
           <t>heidelberg-vilnius-sandeliu</t>
         </is>
       </c>
-      <c r="B9" s="2" t="inlineStr"/>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>304102190</t>
+        </is>
+      </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
           <t>UAB Heidelberg Materials Lietuva Betonas</t>
@@ -1447,7 +1479,11 @@
           <t>heidelberg-kaunas</t>
         </is>
       </c>
-      <c r="B10" s="2" t="inlineStr"/>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>304102190</t>
+        </is>
+      </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
           <t>UAB Heidelberg Materials Lietuva Betonas</t>
@@ -1543,7 +1579,11 @@
           <t>heidelberg-klaipeda</t>
         </is>
       </c>
-      <c r="B11" s="2" t="inlineStr"/>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>304102190</t>
+        </is>
+      </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
           <t>UAB Heidelberg Materials Lietuva Betonas</t>
@@ -1639,7 +1679,11 @@
           <t>heidelberg-alytus</t>
         </is>
       </c>
-      <c r="B12" s="2" t="inlineStr"/>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>304102190</t>
+        </is>
+      </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
           <t>UAB Heidelberg Materials Lietuva Betonas</t>
@@ -1735,7 +1779,11 @@
           <t>heidelberg-pasvalys</t>
         </is>
       </c>
-      <c r="B13" s="2" t="inlineStr"/>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>304102190</t>
+        </is>
+      </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
           <t>UAB Heidelberg Materials Lietuva Betonas</t>
@@ -1831,7 +1879,11 @@
           <t>palmusta-vilnius</t>
         </is>
       </c>
-      <c r="B14" s="2" t="inlineStr"/>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>122619426</t>
+        </is>
+      </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
           <t>UAB Palmusta</t>
@@ -2791,7 +2843,11 @@
           <t>statkasta-kaunas</t>
         </is>
       </c>
-      <c r="B24" s="2" t="inlineStr"/>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>185607978</t>
+        </is>
+      </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
           <t>UAB Statkasta</t>
@@ -2983,7 +3039,11 @@
           <t>betono-baze-visaginas</t>
         </is>
       </c>
-      <c r="B26" s="2" t="inlineStr"/>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>302725961</t>
+        </is>
+      </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
           <t>UAB Betono bazė</t>
@@ -3283,7 +3343,11 @@
           <t>alytaus-gelzbetonis-alytus</t>
         </is>
       </c>
-      <c r="B29" s="2" t="inlineStr"/>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>149720232</t>
+        </is>
+      </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
           <t>AB Alytaus gelžbetonis</t>
@@ -3322,12 +3386,12 @@
       </c>
       <c r="K29" s="2" t="inlineStr">
         <is>
-          <t>precast_concrete</t>
+          <t>ready_mix_concrete</t>
         </is>
       </c>
       <c r="L29" s="2" t="inlineStr">
         <is>
-          <t>Betono gaminiai</t>
+          <t>Betono mišiniai</t>
         </is>
       </c>
       <c r="M29" s="2" t="inlineStr">
@@ -3338,7 +3402,7 @@
       <c r="N29" s="2" t="inlineStr"/>
       <c r="O29" s="2" t="inlineStr">
         <is>
-          <t>Viešai skelbiami betono ir gelžbetonio gaminiai Alytuje.</t>
+          <t>Registrų centro/VDA atviruose duomenyse pagrindinė veikla nurodyta kaip prekinio betono mišinio gamyba (EVRK 23.63).</t>
         </is>
       </c>
       <c r="P29" s="4" t="n">
@@ -3355,7 +3419,7 @@
       </c>
       <c r="V29" s="2" t="inlineStr">
         <is>
-          <t>https://alytausgelzbetonis.lt/kontaktai/</t>
+          <t>https://data.gov.lt/dataset/juridiniu-asmenu-ekonomines-veiklos-rusys-ir-instituciniai-sektoriai/</t>
         </is>
       </c>
       <c r="W29" s="2" t="inlineStr"/>
@@ -3368,7 +3432,7 @@
       </c>
       <c r="AA29" s="2" t="inlineStr">
         <is>
-          <t>Anksčiau ieškota pagal Presbetonas / Alytaus gelžbetonis požymius.</t>
+          <t>Įmonė jau buvo sąraše kaip gelžbetonio gamintoja; veikla patikslinta pagal EVRK 23.63 atvirų duomenų sąrašą.</t>
         </is>
       </c>
       <c r="AB29" s="2" t="inlineStr">
@@ -3511,7 +3575,7 @@
       </c>
       <c r="H31" s="2" t="inlineStr">
         <is>
-          <t>Tiek?j? g. 27B, Kretinga</t>
+          <t>Tiekėjų g. 27B, Kretinga</t>
         </is>
       </c>
       <c r="I31" s="3" t="n">
@@ -3532,7 +3596,7 @@
       </c>
       <c r="M31" s="2" t="inlineStr">
         <is>
-          <t>RE Betono konstrukcij? gamyba</t>
+          <t>RE Betono konstrukcijų gamyba</t>
         </is>
       </c>
       <c r="N31" s="2" t="inlineStr"/>
@@ -3824,7 +3888,7 @@
       </c>
       <c r="M34" s="2" t="inlineStr">
         <is>
-          <t>Pamatas betono gamini? gamyba</t>
+          <t>Pamatas betono gaminių gamyba</t>
         </is>
       </c>
       <c r="N34" s="2" t="inlineStr"/>
@@ -4175,7 +4239,11 @@
           <t>topbeton-panevezys</t>
         </is>
       </c>
-      <c r="B38" s="2" t="inlineStr"/>
+      <c r="B38" s="2" t="inlineStr">
+        <is>
+          <t>307083610</t>
+        </is>
+      </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
           <t>UAB Topbeton</t>
@@ -4571,7 +4639,11 @@
           <t>utenos-betonas-utena</t>
         </is>
       </c>
-      <c r="B42" s="2" t="inlineStr"/>
+      <c r="B42" s="2" t="inlineStr">
+        <is>
+          <t>300904691</t>
+        </is>
+      </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
           <t>UAB Utenos betonas</t>
@@ -4671,7 +4743,11 @@
           <t>sbetonas-jonava</t>
         </is>
       </c>
-      <c r="B43" s="2" t="inlineStr"/>
+      <c r="B43" s="2" t="inlineStr">
+        <is>
+          <t>300902683</t>
+        </is>
+      </c>
       <c r="C43" s="2" t="inlineStr">
         <is>
           <t>UAB Sbetonas</t>
@@ -4895,7 +4971,7 @@
       </c>
       <c r="H45" s="2" t="inlineStr">
         <is>
-          <t>Gelgaudi?kis, ?aki? r.</t>
+          <t>Nemuno g. 1, Gelgaudiškis</t>
         </is>
       </c>
       <c r="I45" s="3" t="n">
@@ -4967,7 +5043,11 @@
           <t>sausta-trakai</t>
         </is>
       </c>
-      <c r="B46" s="2" t="inlineStr"/>
+      <c r="B46" s="2" t="inlineStr">
+        <is>
+          <t>145744638</t>
+        </is>
+      </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
           <t>UAB Sausta</t>
@@ -5057,8 +5137,1264 @@
         </is>
       </c>
     </row>
+    <row r="47">
+      <c r="A47" s="2" t="inlineStr">
+        <is>
+          <t>ginfa-kutiskiai</t>
+        </is>
+      </c>
+      <c r="B47" s="2" t="inlineStr">
+        <is>
+          <t>302680943</t>
+        </is>
+      </c>
+      <c r="C47" s="2" t="inlineStr">
+        <is>
+          <t>UAB GinFa</t>
+        </is>
+      </c>
+      <c r="D47" s="2" t="inlineStr">
+        <is>
+          <t>GinFa</t>
+        </is>
+      </c>
+      <c r="E47" s="2" t="inlineStr">
+        <is>
+          <t>Papildomai rasta EVRK 23.63</t>
+        </is>
+      </c>
+      <c r="F47" s="2" t="inlineStr">
+        <is>
+          <t>Kutiškiai</t>
+        </is>
+      </c>
+      <c r="G47" s="2" t="inlineStr">
+        <is>
+          <t>Radviliškio r. sav.</t>
+        </is>
+      </c>
+      <c r="H47" s="2" t="inlineStr">
+        <is>
+          <t>Alyvų g. 8, Kutiškiai, Radviliškio r.</t>
+        </is>
+      </c>
+      <c r="I47" s="3" t="n">
+        <v>55.8327846</v>
+      </c>
+      <c r="J47" s="3" t="n">
+        <v>23.499724</v>
+      </c>
+      <c r="K47" s="2" t="inlineStr">
+        <is>
+          <t>ready_mix_concrete</t>
+        </is>
+      </c>
+      <c r="L47" s="2" t="inlineStr">
+        <is>
+          <t>Betono mišiniai</t>
+        </is>
+      </c>
+      <c r="M47" s="2" t="inlineStr">
+        <is>
+          <t>GinFa betono gamyba</t>
+        </is>
+      </c>
+      <c r="N47" s="2" t="inlineStr"/>
+      <c r="O47" s="2" t="inlineStr">
+        <is>
+          <t>Registrų centro/VDA atviruose duomenyse pagrindinė veikla nurodyta kaip prekinio betono mišinio gamyba (EVRK 23.63).</t>
+        </is>
+      </c>
+      <c r="P47" s="4" t="n">
+        <v>0.82</v>
+      </c>
+      <c r="Q47" s="5" t="n"/>
+      <c r="R47" s="5" t="n"/>
+      <c r="S47" s="5" t="n"/>
+      <c r="T47" s="5" t="n"/>
+      <c r="U47" s="2" t="inlineStr"/>
+      <c r="V47" s="2" t="inlineStr">
+        <is>
+          <t>https://data.gov.lt/dataset/juridiniu-asmenu-ekonomines-veiklos-rusys-ir-instituciniai-sektoriai/</t>
+        </is>
+      </c>
+      <c r="W47" s="2" t="inlineStr"/>
+      <c r="X47" s="2" t="inlineStr"/>
+      <c r="Y47" s="2" t="inlineStr"/>
+      <c r="Z47" s="2" t="inlineStr"/>
+      <c r="AA47" s="2" t="inlineStr">
+        <is>
+          <t>Adresas geokoduotas pagal viešai randamą įmonės adresą; betono mazgo vietą verta patikslinti atskiru šaltiniu.</t>
+        </is>
+      </c>
+      <c r="AB47" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="2" t="inlineStr">
+        <is>
+          <t>antano-gribino-imone-prienai</t>
+        </is>
+      </c>
+      <c r="B48" s="2" t="inlineStr">
+        <is>
+          <t>170687267</t>
+        </is>
+      </c>
+      <c r="C48" s="2" t="inlineStr">
+        <is>
+          <t>IĮ Antano Gribino gamybos ir komercinės veiklos įmonė</t>
+        </is>
+      </c>
+      <c r="D48" s="2" t="inlineStr">
+        <is>
+          <t>Antano Gribino įmonė</t>
+        </is>
+      </c>
+      <c r="E48" s="2" t="inlineStr">
+        <is>
+          <t>Papildomai rasta EVRK 23.63</t>
+        </is>
+      </c>
+      <c r="F48" s="2" t="inlineStr">
+        <is>
+          <t>Prienai</t>
+        </is>
+      </c>
+      <c r="G48" s="2" t="inlineStr">
+        <is>
+          <t>Prienų r. sav.</t>
+        </is>
+      </c>
+      <c r="H48" s="2" t="inlineStr">
+        <is>
+          <t>Kęstučio g. 95A, Prienai</t>
+        </is>
+      </c>
+      <c r="I48" s="3" t="n">
+        <v>54.6523184</v>
+      </c>
+      <c r="J48" s="3" t="n">
+        <v>23.9696591</v>
+      </c>
+      <c r="K48" s="2" t="inlineStr">
+        <is>
+          <t>ready_mix_concrete</t>
+        </is>
+      </c>
+      <c r="L48" s="2" t="inlineStr">
+        <is>
+          <t>Betono mišiniai</t>
+        </is>
+      </c>
+      <c r="M48" s="2" t="inlineStr">
+        <is>
+          <t>Antano Gribino įmonės betono gamyba</t>
+        </is>
+      </c>
+      <c r="N48" s="2" t="inlineStr"/>
+      <c r="O48" s="2" t="inlineStr">
+        <is>
+          <t>Registrų centro/VDA atviruose duomenyse pagrindinė veikla nurodyta kaip prekinio betono mišinio gamyba (EVRK 23.63).</t>
+        </is>
+      </c>
+      <c r="P48" s="4" t="n">
+        <v>0.82</v>
+      </c>
+      <c r="Q48" s="5" t="n"/>
+      <c r="R48" s="5" t="n"/>
+      <c r="S48" s="5" t="n"/>
+      <c r="T48" s="5" t="n"/>
+      <c r="U48" s="2" t="inlineStr"/>
+      <c r="V48" s="2" t="inlineStr">
+        <is>
+          <t>https://data.gov.lt/dataset/juridiniu-asmenu-ekonomines-veiklos-rusys-ir-instituciniai-sektoriai/</t>
+        </is>
+      </c>
+      <c r="W48" s="2" t="inlineStr"/>
+      <c r="X48" s="2" t="inlineStr"/>
+      <c r="Y48" s="2" t="inlineStr"/>
+      <c r="Z48" s="2" t="inlineStr"/>
+      <c r="AA48" s="2" t="inlineStr">
+        <is>
+          <t>Adresas geokoduotas pagal viešai randamą įmonės adresą; betono mazgo vietą verta patikslinti atskiru šaltiniu.</t>
+        </is>
+      </c>
+      <c r="AB48" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="2" t="inlineStr">
+        <is>
+          <t>kelsera-anavilis</t>
+        </is>
+      </c>
+      <c r="B49" s="2" t="inlineStr">
+        <is>
+          <t>304642165</t>
+        </is>
+      </c>
+      <c r="C49" s="2" t="inlineStr">
+        <is>
+          <t>UAB Kelsera</t>
+        </is>
+      </c>
+      <c r="D49" s="2" t="inlineStr">
+        <is>
+          <t>Kelsera</t>
+        </is>
+      </c>
+      <c r="E49" s="2" t="inlineStr">
+        <is>
+          <t>Papildomai rasta EVRK 23.63</t>
+        </is>
+      </c>
+      <c r="F49" s="2" t="inlineStr">
+        <is>
+          <t>Anavilis</t>
+        </is>
+      </c>
+      <c r="G49" s="2" t="inlineStr">
+        <is>
+          <t>Vilniaus r. sav.</t>
+        </is>
+      </c>
+      <c r="H49" s="2" t="inlineStr">
+        <is>
+          <t>Bitininkų g. 13, Anavilis, Vilniaus r.</t>
+        </is>
+      </c>
+      <c r="I49" s="3" t="n">
+        <v>54.9464296</v>
+      </c>
+      <c r="J49" s="3" t="n">
+        <v>25.2168004</v>
+      </c>
+      <c r="K49" s="2" t="inlineStr">
+        <is>
+          <t>ready_mix_concrete</t>
+        </is>
+      </c>
+      <c r="L49" s="2" t="inlineStr">
+        <is>
+          <t>Betono mišiniai</t>
+        </is>
+      </c>
+      <c r="M49" s="2" t="inlineStr">
+        <is>
+          <t>Kelsera betono gamyba</t>
+        </is>
+      </c>
+      <c r="N49" s="2" t="inlineStr"/>
+      <c r="O49" s="2" t="inlineStr">
+        <is>
+          <t>Registrų centro/VDA atviruose duomenyse pagrindinė veikla nurodyta kaip prekinio betono mišinio gamyba (EVRK 23.63).</t>
+        </is>
+      </c>
+      <c r="P49" s="4" t="n">
+        <v>0.82</v>
+      </c>
+      <c r="Q49" s="5" t="n"/>
+      <c r="R49" s="5" t="n"/>
+      <c r="S49" s="5" t="n"/>
+      <c r="T49" s="5" t="n"/>
+      <c r="U49" s="2" t="inlineStr"/>
+      <c r="V49" s="2" t="inlineStr">
+        <is>
+          <t>https://data.gov.lt/dataset/juridiniu-asmenu-ekonomines-veiklos-rusys-ir-instituciniai-sektoriai/</t>
+        </is>
+      </c>
+      <c r="W49" s="2" t="inlineStr"/>
+      <c r="X49" s="2" t="inlineStr"/>
+      <c r="Y49" s="2" t="inlineStr"/>
+      <c r="Z49" s="2" t="inlineStr"/>
+      <c r="AA49" s="2" t="inlineStr">
+        <is>
+          <t>Adresas geokoduotas pagal viešai randamą įmonės adresą; betono mazgo vietą verta patikslinti atskiru šaltiniu.</t>
+        </is>
+      </c>
+      <c r="AB49" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="2" t="inlineStr">
+        <is>
+          <t>altimas-avizieniai</t>
+        </is>
+      </c>
+      <c r="B50" s="2" t="inlineStr">
+        <is>
+          <t>301699702</t>
+        </is>
+      </c>
+      <c r="C50" s="2" t="inlineStr">
+        <is>
+          <t>UAB Altimas</t>
+        </is>
+      </c>
+      <c r="D50" s="2" t="inlineStr">
+        <is>
+          <t>Altimas</t>
+        </is>
+      </c>
+      <c r="E50" s="2" t="inlineStr">
+        <is>
+          <t>Papildomai rasta EVRK 23.63</t>
+        </is>
+      </c>
+      <c r="F50" s="2" t="inlineStr">
+        <is>
+          <t>Avižieniai</t>
+        </is>
+      </c>
+      <c r="G50" s="2" t="inlineStr">
+        <is>
+          <t>Vilniaus r. sav.</t>
+        </is>
+      </c>
+      <c r="H50" s="2" t="inlineStr">
+        <is>
+          <t>Vaikystės g. 10, Avižieniai, Vilniaus r.</t>
+        </is>
+      </c>
+      <c r="I50" s="3" t="n">
+        <v>54.7574304</v>
+      </c>
+      <c r="J50" s="3" t="n">
+        <v>25.1871813</v>
+      </c>
+      <c r="K50" s="2" t="inlineStr">
+        <is>
+          <t>ready_mix_concrete</t>
+        </is>
+      </c>
+      <c r="L50" s="2" t="inlineStr">
+        <is>
+          <t>Betono mišiniai</t>
+        </is>
+      </c>
+      <c r="M50" s="2" t="inlineStr">
+        <is>
+          <t>Altimas betono gamyba</t>
+        </is>
+      </c>
+      <c r="N50" s="2" t="inlineStr"/>
+      <c r="O50" s="2" t="inlineStr">
+        <is>
+          <t>Registrų centro/VDA atviruose duomenyse pagrindinė veikla nurodyta kaip prekinio betono mišinio gamyba (EVRK 23.63).</t>
+        </is>
+      </c>
+      <c r="P50" s="4" t="n">
+        <v>0.82</v>
+      </c>
+      <c r="Q50" s="5" t="n"/>
+      <c r="R50" s="5" t="n"/>
+      <c r="S50" s="5" t="n"/>
+      <c r="T50" s="5" t="n"/>
+      <c r="U50" s="2" t="inlineStr"/>
+      <c r="V50" s="2" t="inlineStr">
+        <is>
+          <t>https://data.gov.lt/dataset/juridiniu-asmenu-ekonomines-veiklos-rusys-ir-instituciniai-sektoriai/</t>
+        </is>
+      </c>
+      <c r="W50" s="2" t="inlineStr"/>
+      <c r="X50" s="2" t="inlineStr"/>
+      <c r="Y50" s="2" t="inlineStr"/>
+      <c r="Z50" s="2" t="inlineStr"/>
+      <c r="AA50" s="2" t="inlineStr">
+        <is>
+          <t>Adresas geokoduotas pagal viešai randamą įmonės adresą; betono mazgo vietą verta patikslinti atskiru šaltiniu.</t>
+        </is>
+      </c>
+      <c r="AB50" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="2" t="inlineStr">
+        <is>
+          <t>vinido-taurage</t>
+        </is>
+      </c>
+      <c r="B51" s="2" t="inlineStr">
+        <is>
+          <t>306258220</t>
+        </is>
+      </c>
+      <c r="C51" s="2" t="inlineStr">
+        <is>
+          <t>UAB Vinido</t>
+        </is>
+      </c>
+      <c r="D51" s="2" t="inlineStr">
+        <is>
+          <t>Vinido</t>
+        </is>
+      </c>
+      <c r="E51" s="2" t="inlineStr">
+        <is>
+          <t>Papildomai rasta EVRK 23.63</t>
+        </is>
+      </c>
+      <c r="F51" s="2" t="inlineStr">
+        <is>
+          <t>Tauragė</t>
+        </is>
+      </c>
+      <c r="G51" s="2" t="inlineStr">
+        <is>
+          <t>Tauragės r. sav.</t>
+        </is>
+      </c>
+      <c r="H51" s="2" t="inlineStr">
+        <is>
+          <t>Gaurės g. 32, Tauragė</t>
+        </is>
+      </c>
+      <c r="I51" s="3" t="n">
+        <v>55.249189</v>
+      </c>
+      <c r="J51" s="3" t="n">
+        <v>22.3185783</v>
+      </c>
+      <c r="K51" s="2" t="inlineStr">
+        <is>
+          <t>ready_mix_concrete</t>
+        </is>
+      </c>
+      <c r="L51" s="2" t="inlineStr">
+        <is>
+          <t>Betono mišiniai</t>
+        </is>
+      </c>
+      <c r="M51" s="2" t="inlineStr">
+        <is>
+          <t>Vinido betono gamyba</t>
+        </is>
+      </c>
+      <c r="N51" s="2" t="inlineStr"/>
+      <c r="O51" s="2" t="inlineStr">
+        <is>
+          <t>Registrų centro/VDA atviruose duomenyse pagrindinė veikla nurodyta kaip prekinio betono mišinio gamyba (EVRK 23.63).</t>
+        </is>
+      </c>
+      <c r="P51" s="4" t="n">
+        <v>0.82</v>
+      </c>
+      <c r="Q51" s="5" t="n"/>
+      <c r="R51" s="5" t="n"/>
+      <c r="S51" s="5" t="n"/>
+      <c r="T51" s="5" t="n"/>
+      <c r="U51" s="2" t="inlineStr"/>
+      <c r="V51" s="2" t="inlineStr">
+        <is>
+          <t>https://data.gov.lt/dataset/juridiniu-asmenu-ekonomines-veiklos-rusys-ir-instituciniai-sektoriai/</t>
+        </is>
+      </c>
+      <c r="W51" s="2" t="inlineStr"/>
+      <c r="X51" s="2" t="inlineStr"/>
+      <c r="Y51" s="2" t="inlineStr"/>
+      <c r="Z51" s="2" t="inlineStr"/>
+      <c r="AA51" s="2" t="inlineStr">
+        <is>
+          <t>Adresas geokoduotas pagal viešai randamą įmonės adresą; betono mazgo vietą verta patikslinti atskiru šaltiniu.</t>
+        </is>
+      </c>
+      <c r="AB51" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="2" t="inlineStr">
+        <is>
+          <t>santvara-kedainiai</t>
+        </is>
+      </c>
+      <c r="B52" s="2" t="inlineStr">
+        <is>
+          <t>304915297</t>
+        </is>
+      </c>
+      <c r="C52" s="2" t="inlineStr">
+        <is>
+          <t>UAB Santvara</t>
+        </is>
+      </c>
+      <c r="D52" s="2" t="inlineStr">
+        <is>
+          <t>Santvara</t>
+        </is>
+      </c>
+      <c r="E52" s="2" t="inlineStr">
+        <is>
+          <t>Papildomai rasta EVRK 23.63</t>
+        </is>
+      </c>
+      <c r="F52" s="2" t="inlineStr">
+        <is>
+          <t>Kėdainiai</t>
+        </is>
+      </c>
+      <c r="G52" s="2" t="inlineStr">
+        <is>
+          <t>Kėdainių r. sav.</t>
+        </is>
+      </c>
+      <c r="H52" s="2" t="inlineStr">
+        <is>
+          <t>Aruodų g. 34, Kėdainiai</t>
+        </is>
+      </c>
+      <c r="I52" s="3" t="n">
+        <v>55.2634765</v>
+      </c>
+      <c r="J52" s="3" t="n">
+        <v>23.9440395</v>
+      </c>
+      <c r="K52" s="2" t="inlineStr">
+        <is>
+          <t>ready_mix_concrete</t>
+        </is>
+      </c>
+      <c r="L52" s="2" t="inlineStr">
+        <is>
+          <t>Betono mišiniai</t>
+        </is>
+      </c>
+      <c r="M52" s="2" t="inlineStr">
+        <is>
+          <t>Santvara betono gamyba</t>
+        </is>
+      </c>
+      <c r="N52" s="2" t="inlineStr"/>
+      <c r="O52" s="2" t="inlineStr">
+        <is>
+          <t>Registrų centro/VDA atviruose duomenyse pagrindinė veikla nurodyta kaip prekinio betono mišinio gamyba (EVRK 23.63).</t>
+        </is>
+      </c>
+      <c r="P52" s="4" t="n">
+        <v>0.82</v>
+      </c>
+      <c r="Q52" s="5" t="n"/>
+      <c r="R52" s="5" t="n"/>
+      <c r="S52" s="5" t="n"/>
+      <c r="T52" s="5" t="n"/>
+      <c r="U52" s="2" t="inlineStr"/>
+      <c r="V52" s="2" t="inlineStr">
+        <is>
+          <t>https://data.gov.lt/dataset/juridiniu-asmenu-ekonomines-veiklos-rusys-ir-instituciniai-sektoriai/</t>
+        </is>
+      </c>
+      <c r="W52" s="2" t="inlineStr"/>
+      <c r="X52" s="2" t="inlineStr"/>
+      <c r="Y52" s="2" t="inlineStr"/>
+      <c r="Z52" s="2" t="inlineStr">
+        <is>
+          <t>https://chamber.lt/bendruomene/rumu-nariu-sarasas/nariai/santvara/</t>
+        </is>
+      </c>
+      <c r="AA52" s="2" t="inlineStr">
+        <is>
+          <t>Adresas geokoduotas pagal viešai randamą įmonės adresą; betono mazgo vietą verta patikslinti atskiru šaltiniu.</t>
+        </is>
+      </c>
+      <c r="AB52" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="2" t="inlineStr">
+        <is>
+          <t>eurobetonas-visaginas</t>
+        </is>
+      </c>
+      <c r="B53" s="2" t="inlineStr">
+        <is>
+          <t>305191384</t>
+        </is>
+      </c>
+      <c r="C53" s="2" t="inlineStr">
+        <is>
+          <t>UAB Eurobetonas</t>
+        </is>
+      </c>
+      <c r="D53" s="2" t="inlineStr">
+        <is>
+          <t>Eurobetonas</t>
+        </is>
+      </c>
+      <c r="E53" s="2" t="inlineStr">
+        <is>
+          <t>Papildomai rasta EVRK 23.63</t>
+        </is>
+      </c>
+      <c r="F53" s="2" t="inlineStr">
+        <is>
+          <t>Visaginas</t>
+        </is>
+      </c>
+      <c r="G53" s="2" t="inlineStr">
+        <is>
+          <t>Visagino sav.</t>
+        </is>
+      </c>
+      <c r="H53" s="2" t="inlineStr">
+        <is>
+          <t>Sandėlių g. 1, Karlų k., Visagino sav.</t>
+        </is>
+      </c>
+      <c r="I53" s="3" t="n">
+        <v>55.59966</v>
+      </c>
+      <c r="J53" s="3" t="n">
+        <v>26.4370071</v>
+      </c>
+      <c r="K53" s="2" t="inlineStr">
+        <is>
+          <t>ready_mix_concrete</t>
+        </is>
+      </c>
+      <c r="L53" s="2" t="inlineStr">
+        <is>
+          <t>Betono mišiniai</t>
+        </is>
+      </c>
+      <c r="M53" s="2" t="inlineStr">
+        <is>
+          <t>Eurobetonas betono gamyba</t>
+        </is>
+      </c>
+      <c r="N53" s="2" t="inlineStr"/>
+      <c r="O53" s="2" t="inlineStr">
+        <is>
+          <t>Registrų centro/VDA atviruose duomenyse pagrindinė veikla nurodyta kaip prekinio betono mišinio gamyba (EVRK 23.63).</t>
+        </is>
+      </c>
+      <c r="P53" s="4" t="n">
+        <v>0.72</v>
+      </c>
+      <c r="Q53" s="5" t="n"/>
+      <c r="R53" s="5" t="n"/>
+      <c r="S53" s="5" t="n"/>
+      <c r="T53" s="5" t="n"/>
+      <c r="U53" s="2" t="inlineStr"/>
+      <c r="V53" s="2" t="inlineStr">
+        <is>
+          <t>https://data.gov.lt/dataset/juridiniu-asmenu-ekonomines-veiklos-rusys-ir-instituciniai-sektoriai/</t>
+        </is>
+      </c>
+      <c r="W53" s="2" t="inlineStr"/>
+      <c r="X53" s="2" t="inlineStr"/>
+      <c r="Y53" s="2" t="inlineStr"/>
+      <c r="Z53" s="2" t="inlineStr"/>
+      <c r="AA53" s="2" t="inlineStr">
+        <is>
+          <t>Adresas rastas viešuose kataloguose, bet geokoduotas tik iki Visagino miesto taško; reikia patikslinti tikslų betono mazgo GPS.</t>
+        </is>
+      </c>
+      <c r="AB53" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="2" t="inlineStr">
+        <is>
+          <t>medis-ir-betonas-naujoji-akmene</t>
+        </is>
+      </c>
+      <c r="B54" s="2" t="inlineStr">
+        <is>
+          <t>153074073</t>
+        </is>
+      </c>
+      <c r="C54" s="2" t="inlineStr">
+        <is>
+          <t>AB Medis ir betonas</t>
+        </is>
+      </c>
+      <c r="D54" s="2" t="inlineStr">
+        <is>
+          <t>Medis ir betonas</t>
+        </is>
+      </c>
+      <c r="E54" s="2" t="inlineStr">
+        <is>
+          <t>Papildomai rasta EVRK 23.63</t>
+        </is>
+      </c>
+      <c r="F54" s="2" t="inlineStr">
+        <is>
+          <t>Naujoji Akmenė</t>
+        </is>
+      </c>
+      <c r="G54" s="2" t="inlineStr">
+        <is>
+          <t>Akmenės r. sav.</t>
+        </is>
+      </c>
+      <c r="H54" s="2" t="inlineStr">
+        <is>
+          <t>J. Dalinkevičiaus g. 2, Naujoji Akmenė</t>
+        </is>
+      </c>
+      <c r="I54" s="3" t="n">
+        <v>56.3155328</v>
+      </c>
+      <c r="J54" s="3" t="n">
+        <v>22.9143308</v>
+      </c>
+      <c r="K54" s="2" t="inlineStr">
+        <is>
+          <t>ready_mix_concrete</t>
+        </is>
+      </c>
+      <c r="L54" s="2" t="inlineStr">
+        <is>
+          <t>Betono mišiniai</t>
+        </is>
+      </c>
+      <c r="M54" s="2" t="inlineStr">
+        <is>
+          <t>Medis ir betonas gamyba</t>
+        </is>
+      </c>
+      <c r="N54" s="2" t="inlineStr"/>
+      <c r="O54" s="2" t="inlineStr">
+        <is>
+          <t>Registrų centro/VDA atviruose duomenyse pagrindinė veikla nurodyta kaip prekinio betono mišinio gamyba (EVRK 23.63).</t>
+        </is>
+      </c>
+      <c r="P54" s="4" t="n">
+        <v>0.82</v>
+      </c>
+      <c r="Q54" s="5" t="n"/>
+      <c r="R54" s="5" t="n"/>
+      <c r="S54" s="5" t="n"/>
+      <c r="T54" s="5" t="n"/>
+      <c r="U54" s="2" t="inlineStr"/>
+      <c r="V54" s="2" t="inlineStr">
+        <is>
+          <t>https://data.gov.lt/dataset/juridiniu-asmenu-ekonomines-veiklos-rusys-ir-instituciniai-sektoriai/</t>
+        </is>
+      </c>
+      <c r="W54" s="2" t="inlineStr"/>
+      <c r="X54" s="2" t="inlineStr"/>
+      <c r="Y54" s="2" t="inlineStr"/>
+      <c r="Z54" s="2" t="inlineStr"/>
+      <c r="AA54" s="2" t="inlineStr">
+        <is>
+          <t>Adresas geokoduotas pagal viešai randamą įmonės adresą; betono mazgo vietą verta patikslinti atskiru šaltiniu.</t>
+        </is>
+      </c>
+      <c r="AB54" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="2" t="inlineStr">
+        <is>
+          <t>ekobetonas-marijampole</t>
+        </is>
+      </c>
+      <c r="B55" s="2" t="inlineStr">
+        <is>
+          <t>300636364</t>
+        </is>
+      </c>
+      <c r="C55" s="2" t="inlineStr">
+        <is>
+          <t>UAB Ekobetonas</t>
+        </is>
+      </c>
+      <c r="D55" s="2" t="inlineStr">
+        <is>
+          <t>Ekobetonas</t>
+        </is>
+      </c>
+      <c r="E55" s="2" t="inlineStr">
+        <is>
+          <t>Papildomai rasta EVRK 23.63</t>
+        </is>
+      </c>
+      <c r="F55" s="2" t="inlineStr">
+        <is>
+          <t>Marijampolė</t>
+        </is>
+      </c>
+      <c r="G55" s="2" t="inlineStr">
+        <is>
+          <t>Marijampolės sav.</t>
+        </is>
+      </c>
+      <c r="H55" s="2" t="inlineStr">
+        <is>
+          <t>Gamyklų g. 3, Marijampolė</t>
+        </is>
+      </c>
+      <c r="I55" s="3" t="n">
+        <v>54.5750139</v>
+      </c>
+      <c r="J55" s="3" t="n">
+        <v>23.3796432</v>
+      </c>
+      <c r="K55" s="2" t="inlineStr">
+        <is>
+          <t>ready_mix_concrete</t>
+        </is>
+      </c>
+      <c r="L55" s="2" t="inlineStr">
+        <is>
+          <t>Betono mišiniai</t>
+        </is>
+      </c>
+      <c r="M55" s="2" t="inlineStr">
+        <is>
+          <t>Ekobetonas betono gamyba</t>
+        </is>
+      </c>
+      <c r="N55" s="2" t="inlineStr"/>
+      <c r="O55" s="2" t="inlineStr">
+        <is>
+          <t>Registrų centro/VDA atviruose duomenyse pagrindinė veikla nurodyta kaip prekinio betono mišinio gamyba (EVRK 23.63).</t>
+        </is>
+      </c>
+      <c r="P55" s="4" t="n">
+        <v>0.82</v>
+      </c>
+      <c r="Q55" s="5" t="n"/>
+      <c r="R55" s="5" t="n"/>
+      <c r="S55" s="5" t="n"/>
+      <c r="T55" s="5" t="n"/>
+      <c r="U55" s="2" t="inlineStr"/>
+      <c r="V55" s="2" t="inlineStr">
+        <is>
+          <t>https://data.gov.lt/dataset/juridiniu-asmenu-ekonomines-veiklos-rusys-ir-instituciniai-sektoriai/</t>
+        </is>
+      </c>
+      <c r="W55" s="2" t="inlineStr"/>
+      <c r="X55" s="2" t="inlineStr"/>
+      <c r="Y55" s="2" t="inlineStr"/>
+      <c r="Z55" s="2" t="inlineStr"/>
+      <c r="AA55" s="2" t="inlineStr">
+        <is>
+          <t>Adresas geokoduotas pagal viešai randamą įmonės adresą; betono mazgo vietą verta patikslinti atskiru šaltiniu.</t>
+        </is>
+      </c>
+      <c r="AB55" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="2" t="inlineStr">
+        <is>
+          <t>rokbetonis-rokiskis</t>
+        </is>
+      </c>
+      <c r="B56" s="2" t="inlineStr">
+        <is>
+          <t>304184091</t>
+        </is>
+      </c>
+      <c r="C56" s="2" t="inlineStr">
+        <is>
+          <t>MB Rokbetonis</t>
+        </is>
+      </c>
+      <c r="D56" s="2" t="inlineStr">
+        <is>
+          <t>Rokbetonis</t>
+        </is>
+      </c>
+      <c r="E56" s="2" t="inlineStr">
+        <is>
+          <t>Papildomai rasta EVRK 23.63</t>
+        </is>
+      </c>
+      <c r="F56" s="2" t="inlineStr">
+        <is>
+          <t>Rokiškis</t>
+        </is>
+      </c>
+      <c r="G56" s="2" t="inlineStr">
+        <is>
+          <t>Rokiškio r. sav.</t>
+        </is>
+      </c>
+      <c r="H56" s="2" t="inlineStr">
+        <is>
+          <t>Vydūno g. 12A, Parokiškė, Rokiškio r.</t>
+        </is>
+      </c>
+      <c r="I56" s="3" t="n">
+        <v>55.954025</v>
+      </c>
+      <c r="J56" s="3" t="n">
+        <v>25.591746</v>
+      </c>
+      <c r="K56" s="2" t="inlineStr">
+        <is>
+          <t>ready_mix_concrete</t>
+        </is>
+      </c>
+      <c r="L56" s="2" t="inlineStr">
+        <is>
+          <t>Betono mišiniai</t>
+        </is>
+      </c>
+      <c r="M56" s="2" t="inlineStr">
+        <is>
+          <t>Rokbetonis betono gamyba</t>
+        </is>
+      </c>
+      <c r="N56" s="2" t="inlineStr"/>
+      <c r="O56" s="2" t="inlineStr">
+        <is>
+          <t>Registrų centro/VDA atviruose duomenyse pagrindinė veikla nurodyta kaip prekinio betono mišinio gamyba (EVRK 23.63).</t>
+        </is>
+      </c>
+      <c r="P56" s="4" t="n">
+        <v>0.72</v>
+      </c>
+      <c r="Q56" s="5" t="n"/>
+      <c r="R56" s="5" t="n"/>
+      <c r="S56" s="5" t="n"/>
+      <c r="T56" s="5" t="n"/>
+      <c r="U56" s="2" t="inlineStr"/>
+      <c r="V56" s="2" t="inlineStr">
+        <is>
+          <t>https://data.gov.lt/dataset/juridiniu-asmenu-ekonomines-veiklos-rusys-ir-instituciniai-sektoriai/</t>
+        </is>
+      </c>
+      <c r="W56" s="2" t="inlineStr"/>
+      <c r="X56" s="2" t="inlineStr"/>
+      <c r="Y56" s="2" t="inlineStr"/>
+      <c r="Z56" s="2" t="inlineStr"/>
+      <c r="AA56" s="2" t="inlineStr">
+        <is>
+          <t>Adresas rastas viešuose kataloguose, bet geokoduotas tik iki Rokiškio miesto taško; reikia patikslinti tikslų betono mazgo GPS.</t>
+        </is>
+      </c>
+      <c r="AB56" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="2" t="inlineStr">
+        <is>
+          <t>beton-eura-dovainonys</t>
+        </is>
+      </c>
+      <c r="B57" s="2" t="inlineStr">
+        <is>
+          <t>302745280</t>
+        </is>
+      </c>
+      <c r="C57" s="2" t="inlineStr">
+        <is>
+          <t>UAB Beton Eura</t>
+        </is>
+      </c>
+      <c r="D57" s="2" t="inlineStr">
+        <is>
+          <t>Beton Eura</t>
+        </is>
+      </c>
+      <c r="E57" s="2" t="inlineStr">
+        <is>
+          <t>Papildomai rasta EVRK 23.63</t>
+        </is>
+      </c>
+      <c r="F57" s="2" t="inlineStr">
+        <is>
+          <t>Dovainonys</t>
+        </is>
+      </c>
+      <c r="G57" s="2" t="inlineStr">
+        <is>
+          <t>Kaišiadorių r. sav.</t>
+        </is>
+      </c>
+      <c r="H57" s="2" t="inlineStr">
+        <is>
+          <t>Žilvičių g. 2, Dovainonys, Kaišiadorių r.</t>
+        </is>
+      </c>
+      <c r="I57" s="3" t="n">
+        <v>54.8395962</v>
+      </c>
+      <c r="J57" s="3" t="n">
+        <v>24.2360189</v>
+      </c>
+      <c r="K57" s="2" t="inlineStr">
+        <is>
+          <t>ready_mix_concrete</t>
+        </is>
+      </c>
+      <c r="L57" s="2" t="inlineStr">
+        <is>
+          <t>Betono mišiniai</t>
+        </is>
+      </c>
+      <c r="M57" s="2" t="inlineStr">
+        <is>
+          <t>Beton Eura betono gamyba</t>
+        </is>
+      </c>
+      <c r="N57" s="2" t="inlineStr"/>
+      <c r="O57" s="2" t="inlineStr">
+        <is>
+          <t>Registrų centro/VDA atviruose duomenyse pagrindinė veikla nurodyta kaip prekinio betono mišinio gamyba (EVRK 23.63).</t>
+        </is>
+      </c>
+      <c r="P57" s="4" t="n">
+        <v>0.82</v>
+      </c>
+      <c r="Q57" s="5" t="n"/>
+      <c r="R57" s="5" t="n"/>
+      <c r="S57" s="5" t="n"/>
+      <c r="T57" s="5" t="n"/>
+      <c r="U57" s="2" t="inlineStr"/>
+      <c r="V57" s="2" t="inlineStr">
+        <is>
+          <t>https://data.gov.lt/dataset/juridiniu-asmenu-ekonomines-veiklos-rusys-ir-instituciniai-sektoriai/</t>
+        </is>
+      </c>
+      <c r="W57" s="2" t="inlineStr"/>
+      <c r="X57" s="2" t="inlineStr"/>
+      <c r="Y57" s="2" t="inlineStr"/>
+      <c r="Z57" s="2" t="inlineStr"/>
+      <c r="AA57" s="2" t="inlineStr">
+        <is>
+          <t>Adresas geokoduotas pagal viešai randamą įmonės adresą; betono mazgo vietą verta patikslinti atskiru šaltiniu.</t>
+        </is>
+      </c>
+      <c r="AB57" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="2" t="inlineStr">
+        <is>
+          <t>silutes-betonas-silute</t>
+        </is>
+      </c>
+      <c r="B58" s="2" t="inlineStr">
+        <is>
+          <t>177392928</t>
+        </is>
+      </c>
+      <c r="C58" s="2" t="inlineStr">
+        <is>
+          <t>UAB Šilutės betonas</t>
+        </is>
+      </c>
+      <c r="D58" s="2" t="inlineStr">
+        <is>
+          <t>Šilutės betonas</t>
+        </is>
+      </c>
+      <c r="E58" s="2" t="inlineStr">
+        <is>
+          <t>Papildomai rasta EVRK 23.63</t>
+        </is>
+      </c>
+      <c r="F58" s="2" t="inlineStr">
+        <is>
+          <t>Šilutė</t>
+        </is>
+      </c>
+      <c r="G58" s="2" t="inlineStr">
+        <is>
+          <t>Šilutės r. sav.</t>
+        </is>
+      </c>
+      <c r="H58" s="2" t="inlineStr">
+        <is>
+          <t>Ramučių g. 1, Šilutė</t>
+        </is>
+      </c>
+      <c r="I58" s="3" t="n">
+        <v>55.3540625</v>
+      </c>
+      <c r="J58" s="3" t="n">
+        <v>21.4798764</v>
+      </c>
+      <c r="K58" s="2" t="inlineStr">
+        <is>
+          <t>ready_mix_concrete</t>
+        </is>
+      </c>
+      <c r="L58" s="2" t="inlineStr">
+        <is>
+          <t>Betono mišiniai</t>
+        </is>
+      </c>
+      <c r="M58" s="2" t="inlineStr">
+        <is>
+          <t>Šilutės betono gamyba</t>
+        </is>
+      </c>
+      <c r="N58" s="2" t="inlineStr"/>
+      <c r="O58" s="2" t="inlineStr">
+        <is>
+          <t>Registrų centro/VDA atviruose duomenyse pagrindinė veikla nurodyta kaip prekinio betono mišinio gamyba (EVRK 23.63).</t>
+        </is>
+      </c>
+      <c r="P58" s="4" t="n">
+        <v>0.82</v>
+      </c>
+      <c r="Q58" s="5" t="n"/>
+      <c r="R58" s="5" t="n"/>
+      <c r="S58" s="5" t="n"/>
+      <c r="T58" s="5" t="n"/>
+      <c r="U58" s="2" t="inlineStr"/>
+      <c r="V58" s="2" t="inlineStr">
+        <is>
+          <t>https://data.gov.lt/dataset/juridiniu-asmenu-ekonomines-veiklos-rusys-ir-instituciniai-sektoriai/</t>
+        </is>
+      </c>
+      <c r="W58" s="2" t="inlineStr"/>
+      <c r="X58" s="2" t="inlineStr"/>
+      <c r="Y58" s="2" t="inlineStr"/>
+      <c r="Z58" s="2" t="inlineStr">
+        <is>
+          <t>https://fsaskaita.lt/imone/uzdaroji-akcine-bendrove-silutes-betonas-177392928</t>
+        </is>
+      </c>
+      <c r="AA58" s="2" t="inlineStr">
+        <is>
+          <t>Adresas geokoduotas pagal viešai randamą įmonės adresą; betono mazgo vietą verta patikslinti atskiru šaltiniu.</t>
+        </is>
+      </c>
+      <c r="AB58" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="2" t="inlineStr">
+        <is>
+          <t>kruszbet-lithuania-jure</t>
+        </is>
+      </c>
+      <c r="B59" s="2" t="inlineStr">
+        <is>
+          <t>305173596</t>
+        </is>
+      </c>
+      <c r="C59" s="2" t="inlineStr">
+        <is>
+          <t>UAB KRUSZBET Lithuania</t>
+        </is>
+      </c>
+      <c r="D59" s="2" t="inlineStr">
+        <is>
+          <t>KRUSZBET Lithuania</t>
+        </is>
+      </c>
+      <c r="E59" s="2" t="inlineStr">
+        <is>
+          <t>Papildomai rasta EVRK 23.63</t>
+        </is>
+      </c>
+      <c r="F59" s="2" t="inlineStr">
+        <is>
+          <t>Jūrė</t>
+        </is>
+      </c>
+      <c r="G59" s="2" t="inlineStr">
+        <is>
+          <t>Kazlų Rūdos sav.</t>
+        </is>
+      </c>
+      <c r="H59" s="2" t="inlineStr">
+        <is>
+          <t>Medelyno g. 30A, Jūrė, Kazlų Rūdos sav.</t>
+        </is>
+      </c>
+      <c r="I59" s="3" t="n">
+        <v>54.7704618</v>
+      </c>
+      <c r="J59" s="3" t="n">
+        <v>23.4998425</v>
+      </c>
+      <c r="K59" s="2" t="inlineStr">
+        <is>
+          <t>ready_mix_concrete</t>
+        </is>
+      </c>
+      <c r="L59" s="2" t="inlineStr">
+        <is>
+          <t>Betono mišiniai</t>
+        </is>
+      </c>
+      <c r="M59" s="2" t="inlineStr">
+        <is>
+          <t>KRUSZBET Lithuania betono gamyba</t>
+        </is>
+      </c>
+      <c r="N59" s="2" t="inlineStr"/>
+      <c r="O59" s="2" t="inlineStr">
+        <is>
+          <t>Registrų centro/VDA atviruose duomenyse pagrindinė veikla nurodyta kaip prekinio betono mišinio gamyba (EVRK 23.63).</t>
+        </is>
+      </c>
+      <c r="P59" s="4" t="n">
+        <v>0.82</v>
+      </c>
+      <c r="Q59" s="5" t="n"/>
+      <c r="R59" s="5" t="n"/>
+      <c r="S59" s="5" t="n"/>
+      <c r="T59" s="5" t="n"/>
+      <c r="U59" s="2" t="inlineStr"/>
+      <c r="V59" s="2" t="inlineStr">
+        <is>
+          <t>https://data.gov.lt/dataset/juridiniu-asmenu-ekonomines-veiklos-rusys-ir-instituciniai-sektoriai/</t>
+        </is>
+      </c>
+      <c r="W59" s="2" t="inlineStr"/>
+      <c r="X59" s="2" t="inlineStr"/>
+      <c r="Y59" s="2" t="inlineStr"/>
+      <c r="Z59" s="2" t="inlineStr"/>
+      <c r="AA59" s="2" t="inlineStr">
+        <is>
+          <t>Adresas geokoduotas pagal viešai randamą įmonės adresą; betono mazgo vietą verta patikslinti atskiru šaltiniu.</t>
+        </is>
+      </c>
+      <c r="AB59" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:AB46"/>
+  <autoFilter ref="A1:AB59"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -5147,7 +6483,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-06-30T04:22:16.649112+00:00</t>
+          <t>2026-06-30T11:26:53.379253+00:00</t>
         </is>
       </c>
     </row>
@@ -5202,7 +6538,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-06-30T04:22:16.650112+00:00</t>
+          <t>2026-06-30T11:26:53.379253+00:00</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -5216,7 +6552,7 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>45</v>
+        <v>58</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Add Telsiu keliai concrete producer
</commit_message>
<xml_diff>
--- a/data/companies.xlsx
+++ b/data/companies.xlsx
@@ -12,7 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Importo žurnalas" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Įmonės'!$A$1:$AE$59</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Įmonės'!$A$1:$AE$60</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -169,8 +169,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ImonesTable" displayName="ImonesTable" ref="A1:AE59" headerRowCount="1">
-  <autoFilter ref="A1:AE59"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ImonesTable" displayName="ImonesTable" ref="A1:AE60" headerRowCount="1">
+  <autoFilter ref="A1:AE60"/>
   <tableColumns count="31">
     <tableColumn id="1" name="Įrašo ID"/>
     <tableColumn id="2" name="Įmonės kodas"/>
@@ -497,14 +497,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE59"/>
+  <dimension ref="A1:AE60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="39" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
     <col width="42" customWidth="1" min="3" max="3"/>
     <col width="33" customWidth="1" min="4" max="4"/>
-    <col width="29" customWidth="1" min="5" max="5"/>
+    <col width="42" customWidth="1" min="5" max="5"/>
     <col width="16" customWidth="1" min="6" max="6"/>
     <col width="21" customWidth="1" min="7" max="7"/>
     <col width="42" customWidth="1" min="8" max="8"/>
@@ -7288,8 +7288,127 @@
         </is>
       </c>
     </row>
+    <row r="60">
+      <c r="A60" s="2" t="inlineStr">
+        <is>
+          <t>telsiu-keliai-telsiai</t>
+        </is>
+      </c>
+      <c r="B60" s="2" t="inlineStr">
+        <is>
+          <t>180200843</t>
+        </is>
+      </c>
+      <c r="C60" s="2" t="inlineStr">
+        <is>
+          <t>UAB Telšių keliai</t>
+        </is>
+      </c>
+      <c r="D60" s="2" t="inlineStr">
+        <is>
+          <t>Telšių keliai</t>
+        </is>
+      </c>
+      <c r="E60" s="2" t="inlineStr">
+        <is>
+          <t>Papildomai įtraukta pagal naudotojo informaciją</t>
+        </is>
+      </c>
+      <c r="F60" s="2" t="inlineStr">
+        <is>
+          <t>Telšiai</t>
+        </is>
+      </c>
+      <c r="G60" s="2" t="inlineStr">
+        <is>
+          <t>Telšių r. sav.</t>
+        </is>
+      </c>
+      <c r="H60" s="2" t="inlineStr">
+        <is>
+          <t>Mažeikių g. 18, Telšiai</t>
+        </is>
+      </c>
+      <c r="I60" s="3" t="n">
+        <v>56.0004158</v>
+      </c>
+      <c r="J60" s="3" t="n">
+        <v>22.2581129</v>
+      </c>
+      <c r="K60" s="2" t="inlineStr">
+        <is>
+          <t>Tikslus adreso taškas</t>
+        </is>
+      </c>
+      <c r="L60" s="2" t="inlineStr">
+        <is>
+          <t>Lietuvos geolokatorius</t>
+        </is>
+      </c>
+      <c r="M60" s="2" t="inlineStr">
+        <is>
+          <t>https://hub.arcgis.com/content/b9e27b4266524b39bc651d6a26480b87</t>
+        </is>
+      </c>
+      <c r="N60" s="2" t="inlineStr">
+        <is>
+          <t>ready_mix_concrete</t>
+        </is>
+      </c>
+      <c r="O60" s="2" t="inlineStr">
+        <is>
+          <t>Betono mišiniai</t>
+        </is>
+      </c>
+      <c r="P60" s="2" t="inlineStr">
+        <is>
+          <t>Telšių kelių betono mišinių gamyba</t>
+        </is>
+      </c>
+      <c r="Q60" s="2" t="inlineStr"/>
+      <c r="R60" s="2" t="inlineStr">
+        <is>
+          <t>Oficialiame įmonės puslapyje skelbiama betono mišinių gamyba ir prekyba.</t>
+        </is>
+      </c>
+      <c r="S60" s="4" t="n">
+        <v>0.86</v>
+      </c>
+      <c r="T60" s="5" t="n"/>
+      <c r="U60" s="5" t="n"/>
+      <c r="V60" s="5" t="n"/>
+      <c r="W60" s="5" t="n"/>
+      <c r="X60" s="2" t="inlineStr">
+        <is>
+          <t>https://www.tkeliai.lt/</t>
+        </is>
+      </c>
+      <c r="Y60" s="2" t="inlineStr">
+        <is>
+          <t>https://www.tkeliai.lt/kitos-paslaugos/</t>
+        </is>
+      </c>
+      <c r="Z60" s="2" t="inlineStr"/>
+      <c r="AA60" s="2" t="inlineStr"/>
+      <c r="AB60" s="2" t="inlineStr"/>
+      <c r="AC60" s="2" t="inlineStr">
+        <is>
+          <t>https://www.tkeliai.lt/kitos-paslaugos/</t>
+        </is>
+      </c>
+      <c r="AD60" s="2" t="inlineStr">
+        <is>
+          <t>Įtraukta pagal naudotojo informaciją; veikla patvirtinta oficialiame lietuviškame įmonės puslapyje. Koordinatės nustatytos Lietuvos geolokatoriumi pagal Mažeikių g. 18 adresą.</t>
+        </is>
+      </c>
+      <c r="AE60" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:AE59"/>
+  <autoFilter ref="A1:AE60"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -7378,7 +7497,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-06-30T11:58:32.368372+00:00</t>
+          <t>2026-06-30T12:13:10.847047+00:00</t>
         </is>
       </c>
     </row>
@@ -7433,7 +7552,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-06-30T11:58:32.368372+00:00</t>
+          <t>2026-06-30T12:13:10.849054+00:00</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -7447,7 +7566,7 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Add silos count to competitor map
</commit_message>
<xml_diff>
--- a/data/companies.xlsx
+++ b/data/companies.xlsx
@@ -12,7 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Importo žurnalas" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Įmonės'!$A$1:$AE$60</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Įmonės'!$A$1:$AF$60</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -71,7 +71,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top"/>
@@ -86,6 +86,9 @@
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -169,9 +172,9 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ImonesTable" displayName="ImonesTable" ref="A1:AE60" headerRowCount="1">
-  <autoFilter ref="A1:AE60"/>
-  <tableColumns count="31">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ImonesTable" displayName="ImonesTable" ref="A1:AF60" headerRowCount="1">
+  <autoFilter ref="A1:AF60"/>
+  <tableColumns count="32">
     <tableColumn id="1" name="Įrašo ID"/>
     <tableColumn id="2" name="Įmonės kodas"/>
     <tableColumn id="3" name="Įmonės pavadinimas"/>
@@ -189,20 +192,21 @@
     <tableColumn id="15" name="Veikla"/>
     <tableColumn id="16" name="Betono mazgo / gamyklos pavadinimas"/>
     <tableColumn id="17" name="Betono mazgo našumas"/>
-    <tableColumn id="18" name="Viešas betono mazgo / gamyklos aprašymas"/>
-    <tableColumn id="19" name="Klasifikavimo pasitikėjimas"/>
-    <tableColumn id="20" name="Įmonės apyvarta"/>
-    <tableColumn id="21" name="Apyvartos metai"/>
-    <tableColumn id="22" name="Darbuotojų skaičius"/>
-    <tableColumn id="23" name="Automobilių / transporto priemonių skaičius"/>
-    <tableColumn id="24" name="Interneto svetainė"/>
-    <tableColumn id="25" name="Pagrindinis šaltinis"/>
-    <tableColumn id="26" name="Apyvartos šaltinis"/>
-    <tableColumn id="27" name="Darbuotojų šaltinis"/>
-    <tableColumn id="28" name="Transporto šaltinis"/>
-    <tableColumn id="29" name="Betono mazgo / gamyklos šaltinis"/>
-    <tableColumn id="30" name="Pastaba / rankinis papildymas"/>
-    <tableColumn id="31" name="Paskutinio atnaujinimo data"/>
+    <tableColumn id="18" name="Silosų skaičius"/>
+    <tableColumn id="19" name="Viešas betono mazgo / gamyklos aprašymas"/>
+    <tableColumn id="20" name="Klasifikavimo pasitikėjimas"/>
+    <tableColumn id="21" name="Įmonės apyvarta"/>
+    <tableColumn id="22" name="Apyvartos metai"/>
+    <tableColumn id="23" name="Darbuotojų skaičius"/>
+    <tableColumn id="24" name="Automobilių / transporto priemonių skaičius"/>
+    <tableColumn id="25" name="Interneto svetainė"/>
+    <tableColumn id="26" name="Pagrindinis šaltinis"/>
+    <tableColumn id="27" name="Apyvartos šaltinis"/>
+    <tableColumn id="28" name="Darbuotojų šaltinis"/>
+    <tableColumn id="29" name="Transporto šaltinis"/>
+    <tableColumn id="30" name="Betono mazgo / gamyklos šaltinis"/>
+    <tableColumn id="31" name="Pastaba / rankinis papildymas"/>
+    <tableColumn id="32" name="Paskutinio atnaujinimo data"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -497,7 +501,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE60"/>
+  <dimension ref="A1:AF60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="39" customWidth="1" min="1" max="1"/>
@@ -517,20 +521,21 @@
     <col width="24" customWidth="1" min="15" max="15"/>
     <col width="40" customWidth="1" min="16" max="16"/>
     <col width="30" customWidth="1" min="17" max="17"/>
-    <col width="42" customWidth="1" min="18" max="18"/>
-    <col width="29" customWidth="1" min="19" max="19"/>
-    <col width="17" customWidth="1" min="20" max="20"/>
+    <col width="17" customWidth="1" min="18" max="18"/>
+    <col width="42" customWidth="1" min="19" max="19"/>
+    <col width="29" customWidth="1" min="20" max="20"/>
     <col width="17" customWidth="1" min="21" max="21"/>
-    <col width="21" customWidth="1" min="22" max="22"/>
-    <col width="42" customWidth="1" min="23" max="23"/>
+    <col width="17" customWidth="1" min="22" max="22"/>
+    <col width="21" customWidth="1" min="23" max="23"/>
     <col width="42" customWidth="1" min="24" max="24"/>
     <col width="42" customWidth="1" min="25" max="25"/>
-    <col width="20" customWidth="1" min="26" max="26"/>
-    <col width="21" customWidth="1" min="27" max="27"/>
+    <col width="42" customWidth="1" min="26" max="26"/>
+    <col width="20" customWidth="1" min="27" max="27"/>
     <col width="21" customWidth="1" min="28" max="28"/>
-    <col width="42" customWidth="1" min="29" max="29"/>
+    <col width="21" customWidth="1" min="29" max="29"/>
     <col width="42" customWidth="1" min="30" max="30"/>
-    <col width="29" customWidth="1" min="31" max="31"/>
+    <col width="42" customWidth="1" min="31" max="31"/>
+    <col width="29" customWidth="1" min="32" max="32"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -621,70 +626,75 @@
       </c>
       <c r="R1" s="1" t="inlineStr">
         <is>
+          <t>Silosų skaičius</t>
+        </is>
+      </c>
+      <c r="S1" s="1" t="inlineStr">
+        <is>
           <t>Viešas betono mazgo / gamyklos aprašymas</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>Klasifikavimo pasitikėjimas</t>
         </is>
       </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>Įmonės apyvarta</t>
         </is>
       </c>
-      <c r="U1" s="1" t="inlineStr">
+      <c r="V1" s="1" t="inlineStr">
         <is>
           <t>Apyvartos metai</t>
         </is>
       </c>
-      <c r="V1" s="1" t="inlineStr">
+      <c r="W1" s="1" t="inlineStr">
         <is>
           <t>Darbuotojų skaičius</t>
         </is>
       </c>
-      <c r="W1" s="1" t="inlineStr">
+      <c r="X1" s="1" t="inlineStr">
         <is>
           <t>Automobilių / transporto priemonių skaičius</t>
         </is>
       </c>
-      <c r="X1" s="1" t="inlineStr">
+      <c r="Y1" s="1" t="inlineStr">
         <is>
           <t>Interneto svetainė</t>
         </is>
       </c>
-      <c r="Y1" s="1" t="inlineStr">
+      <c r="Z1" s="1" t="inlineStr">
         <is>
           <t>Pagrindinis šaltinis</t>
         </is>
       </c>
-      <c r="Z1" s="1" t="inlineStr">
+      <c r="AA1" s="1" t="inlineStr">
         <is>
           <t>Apyvartos šaltinis</t>
         </is>
       </c>
-      <c r="AA1" s="1" t="inlineStr">
+      <c r="AB1" s="1" t="inlineStr">
         <is>
           <t>Darbuotojų šaltinis</t>
         </is>
       </c>
-      <c r="AB1" s="1" t="inlineStr">
+      <c r="AC1" s="1" t="inlineStr">
         <is>
           <t>Transporto šaltinis</t>
         </is>
       </c>
-      <c r="AC1" s="1" t="inlineStr">
+      <c r="AD1" s="1" t="inlineStr">
         <is>
           <t>Betono mazgo / gamyklos šaltinis</t>
         </is>
       </c>
-      <c r="AD1" s="1" t="inlineStr">
+      <c r="AE1" s="1" t="inlineStr">
         <is>
           <t>Pastaba / rankinis papildymas</t>
         </is>
       </c>
-      <c r="AE1" s="1" t="inlineStr">
+      <c r="AF1" s="1" t="inlineStr">
         <is>
           <t>Paskutinio atnaujinimo data</t>
         </is>
@@ -768,38 +778,39 @@
         </is>
       </c>
       <c r="Q2" s="2" t="inlineStr"/>
-      <c r="R2" s="2" t="inlineStr">
+      <c r="R2" s="2" t="inlineStr"/>
+      <c r="S2" s="2" t="inlineStr">
         <is>
           <t>Viešai skelbiamas Betono centro betono mazgas Vilniuje.</t>
         </is>
       </c>
-      <c r="S2" s="4" t="n">
+      <c r="T2" s="4" t="n">
         <v>0.9</v>
       </c>
-      <c r="T2" s="5" t="n"/>
       <c r="U2" s="5" t="n"/>
-      <c r="V2" s="5" t="n"/>
+      <c r="V2" s="6" t="n"/>
       <c r="W2" s="5" t="n"/>
-      <c r="X2" s="2" t="inlineStr">
+      <c r="X2" s="5" t="n"/>
+      <c r="Y2" s="2" t="inlineStr">
         <is>
           <t>https://betonocentras.lt/</t>
         </is>
       </c>
-      <c r="Y2" s="2" t="inlineStr">
+      <c r="Z2" s="2" t="inlineStr">
         <is>
           <t>https://betonocentras.lt/kontaktai/</t>
         </is>
       </c>
-      <c r="Z2" s="2" t="inlineStr"/>
       <c r="AA2" s="2" t="inlineStr"/>
       <c r="AB2" s="2" t="inlineStr"/>
-      <c r="AC2" s="2" t="inlineStr">
+      <c r="AC2" s="2" t="inlineStr"/>
+      <c r="AD2" s="2" t="inlineStr">
         <is>
           <t>https://betonocentras.lt/kontaktai/</t>
         </is>
       </c>
-      <c r="AD2" s="2" t="inlineStr"/>
-      <c r="AE2" s="2" t="inlineStr">
+      <c r="AE2" s="2" t="inlineStr"/>
+      <c r="AF2" s="2" t="inlineStr">
         <is>
           <t>2026-06-29</t>
         </is>
@@ -883,38 +894,39 @@
         </is>
       </c>
       <c r="Q3" s="2" t="inlineStr"/>
-      <c r="R3" s="2" t="inlineStr">
+      <c r="R3" s="2" t="inlineStr"/>
+      <c r="S3" s="2" t="inlineStr">
         <is>
           <t>Viešai skelbiamas Betono centro betono mazgas Kaune.</t>
         </is>
       </c>
-      <c r="S3" s="4" t="n">
+      <c r="T3" s="4" t="n">
         <v>0.9</v>
       </c>
-      <c r="T3" s="5" t="n"/>
       <c r="U3" s="5" t="n"/>
-      <c r="V3" s="5" t="n"/>
+      <c r="V3" s="6" t="n"/>
       <c r="W3" s="5" t="n"/>
-      <c r="X3" s="2" t="inlineStr">
+      <c r="X3" s="5" t="n"/>
+      <c r="Y3" s="2" t="inlineStr">
         <is>
           <t>https://betonocentras.lt/</t>
         </is>
       </c>
-      <c r="Y3" s="2" t="inlineStr">
+      <c r="Z3" s="2" t="inlineStr">
         <is>
           <t>https://betonocentras.lt/kontaktai/</t>
         </is>
       </c>
-      <c r="Z3" s="2" t="inlineStr"/>
       <c r="AA3" s="2" t="inlineStr"/>
       <c r="AB3" s="2" t="inlineStr"/>
-      <c r="AC3" s="2" t="inlineStr">
+      <c r="AC3" s="2" t="inlineStr"/>
+      <c r="AD3" s="2" t="inlineStr">
         <is>
           <t>https://betonocentras.lt/kontaktai/</t>
         </is>
       </c>
-      <c r="AD3" s="2" t="inlineStr"/>
-      <c r="AE3" s="2" t="inlineStr">
+      <c r="AE3" s="2" t="inlineStr"/>
+      <c r="AF3" s="2" t="inlineStr">
         <is>
           <t>2026-06-29</t>
         </is>
@@ -998,42 +1010,43 @@
         </is>
       </c>
       <c r="Q4" s="2" t="inlineStr"/>
-      <c r="R4" s="2" t="inlineStr">
+      <c r="R4" s="2" t="inlineStr"/>
+      <c r="S4" s="2" t="inlineStr">
         <is>
           <t>Viešai skelbiamas Betono centro betono mazgas Klaipėdoje.</t>
         </is>
       </c>
-      <c r="S4" s="4" t="n">
+      <c r="T4" s="4" t="n">
         <v>0.9</v>
       </c>
-      <c r="T4" s="5" t="n"/>
       <c r="U4" s="5" t="n"/>
-      <c r="V4" s="5" t="n"/>
+      <c r="V4" s="6" t="n"/>
       <c r="W4" s="5" t="n"/>
-      <c r="X4" s="2" t="inlineStr">
+      <c r="X4" s="5" t="n"/>
+      <c r="Y4" s="2" t="inlineStr">
         <is>
           <t>https://betonocentras.lt/</t>
         </is>
       </c>
-      <c r="Y4" s="2" t="inlineStr">
+      <c r="Z4" s="2" t="inlineStr">
         <is>
           <t>https://spsc.lt/registrai/regsapp/ser_produktai_view.php?editid1=13020</t>
         </is>
       </c>
-      <c r="Z4" s="2" t="inlineStr"/>
       <c r="AA4" s="2" t="inlineStr"/>
       <c r="AB4" s="2" t="inlineStr"/>
-      <c r="AC4" s="2" t="inlineStr">
+      <c r="AC4" s="2" t="inlineStr"/>
+      <c r="AD4" s="2" t="inlineStr">
         <is>
           <t>https://spsc.lt/registrai/regsapp/ser_produktai_view.php?editid1=13020</t>
         </is>
       </c>
-      <c r="AD4" s="2" t="inlineStr">
+      <c r="AE4" s="2" t="inlineStr">
         <is>
           <t>Adresas ir koordinatės patikslinti pagal Google Maps ir SPSC registro įrašą.</t>
         </is>
       </c>
-      <c r="AE4" s="2" t="inlineStr">
+      <c r="AF4" s="2" t="inlineStr">
         <is>
           <t>2026-06-30</t>
         </is>
@@ -1117,38 +1130,39 @@
         </is>
       </c>
       <c r="Q5" s="2" t="inlineStr"/>
-      <c r="R5" s="2" t="inlineStr">
+      <c r="R5" s="2" t="inlineStr"/>
+      <c r="S5" s="2" t="inlineStr">
         <is>
           <t>Viešai skelbiamas Betono centro betono mazgas Šiauliuose.</t>
         </is>
       </c>
-      <c r="S5" s="4" t="n">
+      <c r="T5" s="4" t="n">
         <v>0.9</v>
       </c>
-      <c r="T5" s="5" t="n"/>
       <c r="U5" s="5" t="n"/>
-      <c r="V5" s="5" t="n"/>
+      <c r="V5" s="6" t="n"/>
       <c r="W5" s="5" t="n"/>
-      <c r="X5" s="2" t="inlineStr">
+      <c r="X5" s="5" t="n"/>
+      <c r="Y5" s="2" t="inlineStr">
         <is>
           <t>https://betonocentras.lt/</t>
         </is>
       </c>
-      <c r="Y5" s="2" t="inlineStr">
+      <c r="Z5" s="2" t="inlineStr">
         <is>
           <t>https://betonocentras.lt/kontaktai/</t>
         </is>
       </c>
-      <c r="Z5" s="2" t="inlineStr"/>
       <c r="AA5" s="2" t="inlineStr"/>
       <c r="AB5" s="2" t="inlineStr"/>
-      <c r="AC5" s="2" t="inlineStr">
+      <c r="AC5" s="2" t="inlineStr"/>
+      <c r="AD5" s="2" t="inlineStr">
         <is>
           <t>https://betonocentras.lt/kontaktai/</t>
         </is>
       </c>
-      <c r="AD5" s="2" t="inlineStr"/>
-      <c r="AE5" s="2" t="inlineStr">
+      <c r="AE5" s="2" t="inlineStr"/>
+      <c r="AF5" s="2" t="inlineStr">
         <is>
           <t>2026-06-29</t>
         </is>
@@ -1232,38 +1246,39 @@
         </is>
       </c>
       <c r="Q6" s="2" t="inlineStr"/>
-      <c r="R6" s="2" t="inlineStr">
+      <c r="R6" s="2" t="inlineStr"/>
+      <c r="S6" s="2" t="inlineStr">
         <is>
           <t>Viešai skelbiamas Betono centro betono mazgas Mažeikiuose.</t>
         </is>
       </c>
-      <c r="S6" s="4" t="n">
+      <c r="T6" s="4" t="n">
         <v>0.9</v>
       </c>
-      <c r="T6" s="5" t="n"/>
       <c r="U6" s="5" t="n"/>
-      <c r="V6" s="5" t="n"/>
+      <c r="V6" s="6" t="n"/>
       <c r="W6" s="5" t="n"/>
-      <c r="X6" s="2" t="inlineStr">
+      <c r="X6" s="5" t="n"/>
+      <c r="Y6" s="2" t="inlineStr">
         <is>
           <t>https://betonocentras.lt/</t>
         </is>
       </c>
-      <c r="Y6" s="2" t="inlineStr">
+      <c r="Z6" s="2" t="inlineStr">
         <is>
           <t>https://betonocentras.lt/kontaktai/</t>
         </is>
       </c>
-      <c r="Z6" s="2" t="inlineStr"/>
       <c r="AA6" s="2" t="inlineStr"/>
       <c r="AB6" s="2" t="inlineStr"/>
-      <c r="AC6" s="2" t="inlineStr">
+      <c r="AC6" s="2" t="inlineStr"/>
+      <c r="AD6" s="2" t="inlineStr">
         <is>
           <t>https://betonocentras.lt/kontaktai/</t>
         </is>
       </c>
-      <c r="AD6" s="2" t="inlineStr"/>
-      <c r="AE6" s="2" t="inlineStr">
+      <c r="AE6" s="2" t="inlineStr"/>
+      <c r="AF6" s="2" t="inlineStr">
         <is>
           <t>2026-06-29</t>
         </is>
@@ -1347,38 +1362,39 @@
         </is>
       </c>
       <c r="Q7" s="2" t="inlineStr"/>
-      <c r="R7" s="2" t="inlineStr">
+      <c r="R7" s="2" t="inlineStr"/>
+      <c r="S7" s="2" t="inlineStr">
         <is>
           <t>Viešai skelbiamas Betono centro betono mazgas Panevėžyje.</t>
         </is>
       </c>
-      <c r="S7" s="4" t="n">
+      <c r="T7" s="4" t="n">
         <v>0.9</v>
       </c>
-      <c r="T7" s="5" t="n"/>
       <c r="U7" s="5" t="n"/>
-      <c r="V7" s="5" t="n"/>
+      <c r="V7" s="6" t="n"/>
       <c r="W7" s="5" t="n"/>
-      <c r="X7" s="2" t="inlineStr">
+      <c r="X7" s="5" t="n"/>
+      <c r="Y7" s="2" t="inlineStr">
         <is>
           <t>https://betonocentras.lt/</t>
         </is>
       </c>
-      <c r="Y7" s="2" t="inlineStr">
+      <c r="Z7" s="2" t="inlineStr">
         <is>
           <t>https://betonocentras.lt/kontaktai/</t>
         </is>
       </c>
-      <c r="Z7" s="2" t="inlineStr"/>
       <c r="AA7" s="2" t="inlineStr"/>
       <c r="AB7" s="2" t="inlineStr"/>
-      <c r="AC7" s="2" t="inlineStr">
+      <c r="AC7" s="2" t="inlineStr"/>
+      <c r="AD7" s="2" t="inlineStr">
         <is>
           <t>https://betonocentras.lt/kontaktai/</t>
         </is>
       </c>
-      <c r="AD7" s="2" t="inlineStr"/>
-      <c r="AE7" s="2" t="inlineStr">
+      <c r="AE7" s="2" t="inlineStr"/>
+      <c r="AF7" s="2" t="inlineStr">
         <is>
           <t>2026-06-29</t>
         </is>
@@ -1462,38 +1478,39 @@
         </is>
       </c>
       <c r="Q8" s="2" t="inlineStr"/>
-      <c r="R8" s="2" t="inlineStr">
+      <c r="R8" s="2" t="inlineStr"/>
+      <c r="S8" s="2" t="inlineStr">
         <is>
           <t>Viešai skelbiamas Heidelberg Materials betono gamyklų tinklo taškas Vilniuje.</t>
         </is>
       </c>
-      <c r="S8" s="4" t="n">
+      <c r="T8" s="4" t="n">
         <v>0.85</v>
       </c>
-      <c r="T8" s="5" t="n"/>
       <c r="U8" s="5" t="n"/>
-      <c r="V8" s="5" t="n"/>
+      <c r="V8" s="6" t="n"/>
       <c r="W8" s="5" t="n"/>
-      <c r="X8" s="2" t="inlineStr">
+      <c r="X8" s="5" t="n"/>
+      <c r="Y8" s="2" t="inlineStr">
         <is>
           <t>https://www.heidelbergmaterials.lt/</t>
         </is>
       </c>
-      <c r="Y8" s="2" t="inlineStr">
+      <c r="Z8" s="2" t="inlineStr">
         <is>
           <t>https://www.heidelbergmaterials.lt/</t>
         </is>
       </c>
-      <c r="Z8" s="2" t="inlineStr"/>
       <c r="AA8" s="2" t="inlineStr"/>
       <c r="AB8" s="2" t="inlineStr"/>
-      <c r="AC8" s="2" t="inlineStr">
+      <c r="AC8" s="2" t="inlineStr"/>
+      <c r="AD8" s="2" t="inlineStr">
         <is>
           <t>https://www.heidelbergmaterials.lt/</t>
         </is>
       </c>
-      <c r="AD8" s="2" t="inlineStr"/>
-      <c r="AE8" s="2" t="inlineStr">
+      <c r="AE8" s="2" t="inlineStr"/>
+      <c r="AF8" s="2" t="inlineStr">
         <is>
           <t>2026-06-29</t>
         </is>
@@ -1577,38 +1594,39 @@
         </is>
       </c>
       <c r="Q9" s="2" t="inlineStr"/>
-      <c r="R9" s="2" t="inlineStr">
+      <c r="R9" s="2" t="inlineStr"/>
+      <c r="S9" s="2" t="inlineStr">
         <is>
           <t>Viešai skelbiamas Heidelberg Materials betono gamyklų tinklo taškas Vilniuje.</t>
         </is>
       </c>
-      <c r="S9" s="4" t="n">
+      <c r="T9" s="4" t="n">
         <v>0.85</v>
       </c>
-      <c r="T9" s="5" t="n"/>
       <c r="U9" s="5" t="n"/>
-      <c r="V9" s="5" t="n"/>
+      <c r="V9" s="6" t="n"/>
       <c r="W9" s="5" t="n"/>
-      <c r="X9" s="2" t="inlineStr">
+      <c r="X9" s="5" t="n"/>
+      <c r="Y9" s="2" t="inlineStr">
         <is>
           <t>https://www.heidelbergmaterials.lt/</t>
         </is>
       </c>
-      <c r="Y9" s="2" t="inlineStr">
+      <c r="Z9" s="2" t="inlineStr">
         <is>
           <t>https://www.heidelbergmaterials.lt/</t>
         </is>
       </c>
-      <c r="Z9" s="2" t="inlineStr"/>
       <c r="AA9" s="2" t="inlineStr"/>
       <c r="AB9" s="2" t="inlineStr"/>
-      <c r="AC9" s="2" t="inlineStr">
+      <c r="AC9" s="2" t="inlineStr"/>
+      <c r="AD9" s="2" t="inlineStr">
         <is>
           <t>https://www.heidelbergmaterials.lt/</t>
         </is>
       </c>
-      <c r="AD9" s="2" t="inlineStr"/>
-      <c r="AE9" s="2" t="inlineStr">
+      <c r="AE9" s="2" t="inlineStr"/>
+      <c r="AF9" s="2" t="inlineStr">
         <is>
           <t>2026-06-29</t>
         </is>
@@ -1692,38 +1710,39 @@
         </is>
       </c>
       <c r="Q10" s="2" t="inlineStr"/>
-      <c r="R10" s="2" t="inlineStr">
+      <c r="R10" s="2" t="inlineStr"/>
+      <c r="S10" s="2" t="inlineStr">
         <is>
           <t>Viešai skelbiamas Heidelberg Materials betono gamyklų tinklo taškas Kaune.</t>
         </is>
       </c>
-      <c r="S10" s="4" t="n">
+      <c r="T10" s="4" t="n">
         <v>0.85</v>
       </c>
-      <c r="T10" s="5" t="n"/>
       <c r="U10" s="5" t="n"/>
-      <c r="V10" s="5" t="n"/>
+      <c r="V10" s="6" t="n"/>
       <c r="W10" s="5" t="n"/>
-      <c r="X10" s="2" t="inlineStr">
+      <c r="X10" s="5" t="n"/>
+      <c r="Y10" s="2" t="inlineStr">
         <is>
           <t>https://www.heidelbergmaterials.lt/</t>
         </is>
       </c>
-      <c r="Y10" s="2" t="inlineStr">
+      <c r="Z10" s="2" t="inlineStr">
         <is>
           <t>https://www.heidelbergmaterials.lt/</t>
         </is>
       </c>
-      <c r="Z10" s="2" t="inlineStr"/>
       <c r="AA10" s="2" t="inlineStr"/>
       <c r="AB10" s="2" t="inlineStr"/>
-      <c r="AC10" s="2" t="inlineStr">
+      <c r="AC10" s="2" t="inlineStr"/>
+      <c r="AD10" s="2" t="inlineStr">
         <is>
           <t>https://www.heidelbergmaterials.lt/</t>
         </is>
       </c>
-      <c r="AD10" s="2" t="inlineStr"/>
-      <c r="AE10" s="2" t="inlineStr">
+      <c r="AE10" s="2" t="inlineStr"/>
+      <c r="AF10" s="2" t="inlineStr">
         <is>
           <t>2026-06-29</t>
         </is>
@@ -1807,38 +1826,39 @@
         </is>
       </c>
       <c r="Q11" s="2" t="inlineStr"/>
-      <c r="R11" s="2" t="inlineStr">
+      <c r="R11" s="2" t="inlineStr"/>
+      <c r="S11" s="2" t="inlineStr">
         <is>
           <t>Viešai skelbiamas Heidelberg Materials betono gamyklų tinklo taškas Klaipėdoje.</t>
         </is>
       </c>
-      <c r="S11" s="4" t="n">
+      <c r="T11" s="4" t="n">
         <v>0.85</v>
       </c>
-      <c r="T11" s="5" t="n"/>
       <c r="U11" s="5" t="n"/>
-      <c r="V11" s="5" t="n"/>
+      <c r="V11" s="6" t="n"/>
       <c r="W11" s="5" t="n"/>
-      <c r="X11" s="2" t="inlineStr">
+      <c r="X11" s="5" t="n"/>
+      <c r="Y11" s="2" t="inlineStr">
         <is>
           <t>https://www.heidelbergmaterials.lt/</t>
         </is>
       </c>
-      <c r="Y11" s="2" t="inlineStr">
+      <c r="Z11" s="2" t="inlineStr">
         <is>
           <t>https://www.heidelbergmaterials.lt/</t>
         </is>
       </c>
-      <c r="Z11" s="2" t="inlineStr"/>
       <c r="AA11" s="2" t="inlineStr"/>
       <c r="AB11" s="2" t="inlineStr"/>
-      <c r="AC11" s="2" t="inlineStr">
+      <c r="AC11" s="2" t="inlineStr"/>
+      <c r="AD11" s="2" t="inlineStr">
         <is>
           <t>https://www.heidelbergmaterials.lt/</t>
         </is>
       </c>
-      <c r="AD11" s="2" t="inlineStr"/>
-      <c r="AE11" s="2" t="inlineStr">
+      <c r="AE11" s="2" t="inlineStr"/>
+      <c r="AF11" s="2" t="inlineStr">
         <is>
           <t>2026-06-29</t>
         </is>
@@ -1922,38 +1942,39 @@
         </is>
       </c>
       <c r="Q12" s="2" t="inlineStr"/>
-      <c r="R12" s="2" t="inlineStr">
+      <c r="R12" s="2" t="inlineStr"/>
+      <c r="S12" s="2" t="inlineStr">
         <is>
           <t>Viešai skelbiamas Heidelberg Materials betono gamyklų tinklo taškas Alytuje.</t>
         </is>
       </c>
-      <c r="S12" s="4" t="n">
+      <c r="T12" s="4" t="n">
         <v>0.85</v>
       </c>
-      <c r="T12" s="5" t="n"/>
       <c r="U12" s="5" t="n"/>
-      <c r="V12" s="5" t="n"/>
+      <c r="V12" s="6" t="n"/>
       <c r="W12" s="5" t="n"/>
-      <c r="X12" s="2" t="inlineStr">
+      <c r="X12" s="5" t="n"/>
+      <c r="Y12" s="2" t="inlineStr">
         <is>
           <t>https://www.heidelbergmaterials.lt/</t>
         </is>
       </c>
-      <c r="Y12" s="2" t="inlineStr">
+      <c r="Z12" s="2" t="inlineStr">
         <is>
           <t>https://www.heidelbergmaterials.lt/</t>
         </is>
       </c>
-      <c r="Z12" s="2" t="inlineStr"/>
       <c r="AA12" s="2" t="inlineStr"/>
       <c r="AB12" s="2" t="inlineStr"/>
-      <c r="AC12" s="2" t="inlineStr">
+      <c r="AC12" s="2" t="inlineStr"/>
+      <c r="AD12" s="2" t="inlineStr">
         <is>
           <t>https://www.heidelbergmaterials.lt/</t>
         </is>
       </c>
-      <c r="AD12" s="2" t="inlineStr"/>
-      <c r="AE12" s="2" t="inlineStr">
+      <c r="AE12" s="2" t="inlineStr"/>
+      <c r="AF12" s="2" t="inlineStr">
         <is>
           <t>2026-06-29</t>
         </is>
@@ -2037,42 +2058,43 @@
         </is>
       </c>
       <c r="Q13" s="2" t="inlineStr"/>
-      <c r="R13" s="2" t="inlineStr">
+      <c r="R13" s="2" t="inlineStr"/>
+      <c r="S13" s="2" t="inlineStr">
         <is>
           <t>Viešai skelbiamas Heidelberg Materials betono gamyklų tinklo taškas Pasvalyje.</t>
         </is>
       </c>
-      <c r="S13" s="4" t="n">
+      <c r="T13" s="4" t="n">
         <v>0.8</v>
       </c>
-      <c r="T13" s="5" t="n"/>
       <c r="U13" s="5" t="n"/>
-      <c r="V13" s="5" t="n"/>
+      <c r="V13" s="6" t="n"/>
       <c r="W13" s="5" t="n"/>
-      <c r="X13" s="2" t="inlineStr">
+      <c r="X13" s="5" t="n"/>
+      <c r="Y13" s="2" t="inlineStr">
         <is>
           <t>https://www.heidelbergmaterials.lt/</t>
         </is>
       </c>
-      <c r="Y13" s="2" t="inlineStr">
+      <c r="Z13" s="2" t="inlineStr">
         <is>
           <t>https://www.heidelbergmaterials.lt/</t>
         </is>
       </c>
-      <c r="Z13" s="2" t="inlineStr"/>
       <c r="AA13" s="2" t="inlineStr"/>
       <c r="AB13" s="2" t="inlineStr"/>
-      <c r="AC13" s="2" t="inlineStr">
+      <c r="AC13" s="2" t="inlineStr"/>
+      <c r="AD13" s="2" t="inlineStr">
         <is>
           <t>https://www.heidelbergmaterials.lt/</t>
         </is>
       </c>
-      <c r="AD13" s="2" t="inlineStr">
+      <c r="AE13" s="2" t="inlineStr">
         <is>
           <t>Koordinatės patikrintos Lietuvos geolokatoriumi, bet rastas tik gatvės arba vietovės lygio taškas.</t>
         </is>
       </c>
-      <c r="AE13" s="2" t="inlineStr">
+      <c r="AF13" s="2" t="inlineStr">
         <is>
           <t>2026-06-29</t>
         </is>
@@ -2156,38 +2178,39 @@
         </is>
       </c>
       <c r="Q14" s="2" t="inlineStr"/>
-      <c r="R14" s="2" t="inlineStr">
+      <c r="R14" s="2" t="inlineStr"/>
+      <c r="S14" s="2" t="inlineStr">
         <is>
           <t>Viešai skelbiamas betono mišinių tiekėjas Vilniaus regione.</t>
         </is>
       </c>
-      <c r="S14" s="4" t="n">
+      <c r="T14" s="4" t="n">
         <v>0.8</v>
       </c>
-      <c r="T14" s="5" t="n"/>
       <c r="U14" s="5" t="n"/>
-      <c r="V14" s="5" t="n"/>
+      <c r="V14" s="6" t="n"/>
       <c r="W14" s="5" t="n"/>
-      <c r="X14" s="2" t="inlineStr">
+      <c r="X14" s="5" t="n"/>
+      <c r="Y14" s="2" t="inlineStr">
         <is>
           <t>https://www.palmusta.lt/</t>
         </is>
       </c>
-      <c r="Y14" s="2" t="inlineStr">
+      <c r="Z14" s="2" t="inlineStr">
         <is>
           <t>https://www.palmusta.lt/</t>
         </is>
       </c>
-      <c r="Z14" s="2" t="inlineStr"/>
       <c r="AA14" s="2" t="inlineStr"/>
       <c r="AB14" s="2" t="inlineStr"/>
-      <c r="AC14" s="2" t="inlineStr">
+      <c r="AC14" s="2" t="inlineStr"/>
+      <c r="AD14" s="2" t="inlineStr">
         <is>
           <t>https://www.palmusta.lt/</t>
         </is>
       </c>
-      <c r="AD14" s="2" t="inlineStr"/>
-      <c r="AE14" s="2" t="inlineStr">
+      <c r="AE14" s="2" t="inlineStr"/>
+      <c r="AF14" s="2" t="inlineStr">
         <is>
           <t>2026-06-29</t>
         </is>
@@ -2267,38 +2290,39 @@
         </is>
       </c>
       <c r="Q15" s="2" t="inlineStr"/>
-      <c r="R15" s="2" t="inlineStr">
+      <c r="R15" s="2" t="inlineStr"/>
+      <c r="S15" s="2" t="inlineStr">
         <is>
           <t>Gelžbetoninių konstrukcijų gamyba Vilniuje.</t>
         </is>
       </c>
-      <c r="S15" s="4" t="n">
+      <c r="T15" s="4" t="n">
         <v>0.9</v>
       </c>
-      <c r="T15" s="5" t="n"/>
       <c r="U15" s="5" t="n"/>
-      <c r="V15" s="5" t="n"/>
+      <c r="V15" s="6" t="n"/>
       <c r="W15" s="5" t="n"/>
-      <c r="X15" s="2" t="inlineStr">
+      <c r="X15" s="5" t="n"/>
+      <c r="Y15" s="2" t="inlineStr">
         <is>
           <t>https://www.gkg3.lt/</t>
         </is>
       </c>
-      <c r="Y15" s="2" t="inlineStr">
+      <c r="Z15" s="2" t="inlineStr">
         <is>
           <t>https://www.gkg3.lt/</t>
         </is>
       </c>
-      <c r="Z15" s="2" t="inlineStr"/>
       <c r="AA15" s="2" t="inlineStr"/>
       <c r="AB15" s="2" t="inlineStr"/>
-      <c r="AC15" s="2" t="inlineStr">
+      <c r="AC15" s="2" t="inlineStr"/>
+      <c r="AD15" s="2" t="inlineStr">
         <is>
           <t>https://www.gkg3.lt/</t>
         </is>
       </c>
-      <c r="AD15" s="2" t="inlineStr"/>
-      <c r="AE15" s="2" t="inlineStr">
+      <c r="AE15" s="2" t="inlineStr"/>
+      <c r="AF15" s="2" t="inlineStr">
         <is>
           <t>2026-06-29</t>
         </is>
@@ -2382,38 +2406,39 @@
           <t>150 m³/val.</t>
         </is>
       </c>
-      <c r="R16" s="2" t="inlineStr">
+      <c r="R16" s="2" t="inlineStr"/>
+      <c r="S16" s="2" t="inlineStr">
         <is>
           <t>Viešai nurodoma nauja gelžbetonio elementų gamybos linija, kurios našumas 150 m³/val.</t>
         </is>
       </c>
-      <c r="S16" s="4" t="n">
+      <c r="T16" s="4" t="n">
         <v>0.9</v>
       </c>
-      <c r="T16" s="5" t="n"/>
       <c r="U16" s="5" t="n"/>
-      <c r="V16" s="5" t="n"/>
+      <c r="V16" s="6" t="n"/>
       <c r="W16" s="5" t="n"/>
-      <c r="X16" s="2" t="inlineStr">
+      <c r="X16" s="5" t="n"/>
+      <c r="Y16" s="2" t="inlineStr">
         <is>
           <t>https://www.perdanga.lt/</t>
         </is>
       </c>
-      <c r="Y16" s="2" t="inlineStr">
+      <c r="Z16" s="2" t="inlineStr">
         <is>
           <t>https://www.perdanga.lt/</t>
         </is>
       </c>
-      <c r="Z16" s="2" t="inlineStr"/>
       <c r="AA16" s="2" t="inlineStr"/>
       <c r="AB16" s="2" t="inlineStr"/>
-      <c r="AC16" s="2" t="inlineStr">
+      <c r="AC16" s="2" t="inlineStr"/>
+      <c r="AD16" s="2" t="inlineStr">
         <is>
           <t>https://www.perdanga.lt/</t>
         </is>
       </c>
-      <c r="AD16" s="2" t="inlineStr"/>
-      <c r="AE16" s="2" t="inlineStr">
+      <c r="AE16" s="2" t="inlineStr"/>
+      <c r="AF16" s="2" t="inlineStr">
         <is>
           <t>2026-06-29</t>
         </is>
@@ -2493,38 +2518,39 @@
         </is>
       </c>
       <c r="Q17" s="2" t="inlineStr"/>
-      <c r="R17" s="2" t="inlineStr">
+      <c r="R17" s="2" t="inlineStr"/>
+      <c r="S17" s="2" t="inlineStr">
         <is>
           <t>Viešai skelbiamas Perdangos padalinys Klaipėdoje.</t>
         </is>
       </c>
-      <c r="S17" s="4" t="n">
+      <c r="T17" s="4" t="n">
         <v>0.85</v>
       </c>
-      <c r="T17" s="5" t="n"/>
       <c r="U17" s="5" t="n"/>
-      <c r="V17" s="5" t="n"/>
+      <c r="V17" s="6" t="n"/>
       <c r="W17" s="5" t="n"/>
-      <c r="X17" s="2" t="inlineStr">
+      <c r="X17" s="5" t="n"/>
+      <c r="Y17" s="2" t="inlineStr">
         <is>
           <t>https://www.perdanga.lt/</t>
         </is>
       </c>
-      <c r="Y17" s="2" t="inlineStr">
+      <c r="Z17" s="2" t="inlineStr">
         <is>
           <t>https://www.perdanga.lt/</t>
         </is>
       </c>
-      <c r="Z17" s="2" t="inlineStr"/>
       <c r="AA17" s="2" t="inlineStr"/>
       <c r="AB17" s="2" t="inlineStr"/>
-      <c r="AC17" s="2" t="inlineStr">
+      <c r="AC17" s="2" t="inlineStr"/>
+      <c r="AD17" s="2" t="inlineStr">
         <is>
           <t>https://www.perdanga.lt/</t>
         </is>
       </c>
-      <c r="AD17" s="2" t="inlineStr"/>
-      <c r="AE17" s="2" t="inlineStr">
+      <c r="AE17" s="2" t="inlineStr"/>
+      <c r="AF17" s="2" t="inlineStr">
         <is>
           <t>2026-06-29</t>
         </is>
@@ -2604,34 +2630,35 @@
         </is>
       </c>
       <c r="Q18" s="2" t="inlineStr"/>
-      <c r="R18" s="2" t="inlineStr">
+      <c r="R18" s="2" t="inlineStr"/>
+      <c r="S18" s="2" t="inlineStr">
         <is>
           <t>Viešai skelbiamas gelžbetonio gamintojas Kaune.</t>
         </is>
       </c>
-      <c r="S18" s="4" t="n">
+      <c r="T18" s="4" t="n">
         <v>0.8</v>
       </c>
-      <c r="T18" s="5" t="n"/>
       <c r="U18" s="5" t="n"/>
-      <c r="V18" s="5" t="n"/>
+      <c r="V18" s="6" t="n"/>
       <c r="W18" s="5" t="n"/>
-      <c r="X18" s="2" t="inlineStr"/>
-      <c r="Y18" s="2" t="inlineStr">
+      <c r="X18" s="5" t="n"/>
+      <c r="Y18" s="2" t="inlineStr"/>
+      <c r="Z18" s="2" t="inlineStr">
         <is>
           <t>https://www.kaunogelzbetonis.lt/</t>
         </is>
       </c>
-      <c r="Z18" s="2" t="inlineStr"/>
       <c r="AA18" s="2" t="inlineStr"/>
       <c r="AB18" s="2" t="inlineStr"/>
-      <c r="AC18" s="2" t="inlineStr">
+      <c r="AC18" s="2" t="inlineStr"/>
+      <c r="AD18" s="2" t="inlineStr">
         <is>
           <t>https://www.kaunogelzbetonis.lt/</t>
         </is>
       </c>
-      <c r="AD18" s="2" t="inlineStr"/>
-      <c r="AE18" s="2" t="inlineStr">
+      <c r="AE18" s="2" t="inlineStr"/>
+      <c r="AF18" s="2" t="inlineStr">
         <is>
           <t>2026-06-29</t>
         </is>
@@ -2711,34 +2738,35 @@
         </is>
       </c>
       <c r="Q19" s="2" t="inlineStr"/>
-      <c r="R19" s="2" t="inlineStr">
+      <c r="R19" s="2" t="inlineStr"/>
+      <c r="S19" s="2" t="inlineStr">
         <is>
           <t>Viešai skelbiamas gelžbetonio gamintojas Ukmergėje.</t>
         </is>
       </c>
-      <c r="S19" s="4" t="n">
+      <c r="T19" s="4" t="n">
         <v>0.8</v>
       </c>
-      <c r="T19" s="5" t="n"/>
       <c r="U19" s="5" t="n"/>
-      <c r="V19" s="5" t="n"/>
+      <c r="V19" s="6" t="n"/>
       <c r="W19" s="5" t="n"/>
-      <c r="X19" s="2" t="inlineStr"/>
-      <c r="Y19" s="2" t="inlineStr">
+      <c r="X19" s="5" t="n"/>
+      <c r="Y19" s="2" t="inlineStr"/>
+      <c r="Z19" s="2" t="inlineStr">
         <is>
           <t>https://ukmergesgelzbetonis.lt/</t>
         </is>
       </c>
-      <c r="Z19" s="2" t="inlineStr"/>
       <c r="AA19" s="2" t="inlineStr"/>
       <c r="AB19" s="2" t="inlineStr"/>
-      <c r="AC19" s="2" t="inlineStr">
+      <c r="AC19" s="2" t="inlineStr"/>
+      <c r="AD19" s="2" t="inlineStr">
         <is>
           <t>https://ukmergesgelzbetonis.lt/</t>
         </is>
       </c>
-      <c r="AD19" s="2" t="inlineStr"/>
-      <c r="AE19" s="2" t="inlineStr">
+      <c r="AE19" s="2" t="inlineStr"/>
+      <c r="AF19" s="2" t="inlineStr">
         <is>
           <t>2026-06-29</t>
         </is>
@@ -2818,38 +2846,39 @@
         </is>
       </c>
       <c r="Q20" s="2" t="inlineStr"/>
-      <c r="R20" s="2" t="inlineStr">
+      <c r="R20" s="2" t="inlineStr"/>
+      <c r="S20" s="2" t="inlineStr">
         <is>
           <t>Viešai skelbiamas gelžbetonio gamintojas Šiauliuose.</t>
         </is>
       </c>
-      <c r="S20" s="4" t="n">
+      <c r="T20" s="4" t="n">
         <v>0.8</v>
       </c>
-      <c r="T20" s="5" t="n"/>
       <c r="U20" s="5" t="n"/>
-      <c r="V20" s="5" t="n"/>
+      <c r="V20" s="6" t="n"/>
       <c r="W20" s="5" t="n"/>
-      <c r="X20" s="2" t="inlineStr">
+      <c r="X20" s="5" t="n"/>
+      <c r="Y20" s="2" t="inlineStr">
         <is>
           <t>https://www.gelzbetonineskonstrukcijos.lt/</t>
         </is>
       </c>
-      <c r="Y20" s="2" t="inlineStr">
+      <c r="Z20" s="2" t="inlineStr">
         <is>
           <t>https://www.gelzbetonineskonstrukcijos.lt/</t>
         </is>
       </c>
-      <c r="Z20" s="2" t="inlineStr"/>
       <c r="AA20" s="2" t="inlineStr"/>
       <c r="AB20" s="2" t="inlineStr"/>
-      <c r="AC20" s="2" t="inlineStr">
+      <c r="AC20" s="2" t="inlineStr"/>
+      <c r="AD20" s="2" t="inlineStr">
         <is>
           <t>https://www.gelzbetonineskonstrukcijos.lt/</t>
         </is>
       </c>
-      <c r="AD20" s="2" t="inlineStr"/>
-      <c r="AE20" s="2" t="inlineStr">
+      <c r="AE20" s="2" t="inlineStr"/>
+      <c r="AF20" s="2" t="inlineStr">
         <is>
           <t>2026-06-29</t>
         </is>
@@ -2929,38 +2958,39 @@
         </is>
       </c>
       <c r="Q21" s="2" t="inlineStr"/>
-      <c r="R21" s="2" t="inlineStr">
+      <c r="R21" s="2" t="inlineStr"/>
+      <c r="S21" s="2" t="inlineStr">
         <is>
           <t>Viešai skelbiamas surenkamojo gelžbetonio konstrukcijų gamintojas.</t>
         </is>
       </c>
-      <c r="S21" s="4" t="n">
+      <c r="T21" s="4" t="n">
         <v>0.8</v>
       </c>
-      <c r="T21" s="5" t="n"/>
       <c r="U21" s="5" t="n"/>
-      <c r="V21" s="5" t="n"/>
+      <c r="V21" s="6" t="n"/>
       <c r="W21" s="5" t="n"/>
-      <c r="X21" s="2" t="inlineStr">
+      <c r="X21" s="5" t="n"/>
+      <c r="Y21" s="2" t="inlineStr">
         <is>
           <t>https://inhus.eu/</t>
         </is>
       </c>
-      <c r="Y21" s="2" t="inlineStr">
+      <c r="Z21" s="2" t="inlineStr">
         <is>
           <t>https://inhus.eu/</t>
         </is>
       </c>
-      <c r="Z21" s="2" t="inlineStr"/>
       <c r="AA21" s="2" t="inlineStr"/>
       <c r="AB21" s="2" t="inlineStr"/>
-      <c r="AC21" s="2" t="inlineStr">
+      <c r="AC21" s="2" t="inlineStr"/>
+      <c r="AD21" s="2" t="inlineStr">
         <is>
           <t>https://inhus.eu/</t>
         </is>
       </c>
-      <c r="AD21" s="2" t="inlineStr"/>
-      <c r="AE21" s="2" t="inlineStr">
+      <c r="AE21" s="2" t="inlineStr"/>
+      <c r="AF21" s="2" t="inlineStr">
         <is>
           <t>2026-06-29</t>
         </is>
@@ -3040,38 +3070,39 @@
         </is>
       </c>
       <c r="Q22" s="2" t="inlineStr"/>
-      <c r="R22" s="2" t="inlineStr">
+      <c r="R22" s="2" t="inlineStr"/>
+      <c r="S22" s="2" t="inlineStr">
         <is>
           <t>Viešai skelbiamas betono mišinių tiekėjas.</t>
         </is>
       </c>
-      <c r="S22" s="4" t="n">
+      <c r="T22" s="4" t="n">
         <v>0.75</v>
       </c>
-      <c r="T22" s="5" t="n"/>
       <c r="U22" s="5" t="n"/>
-      <c r="V22" s="5" t="n"/>
+      <c r="V22" s="6" t="n"/>
       <c r="W22" s="5" t="n"/>
-      <c r="X22" s="2" t="inlineStr">
+      <c r="X22" s="5" t="n"/>
+      <c r="Y22" s="2" t="inlineStr">
         <is>
           <t>https://gelmesta.lt/</t>
         </is>
       </c>
-      <c r="Y22" s="2" t="inlineStr">
+      <c r="Z22" s="2" t="inlineStr">
         <is>
           <t>https://gelmesta.lt/</t>
         </is>
       </c>
-      <c r="Z22" s="2" t="inlineStr"/>
       <c r="AA22" s="2" t="inlineStr"/>
       <c r="AB22" s="2" t="inlineStr"/>
-      <c r="AC22" s="2" t="inlineStr">
+      <c r="AC22" s="2" t="inlineStr"/>
+      <c r="AD22" s="2" t="inlineStr">
         <is>
           <t>https://gelmesta.lt/</t>
         </is>
       </c>
-      <c r="AD22" s="2" t="inlineStr"/>
-      <c r="AE22" s="2" t="inlineStr">
+      <c r="AE22" s="2" t="inlineStr"/>
+      <c r="AF22" s="2" t="inlineStr">
         <is>
           <t>2026-06-29</t>
         </is>
@@ -3155,38 +3186,39 @@
           <t>iki 200 m³ per darbo pamainą</t>
         </is>
       </c>
-      <c r="R23" s="2" t="inlineStr">
+      <c r="R23" s="2" t="inlineStr"/>
+      <c r="S23" s="2" t="inlineStr">
         <is>
           <t>Viešai skelbiamas betono mišinių gamintojas; nurodomas našumas iki 200 m³ per darbo pamainą.</t>
         </is>
       </c>
-      <c r="S23" s="4" t="n">
+      <c r="T23" s="4" t="n">
         <v>0.75</v>
       </c>
-      <c r="T23" s="5" t="n"/>
       <c r="U23" s="5" t="n"/>
-      <c r="V23" s="5" t="n"/>
+      <c r="V23" s="6" t="n"/>
       <c r="W23" s="5" t="n"/>
-      <c r="X23" s="2" t="inlineStr">
+      <c r="X23" s="5" t="n"/>
+      <c r="Y23" s="2" t="inlineStr">
         <is>
           <t>https://www.suduvos-betonas.lt/</t>
         </is>
       </c>
-      <c r="Y23" s="2" t="inlineStr">
+      <c r="Z23" s="2" t="inlineStr">
         <is>
           <t>https://www.suduvos-betonas.lt/kontaktai/</t>
         </is>
       </c>
-      <c r="Z23" s="2" t="inlineStr"/>
       <c r="AA23" s="2" t="inlineStr"/>
       <c r="AB23" s="2" t="inlineStr"/>
-      <c r="AC23" s="2" t="inlineStr">
+      <c r="AC23" s="2" t="inlineStr"/>
+      <c r="AD23" s="2" t="inlineStr">
         <is>
           <t>https://www.suduvos-betonas.lt/</t>
         </is>
       </c>
-      <c r="AD23" s="2" t="inlineStr"/>
-      <c r="AE23" s="2" t="inlineStr">
+      <c r="AE23" s="2" t="inlineStr"/>
+      <c r="AF23" s="2" t="inlineStr">
         <is>
           <t>2026-06-29</t>
         </is>
@@ -3270,38 +3302,39 @@
         </is>
       </c>
       <c r="Q24" s="2" t="inlineStr"/>
-      <c r="R24" s="2" t="inlineStr">
+      <c r="R24" s="2" t="inlineStr"/>
+      <c r="S24" s="2" t="inlineStr">
         <is>
           <t>Viešai skelbiamas betono mišinių tiekėjas.</t>
         </is>
       </c>
-      <c r="S24" s="4" t="n">
+      <c r="T24" s="4" t="n">
         <v>0.75</v>
       </c>
-      <c r="T24" s="5" t="n"/>
       <c r="U24" s="5" t="n"/>
-      <c r="V24" s="5" t="n"/>
+      <c r="V24" s="6" t="n"/>
       <c r="W24" s="5" t="n"/>
-      <c r="X24" s="2" t="inlineStr">
+      <c r="X24" s="5" t="n"/>
+      <c r="Y24" s="2" t="inlineStr">
         <is>
           <t>https://statkasta.lt/</t>
         </is>
       </c>
-      <c r="Y24" s="2" t="inlineStr">
+      <c r="Z24" s="2" t="inlineStr">
         <is>
           <t>https://statkasta.lt/</t>
         </is>
       </c>
-      <c r="Z24" s="2" t="inlineStr"/>
       <c r="AA24" s="2" t="inlineStr"/>
       <c r="AB24" s="2" t="inlineStr"/>
-      <c r="AC24" s="2" t="inlineStr">
+      <c r="AC24" s="2" t="inlineStr"/>
+      <c r="AD24" s="2" t="inlineStr">
         <is>
           <t>https://statkasta.lt/</t>
         </is>
       </c>
-      <c r="AD24" s="2" t="inlineStr"/>
-      <c r="AE24" s="2" t="inlineStr">
+      <c r="AE24" s="2" t="inlineStr"/>
+      <c r="AF24" s="2" t="inlineStr">
         <is>
           <t>2026-06-29</t>
         </is>
@@ -3377,42 +3410,43 @@
       </c>
       <c r="P25" s="2" t="inlineStr"/>
       <c r="Q25" s="2" t="inlineStr"/>
-      <c r="R25" s="2" t="inlineStr">
+      <c r="R25" s="2" t="inlineStr"/>
+      <c r="S25" s="2" t="inlineStr">
         <is>
           <t>Viešuose šaltiniuose minima betono mišinių veikla; tikslų mazgo pavadinimą reikia patikslinti.</t>
         </is>
       </c>
-      <c r="S25" s="4" t="n">
+      <c r="T25" s="4" t="n">
         <v>0.6</v>
       </c>
-      <c r="T25" s="5" t="n"/>
       <c r="U25" s="5" t="n"/>
-      <c r="V25" s="5" t="n"/>
+      <c r="V25" s="6" t="n"/>
       <c r="W25" s="5" t="n"/>
-      <c r="X25" s="2" t="inlineStr">
+      <c r="X25" s="5" t="n"/>
+      <c r="Y25" s="2" t="inlineStr">
         <is>
           <t>https://autokausta.lt/</t>
         </is>
       </c>
-      <c r="Y25" s="2" t="inlineStr">
+      <c r="Z25" s="2" t="inlineStr">
         <is>
           <t>https://autokausta.lt/</t>
         </is>
       </c>
-      <c r="Z25" s="2" t="inlineStr"/>
       <c r="AA25" s="2" t="inlineStr"/>
       <c r="AB25" s="2" t="inlineStr"/>
-      <c r="AC25" s="2" t="inlineStr">
+      <c r="AC25" s="2" t="inlineStr"/>
+      <c r="AD25" s="2" t="inlineStr">
         <is>
           <t>https://autokausta.lt/</t>
         </is>
       </c>
-      <c r="AD25" s="2" t="inlineStr">
+      <c r="AE25" s="2" t="inlineStr">
         <is>
           <t>Betono mazgo adresas patikslintas pagal lietuviškus viešus šaltinius; koordinatės nustatytos Lietuvos geolokatoriumi.</t>
         </is>
       </c>
-      <c r="AE25" s="2" t="inlineStr">
+      <c r="AF25" s="2" t="inlineStr">
         <is>
           <t>2026-06-29</t>
         </is>
@@ -3496,42 +3530,43 @@
         </is>
       </c>
       <c r="Q26" s="2" t="inlineStr"/>
-      <c r="R26" s="2" t="inlineStr">
+      <c r="R26" s="2" t="inlineStr"/>
+      <c r="S26" s="2" t="inlineStr">
         <is>
           <t>Viešuose šaltiniuose minima betono mišinių veikla; tikslų mazgo adresą reikia patikslinti.</t>
         </is>
       </c>
-      <c r="S26" s="4" t="n">
+      <c r="T26" s="4" t="n">
         <v>0.65</v>
       </c>
-      <c r="T26" s="5" t="n"/>
       <c r="U26" s="5" t="n"/>
-      <c r="V26" s="5" t="n"/>
+      <c r="V26" s="6" t="n"/>
       <c r="W26" s="5" t="n"/>
-      <c r="X26" s="2" t="inlineStr">
+      <c r="X26" s="5" t="n"/>
+      <c r="Y26" s="2" t="inlineStr">
         <is>
           <t>https://betonobaze.lt/</t>
         </is>
       </c>
-      <c r="Y26" s="2" t="inlineStr">
+      <c r="Z26" s="2" t="inlineStr">
         <is>
           <t>https://betonobaze.lt/</t>
         </is>
       </c>
-      <c r="Z26" s="2" t="inlineStr"/>
       <c r="AA26" s="2" t="inlineStr"/>
       <c r="AB26" s="2" t="inlineStr"/>
-      <c r="AC26" s="2" t="inlineStr">
+      <c r="AC26" s="2" t="inlineStr"/>
+      <c r="AD26" s="2" t="inlineStr">
         <is>
           <t>https://betonobaze.lt/</t>
         </is>
       </c>
-      <c r="AD26" s="2" t="inlineStr">
+      <c r="AE26" s="2" t="inlineStr">
         <is>
           <t>Adresas patikslintas pagal lietuviškus viešus šaltinius; koordinatės nustatytos Lietuvos geolokatoriumi.</t>
         </is>
       </c>
-      <c r="AE26" s="2" t="inlineStr">
+      <c r="AF26" s="2" t="inlineStr">
         <is>
           <t>2026-06-29</t>
         </is>
@@ -3611,42 +3646,43 @@
         </is>
       </c>
       <c r="Q27" s="2" t="inlineStr"/>
-      <c r="R27" s="2" t="inlineStr">
+      <c r="R27" s="2" t="inlineStr"/>
+      <c r="S27" s="2" t="inlineStr">
         <is>
           <t>Viešai skelbiamas betono mišinių tiekėjas Druskininkų regione.</t>
         </is>
       </c>
-      <c r="S27" s="4" t="n">
+      <c r="T27" s="4" t="n">
         <v>0.7</v>
       </c>
-      <c r="T27" s="5" t="n"/>
       <c r="U27" s="5" t="n"/>
-      <c r="V27" s="5" t="n"/>
+      <c r="V27" s="6" t="n"/>
       <c r="W27" s="5" t="n"/>
-      <c r="X27" s="2" t="inlineStr">
+      <c r="X27" s="5" t="n"/>
+      <c r="Y27" s="2" t="inlineStr">
         <is>
           <t>https://transdosa.lt/</t>
         </is>
       </c>
-      <c r="Y27" s="2" t="inlineStr">
+      <c r="Z27" s="2" t="inlineStr">
         <is>
           <t>https://transdosa.lt/</t>
         </is>
       </c>
-      <c r="Z27" s="2" t="inlineStr"/>
       <c r="AA27" s="2" t="inlineStr"/>
       <c r="AB27" s="2" t="inlineStr"/>
-      <c r="AC27" s="2" t="inlineStr">
+      <c r="AC27" s="2" t="inlineStr"/>
+      <c r="AD27" s="2" t="inlineStr">
         <is>
           <t>https://transdosa.lt/</t>
         </is>
       </c>
-      <c r="AD27" s="2" t="inlineStr">
+      <c r="AE27" s="2" t="inlineStr">
         <is>
           <t>Adresas patikslintas pagal lietuviškus viešus šaltinius; koordinatės nustatytos Lietuvos geolokatoriumi.</t>
         </is>
       </c>
-      <c r="AE27" s="2" t="inlineStr">
+      <c r="AF27" s="2" t="inlineStr">
         <is>
           <t>2026-06-29</t>
         </is>
@@ -3726,42 +3762,43 @@
         </is>
       </c>
       <c r="Q28" s="2" t="inlineStr"/>
-      <c r="R28" s="2" t="inlineStr">
+      <c r="R28" s="2" t="inlineStr"/>
+      <c r="S28" s="2" t="inlineStr">
         <is>
           <t>Viešai skelbiama gelžbetonio ir betono gaminių gamyba Šiauliuose.</t>
         </is>
       </c>
-      <c r="S28" s="4" t="n">
+      <c r="T28" s="4" t="n">
         <v>0.82</v>
       </c>
-      <c r="T28" s="5" t="n"/>
       <c r="U28" s="5" t="n"/>
-      <c r="V28" s="5" t="n"/>
+      <c r="V28" s="6" t="n"/>
       <c r="W28" s="5" t="n"/>
-      <c r="X28" s="2" t="inlineStr">
+      <c r="X28" s="5" t="n"/>
+      <c r="Y28" s="2" t="inlineStr">
         <is>
           <t>https://sodbeta.lt/</t>
         </is>
       </c>
-      <c r="Y28" s="2" t="inlineStr">
+      <c r="Z28" s="2" t="inlineStr">
         <is>
           <t>https://sodbeta.lt/</t>
         </is>
       </c>
-      <c r="Z28" s="2" t="inlineStr"/>
       <c r="AA28" s="2" t="inlineStr"/>
       <c r="AB28" s="2" t="inlineStr"/>
-      <c r="AC28" s="2" t="inlineStr">
+      <c r="AC28" s="2" t="inlineStr"/>
+      <c r="AD28" s="2" t="inlineStr">
         <is>
           <t>https://sodbeta.lt/</t>
         </is>
       </c>
-      <c r="AD28" s="2" t="inlineStr">
+      <c r="AE28" s="2" t="inlineStr">
         <is>
           <t>Papildomai rasta pagal požymį betono gaminiai.</t>
         </is>
       </c>
-      <c r="AE28" s="2" t="inlineStr">
+      <c r="AF28" s="2" t="inlineStr">
         <is>
           <t>2026-06-30</t>
         </is>
@@ -3845,42 +3882,43 @@
         </is>
       </c>
       <c r="Q29" s="2" t="inlineStr"/>
-      <c r="R29" s="2" t="inlineStr">
+      <c r="R29" s="2" t="inlineStr"/>
+      <c r="S29" s="2" t="inlineStr">
         <is>
           <t>Registrų centro/VDA atviruose duomenyse pagrindinė veikla nurodyta kaip prekinio betono mišinio gamyba (EVRK 23.63).</t>
         </is>
       </c>
-      <c r="S29" s="4" t="n">
+      <c r="T29" s="4" t="n">
         <v>0.85</v>
       </c>
-      <c r="T29" s="5" t="n"/>
       <c r="U29" s="5" t="n"/>
-      <c r="V29" s="5" t="n"/>
+      <c r="V29" s="6" t="n"/>
       <c r="W29" s="5" t="n"/>
-      <c r="X29" s="2" t="inlineStr">
+      <c r="X29" s="5" t="n"/>
+      <c r="Y29" s="2" t="inlineStr">
         <is>
           <t>https://alytausgelzbetonis.lt/</t>
         </is>
       </c>
-      <c r="Y29" s="2" t="inlineStr">
+      <c r="Z29" s="2" t="inlineStr">
         <is>
           <t>https://data.gov.lt/dataset/juridiniu-asmenu-ekonomines-veiklos-rusys-ir-instituciniai-sektoriai/</t>
         </is>
       </c>
-      <c r="Z29" s="2" t="inlineStr"/>
       <c r="AA29" s="2" t="inlineStr"/>
       <c r="AB29" s="2" t="inlineStr"/>
-      <c r="AC29" s="2" t="inlineStr">
+      <c r="AC29" s="2" t="inlineStr"/>
+      <c r="AD29" s="2" t="inlineStr">
         <is>
           <t>https://alytausgelzbetonis.lt/kontaktai/</t>
         </is>
       </c>
-      <c r="AD29" s="2" t="inlineStr">
+      <c r="AE29" s="2" t="inlineStr">
         <is>
           <t>Įmonė jau buvo sąraše kaip gelžbetonio gamintoja; veikla patikslinta pagal EVRK 23.63 atvirų duomenų sąrašą.</t>
         </is>
       </c>
-      <c r="AE29" s="2" t="inlineStr">
+      <c r="AF29" s="2" t="inlineStr">
         <is>
           <t>2026-06-30</t>
         </is>
@@ -3960,42 +3998,43 @@
         </is>
       </c>
       <c r="Q30" s="2" t="inlineStr"/>
-      <c r="R30" s="2" t="inlineStr">
+      <c r="R30" s="2" t="inlineStr"/>
+      <c r="S30" s="2" t="inlineStr">
         <is>
           <t>Viešai skelbiamas betono mišinių tiekėjas Marijampolėje.</t>
         </is>
       </c>
-      <c r="S30" s="4" t="n">
+      <c r="T30" s="4" t="n">
         <v>0.75</v>
       </c>
-      <c r="T30" s="5" t="n"/>
       <c r="U30" s="5" t="n"/>
-      <c r="V30" s="5" t="n"/>
+      <c r="V30" s="6" t="n"/>
       <c r="W30" s="5" t="n"/>
-      <c r="X30" s="2" t="inlineStr">
+      <c r="X30" s="5" t="n"/>
+      <c r="Y30" s="2" t="inlineStr">
         <is>
           <t>https://gernora.lt/</t>
         </is>
       </c>
-      <c r="Y30" s="2" t="inlineStr">
+      <c r="Z30" s="2" t="inlineStr">
         <is>
           <t>https://gernora.lt/</t>
         </is>
       </c>
-      <c r="Z30" s="2" t="inlineStr"/>
       <c r="AA30" s="2" t="inlineStr"/>
       <c r="AB30" s="2" t="inlineStr"/>
-      <c r="AC30" s="2" t="inlineStr">
+      <c r="AC30" s="2" t="inlineStr"/>
+      <c r="AD30" s="2" t="inlineStr">
         <is>
           <t>https://gernora.lt/</t>
         </is>
       </c>
-      <c r="AD30" s="2" t="inlineStr">
+      <c r="AE30" s="2" t="inlineStr">
         <is>
           <t>Reikia patikslinti našumą.</t>
         </is>
       </c>
-      <c r="AE30" s="2" t="inlineStr">
+      <c r="AF30" s="2" t="inlineStr">
         <is>
           <t>2026-06-30</t>
         </is>
@@ -4075,38 +4114,39 @@
         </is>
       </c>
       <c r="Q31" s="2" t="inlineStr"/>
-      <c r="R31" s="2" t="inlineStr">
+      <c r="R31" s="2" t="inlineStr"/>
+      <c r="S31" s="2" t="inlineStr">
         <is>
           <t>Viešame kataloge nurodomi betonas, cemento gaminiai, betono siurblys ir pamatų blokai Kretingoje.</t>
         </is>
       </c>
-      <c r="S31" s="4" t="n">
+      <c r="T31" s="4" t="n">
         <v>0.78</v>
       </c>
-      <c r="T31" s="5" t="n"/>
       <c r="U31" s="5" t="n"/>
-      <c r="V31" s="5" t="n"/>
+      <c r="V31" s="6" t="n"/>
       <c r="W31" s="5" t="n"/>
-      <c r="X31" s="2" t="inlineStr"/>
-      <c r="Y31" s="2" t="inlineStr">
+      <c r="X31" s="5" t="n"/>
+      <c r="Y31" s="2" t="inlineStr"/>
+      <c r="Z31" s="2" t="inlineStr">
         <is>
           <t>https://www.1551.lt/re-betono-konstrukcijos-uab-betonas-cementas-betono-siurblys-pamatu-blokai-kretingoje-104253/</t>
         </is>
       </c>
-      <c r="Z31" s="2" t="inlineStr"/>
       <c r="AA31" s="2" t="inlineStr"/>
       <c r="AB31" s="2" t="inlineStr"/>
-      <c r="AC31" s="2" t="inlineStr">
+      <c r="AC31" s="2" t="inlineStr"/>
+      <c r="AD31" s="2" t="inlineStr">
         <is>
           <t>https://www.1551.lt/re-betono-konstrukcijos-uab-betonas-cementas-betono-siurblys-pamatu-blokai-kretingoje-104253/</t>
         </is>
       </c>
-      <c r="AD31" s="2" t="inlineStr">
+      <c r="AE31" s="2" t="inlineStr">
         <is>
           <t>Katalogo šaltinis, reikia patikslinti gamybos apimtį.</t>
         </is>
       </c>
-      <c r="AE31" s="2" t="inlineStr">
+      <c r="AF31" s="2" t="inlineStr">
         <is>
           <t>2026-06-30</t>
         </is>
@@ -4186,42 +4226,43 @@
         </is>
       </c>
       <c r="Q32" s="2" t="inlineStr"/>
-      <c r="R32" s="2" t="inlineStr">
+      <c r="R32" s="2" t="inlineStr"/>
+      <c r="S32" s="2" t="inlineStr">
         <is>
           <t>Viešai skelbiama betono gaminių ir statybinių konstrukcijų veikla Šilalės rajone.</t>
         </is>
       </c>
-      <c r="S32" s="4" t="n">
+      <c r="T32" s="4" t="n">
         <v>0.72</v>
       </c>
-      <c r="T32" s="5" t="n"/>
       <c r="U32" s="5" t="n"/>
-      <c r="V32" s="5" t="n"/>
+      <c r="V32" s="6" t="n"/>
       <c r="W32" s="5" t="n"/>
-      <c r="X32" s="2" t="inlineStr">
+      <c r="X32" s="5" t="n"/>
+      <c r="Y32" s="2" t="inlineStr">
         <is>
           <t>https://www.silalesstatyba.lt/</t>
         </is>
       </c>
-      <c r="Y32" s="2" t="inlineStr">
+      <c r="Z32" s="2" t="inlineStr">
         <is>
           <t>https://www.silalesstatyba.lt/</t>
         </is>
       </c>
-      <c r="Z32" s="2" t="inlineStr"/>
       <c r="AA32" s="2" t="inlineStr"/>
       <c r="AB32" s="2" t="inlineStr"/>
-      <c r="AC32" s="2" t="inlineStr">
+      <c r="AC32" s="2" t="inlineStr"/>
+      <c r="AD32" s="2" t="inlineStr">
         <is>
           <t>https://www.silalesstatyba.lt/</t>
         </is>
       </c>
-      <c r="AD32" s="2" t="inlineStr">
+      <c r="AE32" s="2" t="inlineStr">
         <is>
           <t>Reikia patikslinti tikslų gaminių asortimentą.</t>
         </is>
       </c>
-      <c r="AE32" s="2" t="inlineStr">
+      <c r="AF32" s="2" t="inlineStr">
         <is>
           <t>2026-06-30</t>
         </is>
@@ -4301,38 +4342,39 @@
         </is>
       </c>
       <c r="Q33" s="2" t="inlineStr"/>
-      <c r="R33" s="2" t="inlineStr">
+      <c r="R33" s="2" t="inlineStr"/>
+      <c r="S33" s="2" t="inlineStr">
         <is>
           <t>Viešame įmonių kataloge nurodomas gelžbetonio gaminių profilis Panevėžyje.</t>
         </is>
       </c>
-      <c r="S33" s="4" t="n">
+      <c r="T33" s="4" t="n">
         <v>0.78</v>
       </c>
-      <c r="T33" s="5" t="n"/>
       <c r="U33" s="5" t="n"/>
-      <c r="V33" s="5" t="n"/>
+      <c r="V33" s="6" t="n"/>
       <c r="W33" s="5" t="n"/>
-      <c r="X33" s="2" t="inlineStr"/>
-      <c r="Y33" s="2" t="inlineStr">
+      <c r="X33" s="5" t="n"/>
+      <c r="Y33" s="2" t="inlineStr"/>
+      <c r="Z33" s="2" t="inlineStr">
         <is>
           <t>https://www.spec.lt/imone/panevezio-gelzbetonis-uab</t>
         </is>
       </c>
-      <c r="Z33" s="2" t="inlineStr"/>
       <c r="AA33" s="2" t="inlineStr"/>
       <c r="AB33" s="2" t="inlineStr"/>
-      <c r="AC33" s="2" t="inlineStr">
+      <c r="AC33" s="2" t="inlineStr"/>
+      <c r="AD33" s="2" t="inlineStr">
         <is>
           <t>https://www.spec.lt/imone/panevezio-gelzbetonis-uab</t>
         </is>
       </c>
-      <c r="AD33" s="2" t="inlineStr">
+      <c r="AE33" s="2" t="inlineStr">
         <is>
           <t>Reikia patikrinti veiklos aktyvumą ir produkcijos apimtį.</t>
         </is>
       </c>
-      <c r="AE33" s="2" t="inlineStr">
+      <c r="AF33" s="2" t="inlineStr">
         <is>
           <t>2026-06-30</t>
         </is>
@@ -4412,42 +4454,43 @@
         </is>
       </c>
       <c r="Q34" s="2" t="inlineStr"/>
-      <c r="R34" s="2" t="inlineStr">
+      <c r="R34" s="2" t="inlineStr"/>
+      <c r="S34" s="2" t="inlineStr">
         <is>
           <t>Viešai skelbiami pamatų ir kiti betono gaminiai Telšių rajone.</t>
         </is>
       </c>
-      <c r="S34" s="4" t="n">
+      <c r="T34" s="4" t="n">
         <v>0.72</v>
       </c>
-      <c r="T34" s="5" t="n"/>
       <c r="U34" s="5" t="n"/>
-      <c r="V34" s="5" t="n"/>
+      <c r="V34" s="6" t="n"/>
       <c r="W34" s="5" t="n"/>
-      <c r="X34" s="2" t="inlineStr">
+      <c r="X34" s="5" t="n"/>
+      <c r="Y34" s="2" t="inlineStr">
         <is>
           <t>https://pamatas.lt/</t>
         </is>
       </c>
-      <c r="Y34" s="2" t="inlineStr">
+      <c r="Z34" s="2" t="inlineStr">
         <is>
           <t>https://pamatas.lt/</t>
         </is>
       </c>
-      <c r="Z34" s="2" t="inlineStr"/>
       <c r="AA34" s="2" t="inlineStr"/>
       <c r="AB34" s="2" t="inlineStr"/>
-      <c r="AC34" s="2" t="inlineStr">
+      <c r="AC34" s="2" t="inlineStr"/>
+      <c r="AD34" s="2" t="inlineStr">
         <is>
           <t>https://pamatas.lt/</t>
         </is>
       </c>
-      <c r="AD34" s="2" t="inlineStr">
+      <c r="AE34" s="2" t="inlineStr">
         <is>
           <t>Adresas patikslintas pagal lietuvišką įmonės puslapį; koordinatės nustatytos Lietuvos geolokatoriumi.</t>
         </is>
       </c>
-      <c r="AE34" s="2" t="inlineStr">
+      <c r="AF34" s="2" t="inlineStr">
         <is>
           <t>2026-06-30</t>
         </is>
@@ -4527,42 +4570,43 @@
         </is>
       </c>
       <c r="Q35" s="2" t="inlineStr"/>
-      <c r="R35" s="2" t="inlineStr">
+      <c r="R35" s="2" t="inlineStr"/>
+      <c r="S35" s="2" t="inlineStr">
         <is>
           <t>Viešai skelbiamas HAUS blokelių ir betono gaminių gamintojas.</t>
         </is>
       </c>
-      <c r="S35" s="4" t="n">
+      <c r="T35" s="4" t="n">
         <v>0.8</v>
       </c>
-      <c r="T35" s="5" t="n"/>
       <c r="U35" s="5" t="n"/>
-      <c r="V35" s="5" t="n"/>
+      <c r="V35" s="6" t="n"/>
       <c r="W35" s="5" t="n"/>
-      <c r="X35" s="2" t="inlineStr">
+      <c r="X35" s="5" t="n"/>
+      <c r="Y35" s="2" t="inlineStr">
         <is>
           <t>https://www.vbg.lt/</t>
         </is>
       </c>
-      <c r="Y35" s="2" t="inlineStr">
+      <c r="Z35" s="2" t="inlineStr">
         <is>
           <t>https://www.vbg.lt/</t>
         </is>
       </c>
-      <c r="Z35" s="2" t="inlineStr"/>
       <c r="AA35" s="2" t="inlineStr"/>
       <c r="AB35" s="2" t="inlineStr"/>
-      <c r="AC35" s="2" t="inlineStr">
+      <c r="AC35" s="2" t="inlineStr"/>
+      <c r="AD35" s="2" t="inlineStr">
         <is>
           <t>https://www.vbg.lt/</t>
         </is>
       </c>
-      <c r="AD35" s="2" t="inlineStr">
+      <c r="AE35" s="2" t="inlineStr">
         <is>
           <t>Žemėlapyje naudotas viešai skelbiamas įmonės adresas; gamybos vietą reikia patikslinti.</t>
         </is>
       </c>
-      <c r="AE35" s="2" t="inlineStr">
+      <c r="AF35" s="2" t="inlineStr">
         <is>
           <t>2026-06-30</t>
         </is>
@@ -4642,42 +4686,43 @@
         </is>
       </c>
       <c r="Q36" s="2" t="inlineStr"/>
-      <c r="R36" s="2" t="inlineStr">
+      <c r="R36" s="2" t="inlineStr"/>
+      <c r="S36" s="2" t="inlineStr">
         <is>
           <t>Viešai skelbiama betono mišinių veikla Klaipėdos rajone.</t>
         </is>
       </c>
-      <c r="S36" s="4" t="n">
+      <c r="T36" s="4" t="n">
         <v>0.75</v>
       </c>
-      <c r="T36" s="5" t="n"/>
       <c r="U36" s="5" t="n"/>
-      <c r="V36" s="5" t="n"/>
+      <c r="V36" s="6" t="n"/>
       <c r="W36" s="5" t="n"/>
-      <c r="X36" s="2" t="inlineStr">
+      <c r="X36" s="5" t="n"/>
+      <c r="Y36" s="2" t="inlineStr">
         <is>
           <t>https://pamariogrupe.lt/</t>
         </is>
       </c>
-      <c r="Y36" s="2" t="inlineStr">
+      <c r="Z36" s="2" t="inlineStr">
         <is>
           <t>https://pamariogrupe.lt/</t>
         </is>
       </c>
-      <c r="Z36" s="2" t="inlineStr"/>
       <c r="AA36" s="2" t="inlineStr"/>
       <c r="AB36" s="2" t="inlineStr"/>
-      <c r="AC36" s="2" t="inlineStr">
+      <c r="AC36" s="2" t="inlineStr"/>
+      <c r="AD36" s="2" t="inlineStr">
         <is>
           <t>https://pamariogrupe.lt/</t>
         </is>
       </c>
-      <c r="AD36" s="2" t="inlineStr">
+      <c r="AE36" s="2" t="inlineStr">
         <is>
           <t>Reikia patikslinti našumą ir gamybos režimą.</t>
         </is>
       </c>
-      <c r="AE36" s="2" t="inlineStr">
+      <c r="AF36" s="2" t="inlineStr">
         <is>
           <t>2026-06-30</t>
         </is>
@@ -4757,42 +4802,43 @@
         </is>
       </c>
       <c r="Q37" s="2" t="inlineStr"/>
-      <c r="R37" s="2" t="inlineStr">
+      <c r="R37" s="2" t="inlineStr"/>
+      <c r="S37" s="2" t="inlineStr">
         <is>
           <t>Viešai skelbiama betono gaminių veikla Klaipėdoje.</t>
         </is>
       </c>
-      <c r="S37" s="4" t="n">
+      <c r="T37" s="4" t="n">
         <v>0.65</v>
       </c>
-      <c r="T37" s="5" t="n"/>
       <c r="U37" s="5" t="n"/>
-      <c r="V37" s="5" t="n"/>
+      <c r="V37" s="6" t="n"/>
       <c r="W37" s="5" t="n"/>
-      <c r="X37" s="2" t="inlineStr">
+      <c r="X37" s="5" t="n"/>
+      <c r="Y37" s="2" t="inlineStr">
         <is>
           <t>https://betonozona.lt/</t>
         </is>
       </c>
-      <c r="Y37" s="2" t="inlineStr">
+      <c r="Z37" s="2" t="inlineStr">
         <is>
           <t>https://betonozona.lt/</t>
         </is>
       </c>
-      <c r="Z37" s="2" t="inlineStr"/>
       <c r="AA37" s="2" t="inlineStr"/>
       <c r="AB37" s="2" t="inlineStr"/>
-      <c r="AC37" s="2" t="inlineStr">
+      <c r="AC37" s="2" t="inlineStr"/>
+      <c r="AD37" s="2" t="inlineStr">
         <is>
           <t>https://betonozona.lt/</t>
         </is>
       </c>
-      <c r="AD37" s="2" t="inlineStr">
+      <c r="AE37" s="2" t="inlineStr">
         <is>
           <t>Patikrinti, ar įmonė pati gamina, ar tik prekiauja betono gaminiais.</t>
         </is>
       </c>
-      <c r="AE37" s="2" t="inlineStr">
+      <c r="AF37" s="2" t="inlineStr">
         <is>
           <t>2026-06-30</t>
         </is>
@@ -4876,42 +4922,43 @@
         </is>
       </c>
       <c r="Q38" s="2" t="inlineStr"/>
-      <c r="R38" s="2" t="inlineStr">
+      <c r="R38" s="2" t="inlineStr"/>
+      <c r="S38" s="2" t="inlineStr">
         <is>
           <t>Viešai skelbiama betono mišinių gamyba Panevėžyje.</t>
         </is>
       </c>
-      <c r="S38" s="4" t="n">
+      <c r="T38" s="4" t="n">
         <v>0.78</v>
       </c>
-      <c r="T38" s="5" t="n"/>
       <c r="U38" s="5" t="n"/>
-      <c r="V38" s="5" t="n"/>
+      <c r="V38" s="6" t="n"/>
       <c r="W38" s="5" t="n"/>
-      <c r="X38" s="2" t="inlineStr">
+      <c r="X38" s="5" t="n"/>
+      <c r="Y38" s="2" t="inlineStr">
         <is>
           <t>https://topbeton.lt/</t>
         </is>
       </c>
-      <c r="Y38" s="2" t="inlineStr">
+      <c r="Z38" s="2" t="inlineStr">
         <is>
           <t>https://topbeton.lt/</t>
         </is>
       </c>
-      <c r="Z38" s="2" t="inlineStr"/>
       <c r="AA38" s="2" t="inlineStr"/>
       <c r="AB38" s="2" t="inlineStr"/>
-      <c r="AC38" s="2" t="inlineStr">
+      <c r="AC38" s="2" t="inlineStr"/>
+      <c r="AD38" s="2" t="inlineStr">
         <is>
           <t>https://topbeton.lt/</t>
         </is>
       </c>
-      <c r="AD38" s="2" t="inlineStr">
+      <c r="AE38" s="2" t="inlineStr">
         <is>
           <t>Papildomai rasta pagal prekinio betono požymį.</t>
         </is>
       </c>
-      <c r="AE38" s="2" t="inlineStr">
+      <c r="AF38" s="2" t="inlineStr">
         <is>
           <t>2026-06-30</t>
         </is>
@@ -4991,42 +5038,43 @@
         </is>
       </c>
       <c r="Q39" s="2" t="inlineStr"/>
-      <c r="R39" s="2" t="inlineStr">
+      <c r="R39" s="2" t="inlineStr"/>
+      <c r="S39" s="2" t="inlineStr">
         <is>
           <t>Viešai skelbiama gelžbetonio gaminių gamyba Panevėžyje.</t>
         </is>
       </c>
-      <c r="S39" s="4" t="n">
+      <c r="T39" s="4" t="n">
         <v>0.72</v>
       </c>
-      <c r="T39" s="5" t="n"/>
       <c r="U39" s="5" t="n"/>
-      <c r="V39" s="5" t="n"/>
+      <c r="V39" s="6" t="n"/>
       <c r="W39" s="5" t="n"/>
-      <c r="X39" s="2" t="inlineStr">
+      <c r="X39" s="5" t="n"/>
+      <c r="Y39" s="2" t="inlineStr">
         <is>
           <t>https://gelzbetoniogamyba.lt/</t>
         </is>
       </c>
-      <c r="Y39" s="2" t="inlineStr">
+      <c r="Z39" s="2" t="inlineStr">
         <is>
           <t>https://gelzbetoniogamyba.lt/</t>
         </is>
       </c>
-      <c r="Z39" s="2" t="inlineStr"/>
       <c r="AA39" s="2" t="inlineStr"/>
       <c r="AB39" s="2" t="inlineStr"/>
-      <c r="AC39" s="2" t="inlineStr">
+      <c r="AC39" s="2" t="inlineStr"/>
+      <c r="AD39" s="2" t="inlineStr">
         <is>
           <t>https://gelzbetoniogamyba.lt/</t>
         </is>
       </c>
-      <c r="AD39" s="2" t="inlineStr">
+      <c r="AE39" s="2" t="inlineStr">
         <is>
           <t>Reikia patikslinti ryšį su kitomis S. Kerbedžio g. 52 įmonėmis.</t>
         </is>
       </c>
-      <c r="AE39" s="2" t="inlineStr">
+      <c r="AF39" s="2" t="inlineStr">
         <is>
           <t>2026-06-30</t>
         </is>
@@ -5106,42 +5154,43 @@
         </is>
       </c>
       <c r="Q40" s="2" t="inlineStr"/>
-      <c r="R40" s="2" t="inlineStr">
+      <c r="R40" s="2" t="inlineStr"/>
+      <c r="S40" s="2" t="inlineStr">
         <is>
           <t>Viešai skelbiama betono mišinių veikla Pakruojyje.</t>
         </is>
       </c>
-      <c r="S40" s="4" t="n">
+      <c r="T40" s="4" t="n">
         <v>0.72</v>
       </c>
-      <c r="T40" s="5" t="n"/>
       <c r="U40" s="5" t="n"/>
-      <c r="V40" s="5" t="n"/>
+      <c r="V40" s="6" t="n"/>
       <c r="W40" s="5" t="n"/>
-      <c r="X40" s="2" t="inlineStr">
+      <c r="X40" s="5" t="n"/>
+      <c r="Y40" s="2" t="inlineStr">
         <is>
           <t>https://inroma.lt/</t>
         </is>
       </c>
-      <c r="Y40" s="2" t="inlineStr">
+      <c r="Z40" s="2" t="inlineStr">
         <is>
           <t>https://inroma.lt/</t>
         </is>
       </c>
-      <c r="Z40" s="2" t="inlineStr"/>
       <c r="AA40" s="2" t="inlineStr"/>
       <c r="AB40" s="2" t="inlineStr"/>
-      <c r="AC40" s="2" t="inlineStr">
+      <c r="AC40" s="2" t="inlineStr"/>
+      <c r="AD40" s="2" t="inlineStr">
         <is>
           <t>https://inroma.lt/</t>
         </is>
       </c>
-      <c r="AD40" s="2" t="inlineStr">
+      <c r="AE40" s="2" t="inlineStr">
         <is>
           <t>Reikia patikslinti našumą.</t>
         </is>
       </c>
-      <c r="AE40" s="2" t="inlineStr">
+      <c r="AF40" s="2" t="inlineStr">
         <is>
           <t>2026-06-30</t>
         </is>
@@ -5221,38 +5270,39 @@
         </is>
       </c>
       <c r="Q41" s="2" t="inlineStr"/>
-      <c r="R41" s="2" t="inlineStr">
+      <c r="R41" s="2" t="inlineStr"/>
+      <c r="S41" s="2" t="inlineStr">
         <is>
           <t>Viešame kataloge nurodoma prekinio betono gamyba ir prekyba Vilniuje.</t>
         </is>
       </c>
-      <c r="S41" s="4" t="n">
+      <c r="T41" s="4" t="n">
         <v>0.7</v>
       </c>
-      <c r="T41" s="5" t="n"/>
       <c r="U41" s="5" t="n"/>
-      <c r="V41" s="5" t="n"/>
+      <c r="V41" s="6" t="n"/>
       <c r="W41" s="5" t="n"/>
-      <c r="X41" s="2" t="inlineStr"/>
-      <c r="Y41" s="2" t="inlineStr">
+      <c r="X41" s="5" t="n"/>
+      <c r="Y41" s="2" t="inlineStr"/>
+      <c r="Z41" s="2" t="inlineStr">
         <is>
           <t>https://www.1551.lt/seldra-uab-prekinio-betono-gamyba-ir-prekyba-vilniuje-219193/</t>
         </is>
       </c>
-      <c r="Z41" s="2" t="inlineStr"/>
       <c r="AA41" s="2" t="inlineStr"/>
       <c r="AB41" s="2" t="inlineStr"/>
-      <c r="AC41" s="2" t="inlineStr">
+      <c r="AC41" s="2" t="inlineStr"/>
+      <c r="AD41" s="2" t="inlineStr">
         <is>
           <t>https://www.1551.lt/seldra-uab-prekinio-betono-gamyba-ir-prekyba-vilniuje-219193/</t>
         </is>
       </c>
-      <c r="AD41" s="2" t="inlineStr">
+      <c r="AE41" s="2" t="inlineStr">
         <is>
           <t>Koordinatė apytikslė pagal adresą; reikia patikslinti gamybos tašką.</t>
         </is>
       </c>
-      <c r="AE41" s="2" t="inlineStr">
+      <c r="AF41" s="2" t="inlineStr">
         <is>
           <t>2026-06-30</t>
         </is>
@@ -5336,42 +5386,43 @@
         </is>
       </c>
       <c r="Q42" s="2" t="inlineStr"/>
-      <c r="R42" s="2" t="inlineStr">
+      <c r="R42" s="2" t="inlineStr"/>
+      <c r="S42" s="2" t="inlineStr">
         <is>
           <t>Viešai skelbiama betono mišinių veikla Utenoje.</t>
         </is>
       </c>
-      <c r="S42" s="4" t="n">
+      <c r="T42" s="4" t="n">
         <v>0.78</v>
       </c>
-      <c r="T42" s="5" t="n"/>
       <c r="U42" s="5" t="n"/>
-      <c r="V42" s="5" t="n"/>
+      <c r="V42" s="6" t="n"/>
       <c r="W42" s="5" t="n"/>
-      <c r="X42" s="2" t="inlineStr">
+      <c r="X42" s="5" t="n"/>
+      <c r="Y42" s="2" t="inlineStr">
         <is>
           <t>https://utenosbetonas.lt/</t>
         </is>
       </c>
-      <c r="Y42" s="2" t="inlineStr">
+      <c r="Z42" s="2" t="inlineStr">
         <is>
           <t>https://utenosbetonas.lt/</t>
         </is>
       </c>
-      <c r="Z42" s="2" t="inlineStr"/>
       <c r="AA42" s="2" t="inlineStr"/>
       <c r="AB42" s="2" t="inlineStr"/>
-      <c r="AC42" s="2" t="inlineStr">
+      <c r="AC42" s="2" t="inlineStr"/>
+      <c r="AD42" s="2" t="inlineStr">
         <is>
           <t>https://utenosbetonas.lt/</t>
         </is>
       </c>
-      <c r="AD42" s="2" t="inlineStr">
+      <c r="AE42" s="2" t="inlineStr">
         <is>
           <t>Reikia patikslinti našumą.</t>
         </is>
       </c>
-      <c r="AE42" s="2" t="inlineStr">
+      <c r="AF42" s="2" t="inlineStr">
         <is>
           <t>2026-06-30</t>
         </is>
@@ -5455,42 +5506,43 @@
         </is>
       </c>
       <c r="Q43" s="2" t="inlineStr"/>
-      <c r="R43" s="2" t="inlineStr">
+      <c r="R43" s="2" t="inlineStr"/>
+      <c r="S43" s="2" t="inlineStr">
         <is>
           <t>Viešai skelbiama prekinio betono gamyba Jonavoje.</t>
         </is>
       </c>
-      <c r="S43" s="4" t="n">
+      <c r="T43" s="4" t="n">
         <v>0.78</v>
       </c>
-      <c r="T43" s="5" t="n"/>
       <c r="U43" s="5" t="n"/>
-      <c r="V43" s="5" t="n"/>
+      <c r="V43" s="6" t="n"/>
       <c r="W43" s="5" t="n"/>
-      <c r="X43" s="2" t="inlineStr">
+      <c r="X43" s="5" t="n"/>
+      <c r="Y43" s="2" t="inlineStr">
         <is>
           <t>https://sbetonas.lt/</t>
         </is>
       </c>
-      <c r="Y43" s="2" t="inlineStr">
+      <c r="Z43" s="2" t="inlineStr">
         <is>
           <t>https://sbetonas.lt/</t>
         </is>
       </c>
-      <c r="Z43" s="2" t="inlineStr"/>
       <c r="AA43" s="2" t="inlineStr"/>
       <c r="AB43" s="2" t="inlineStr"/>
-      <c r="AC43" s="2" t="inlineStr">
+      <c r="AC43" s="2" t="inlineStr"/>
+      <c r="AD43" s="2" t="inlineStr">
         <is>
           <t>https://sbetonas.lt/</t>
         </is>
       </c>
-      <c r="AD43" s="2" t="inlineStr">
+      <c r="AE43" s="2" t="inlineStr">
         <is>
           <t>Papildomai rasta pagal prekinio betono požymį.</t>
         </is>
       </c>
-      <c r="AE43" s="2" t="inlineStr">
+      <c r="AF43" s="2" t="inlineStr">
         <is>
           <t>2026-06-30</t>
         </is>
@@ -5570,38 +5622,39 @@
         </is>
       </c>
       <c r="Q44" s="2" t="inlineStr"/>
-      <c r="R44" s="2" t="inlineStr">
+      <c r="R44" s="2" t="inlineStr"/>
+      <c r="S44" s="2" t="inlineStr">
         <is>
           <t>Viešame kataloge nurodomi betonas, betono mišiniai ir betono gamybos linija Naujojoje Akmenėje.</t>
         </is>
       </c>
-      <c r="S44" s="4" t="n">
+      <c r="T44" s="4" t="n">
         <v>0.78</v>
       </c>
-      <c r="T44" s="5" t="n"/>
       <c r="U44" s="5" t="n"/>
-      <c r="V44" s="5" t="n"/>
+      <c r="V44" s="6" t="n"/>
       <c r="W44" s="5" t="n"/>
-      <c r="X44" s="2" t="inlineStr"/>
-      <c r="Y44" s="2" t="inlineStr">
+      <c r="X44" s="5" t="n"/>
+      <c r="Y44" s="2" t="inlineStr"/>
+      <c r="Z44" s="2" t="inlineStr">
         <is>
           <t>https://www.1551.lt/kalcitas-ab-betonas-betono-misiniai-betono-gamybos-linija-technikos-nuoma-naujojoje-akmeneje-59982/</t>
         </is>
       </c>
-      <c r="Z44" s="2" t="inlineStr"/>
       <c r="AA44" s="2" t="inlineStr"/>
       <c r="AB44" s="2" t="inlineStr"/>
-      <c r="AC44" s="2" t="inlineStr">
+      <c r="AC44" s="2" t="inlineStr"/>
+      <c r="AD44" s="2" t="inlineStr">
         <is>
           <t>https://www.1551.lt/kalcitas-ab-betonas-betono-misiniai-betono-gamybos-linija-technikos-nuoma-naujojoje-akmeneje-59982/</t>
         </is>
       </c>
-      <c r="AD44" s="2" t="inlineStr">
+      <c r="AE44" s="2" t="inlineStr">
         <is>
           <t>Reikia patikslinti, ar veikla yra nuolat aktyvi.</t>
         </is>
       </c>
-      <c r="AE44" s="2" t="inlineStr">
+      <c r="AF44" s="2" t="inlineStr">
         <is>
           <t>2026-06-30</t>
         </is>
@@ -5681,42 +5734,43 @@
         </is>
       </c>
       <c r="Q45" s="2" t="inlineStr"/>
-      <c r="R45" s="2" t="inlineStr">
+      <c r="R45" s="2" t="inlineStr"/>
+      <c r="S45" s="2" t="inlineStr">
         <is>
           <t>Viešai skelbiami gelžbetonio gaminiai.</t>
         </is>
       </c>
-      <c r="S45" s="4" t="n">
+      <c r="T45" s="4" t="n">
         <v>0.78</v>
       </c>
-      <c r="T45" s="5" t="n"/>
       <c r="U45" s="5" t="n"/>
-      <c r="V45" s="5" t="n"/>
+      <c r="V45" s="6" t="n"/>
       <c r="W45" s="5" t="n"/>
-      <c r="X45" s="2" t="inlineStr">
+      <c r="X45" s="5" t="n"/>
+      <c r="Y45" s="2" t="inlineStr">
         <is>
           <t>https://glg.lt/</t>
         </is>
       </c>
-      <c r="Y45" s="2" t="inlineStr">
+      <c r="Z45" s="2" t="inlineStr">
         <is>
           <t>https://glg.lt/kontaktai/</t>
         </is>
       </c>
-      <c r="Z45" s="2" t="inlineStr"/>
       <c r="AA45" s="2" t="inlineStr"/>
       <c r="AB45" s="2" t="inlineStr"/>
-      <c r="AC45" s="2" t="inlineStr">
+      <c r="AC45" s="2" t="inlineStr"/>
+      <c r="AD45" s="2" t="inlineStr">
         <is>
           <t>https://glg.lt/kontaktai/</t>
         </is>
       </c>
-      <c r="AD45" s="2" t="inlineStr">
+      <c r="AE45" s="2" t="inlineStr">
         <is>
           <t>Reikia patikslinti tikslų gamyklos adresą.</t>
         </is>
       </c>
-      <c r="AE45" s="2" t="inlineStr">
+      <c r="AF45" s="2" t="inlineStr">
         <is>
           <t>2026-06-30</t>
         </is>
@@ -5800,38 +5854,39 @@
         </is>
       </c>
       <c r="Q46" s="2" t="inlineStr"/>
-      <c r="R46" s="2" t="inlineStr">
+      <c r="R46" s="2" t="inlineStr"/>
+      <c r="S46" s="2" t="inlineStr">
         <is>
           <t>Viešame kataloge įmonė siejama su betono mišinių veikla.</t>
         </is>
       </c>
-      <c r="S46" s="4" t="n">
+      <c r="T46" s="4" t="n">
         <v>0.62</v>
       </c>
-      <c r="T46" s="5" t="n"/>
       <c r="U46" s="5" t="n"/>
-      <c r="V46" s="5" t="n"/>
+      <c r="V46" s="6" t="n"/>
       <c r="W46" s="5" t="n"/>
-      <c r="X46" s="2" t="inlineStr"/>
-      <c r="Y46" s="2" t="inlineStr">
+      <c r="X46" s="5" t="n"/>
+      <c r="Y46" s="2" t="inlineStr"/>
+      <c r="Z46" s="2" t="inlineStr">
         <is>
           <t>https://www.1551.lt/sausta-uab-240915/</t>
         </is>
       </c>
-      <c r="Z46" s="2" t="inlineStr"/>
       <c r="AA46" s="2" t="inlineStr"/>
       <c r="AB46" s="2" t="inlineStr"/>
-      <c r="AC46" s="2" t="inlineStr">
+      <c r="AC46" s="2" t="inlineStr"/>
+      <c r="AD46" s="2" t="inlineStr">
         <is>
           <t>https://www.1551.lt/sausta-uab-240915/</t>
         </is>
       </c>
-      <c r="AD46" s="2" t="inlineStr">
+      <c r="AE46" s="2" t="inlineStr">
         <is>
           <t>Žemos pasitikėjimo įrašas; reikia patikslinti, ar gamyba vykdoma šiame taške.</t>
         </is>
       </c>
-      <c r="AE46" s="2" t="inlineStr">
+      <c r="AF46" s="2" t="inlineStr">
         <is>
           <t>2026-06-30</t>
         </is>
@@ -5915,34 +5970,35 @@
         </is>
       </c>
       <c r="Q47" s="2" t="inlineStr"/>
-      <c r="R47" s="2" t="inlineStr">
+      <c r="R47" s="2" t="inlineStr"/>
+      <c r="S47" s="2" t="inlineStr">
         <is>
           <t>Registrų centro/VDA atviruose duomenyse pagrindinė veikla nurodyta kaip prekinio betono mišinio gamyba (EVRK 23.63).</t>
         </is>
       </c>
-      <c r="S47" s="4" t="n">
+      <c r="T47" s="4" t="n">
         <v>0.82</v>
       </c>
-      <c r="T47" s="5" t="n"/>
       <c r="U47" s="5" t="n"/>
-      <c r="V47" s="5" t="n"/>
+      <c r="V47" s="6" t="n"/>
       <c r="W47" s="5" t="n"/>
-      <c r="X47" s="2" t="inlineStr"/>
-      <c r="Y47" s="2" t="inlineStr">
+      <c r="X47" s="5" t="n"/>
+      <c r="Y47" s="2" t="inlineStr"/>
+      <c r="Z47" s="2" t="inlineStr">
         <is>
           <t>https://data.gov.lt/dataset/juridiniu-asmenu-ekonomines-veiklos-rusys-ir-instituciniai-sektoriai/</t>
         </is>
       </c>
-      <c r="Z47" s="2" t="inlineStr"/>
       <c r="AA47" s="2" t="inlineStr"/>
       <c r="AB47" s="2" t="inlineStr"/>
       <c r="AC47" s="2" t="inlineStr"/>
-      <c r="AD47" s="2" t="inlineStr">
+      <c r="AD47" s="2" t="inlineStr"/>
+      <c r="AE47" s="2" t="inlineStr">
         <is>
           <t>Adresas geokoduotas pagal viešai randamą įmonės adresą; betono mazgo vietą verta patikslinti atskiru šaltiniu.</t>
         </is>
       </c>
-      <c r="AE47" s="2" t="inlineStr">
+      <c r="AF47" s="2" t="inlineStr">
         <is>
           <t>2026-06-30</t>
         </is>
@@ -6026,34 +6082,35 @@
         </is>
       </c>
       <c r="Q48" s="2" t="inlineStr"/>
-      <c r="R48" s="2" t="inlineStr">
+      <c r="R48" s="2" t="inlineStr"/>
+      <c r="S48" s="2" t="inlineStr">
         <is>
           <t>Registrų centro/VDA atviruose duomenyse pagrindinė veikla nurodyta kaip prekinio betono mišinio gamyba (EVRK 23.63).</t>
         </is>
       </c>
-      <c r="S48" s="4" t="n">
+      <c r="T48" s="4" t="n">
         <v>0.82</v>
       </c>
-      <c r="T48" s="5" t="n"/>
       <c r="U48" s="5" t="n"/>
-      <c r="V48" s="5" t="n"/>
+      <c r="V48" s="6" t="n"/>
       <c r="W48" s="5" t="n"/>
-      <c r="X48" s="2" t="inlineStr"/>
-      <c r="Y48" s="2" t="inlineStr">
+      <c r="X48" s="5" t="n"/>
+      <c r="Y48" s="2" t="inlineStr"/>
+      <c r="Z48" s="2" t="inlineStr">
         <is>
           <t>https://data.gov.lt/dataset/juridiniu-asmenu-ekonomines-veiklos-rusys-ir-instituciniai-sektoriai/</t>
         </is>
       </c>
-      <c r="Z48" s="2" t="inlineStr"/>
       <c r="AA48" s="2" t="inlineStr"/>
       <c r="AB48" s="2" t="inlineStr"/>
       <c r="AC48" s="2" t="inlineStr"/>
-      <c r="AD48" s="2" t="inlineStr">
+      <c r="AD48" s="2" t="inlineStr"/>
+      <c r="AE48" s="2" t="inlineStr">
         <is>
           <t>Adresas geokoduotas pagal viešai randamą įmonės adresą; betono mazgo vietą verta patikslinti atskiru šaltiniu.</t>
         </is>
       </c>
-      <c r="AE48" s="2" t="inlineStr">
+      <c r="AF48" s="2" t="inlineStr">
         <is>
           <t>2026-06-30</t>
         </is>
@@ -6137,34 +6194,35 @@
         </is>
       </c>
       <c r="Q49" s="2" t="inlineStr"/>
-      <c r="R49" s="2" t="inlineStr">
+      <c r="R49" s="2" t="inlineStr"/>
+      <c r="S49" s="2" t="inlineStr">
         <is>
           <t>Registrų centro/VDA atviruose duomenyse pagrindinė veikla nurodyta kaip prekinio betono mišinio gamyba (EVRK 23.63).</t>
         </is>
       </c>
-      <c r="S49" s="4" t="n">
+      <c r="T49" s="4" t="n">
         <v>0.82</v>
       </c>
-      <c r="T49" s="5" t="n"/>
       <c r="U49" s="5" t="n"/>
-      <c r="V49" s="5" t="n"/>
+      <c r="V49" s="6" t="n"/>
       <c r="W49" s="5" t="n"/>
-      <c r="X49" s="2" t="inlineStr"/>
-      <c r="Y49" s="2" t="inlineStr">
+      <c r="X49" s="5" t="n"/>
+      <c r="Y49" s="2" t="inlineStr"/>
+      <c r="Z49" s="2" t="inlineStr">
         <is>
           <t>https://data.gov.lt/dataset/juridiniu-asmenu-ekonomines-veiklos-rusys-ir-instituciniai-sektoriai/</t>
         </is>
       </c>
-      <c r="Z49" s="2" t="inlineStr"/>
       <c r="AA49" s="2" t="inlineStr"/>
       <c r="AB49" s="2" t="inlineStr"/>
       <c r="AC49" s="2" t="inlineStr"/>
-      <c r="AD49" s="2" t="inlineStr">
+      <c r="AD49" s="2" t="inlineStr"/>
+      <c r="AE49" s="2" t="inlineStr">
         <is>
           <t>Adresas geokoduotas pagal viešai randamą įmonės adresą; betono mazgo vietą verta patikslinti atskiru šaltiniu.</t>
         </is>
       </c>
-      <c r="AE49" s="2" t="inlineStr">
+      <c r="AF49" s="2" t="inlineStr">
         <is>
           <t>2026-06-30</t>
         </is>
@@ -6248,34 +6306,35 @@
         </is>
       </c>
       <c r="Q50" s="2" t="inlineStr"/>
-      <c r="R50" s="2" t="inlineStr">
+      <c r="R50" s="2" t="inlineStr"/>
+      <c r="S50" s="2" t="inlineStr">
         <is>
           <t>Registrų centro/VDA atviruose duomenyse pagrindinė veikla nurodyta kaip prekinio betono mišinio gamyba (EVRK 23.63).</t>
         </is>
       </c>
-      <c r="S50" s="4" t="n">
+      <c r="T50" s="4" t="n">
         <v>0.82</v>
       </c>
-      <c r="T50" s="5" t="n"/>
       <c r="U50" s="5" t="n"/>
-      <c r="V50" s="5" t="n"/>
+      <c r="V50" s="6" t="n"/>
       <c r="W50" s="5" t="n"/>
-      <c r="X50" s="2" t="inlineStr"/>
-      <c r="Y50" s="2" t="inlineStr">
+      <c r="X50" s="5" t="n"/>
+      <c r="Y50" s="2" t="inlineStr"/>
+      <c r="Z50" s="2" t="inlineStr">
         <is>
           <t>https://data.gov.lt/dataset/juridiniu-asmenu-ekonomines-veiklos-rusys-ir-instituciniai-sektoriai/</t>
         </is>
       </c>
-      <c r="Z50" s="2" t="inlineStr"/>
       <c r="AA50" s="2" t="inlineStr"/>
       <c r="AB50" s="2" t="inlineStr"/>
       <c r="AC50" s="2" t="inlineStr"/>
-      <c r="AD50" s="2" t="inlineStr">
+      <c r="AD50" s="2" t="inlineStr"/>
+      <c r="AE50" s="2" t="inlineStr">
         <is>
           <t>Adresas geokoduotas pagal viešai randamą įmonės adresą; betono mazgo vietą verta patikslinti atskiru šaltiniu.</t>
         </is>
       </c>
-      <c r="AE50" s="2" t="inlineStr">
+      <c r="AF50" s="2" t="inlineStr">
         <is>
           <t>2026-06-30</t>
         </is>
@@ -6359,34 +6418,35 @@
         </is>
       </c>
       <c r="Q51" s="2" t="inlineStr"/>
-      <c r="R51" s="2" t="inlineStr">
+      <c r="R51" s="2" t="inlineStr"/>
+      <c r="S51" s="2" t="inlineStr">
         <is>
           <t>Registrų centro/VDA atviruose duomenyse pagrindinė veikla nurodyta kaip prekinio betono mišinio gamyba (EVRK 23.63).</t>
         </is>
       </c>
-      <c r="S51" s="4" t="n">
+      <c r="T51" s="4" t="n">
         <v>0.82</v>
       </c>
-      <c r="T51" s="5" t="n"/>
       <c r="U51" s="5" t="n"/>
-      <c r="V51" s="5" t="n"/>
+      <c r="V51" s="6" t="n"/>
       <c r="W51" s="5" t="n"/>
-      <c r="X51" s="2" t="inlineStr"/>
-      <c r="Y51" s="2" t="inlineStr">
+      <c r="X51" s="5" t="n"/>
+      <c r="Y51" s="2" t="inlineStr"/>
+      <c r="Z51" s="2" t="inlineStr">
         <is>
           <t>https://data.gov.lt/dataset/juridiniu-asmenu-ekonomines-veiklos-rusys-ir-instituciniai-sektoriai/</t>
         </is>
       </c>
-      <c r="Z51" s="2" t="inlineStr"/>
       <c r="AA51" s="2" t="inlineStr"/>
       <c r="AB51" s="2" t="inlineStr"/>
       <c r="AC51" s="2" t="inlineStr"/>
-      <c r="AD51" s="2" t="inlineStr">
+      <c r="AD51" s="2" t="inlineStr"/>
+      <c r="AE51" s="2" t="inlineStr">
         <is>
           <t>Adresas geokoduotas pagal viešai randamą įmonės adresą; betono mazgo vietą verta patikslinti atskiru šaltiniu.</t>
         </is>
       </c>
-      <c r="AE51" s="2" t="inlineStr">
+      <c r="AF51" s="2" t="inlineStr">
         <is>
           <t>2026-06-30</t>
         </is>
@@ -6470,38 +6530,39 @@
         </is>
       </c>
       <c r="Q52" s="2" t="inlineStr"/>
-      <c r="R52" s="2" t="inlineStr">
+      <c r="R52" s="2" t="inlineStr"/>
+      <c r="S52" s="2" t="inlineStr">
         <is>
           <t>Registrų centro/VDA atviruose duomenyse pagrindinė veikla nurodyta kaip prekinio betono mišinio gamyba (EVRK 23.63).</t>
         </is>
       </c>
-      <c r="S52" s="4" t="n">
+      <c r="T52" s="4" t="n">
         <v>0.82</v>
       </c>
-      <c r="T52" s="5" t="n"/>
       <c r="U52" s="5" t="n"/>
-      <c r="V52" s="5" t="n"/>
+      <c r="V52" s="6" t="n"/>
       <c r="W52" s="5" t="n"/>
-      <c r="X52" s="2" t="inlineStr"/>
-      <c r="Y52" s="2" t="inlineStr">
+      <c r="X52" s="5" t="n"/>
+      <c r="Y52" s="2" t="inlineStr"/>
+      <c r="Z52" s="2" t="inlineStr">
         <is>
           <t>https://data.gov.lt/dataset/juridiniu-asmenu-ekonomines-veiklos-rusys-ir-instituciniai-sektoriai/</t>
         </is>
       </c>
-      <c r="Z52" s="2" t="inlineStr"/>
       <c r="AA52" s="2" t="inlineStr"/>
       <c r="AB52" s="2" t="inlineStr"/>
-      <c r="AC52" s="2" t="inlineStr">
+      <c r="AC52" s="2" t="inlineStr"/>
+      <c r="AD52" s="2" t="inlineStr">
         <is>
           <t>https://chamber.lt/bendruomene/rumu-nariu-sarasas/nariai/santvara/</t>
         </is>
       </c>
-      <c r="AD52" s="2" t="inlineStr">
+      <c r="AE52" s="2" t="inlineStr">
         <is>
           <t>Adresas geokoduotas pagal viešai randamą įmonės adresą; betono mazgo vietą verta patikslinti atskiru šaltiniu.</t>
         </is>
       </c>
-      <c r="AE52" s="2" t="inlineStr">
+      <c r="AF52" s="2" t="inlineStr">
         <is>
           <t>2026-06-30</t>
         </is>
@@ -6585,34 +6646,35 @@
         </is>
       </c>
       <c r="Q53" s="2" t="inlineStr"/>
-      <c r="R53" s="2" t="inlineStr">
+      <c r="R53" s="2" t="inlineStr"/>
+      <c r="S53" s="2" t="inlineStr">
         <is>
           <t>Registrų centro/VDA atviruose duomenyse pagrindinė veikla nurodyta kaip prekinio betono mišinio gamyba (EVRK 23.63).</t>
         </is>
       </c>
-      <c r="S53" s="4" t="n">
+      <c r="T53" s="4" t="n">
         <v>0.72</v>
       </c>
-      <c r="T53" s="5" t="n"/>
       <c r="U53" s="5" t="n"/>
-      <c r="V53" s="5" t="n"/>
+      <c r="V53" s="6" t="n"/>
       <c r="W53" s="5" t="n"/>
-      <c r="X53" s="2" t="inlineStr"/>
-      <c r="Y53" s="2" t="inlineStr">
+      <c r="X53" s="5" t="n"/>
+      <c r="Y53" s="2" t="inlineStr"/>
+      <c r="Z53" s="2" t="inlineStr">
         <is>
           <t>https://data.gov.lt/dataset/juridiniu-asmenu-ekonomines-veiklos-rusys-ir-instituciniai-sektoriai/</t>
         </is>
       </c>
-      <c r="Z53" s="2" t="inlineStr"/>
       <c r="AA53" s="2" t="inlineStr"/>
       <c r="AB53" s="2" t="inlineStr"/>
       <c r="AC53" s="2" t="inlineStr"/>
-      <c r="AD53" s="2" t="inlineStr">
+      <c r="AD53" s="2" t="inlineStr"/>
+      <c r="AE53" s="2" t="inlineStr">
         <is>
           <t>Adresas rastas viešuose kataloguose, bet geokoduotas tik iki Visagino miesto taško; reikia patikslinti tikslų betono mazgo GPS.</t>
         </is>
       </c>
-      <c r="AE53" s="2" t="inlineStr">
+      <c r="AF53" s="2" t="inlineStr">
         <is>
           <t>2026-06-30</t>
         </is>
@@ -6696,34 +6758,35 @@
         </is>
       </c>
       <c r="Q54" s="2" t="inlineStr"/>
-      <c r="R54" s="2" t="inlineStr">
+      <c r="R54" s="2" t="inlineStr"/>
+      <c r="S54" s="2" t="inlineStr">
         <is>
           <t>Registrų centro/VDA atviruose duomenyse pagrindinė veikla nurodyta kaip prekinio betono mišinio gamyba (EVRK 23.63).</t>
         </is>
       </c>
-      <c r="S54" s="4" t="n">
+      <c r="T54" s="4" t="n">
         <v>0.82</v>
       </c>
-      <c r="T54" s="5" t="n"/>
       <c r="U54" s="5" t="n"/>
-      <c r="V54" s="5" t="n"/>
+      <c r="V54" s="6" t="n"/>
       <c r="W54" s="5" t="n"/>
-      <c r="X54" s="2" t="inlineStr"/>
-      <c r="Y54" s="2" t="inlineStr">
+      <c r="X54" s="5" t="n"/>
+      <c r="Y54" s="2" t="inlineStr"/>
+      <c r="Z54" s="2" t="inlineStr">
         <is>
           <t>https://data.gov.lt/dataset/juridiniu-asmenu-ekonomines-veiklos-rusys-ir-instituciniai-sektoriai/</t>
         </is>
       </c>
-      <c r="Z54" s="2" t="inlineStr"/>
       <c r="AA54" s="2" t="inlineStr"/>
       <c r="AB54" s="2" t="inlineStr"/>
       <c r="AC54" s="2" t="inlineStr"/>
-      <c r="AD54" s="2" t="inlineStr">
+      <c r="AD54" s="2" t="inlineStr"/>
+      <c r="AE54" s="2" t="inlineStr">
         <is>
           <t>Adresas geokoduotas pagal viešai randamą įmonės adresą; betono mazgo vietą verta patikslinti atskiru šaltiniu.</t>
         </is>
       </c>
-      <c r="AE54" s="2" t="inlineStr">
+      <c r="AF54" s="2" t="inlineStr">
         <is>
           <t>2026-06-30</t>
         </is>
@@ -6807,34 +6870,35 @@
         </is>
       </c>
       <c r="Q55" s="2" t="inlineStr"/>
-      <c r="R55" s="2" t="inlineStr">
+      <c r="R55" s="2" t="inlineStr"/>
+      <c r="S55" s="2" t="inlineStr">
         <is>
           <t>Registrų centro/VDA atviruose duomenyse pagrindinė veikla nurodyta kaip prekinio betono mišinio gamyba (EVRK 23.63).</t>
         </is>
       </c>
-      <c r="S55" s="4" t="n">
+      <c r="T55" s="4" t="n">
         <v>0.82</v>
       </c>
-      <c r="T55" s="5" t="n"/>
       <c r="U55" s="5" t="n"/>
-      <c r="V55" s="5" t="n"/>
+      <c r="V55" s="6" t="n"/>
       <c r="W55" s="5" t="n"/>
-      <c r="X55" s="2" t="inlineStr"/>
-      <c r="Y55" s="2" t="inlineStr">
+      <c r="X55" s="5" t="n"/>
+      <c r="Y55" s="2" t="inlineStr"/>
+      <c r="Z55" s="2" t="inlineStr">
         <is>
           <t>https://data.gov.lt/dataset/juridiniu-asmenu-ekonomines-veiklos-rusys-ir-instituciniai-sektoriai/</t>
         </is>
       </c>
-      <c r="Z55" s="2" t="inlineStr"/>
       <c r="AA55" s="2" t="inlineStr"/>
       <c r="AB55" s="2" t="inlineStr"/>
       <c r="AC55" s="2" t="inlineStr"/>
-      <c r="AD55" s="2" t="inlineStr">
+      <c r="AD55" s="2" t="inlineStr"/>
+      <c r="AE55" s="2" t="inlineStr">
         <is>
           <t>Adresas geokoduotas pagal viešai randamą įmonės adresą; betono mazgo vietą verta patikslinti atskiru šaltiniu.</t>
         </is>
       </c>
-      <c r="AE55" s="2" t="inlineStr">
+      <c r="AF55" s="2" t="inlineStr">
         <is>
           <t>2026-06-30</t>
         </is>
@@ -6918,34 +6982,35 @@
         </is>
       </c>
       <c r="Q56" s="2" t="inlineStr"/>
-      <c r="R56" s="2" t="inlineStr">
+      <c r="R56" s="2" t="inlineStr"/>
+      <c r="S56" s="2" t="inlineStr">
         <is>
           <t>Registrų centro/VDA atviruose duomenyse pagrindinė veikla nurodyta kaip prekinio betono mišinio gamyba (EVRK 23.63).</t>
         </is>
       </c>
-      <c r="S56" s="4" t="n">
+      <c r="T56" s="4" t="n">
         <v>0.72</v>
       </c>
-      <c r="T56" s="5" t="n"/>
       <c r="U56" s="5" t="n"/>
-      <c r="V56" s="5" t="n"/>
+      <c r="V56" s="6" t="n"/>
       <c r="W56" s="5" t="n"/>
-      <c r="X56" s="2" t="inlineStr"/>
-      <c r="Y56" s="2" t="inlineStr">
+      <c r="X56" s="5" t="n"/>
+      <c r="Y56" s="2" t="inlineStr"/>
+      <c r="Z56" s="2" t="inlineStr">
         <is>
           <t>https://data.gov.lt/dataset/juridiniu-asmenu-ekonomines-veiklos-rusys-ir-instituciniai-sektoriai/</t>
         </is>
       </c>
-      <c r="Z56" s="2" t="inlineStr"/>
       <c r="AA56" s="2" t="inlineStr"/>
       <c r="AB56" s="2" t="inlineStr"/>
       <c r="AC56" s="2" t="inlineStr"/>
-      <c r="AD56" s="2" t="inlineStr">
+      <c r="AD56" s="2" t="inlineStr"/>
+      <c r="AE56" s="2" t="inlineStr">
         <is>
           <t>Adresas rastas viešuose kataloguose, bet geokoduotas tik iki Rokiškio miesto taško; reikia patikslinti tikslų betono mazgo GPS.</t>
         </is>
       </c>
-      <c r="AE56" s="2" t="inlineStr">
+      <c r="AF56" s="2" t="inlineStr">
         <is>
           <t>2026-06-30</t>
         </is>
@@ -7029,34 +7094,35 @@
         </is>
       </c>
       <c r="Q57" s="2" t="inlineStr"/>
-      <c r="R57" s="2" t="inlineStr">
+      <c r="R57" s="2" t="inlineStr"/>
+      <c r="S57" s="2" t="inlineStr">
         <is>
           <t>Registrų centro/VDA atviruose duomenyse pagrindinė veikla nurodyta kaip prekinio betono mišinio gamyba (EVRK 23.63).</t>
         </is>
       </c>
-      <c r="S57" s="4" t="n">
+      <c r="T57" s="4" t="n">
         <v>0.82</v>
       </c>
-      <c r="T57" s="5" t="n"/>
       <c r="U57" s="5" t="n"/>
-      <c r="V57" s="5" t="n"/>
+      <c r="V57" s="6" t="n"/>
       <c r="W57" s="5" t="n"/>
-      <c r="X57" s="2" t="inlineStr"/>
-      <c r="Y57" s="2" t="inlineStr">
+      <c r="X57" s="5" t="n"/>
+      <c r="Y57" s="2" t="inlineStr"/>
+      <c r="Z57" s="2" t="inlineStr">
         <is>
           <t>https://data.gov.lt/dataset/juridiniu-asmenu-ekonomines-veiklos-rusys-ir-instituciniai-sektoriai/</t>
         </is>
       </c>
-      <c r="Z57" s="2" t="inlineStr"/>
       <c r="AA57" s="2" t="inlineStr"/>
       <c r="AB57" s="2" t="inlineStr"/>
       <c r="AC57" s="2" t="inlineStr"/>
-      <c r="AD57" s="2" t="inlineStr">
+      <c r="AD57" s="2" t="inlineStr"/>
+      <c r="AE57" s="2" t="inlineStr">
         <is>
           <t>Adresas geokoduotas pagal viešai randamą įmonės adresą; betono mazgo vietą verta patikslinti atskiru šaltiniu.</t>
         </is>
       </c>
-      <c r="AE57" s="2" t="inlineStr">
+      <c r="AF57" s="2" t="inlineStr">
         <is>
           <t>2026-06-30</t>
         </is>
@@ -7140,38 +7206,39 @@
         </is>
       </c>
       <c r="Q58" s="2" t="inlineStr"/>
-      <c r="R58" s="2" t="inlineStr">
+      <c r="R58" s="2" t="inlineStr"/>
+      <c r="S58" s="2" t="inlineStr">
         <is>
           <t>Registrų centro/VDA atviruose duomenyse pagrindinė veikla nurodyta kaip prekinio betono mišinio gamyba (EVRK 23.63).</t>
         </is>
       </c>
-      <c r="S58" s="4" t="n">
+      <c r="T58" s="4" t="n">
         <v>0.82</v>
       </c>
-      <c r="T58" s="5" t="n"/>
       <c r="U58" s="5" t="n"/>
-      <c r="V58" s="5" t="n"/>
+      <c r="V58" s="6" t="n"/>
       <c r="W58" s="5" t="n"/>
-      <c r="X58" s="2" t="inlineStr"/>
-      <c r="Y58" s="2" t="inlineStr">
+      <c r="X58" s="5" t="n"/>
+      <c r="Y58" s="2" t="inlineStr"/>
+      <c r="Z58" s="2" t="inlineStr">
         <is>
           <t>https://data.gov.lt/dataset/juridiniu-asmenu-ekonomines-veiklos-rusys-ir-instituciniai-sektoriai/</t>
         </is>
       </c>
-      <c r="Z58" s="2" t="inlineStr"/>
       <c r="AA58" s="2" t="inlineStr"/>
       <c r="AB58" s="2" t="inlineStr"/>
-      <c r="AC58" s="2" t="inlineStr">
+      <c r="AC58" s="2" t="inlineStr"/>
+      <c r="AD58" s="2" t="inlineStr">
         <is>
           <t>https://fsaskaita.lt/imone/uzdaroji-akcine-bendrove-silutes-betonas-177392928</t>
         </is>
       </c>
-      <c r="AD58" s="2" t="inlineStr">
+      <c r="AE58" s="2" t="inlineStr">
         <is>
           <t>Adresas geokoduotas pagal viešai randamą įmonės adresą; betono mazgo vietą verta patikslinti atskiru šaltiniu.</t>
         </is>
       </c>
-      <c r="AE58" s="2" t="inlineStr">
+      <c r="AF58" s="2" t="inlineStr">
         <is>
           <t>2026-06-30</t>
         </is>
@@ -7255,34 +7322,35 @@
         </is>
       </c>
       <c r="Q59" s="2" t="inlineStr"/>
-      <c r="R59" s="2" t="inlineStr">
+      <c r="R59" s="2" t="inlineStr"/>
+      <c r="S59" s="2" t="inlineStr">
         <is>
           <t>Registrų centro/VDA atviruose duomenyse pagrindinė veikla nurodyta kaip prekinio betono mišinio gamyba (EVRK 23.63).</t>
         </is>
       </c>
-      <c r="S59" s="4" t="n">
+      <c r="T59" s="4" t="n">
         <v>0.82</v>
       </c>
-      <c r="T59" s="5" t="n"/>
       <c r="U59" s="5" t="n"/>
-      <c r="V59" s="5" t="n"/>
+      <c r="V59" s="6" t="n"/>
       <c r="W59" s="5" t="n"/>
-      <c r="X59" s="2" t="inlineStr"/>
-      <c r="Y59" s="2" t="inlineStr">
+      <c r="X59" s="5" t="n"/>
+      <c r="Y59" s="2" t="inlineStr"/>
+      <c r="Z59" s="2" t="inlineStr">
         <is>
           <t>https://data.gov.lt/dataset/juridiniu-asmenu-ekonomines-veiklos-rusys-ir-instituciniai-sektoriai/</t>
         </is>
       </c>
-      <c r="Z59" s="2" t="inlineStr"/>
       <c r="AA59" s="2" t="inlineStr"/>
       <c r="AB59" s="2" t="inlineStr"/>
       <c r="AC59" s="2" t="inlineStr"/>
-      <c r="AD59" s="2" t="inlineStr">
+      <c r="AD59" s="2" t="inlineStr"/>
+      <c r="AE59" s="2" t="inlineStr">
         <is>
           <t>Adresas geokoduotas pagal viešai randamą įmonės adresą; betono mazgo vietą verta patikslinti atskiru šaltiniu.</t>
         </is>
       </c>
-      <c r="AE59" s="2" t="inlineStr">
+      <c r="AF59" s="2" t="inlineStr">
         <is>
           <t>2026-06-30</t>
         </is>
@@ -7366,49 +7434,50 @@
         </is>
       </c>
       <c r="Q60" s="2" t="inlineStr"/>
-      <c r="R60" s="2" t="inlineStr">
+      <c r="R60" s="2" t="inlineStr"/>
+      <c r="S60" s="2" t="inlineStr">
         <is>
           <t>Oficialiame įmonės puslapyje skelbiama betono mišinių gamyba ir prekyba.</t>
         </is>
       </c>
-      <c r="S60" s="4" t="n">
+      <c r="T60" s="4" t="n">
         <v>0.86</v>
       </c>
-      <c r="T60" s="5" t="n"/>
       <c r="U60" s="5" t="n"/>
-      <c r="V60" s="5" t="n"/>
+      <c r="V60" s="6" t="n"/>
       <c r="W60" s="5" t="n"/>
-      <c r="X60" s="2" t="inlineStr">
+      <c r="X60" s="5" t="n"/>
+      <c r="Y60" s="2" t="inlineStr">
         <is>
           <t>https://www.tkeliai.lt/</t>
         </is>
       </c>
-      <c r="Y60" s="2" t="inlineStr">
+      <c r="Z60" s="2" t="inlineStr">
         <is>
           <t>https://www.tkeliai.lt/kitos-paslaugos/</t>
         </is>
       </c>
-      <c r="Z60" s="2" t="inlineStr"/>
       <c r="AA60" s="2" t="inlineStr"/>
       <c r="AB60" s="2" t="inlineStr"/>
-      <c r="AC60" s="2" t="inlineStr">
+      <c r="AC60" s="2" t="inlineStr"/>
+      <c r="AD60" s="2" t="inlineStr">
         <is>
           <t>https://www.tkeliai.lt/kitos-paslaugos/</t>
         </is>
       </c>
-      <c r="AD60" s="2" t="inlineStr">
+      <c r="AE60" s="2" t="inlineStr">
         <is>
           <t>Įtraukta pagal naudotojo informaciją; veikla patvirtinta oficialiame lietuviškame įmonės puslapyje. Koordinatės nustatytos Lietuvos geolokatoriumi pagal Mažeikių g. 18 adresą.</t>
         </is>
       </c>
-      <c r="AE60" s="2" t="inlineStr">
+      <c r="AF60" s="2" t="inlineStr">
         <is>
           <t>2026-06-30</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AE60"/>
+  <autoFilter ref="A1:AF60"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -7430,7 +7499,7 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="6" t="inlineStr">
+      <c r="A1" s="7" t="inlineStr">
         <is>
           <t>Projektas</t>
         </is>
@@ -7442,7 +7511,7 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="6" t="inlineStr">
+      <c r="A2" s="7" t="inlineStr">
         <is>
           <t>Apimtis</t>
         </is>
@@ -7454,7 +7523,7 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="6" t="inlineStr">
+      <c r="A3" s="7" t="inlineStr">
         <is>
           <t>Įtraukta</t>
         </is>
@@ -7466,7 +7535,7 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="6" t="inlineStr">
+      <c r="A4" s="7" t="inlineStr">
         <is>
           <t>Neįtraukta</t>
         </is>
@@ -7478,7 +7547,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="6" t="inlineStr">
+      <c r="A5" s="7" t="inlineStr">
         <is>
           <t>Duomenų modelis</t>
         </is>
@@ -7490,14 +7559,14 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="6" t="inlineStr">
+      <c r="A6" s="7" t="inlineStr">
         <is>
           <t>Sugeneruota</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-06-30T12:13:10.847047+00:00</t>
+          <t>2026-06-30T12:21:46.857357+00:00</t>
         </is>
       </c>
     </row>
@@ -7523,27 +7592,27 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="7" t="inlineStr">
+      <c r="A1" s="8" t="inlineStr">
         <is>
           <t>Paleidimo laikas</t>
         </is>
       </c>
-      <c r="B1" s="7" t="inlineStr">
+      <c r="B1" s="8" t="inlineStr">
         <is>
           <t>Būsena</t>
         </is>
       </c>
-      <c r="C1" s="7" t="inlineStr">
+      <c r="C1" s="8" t="inlineStr">
         <is>
           <t>Šaltinis</t>
         </is>
       </c>
-      <c r="D1" s="7" t="inlineStr">
+      <c r="D1" s="8" t="inlineStr">
         <is>
           <t>Eilučių skaičius</t>
         </is>
       </c>
-      <c r="E1" s="7" t="inlineStr">
+      <c r="E1" s="8" t="inlineStr">
         <is>
           <t>Pastabos</t>
         </is>
@@ -7552,7 +7621,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-06-30T12:13:10.849054+00:00</t>
+          <t>2026-06-30T12:21:46.857357+00:00</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">

</xml_diff>

<commit_message>
Update Gelgaudiskio gelzbetonis details
</commit_message>
<xml_diff>
--- a/data/companies.xlsx
+++ b/data/companies.xlsx
@@ -518,7 +518,7 @@
     <col width="24" customWidth="1" min="12" max="12"/>
     <col width="42" customWidth="1" min="13" max="13"/>
     <col width="20" customWidth="1" min="14" max="14"/>
-    <col width="24" customWidth="1" min="15" max="15"/>
+    <col width="32" customWidth="1" min="15" max="15"/>
     <col width="40" customWidth="1" min="16" max="16"/>
     <col width="30" customWidth="1" min="17" max="17"/>
     <col width="17" customWidth="1" min="18" max="18"/>
@@ -531,7 +531,7 @@
     <col width="42" customWidth="1" min="25" max="25"/>
     <col width="42" customWidth="1" min="26" max="26"/>
     <col width="20" customWidth="1" min="27" max="27"/>
-    <col width="21" customWidth="1" min="28" max="28"/>
+    <col width="28" customWidth="1" min="28" max="28"/>
     <col width="21" customWidth="1" min="29" max="29"/>
     <col width="42" customWidth="1" min="30" max="30"/>
     <col width="42" customWidth="1" min="31" max="31"/>
@@ -5694,14 +5694,14 @@
       </c>
       <c r="H45" s="2" t="inlineStr">
         <is>
-          <t>Nemuno g. 1, Gelgaudiškis</t>
+          <t>Vakarų g. 33 D, 71431, Gelgaudiškis</t>
         </is>
       </c>
       <c r="I45" s="3" t="n">
-        <v>55.0823469</v>
+        <v>55.07067</v>
       </c>
       <c r="J45" s="3" t="n">
-        <v>22.9903537</v>
+        <v>22.976723</v>
       </c>
       <c r="K45" s="2" t="inlineStr">
         <is>
@@ -5710,12 +5710,12 @@
       </c>
       <c r="L45" s="2" t="inlineStr">
         <is>
-          <t>Lietuvos geolokatorius</t>
+          <t>GLG kontaktų puslapis</t>
         </is>
       </c>
       <c r="M45" s="2" t="inlineStr">
         <is>
-          <t>https://hub.arcgis.com/content/b9e27b4266524b39bc651d6a26480b87</t>
+          <t>https://glg.lt/kontaktai/</t>
         </is>
       </c>
       <c r="N45" s="2" t="inlineStr">
@@ -5725,7 +5725,7 @@
       </c>
       <c r="O45" s="2" t="inlineStr">
         <is>
-          <t>Gelžbetonis</t>
+          <t>Betono mišiniai ir gelžbetonis</t>
         </is>
       </c>
       <c r="P45" s="2" t="inlineStr">
@@ -5737,15 +5737,17 @@
       <c r="R45" s="2" t="inlineStr"/>
       <c r="S45" s="2" t="inlineStr">
         <is>
-          <t>Viešai skelbiami gelžbetonio gaminiai.</t>
+          <t>Įmonė gamina gelžbetonio gaminius, prekinį ir hidrotechninį betoną bei smėlbetonio mišinius.</t>
         </is>
       </c>
       <c r="T45" s="4" t="n">
-        <v>0.78</v>
+        <v>0.9</v>
       </c>
       <c r="U45" s="5" t="n"/>
       <c r="V45" s="6" t="n"/>
-      <c r="W45" s="5" t="n"/>
+      <c r="W45" s="5" t="n">
+        <v>100</v>
+      </c>
       <c r="X45" s="5" t="n"/>
       <c r="Y45" s="2" t="inlineStr">
         <is>
@@ -5758,16 +5760,20 @@
         </is>
       </c>
       <c r="AA45" s="2" t="inlineStr"/>
-      <c r="AB45" s="2" t="inlineStr"/>
+      <c r="AB45" s="2" t="inlineStr">
+        <is>
+          <t>https://glg.lt/apie-imone/</t>
+        </is>
+      </c>
       <c r="AC45" s="2" t="inlineStr"/>
       <c r="AD45" s="2" t="inlineStr">
         <is>
-          <t>https://glg.lt/kontaktai/</t>
+          <t>https://glg.lt/betonas/betono-misiniai/</t>
         </is>
       </c>
       <c r="AE45" s="2" t="inlineStr">
         <is>
-          <t>Reikia patikslinti tikslų gamyklos adresą.</t>
+          <t>Patikslinta pagal oficialų glg.lt kontaktų ir įmonės aprašymo puslapius.</t>
         </is>
       </c>
       <c r="AF45" s="2" t="inlineStr">
@@ -7566,7 +7572,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-06-30T12:21:46.857357+00:00</t>
+          <t>2026-06-30T18:58:32.115728+00:00</t>
         </is>
       </c>
     </row>
@@ -7621,7 +7627,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-06-30T12:21:46.857357+00:00</t>
+          <t>2026-06-30T18:58:32.115728+00:00</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">

</xml_diff>

<commit_message>
Update official company contact data batch 1
</commit_message>
<xml_diff>
--- a/data/companies.xlsx
+++ b/data/companies.xlsx
@@ -515,7 +515,7 @@
     <col width="12" customWidth="1" min="9" max="9"/>
     <col width="12" customWidth="1" min="10" max="10"/>
     <col width="42" customWidth="1" min="11" max="11"/>
-    <col width="24" customWidth="1" min="12" max="12"/>
+    <col width="42" customWidth="1" min="12" max="12"/>
     <col width="42" customWidth="1" min="13" max="13"/>
     <col width="20" customWidth="1" min="14" max="14"/>
     <col width="32" customWidth="1" min="15" max="15"/>
@@ -1030,7 +1030,7 @@
       </c>
       <c r="Z4" s="2" t="inlineStr">
         <is>
-          <t>https://spsc.lt/registrai/regsapp/ser_produktai_view.php?editid1=13020</t>
+          <t>https://betonocentras.lt/kontaktai/</t>
         </is>
       </c>
       <c r="AA4" s="2" t="inlineStr"/>
@@ -1038,12 +1038,12 @@
       <c r="AC4" s="2" t="inlineStr"/>
       <c r="AD4" s="2" t="inlineStr">
         <is>
-          <t>https://spsc.lt/registrai/regsapp/ser_produktai_view.php?editid1=13020</t>
+          <t>https://betonocentras.lt/kontaktai/</t>
         </is>
       </c>
       <c r="AE4" s="2" t="inlineStr">
         <is>
-          <t>Adresas ir koordinatės patikslinti pagal Google Maps ir SPSC registro įrašą.</t>
+          <t>Oficialiame Betono centro kontaktų puslapyje patvirtintas Klaipėdos padalinys.</t>
         </is>
       </c>
       <c r="AF4" s="2" t="inlineStr">
@@ -2254,24 +2254,24 @@
         </is>
       </c>
       <c r="I15" s="3" t="n">
-        <v>54.6482969</v>
+        <v>54.6471731</v>
       </c>
       <c r="J15" s="3" t="n">
-        <v>25.1958961</v>
+        <v>25.1918488</v>
       </c>
       <c r="K15" s="2" t="inlineStr">
         <is>
-          <t>Tikslus adreso taškas</t>
+          <t>Oficialios Google Maps nuorodos taškas</t>
         </is>
       </c>
       <c r="L15" s="2" t="inlineStr">
         <is>
-          <t>Lietuvos geolokatorius</t>
+          <t>GKG3 kontaktų puslapis</t>
         </is>
       </c>
       <c r="M15" s="2" t="inlineStr">
         <is>
-          <t>https://hub.arcgis.com/content/b9e27b4266524b39bc651d6a26480b87</t>
+          <t>https://gkg3.lt/kontaktai/</t>
         </is>
       </c>
       <c r="N15" s="2" t="inlineStr">
@@ -2310,7 +2310,7 @@
       </c>
       <c r="Z15" s="2" t="inlineStr">
         <is>
-          <t>https://www.gkg3.lt/</t>
+          <t>https://gkg3.lt/kontaktai/</t>
         </is>
       </c>
       <c r="AA15" s="2" t="inlineStr"/>
@@ -2318,10 +2318,14 @@
       <c r="AC15" s="2" t="inlineStr"/>
       <c r="AD15" s="2" t="inlineStr">
         <is>
-          <t>https://www.gkg3.lt/</t>
-        </is>
-      </c>
-      <c r="AE15" s="2" t="inlineStr"/>
+          <t>https://gkg3.lt/kontaktai/</t>
+        </is>
+      </c>
+      <c r="AE15" s="2" t="inlineStr">
+        <is>
+          <t>Koordinatės patikslintos pagal oficialaus GKG3 kontaktų puslapio Google Maps nuorodą.</t>
+        </is>
+      </c>
       <c r="AF15" s="2" t="inlineStr">
         <is>
           <t>2026-06-29</t>
@@ -2810,24 +2814,24 @@
         </is>
       </c>
       <c r="I20" s="3" t="n">
-        <v>55.9494778</v>
+        <v>55.9495824</v>
       </c>
       <c r="J20" s="3" t="n">
-        <v>23.3103706</v>
+        <v>23.3105291</v>
       </c>
       <c r="K20" s="2" t="inlineStr">
         <is>
-          <t>Tikslus adreso taškas</t>
+          <t>Oficialios žemėlapio nuorodos taškas</t>
         </is>
       </c>
       <c r="L20" s="2" t="inlineStr">
         <is>
-          <t>Lietuvos geolokatorius</t>
+          <t>Gelžbetoninės konstrukcijos kontaktų puslapis</t>
         </is>
       </c>
       <c r="M20" s="2" t="inlineStr">
         <is>
-          <t>https://hub.arcgis.com/content/b9e27b4266524b39bc651d6a26480b87</t>
+          <t>https://www.gelzbetonineskonstrukcijos.lt/contacts/</t>
         </is>
       </c>
       <c r="N20" s="2" t="inlineStr">
@@ -2866,7 +2870,7 @@
       </c>
       <c r="Z20" s="2" t="inlineStr">
         <is>
-          <t>https://www.gelzbetonineskonstrukcijos.lt/</t>
+          <t>https://www.gelzbetonineskonstrukcijos.lt/contacts/</t>
         </is>
       </c>
       <c r="AA20" s="2" t="inlineStr"/>
@@ -2874,10 +2878,14 @@
       <c r="AC20" s="2" t="inlineStr"/>
       <c r="AD20" s="2" t="inlineStr">
         <is>
-          <t>https://www.gelzbetonineskonstrukcijos.lt/</t>
-        </is>
-      </c>
-      <c r="AE20" s="2" t="inlineStr"/>
+          <t>https://www.gelzbetonineskonstrukcijos.lt/contacts/</t>
+        </is>
+      </c>
+      <c r="AE20" s="2" t="inlineStr">
+        <is>
+          <t>Koordinatės patikslintos pagal oficialaus kontaktų puslapio žemėlapio tašką.</t>
+        </is>
+      </c>
       <c r="AF20" s="2" t="inlineStr">
         <is>
           <t>2026-06-29</t>
@@ -3252,38 +3260,38 @@
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>Kaunas</t>
+          <t>Serdokai</t>
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr">
         <is>
-          <t>Kauno m. sav.</t>
+          <t>Vilkaviškio r. sav.</t>
         </is>
       </c>
       <c r="H24" s="2" t="inlineStr">
         <is>
-          <t>Marvelės g. 199B, Kaunas</t>
+          <t>Gėlių g. 34, Serdokų k., Vilkaviškio r., LT-70201</t>
         </is>
       </c>
       <c r="I24" s="3" t="n">
-        <v>54.9007881</v>
+        <v>54.6279368</v>
       </c>
       <c r="J24" s="3" t="n">
-        <v>23.8489377</v>
+        <v>23.0871345</v>
       </c>
       <c r="K24" s="2" t="inlineStr">
         <is>
-          <t>Tikslus adreso taškas</t>
+          <t>Vietovės lygio taškas; reikia tikslesnio adreso taško</t>
         </is>
       </c>
       <c r="L24" s="2" t="inlineStr">
         <is>
-          <t>Lietuvos geolokatorius</t>
+          <t>ArcGIS geokodavimas pagal oficialų Statkasta adresą</t>
         </is>
       </c>
       <c r="M24" s="2" t="inlineStr">
         <is>
-          <t>https://hub.arcgis.com/content/b9e27b4266524b39bc651d6a26480b87</t>
+          <t>https://statkasta.lt/kontaktai/</t>
         </is>
       </c>
       <c r="N24" s="2" t="inlineStr">
@@ -3322,7 +3330,7 @@
       </c>
       <c r="Z24" s="2" t="inlineStr">
         <is>
-          <t>https://statkasta.lt/</t>
+          <t>https://statkasta.lt/kontaktai/</t>
         </is>
       </c>
       <c r="AA24" s="2" t="inlineStr"/>
@@ -3330,10 +3338,14 @@
       <c r="AC24" s="2" t="inlineStr"/>
       <c r="AD24" s="2" t="inlineStr">
         <is>
-          <t>https://statkasta.lt/</t>
-        </is>
-      </c>
-      <c r="AE24" s="2" t="inlineStr"/>
+          <t>https://statkasta.lt/kontaktai/</t>
+        </is>
+      </c>
+      <c r="AE24" s="2" t="inlineStr">
+        <is>
+          <t>Oficialiame Statkasta kontaktų puslapyje nurodytas adresas Gėlių g. 34, Serdokų k.; koordinatės geokoduotos iki vietovės lygio.</t>
+        </is>
+      </c>
       <c r="AF24" s="2" t="inlineStr">
         <is>
           <t>2026-06-29</t>
@@ -3430,7 +3442,7 @@
       </c>
       <c r="Z25" s="2" t="inlineStr">
         <is>
-          <t>https://autokausta.lt/</t>
+          <t>https://www.autokausta.lt/apie-mus/betonas/</t>
         </is>
       </c>
       <c r="AA25" s="2" t="inlineStr"/>
@@ -3438,12 +3450,12 @@
       <c r="AC25" s="2" t="inlineStr"/>
       <c r="AD25" s="2" t="inlineStr">
         <is>
-          <t>https://autokausta.lt/</t>
+          <t>https://www.autokausta.lt/apie-mus/betonas/</t>
         </is>
       </c>
       <c r="AE25" s="2" t="inlineStr">
         <is>
-          <t>Betono mazgo adresas patikslintas pagal lietuviškus viešus šaltinius; koordinatės nustatytos Lietuvos geolokatoriumi.</t>
+          <t>Oficialus Autokausta betono puslapis patvirtina betono veiklą ir Marvelės g. 199B kontaktą.</t>
         </is>
       </c>
       <c r="AF25" s="2" t="inlineStr">
@@ -3545,12 +3557,12 @@
       <c r="X26" s="5" t="n"/>
       <c r="Y26" s="2" t="inlineStr">
         <is>
-          <t>https://betonobaze.lt/</t>
+          <t>https://www.betonobaze.lt/</t>
         </is>
       </c>
       <c r="Z26" s="2" t="inlineStr">
         <is>
-          <t>https://betonobaze.lt/</t>
+          <t>https://www.betonobaze.lt/kontaktai</t>
         </is>
       </c>
       <c r="AA26" s="2" t="inlineStr"/>
@@ -3558,12 +3570,12 @@
       <c r="AC26" s="2" t="inlineStr"/>
       <c r="AD26" s="2" t="inlineStr">
         <is>
-          <t>https://betonobaze.lt/</t>
+          <t>https://www.betonobaze.lt/kontaktai</t>
         </is>
       </c>
       <c r="AE26" s="2" t="inlineStr">
         <is>
-          <t>Adresas patikslintas pagal lietuviškus viešus šaltinius; koordinatės nustatytos Lietuvos geolokatoriumi.</t>
+          <t>Oficialus kontaktų puslapis patvirtina Elektrinės g. 11 adresą ir betono bazės veiklą.</t>
         </is>
       </c>
       <c r="AF26" s="2" t="inlineStr">
@@ -3666,7 +3678,7 @@
       </c>
       <c r="Z27" s="2" t="inlineStr">
         <is>
-          <t>https://transdosa.lt/</t>
+          <t>https://www.transdosa.lt/kontaktai/</t>
         </is>
       </c>
       <c r="AA27" s="2" t="inlineStr"/>
@@ -3674,12 +3686,12 @@
       <c r="AC27" s="2" t="inlineStr"/>
       <c r="AD27" s="2" t="inlineStr">
         <is>
-          <t>https://transdosa.lt/</t>
+          <t>https://www.transdosa.lt/betonas/</t>
         </is>
       </c>
       <c r="AE27" s="2" t="inlineStr">
         <is>
-          <t>Adresas patikslintas pagal lietuviškus viešus šaltinius; koordinatės nustatytos Lietuvos geolokatoriumi.</t>
+          <t>Oficialūs Transdosa kontaktų ir betono puslapiai patvirtina Margų karjero betono gamybą adresu Žvyro g. 2A.</t>
         </is>
       </c>
       <c r="AF27" s="2" t="inlineStr">
@@ -3790,12 +3802,12 @@
       <c r="AC28" s="2" t="inlineStr"/>
       <c r="AD28" s="2" t="inlineStr">
         <is>
-          <t>https://sodbeta.lt/</t>
+          <t>https://sodbeta.lt/betonas/betono-misiniai/</t>
         </is>
       </c>
       <c r="AE28" s="2" t="inlineStr">
         <is>
-          <t>Papildomai rasta pagal požymį betono gaminiai.</t>
+          <t>Oficiali Sodbeta svetainė patvirtina Sodo g. 20 adresą ir betono mišinių puslapį.</t>
         </is>
       </c>
       <c r="AF28" s="2" t="inlineStr">
@@ -3846,24 +3858,24 @@
         </is>
       </c>
       <c r="I29" s="3" t="n">
-        <v>54.4260262</v>
+        <v>54.426129</v>
       </c>
       <c r="J29" s="3" t="n">
-        <v>24.014948</v>
+        <v>24.016482</v>
       </c>
       <c r="K29" s="2" t="inlineStr">
         <is>
-          <t>Tikslus adreso taškas</t>
+          <t>Oficialaus kontaktų puslapio žemėlapio taškas</t>
         </is>
       </c>
       <c r="L29" s="2" t="inlineStr">
         <is>
-          <t>Lietuvos geolokatorius</t>
+          <t>Alytaus gelžbetonis kontaktų puslapis</t>
         </is>
       </c>
       <c r="M29" s="2" t="inlineStr">
         <is>
-          <t>https://hub.arcgis.com/content/b9e27b4266524b39bc651d6a26480b87</t>
+          <t>https://alytausgelzbetonis.lt/kontaktai/</t>
         </is>
       </c>
       <c r="N29" s="2" t="inlineStr">
@@ -3902,7 +3914,7 @@
       </c>
       <c r="Z29" s="2" t="inlineStr">
         <is>
-          <t>https://data.gov.lt/dataset/juridiniu-asmenu-ekonomines-veiklos-rusys-ir-instituciniai-sektoriai/</t>
+          <t>https://alytausgelzbetonis.lt/kontaktai/</t>
         </is>
       </c>
       <c r="AA29" s="2" t="inlineStr"/>
@@ -3915,7 +3927,7 @@
       </c>
       <c r="AE29" s="2" t="inlineStr">
         <is>
-          <t>Įmonė jau buvo sąraše kaip gelžbetonio gamintoja; veikla patikslinta pagal EVRK 23.63 atvirų duomenų sąrašą.</t>
+          <t>Patikslinta pagal oficialų kontaktų puslapį.</t>
         </is>
       </c>
       <c r="AF29" s="2" t="inlineStr">
@@ -3958,28 +3970,28 @@
       </c>
       <c r="H30" s="2" t="inlineStr">
         <is>
-          <t>Vingio g. 2M, Marijampolė</t>
+          <t>Vingio g. 2M, LT-68131 Marijampolė</t>
         </is>
       </c>
       <c r="I30" s="3" t="n">
-        <v>54.5358398</v>
+        <v>54.5356806</v>
       </c>
       <c r="J30" s="3" t="n">
-        <v>23.3344441</v>
+        <v>23.3349754</v>
       </c>
       <c r="K30" s="2" t="inlineStr">
         <is>
-          <t>Tikslus adreso taškas</t>
+          <t>Oficialios Google Maps nuorodos taškas</t>
         </is>
       </c>
       <c r="L30" s="2" t="inlineStr">
         <is>
-          <t>Lietuvos geolokatorius</t>
+          <t>Gernora kontaktų puslapis</t>
         </is>
       </c>
       <c r="M30" s="2" t="inlineStr">
         <is>
-          <t>https://hub.arcgis.com/content/b9e27b4266524b39bc651d6a26480b87</t>
+          <t>https://gernora.lt/kontaktai/</t>
         </is>
       </c>
       <c r="N30" s="2" t="inlineStr">
@@ -4018,7 +4030,7 @@
       </c>
       <c r="Z30" s="2" t="inlineStr">
         <is>
-          <t>https://gernora.lt/</t>
+          <t>https://gernora.lt/kontaktai/</t>
         </is>
       </c>
       <c r="AA30" s="2" t="inlineStr"/>
@@ -4026,12 +4038,12 @@
       <c r="AC30" s="2" t="inlineStr"/>
       <c r="AD30" s="2" t="inlineStr">
         <is>
-          <t>https://gernora.lt/</t>
+          <t>https://gernora.lt/kontaktai/</t>
         </is>
       </c>
       <c r="AE30" s="2" t="inlineStr">
         <is>
-          <t>Reikia patikslinti našumą.</t>
+          <t>Koordinatės patikslintos pagal oficialaus Gernora kontaktų puslapio Google Maps nuorodą.</t>
         </is>
       </c>
       <c r="AF30" s="2" t="inlineStr">
@@ -4942,7 +4954,7 @@
       </c>
       <c r="Z38" s="2" t="inlineStr">
         <is>
-          <t>https://topbeton.lt/</t>
+          <t>https://www.topbeton.lt/kontaktai/</t>
         </is>
       </c>
       <c r="AA38" s="2" t="inlineStr"/>
@@ -4950,12 +4962,12 @@
       <c r="AC38" s="2" t="inlineStr"/>
       <c r="AD38" s="2" t="inlineStr">
         <is>
-          <t>https://topbeton.lt/</t>
+          <t>https://www.topbeton.lt/kontaktai/</t>
         </is>
       </c>
       <c r="AE38" s="2" t="inlineStr">
         <is>
-          <t>Papildomai rasta pagal prekinio betono požymį.</t>
+          <t>Oficialus kontaktų puslapis patvirtina Beržų g. 5C adresą.</t>
         </is>
       </c>
       <c r="AF38" s="2" t="inlineStr">
@@ -5406,7 +5418,7 @@
       </c>
       <c r="Z42" s="2" t="inlineStr">
         <is>
-          <t>https://utenosbetonas.lt/</t>
+          <t>https://www.utenosbetonas.lt/kontaktai/</t>
         </is>
       </c>
       <c r="AA42" s="2" t="inlineStr"/>
@@ -5414,12 +5426,12 @@
       <c r="AC42" s="2" t="inlineStr"/>
       <c r="AD42" s="2" t="inlineStr">
         <is>
-          <t>https://utenosbetonas.lt/</t>
+          <t>https://www.utenosbetonas.lt/kontaktai/</t>
         </is>
       </c>
       <c r="AE42" s="2" t="inlineStr">
         <is>
-          <t>Reikia patikslinti našumą.</t>
+          <t>Oficialus kontaktų puslapis patvirtina Metalo g. 9B adresą.</t>
         </is>
       </c>
       <c r="AF42" s="2" t="inlineStr">
@@ -7572,7 +7584,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-06-30T18:58:32.115728+00:00</t>
+          <t>2026-06-30T19:20:50.501274+00:00</t>
         </is>
       </c>
     </row>
@@ -7627,7 +7639,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-06-30T18:58:32.115728+00:00</t>
+          <t>2026-06-30T19:20:50.501274+00:00</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">

</xml_diff>

<commit_message>
Update Heidelberg official contact sources
</commit_message>
<xml_diff>
--- a/data/companies.xlsx
+++ b/data/companies.xlsx
@@ -1493,12 +1493,12 @@
       <c r="X8" s="5" t="n"/>
       <c r="Y8" s="2" t="inlineStr">
         <is>
-          <t>https://www.heidelbergmaterials.lt/</t>
+          <t>https://www.betonas.heidelbergmaterials.lt/lt</t>
         </is>
       </c>
       <c r="Z8" s="2" t="inlineStr">
         <is>
-          <t>https://www.heidelbergmaterials.lt/</t>
+          <t>https://www.betonas.heidelbergmaterials.lt/lt/kontaktine-informacija-0</t>
         </is>
       </c>
       <c r="AA8" s="2" t="inlineStr"/>
@@ -1506,10 +1506,14 @@
       <c r="AC8" s="2" t="inlineStr"/>
       <c r="AD8" s="2" t="inlineStr">
         <is>
-          <t>https://www.heidelbergmaterials.lt/</t>
-        </is>
-      </c>
-      <c r="AE8" s="2" t="inlineStr"/>
+          <t>https://www.betonas.heidelbergmaterials.lt/lt/kontaktine-informacija-0</t>
+        </is>
+      </c>
+      <c r="AE8" s="2" t="inlineStr">
+        <is>
+          <t>Oficialus Heidelberg Materials Lietuva Betonas kontaktų puslapis patvirtina betono užsakymų padalinius Lietuvoje.</t>
+        </is>
+      </c>
       <c r="AF8" s="2" t="inlineStr">
         <is>
           <t>2026-06-29</t>
@@ -1609,12 +1613,12 @@
       <c r="X9" s="5" t="n"/>
       <c r="Y9" s="2" t="inlineStr">
         <is>
-          <t>https://www.heidelbergmaterials.lt/</t>
+          <t>https://www.betonas.heidelbergmaterials.lt/lt</t>
         </is>
       </c>
       <c r="Z9" s="2" t="inlineStr">
         <is>
-          <t>https://www.heidelbergmaterials.lt/</t>
+          <t>https://www.betonas.heidelbergmaterials.lt/lt/kontaktine-informacija-0</t>
         </is>
       </c>
       <c r="AA9" s="2" t="inlineStr"/>
@@ -1622,10 +1626,14 @@
       <c r="AC9" s="2" t="inlineStr"/>
       <c r="AD9" s="2" t="inlineStr">
         <is>
-          <t>https://www.heidelbergmaterials.lt/</t>
-        </is>
-      </c>
-      <c r="AE9" s="2" t="inlineStr"/>
+          <t>https://www.betonas.heidelbergmaterials.lt/lt/kontaktine-informacija-0</t>
+        </is>
+      </c>
+      <c r="AE9" s="2" t="inlineStr">
+        <is>
+          <t>Oficialus Heidelberg Materials Lietuva Betonas kontaktų puslapis patvirtina betono užsakymų padalinius Lietuvoje.</t>
+        </is>
+      </c>
       <c r="AF9" s="2" t="inlineStr">
         <is>
           <t>2026-06-29</t>
@@ -1725,12 +1733,12 @@
       <c r="X10" s="5" t="n"/>
       <c r="Y10" s="2" t="inlineStr">
         <is>
-          <t>https://www.heidelbergmaterials.lt/</t>
+          <t>https://www.betonas.heidelbergmaterials.lt/lt</t>
         </is>
       </c>
       <c r="Z10" s="2" t="inlineStr">
         <is>
-          <t>https://www.heidelbergmaterials.lt/</t>
+          <t>https://www.betonas.heidelbergmaterials.lt/lt/kontaktine-informacija-0</t>
         </is>
       </c>
       <c r="AA10" s="2" t="inlineStr"/>
@@ -1738,10 +1746,14 @@
       <c r="AC10" s="2" t="inlineStr"/>
       <c r="AD10" s="2" t="inlineStr">
         <is>
-          <t>https://www.heidelbergmaterials.lt/</t>
-        </is>
-      </c>
-      <c r="AE10" s="2" t="inlineStr"/>
+          <t>https://www.betonas.heidelbergmaterials.lt/lt/kontaktine-informacija-0</t>
+        </is>
+      </c>
+      <c r="AE10" s="2" t="inlineStr">
+        <is>
+          <t>Oficialus Heidelberg Materials Lietuva Betonas kontaktų puslapis patvirtina betono užsakymų padalinius Lietuvoje.</t>
+        </is>
+      </c>
       <c r="AF10" s="2" t="inlineStr">
         <is>
           <t>2026-06-29</t>
@@ -1841,12 +1853,12 @@
       <c r="X11" s="5" t="n"/>
       <c r="Y11" s="2" t="inlineStr">
         <is>
-          <t>https://www.heidelbergmaterials.lt/</t>
+          <t>https://www.betonas.heidelbergmaterials.lt/lt</t>
         </is>
       </c>
       <c r="Z11" s="2" t="inlineStr">
         <is>
-          <t>https://www.heidelbergmaterials.lt/</t>
+          <t>https://www.betonas.heidelbergmaterials.lt/lt/kontaktine-informacija-0</t>
         </is>
       </c>
       <c r="AA11" s="2" t="inlineStr"/>
@@ -1854,10 +1866,14 @@
       <c r="AC11" s="2" t="inlineStr"/>
       <c r="AD11" s="2" t="inlineStr">
         <is>
-          <t>https://www.heidelbergmaterials.lt/</t>
-        </is>
-      </c>
-      <c r="AE11" s="2" t="inlineStr"/>
+          <t>https://www.betonas.heidelbergmaterials.lt/lt/kontaktine-informacija-0</t>
+        </is>
+      </c>
+      <c r="AE11" s="2" t="inlineStr">
+        <is>
+          <t>Oficialus Heidelberg Materials Lietuva Betonas kontaktų puslapis patvirtina betono užsakymų padalinius Lietuvoje.</t>
+        </is>
+      </c>
       <c r="AF11" s="2" t="inlineStr">
         <is>
           <t>2026-06-29</t>
@@ -1957,12 +1973,12 @@
       <c r="X12" s="5" t="n"/>
       <c r="Y12" s="2" t="inlineStr">
         <is>
-          <t>https://www.heidelbergmaterials.lt/</t>
+          <t>https://www.betonas.heidelbergmaterials.lt/lt</t>
         </is>
       </c>
       <c r="Z12" s="2" t="inlineStr">
         <is>
-          <t>https://www.heidelbergmaterials.lt/</t>
+          <t>https://www.betonas.heidelbergmaterials.lt/lt/kontaktine-informacija-0</t>
         </is>
       </c>
       <c r="AA12" s="2" t="inlineStr"/>
@@ -1970,10 +1986,14 @@
       <c r="AC12" s="2" t="inlineStr"/>
       <c r="AD12" s="2" t="inlineStr">
         <is>
-          <t>https://www.heidelbergmaterials.lt/</t>
-        </is>
-      </c>
-      <c r="AE12" s="2" t="inlineStr"/>
+          <t>https://www.betonas.heidelbergmaterials.lt/lt/kontaktine-informacija-0</t>
+        </is>
+      </c>
+      <c r="AE12" s="2" t="inlineStr">
+        <is>
+          <t>Oficialus Heidelberg Materials Lietuva Betonas kontaktų puslapis patvirtina betono užsakymų padalinius Lietuvoje.</t>
+        </is>
+      </c>
       <c r="AF12" s="2" t="inlineStr">
         <is>
           <t>2026-06-29</t>
@@ -2073,12 +2093,12 @@
       <c r="X13" s="5" t="n"/>
       <c r="Y13" s="2" t="inlineStr">
         <is>
-          <t>https://www.heidelbergmaterials.lt/</t>
+          <t>https://www.betonas.heidelbergmaterials.lt/lt</t>
         </is>
       </c>
       <c r="Z13" s="2" t="inlineStr">
         <is>
-          <t>https://www.heidelbergmaterials.lt/</t>
+          <t>https://www.betonas.heidelbergmaterials.lt/lt/kontaktine-informacija-0</t>
         </is>
       </c>
       <c r="AA13" s="2" t="inlineStr"/>
@@ -2086,12 +2106,12 @@
       <c r="AC13" s="2" t="inlineStr"/>
       <c r="AD13" s="2" t="inlineStr">
         <is>
-          <t>https://www.heidelbergmaterials.lt/</t>
+          <t>https://www.betonas.heidelbergmaterials.lt/lt/kontaktine-informacija-0</t>
         </is>
       </c>
       <c r="AE13" s="2" t="inlineStr">
         <is>
-          <t>Koordinatės patikrintos Lietuvos geolokatoriumi, bet rastas tik gatvės arba vietovės lygio taškas.</t>
+          <t>Oficialus Heidelberg Materials Lietuva Betonas kontaktų puslapis patvirtina betono užsakymų padalinius Lietuvoje.</t>
         </is>
       </c>
       <c r="AF13" s="2" t="inlineStr">
@@ -7584,7 +7604,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-06-30T19:20:50.501274+00:00</t>
+          <t>2026-06-30T19:25:45.266075+00:00</t>
         </is>
       </c>
     </row>
@@ -7639,7 +7659,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-06-30T19:20:50.501274+00:00</t>
+          <t>2026-06-30T19:25:45.266075+00:00</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">

</xml_diff>

<commit_message>
Update additional official company sources
</commit_message>
<xml_diff>
--- a/data/companies.xlsx
+++ b/data/companies.xlsx
@@ -2667,10 +2667,14 @@
       <c r="V18" s="6" t="n"/>
       <c r="W18" s="5" t="n"/>
       <c r="X18" s="5" t="n"/>
-      <c r="Y18" s="2" t="inlineStr"/>
+      <c r="Y18" s="2" t="inlineStr">
+        <is>
+          <t>https://www.kaunogelzbetonis.lt/</t>
+        </is>
+      </c>
       <c r="Z18" s="2" t="inlineStr">
         <is>
-          <t>https://www.kaunogelzbetonis.lt/</t>
+          <t>https://www.kaunogelzbetonis.lt/kontaktai/</t>
         </is>
       </c>
       <c r="AA18" s="2" t="inlineStr"/>
@@ -2678,10 +2682,14 @@
       <c r="AC18" s="2" t="inlineStr"/>
       <c r="AD18" s="2" t="inlineStr">
         <is>
-          <t>https://www.kaunogelzbetonis.lt/</t>
-        </is>
-      </c>
-      <c r="AE18" s="2" t="inlineStr"/>
+          <t>https://www.kaunogelzbetonis.lt/kontaktai/</t>
+        </is>
+      </c>
+      <c r="AE18" s="2" t="inlineStr">
+        <is>
+          <t>Oficialus Kauno gelžbetonio kontaktų puslapis patvirtina Pramonės pr. 8 adresą.</t>
+        </is>
+      </c>
       <c r="AF18" s="2" t="inlineStr">
         <is>
           <t>2026-06-29</t>
@@ -2775,7 +2783,11 @@
       <c r="V19" s="6" t="n"/>
       <c r="W19" s="5" t="n"/>
       <c r="X19" s="5" t="n"/>
-      <c r="Y19" s="2" t="inlineStr"/>
+      <c r="Y19" s="2" t="inlineStr">
+        <is>
+          <t>https://ukmergesgelzbetonis.lt/</t>
+        </is>
+      </c>
       <c r="Z19" s="2" t="inlineStr">
         <is>
           <t>https://ukmergesgelzbetonis.lt/</t>
@@ -2789,7 +2801,11 @@
           <t>https://ukmergesgelzbetonis.lt/</t>
         </is>
       </c>
-      <c r="AE19" s="2" t="inlineStr"/>
+      <c r="AE19" s="2" t="inlineStr">
+        <is>
+          <t>Oficiali Ukmergės gelžbetonio svetainė palikta kaip pagrindinis šaltinis; naujų patikimų koordinačių nerasta.</t>
+        </is>
+      </c>
       <c r="AF19" s="2" t="inlineStr">
         <is>
           <t>2026-06-29</t>
@@ -6469,19 +6485,27 @@
       <c r="V51" s="6" t="n"/>
       <c r="W51" s="5" t="n"/>
       <c r="X51" s="5" t="n"/>
-      <c r="Y51" s="2" t="inlineStr"/>
+      <c r="Y51" s="2" t="inlineStr">
+        <is>
+          <t>https://betonastaurageje.lt/</t>
+        </is>
+      </c>
       <c r="Z51" s="2" t="inlineStr">
         <is>
-          <t>https://data.gov.lt/dataset/juridiniu-asmenu-ekonomines-veiklos-rusys-ir-instituciniai-sektoriai/</t>
+          <t>https://betonastaurageje.lt/kontaktai/</t>
         </is>
       </c>
       <c r="AA51" s="2" t="inlineStr"/>
       <c r="AB51" s="2" t="inlineStr"/>
       <c r="AC51" s="2" t="inlineStr"/>
-      <c r="AD51" s="2" t="inlineStr"/>
+      <c r="AD51" s="2" t="inlineStr">
+        <is>
+          <t>https://betonastaurageje.lt/betonas/</t>
+        </is>
+      </c>
       <c r="AE51" s="2" t="inlineStr">
         <is>
-          <t>Adresas geokoduotas pagal viešai randamą įmonės adresą; betono mazgo vietą verta patikslinti atskiru šaltiniu.</t>
+          <t>Oficiali Vinido svetainė patvirtina Gaurės g. 32 adresą, betono gamybą ir betono mazgą.</t>
         </is>
       </c>
       <c r="AF51" s="2" t="inlineStr">
@@ -6581,10 +6605,14 @@
       <c r="V52" s="6" t="n"/>
       <c r="W52" s="5" t="n"/>
       <c r="X52" s="5" t="n"/>
-      <c r="Y52" s="2" t="inlineStr"/>
+      <c r="Y52" s="2" t="inlineStr">
+        <is>
+          <t>https://santvara.eu/</t>
+        </is>
+      </c>
       <c r="Z52" s="2" t="inlineStr">
         <is>
-          <t>https://data.gov.lt/dataset/juridiniu-asmenu-ekonomines-veiklos-rusys-ir-instituciniai-sektoriai/</t>
+          <t>https://santvara.eu/</t>
         </is>
       </c>
       <c r="AA52" s="2" t="inlineStr"/>
@@ -6592,12 +6620,12 @@
       <c r="AC52" s="2" t="inlineStr"/>
       <c r="AD52" s="2" t="inlineStr">
         <is>
-          <t>https://chamber.lt/bendruomene/rumu-nariu-sarasas/nariai/santvara/</t>
+          <t>https://santvara.eu/</t>
         </is>
       </c>
       <c r="AE52" s="2" t="inlineStr">
         <is>
-          <t>Adresas geokoduotas pagal viešai randamą įmonės adresą; betono mazgo vietą verta patikslinti atskiru šaltiniu.</t>
+          <t>Oficiali Santvara svetainė patvirtina Aruodų g. 34 adresą ir betono bei birių medžiagų veiklą.</t>
         </is>
       </c>
       <c r="AF52" s="2" t="inlineStr">
@@ -6921,19 +6949,27 @@
       <c r="V55" s="6" t="n"/>
       <c r="W55" s="5" t="n"/>
       <c r="X55" s="5" t="n"/>
-      <c r="Y55" s="2" t="inlineStr"/>
+      <c r="Y55" s="2" t="inlineStr">
+        <is>
+          <t>https://ekobetonas.lt/</t>
+        </is>
+      </c>
       <c r="Z55" s="2" t="inlineStr">
         <is>
-          <t>https://data.gov.lt/dataset/juridiniu-asmenu-ekonomines-veiklos-rusys-ir-instituciniai-sektoriai/</t>
+          <t>https://ekobetonas.lt/kontaktai-betono-gamyba-armaturinis-plienas/</t>
         </is>
       </c>
       <c r="AA55" s="2" t="inlineStr"/>
       <c r="AB55" s="2" t="inlineStr"/>
       <c r="AC55" s="2" t="inlineStr"/>
-      <c r="AD55" s="2" t="inlineStr"/>
+      <c r="AD55" s="2" t="inlineStr">
+        <is>
+          <t>https://ekobetonas.lt/kontaktai-betono-gamyba-armaturinis-plienas/</t>
+        </is>
+      </c>
       <c r="AE55" s="2" t="inlineStr">
         <is>
-          <t>Adresas geokoduotas pagal viešai randamą įmonės adresą; betono mazgo vietą verta patikslinti atskiru šaltiniu.</t>
+          <t>Oficialus Ekobetonas kontaktų puslapis patvirtina Gamyklų g. 3 adresą ir betono užsakymų kontaktus.</t>
         </is>
       </c>
       <c r="AF55" s="2" t="inlineStr">
@@ -7145,19 +7181,27 @@
       <c r="V57" s="6" t="n"/>
       <c r="W57" s="5" t="n"/>
       <c r="X57" s="5" t="n"/>
-      <c r="Y57" s="2" t="inlineStr"/>
+      <c r="Y57" s="2" t="inlineStr">
+        <is>
+          <t>https://www.betoneura.lt/</t>
+        </is>
+      </c>
       <c r="Z57" s="2" t="inlineStr">
         <is>
-          <t>https://data.gov.lt/dataset/juridiniu-asmenu-ekonomines-veiklos-rusys-ir-instituciniai-sektoriai/</t>
+          <t>https://www.betoneura.lt/kontaktai/</t>
         </is>
       </c>
       <c r="AA57" s="2" t="inlineStr"/>
       <c r="AB57" s="2" t="inlineStr"/>
       <c r="AC57" s="2" t="inlineStr"/>
-      <c r="AD57" s="2" t="inlineStr"/>
+      <c r="AD57" s="2" t="inlineStr">
+        <is>
+          <t>https://www.betoneura.lt/kontaktai/</t>
+        </is>
+      </c>
       <c r="AE57" s="2" t="inlineStr">
         <is>
-          <t>Adresas geokoduotas pagal viešai randamą įmonės adresą; betono mazgo vietą verta patikslinti atskiru šaltiniu.</t>
+          <t>Oficialus Beton Eura kontaktų puslapis patvirtina Žilvičių g. 2 adresą ir rekvizitus.</t>
         </is>
       </c>
       <c r="AF57" s="2" t="inlineStr">
@@ -7604,7 +7648,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-06-30T19:25:45.266075+00:00</t>
+          <t>2026-06-30T19:33:43.490785+00:00</t>
         </is>
       </c>
     </row>
@@ -7659,7 +7703,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-06-30T19:25:45.266075+00:00</t>
+          <t>2026-06-30T19:33:43.490785+00:00</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">

</xml_diff>

<commit_message>
Update competitor map data
</commit_message>
<xml_diff>
--- a/data/companies.xlsx
+++ b/data/companies.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Įmonės" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Metaduomenys" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Importo žurnalas" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Įmonės" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Metaduomenys" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Importo žurnalas" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Įmonės'!$A$1:$AF$60</definedName>
@@ -7648,7 +7648,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-06-30T19:33:43.490785+00:00</t>
+          <t>2026-07-06T16:45:44.788666+00:00</t>
         </is>
       </c>
     </row>
@@ -7703,7 +7703,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-06-30T19:33:43.490785+00:00</t>
+          <t>2026-07-06T16:45:44.789546+00:00</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">

</xml_diff>

<commit_message>
Add mixer field and update plant technical data
</commit_message>
<xml_diff>
--- a/data/companies.xlsx
+++ b/data/companies.xlsx
@@ -1,18 +1,18 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Įmonės" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Metaduomenys" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Importo žurnalas" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Įmonės" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Metaduomenys" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Importo žurnalas" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Įmonės'!$A$1:$AF$60</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Įmonės'!$A$1:$AG$60</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -172,9 +172,9 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ImonesTable" displayName="ImonesTable" ref="A1:AF60" headerRowCount="1">
-  <autoFilter ref="A1:AF60"/>
-  <tableColumns count="32">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ImonesTable" displayName="ImonesTable" ref="A1:AG60" headerRowCount="1">
+  <autoFilter ref="A1:AG60"/>
+  <tableColumns count="33">
     <tableColumn id="1" name="Įrašo ID"/>
     <tableColumn id="2" name="Įmonės kodas"/>
     <tableColumn id="3" name="Įmonės pavadinimas"/>
@@ -191,22 +191,23 @@
     <tableColumn id="14" name="Veiklos tipas"/>
     <tableColumn id="15" name="Veikla"/>
     <tableColumn id="16" name="Betono mazgo / gamyklos pavadinimas"/>
-    <tableColumn id="17" name="Betono mazgo našumas"/>
-    <tableColumn id="18" name="Silosų skaičius"/>
-    <tableColumn id="19" name="Viešas betono mazgo / gamyklos aprašymas"/>
-    <tableColumn id="20" name="Klasifikavimo pasitikėjimas"/>
-    <tableColumn id="21" name="Įmonės apyvarta"/>
-    <tableColumn id="22" name="Apyvartos metai"/>
-    <tableColumn id="23" name="Darbuotojų skaičius"/>
-    <tableColumn id="24" name="Automobilių / transporto priemonių skaičius"/>
-    <tableColumn id="25" name="Interneto svetainė"/>
-    <tableColumn id="26" name="Pagrindinis šaltinis"/>
-    <tableColumn id="27" name="Apyvartos šaltinis"/>
-    <tableColumn id="28" name="Darbuotojų šaltinis"/>
-    <tableColumn id="29" name="Transporto šaltinis"/>
-    <tableColumn id="30" name="Betono mazgo / gamyklos šaltinis"/>
-    <tableColumn id="31" name="Pastaba / rankinis papildymas"/>
-    <tableColumn id="32" name="Paskutinio atnaujinimo data"/>
+    <tableColumn id="17" name="Maišyklė"/>
+    <tableColumn id="18" name="Našumas (realus)"/>
+    <tableColumn id="19" name="Silosų skaičius"/>
+    <tableColumn id="20" name="Viešas betono mazgo / gamyklos aprašymas"/>
+    <tableColumn id="21" name="Klasifikavimo pasitikėjimas"/>
+    <tableColumn id="22" name="Įmonės apyvarta"/>
+    <tableColumn id="23" name="Apyvartos metai"/>
+    <tableColumn id="24" name="Darbuotojų skaičius"/>
+    <tableColumn id="25" name="Automobilių / transporto priemonių skaičius"/>
+    <tableColumn id="26" name="Interneto svetainė"/>
+    <tableColumn id="27" name="Pagrindinis šaltinis"/>
+    <tableColumn id="28" name="Apyvartos šaltinis"/>
+    <tableColumn id="29" name="Darbuotojų šaltinis"/>
+    <tableColumn id="30" name="Transporto šaltinis"/>
+    <tableColumn id="31" name="Betono mazgo / gamyklos šaltinis"/>
+    <tableColumn id="32" name="Pastaba / rankinis papildymas"/>
+    <tableColumn id="33" name="Paskutinio atnaujinimo data"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -501,7 +502,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AF60"/>
+  <dimension ref="A1:AG60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="39" customWidth="1" min="1" max="1"/>
@@ -520,22 +521,23 @@
     <col width="20" customWidth="1" min="14" max="14"/>
     <col width="32" customWidth="1" min="15" max="15"/>
     <col width="40" customWidth="1" min="16" max="16"/>
-    <col width="30" customWidth="1" min="17" max="17"/>
-    <col width="17" customWidth="1" min="18" max="18"/>
-    <col width="42" customWidth="1" min="19" max="19"/>
-    <col width="29" customWidth="1" min="20" max="20"/>
-    <col width="17" customWidth="1" min="21" max="21"/>
+    <col width="27" customWidth="1" min="17" max="17"/>
+    <col width="30" customWidth="1" min="18" max="18"/>
+    <col width="17" customWidth="1" min="19" max="19"/>
+    <col width="42" customWidth="1" min="20" max="20"/>
+    <col width="29" customWidth="1" min="21" max="21"/>
     <col width="17" customWidth="1" min="22" max="22"/>
-    <col width="21" customWidth="1" min="23" max="23"/>
-    <col width="42" customWidth="1" min="24" max="24"/>
+    <col width="17" customWidth="1" min="23" max="23"/>
+    <col width="21" customWidth="1" min="24" max="24"/>
     <col width="42" customWidth="1" min="25" max="25"/>
     <col width="42" customWidth="1" min="26" max="26"/>
-    <col width="20" customWidth="1" min="27" max="27"/>
-    <col width="28" customWidth="1" min="28" max="28"/>
-    <col width="21" customWidth="1" min="29" max="29"/>
-    <col width="42" customWidth="1" min="30" max="30"/>
+    <col width="42" customWidth="1" min="27" max="27"/>
+    <col width="20" customWidth="1" min="28" max="28"/>
+    <col width="28" customWidth="1" min="29" max="29"/>
+    <col width="21" customWidth="1" min="30" max="30"/>
     <col width="42" customWidth="1" min="31" max="31"/>
-    <col width="29" customWidth="1" min="32" max="32"/>
+    <col width="42" customWidth="1" min="32" max="32"/>
+    <col width="29" customWidth="1" min="33" max="33"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -621,80 +623,85 @@
       </c>
       <c r="Q1" s="1" t="inlineStr">
         <is>
-          <t>Betono mazgo našumas</t>
+          <t>Maišyklė</t>
         </is>
       </c>
       <c r="R1" s="1" t="inlineStr">
         <is>
+          <t>Našumas (realus)</t>
+        </is>
+      </c>
+      <c r="S1" s="1" t="inlineStr">
+        <is>
           <t>Silosų skaičius</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>Viešas betono mazgo / gamyklos aprašymas</t>
         </is>
       </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>Klasifikavimo pasitikėjimas</t>
         </is>
       </c>
-      <c r="U1" s="1" t="inlineStr">
+      <c r="V1" s="1" t="inlineStr">
         <is>
           <t>Įmonės apyvarta</t>
         </is>
       </c>
-      <c r="V1" s="1" t="inlineStr">
+      <c r="W1" s="1" t="inlineStr">
         <is>
           <t>Apyvartos metai</t>
         </is>
       </c>
-      <c r="W1" s="1" t="inlineStr">
+      <c r="X1" s="1" t="inlineStr">
         <is>
           <t>Darbuotojų skaičius</t>
         </is>
       </c>
-      <c r="X1" s="1" t="inlineStr">
+      <c r="Y1" s="1" t="inlineStr">
         <is>
           <t>Automobilių / transporto priemonių skaičius</t>
         </is>
       </c>
-      <c r="Y1" s="1" t="inlineStr">
+      <c r="Z1" s="1" t="inlineStr">
         <is>
           <t>Interneto svetainė</t>
         </is>
       </c>
-      <c r="Z1" s="1" t="inlineStr">
+      <c r="AA1" s="1" t="inlineStr">
         <is>
           <t>Pagrindinis šaltinis</t>
         </is>
       </c>
-      <c r="AA1" s="1" t="inlineStr">
+      <c r="AB1" s="1" t="inlineStr">
         <is>
           <t>Apyvartos šaltinis</t>
         </is>
       </c>
-      <c r="AB1" s="1" t="inlineStr">
+      <c r="AC1" s="1" t="inlineStr">
         <is>
           <t>Darbuotojų šaltinis</t>
         </is>
       </c>
-      <c r="AC1" s="1" t="inlineStr">
+      <c r="AD1" s="1" t="inlineStr">
         <is>
           <t>Transporto šaltinis</t>
         </is>
       </c>
-      <c r="AD1" s="1" t="inlineStr">
+      <c r="AE1" s="1" t="inlineStr">
         <is>
           <t>Betono mazgo / gamyklos šaltinis</t>
         </is>
       </c>
-      <c r="AE1" s="1" t="inlineStr">
+      <c r="AF1" s="1" t="inlineStr">
         <is>
           <t>Pastaba / rankinis papildymas</t>
         </is>
       </c>
-      <c r="AF1" s="1" t="inlineStr">
+      <c r="AG1" s="1" t="inlineStr">
         <is>
           <t>Paskutinio atnaujinimo data</t>
         </is>
@@ -779,38 +786,39 @@
       </c>
       <c r="Q2" s="2" t="inlineStr"/>
       <c r="R2" s="2" t="inlineStr"/>
-      <c r="S2" s="2" t="inlineStr">
+      <c r="S2" s="2" t="inlineStr"/>
+      <c r="T2" s="2" t="inlineStr">
         <is>
           <t>Viešai skelbiamas Betono centro betono mazgas Vilniuje.</t>
         </is>
       </c>
-      <c r="T2" s="4" t="n">
+      <c r="U2" s="4" t="n">
         <v>0.9</v>
       </c>
-      <c r="U2" s="5" t="n"/>
-      <c r="V2" s="6" t="n"/>
-      <c r="W2" s="5" t="n"/>
+      <c r="V2" s="5" t="n"/>
+      <c r="W2" s="6" t="n"/>
       <c r="X2" s="5" t="n"/>
-      <c r="Y2" s="2" t="inlineStr">
+      <c r="Y2" s="5" t="n"/>
+      <c r="Z2" s="2" t="inlineStr">
         <is>
           <t>https://betonocentras.lt/</t>
         </is>
       </c>
-      <c r="Z2" s="2" t="inlineStr">
+      <c r="AA2" s="2" t="inlineStr">
         <is>
           <t>https://betonocentras.lt/kontaktai/</t>
         </is>
       </c>
-      <c r="AA2" s="2" t="inlineStr"/>
       <c r="AB2" s="2" t="inlineStr"/>
       <c r="AC2" s="2" t="inlineStr"/>
-      <c r="AD2" s="2" t="inlineStr">
+      <c r="AD2" s="2" t="inlineStr"/>
+      <c r="AE2" s="2" t="inlineStr">
         <is>
           <t>https://betonocentras.lt/kontaktai/</t>
         </is>
       </c>
-      <c r="AE2" s="2" t="inlineStr"/>
-      <c r="AF2" s="2" t="inlineStr">
+      <c r="AF2" s="2" t="inlineStr"/>
+      <c r="AG2" s="2" t="inlineStr">
         <is>
           <t>2026-06-29</t>
         </is>
@@ -895,38 +903,39 @@
       </c>
       <c r="Q3" s="2" t="inlineStr"/>
       <c r="R3" s="2" t="inlineStr"/>
-      <c r="S3" s="2" t="inlineStr">
+      <c r="S3" s="2" t="inlineStr"/>
+      <c r="T3" s="2" t="inlineStr">
         <is>
           <t>Viešai skelbiamas Betono centro betono mazgas Kaune.</t>
         </is>
       </c>
-      <c r="T3" s="4" t="n">
+      <c r="U3" s="4" t="n">
         <v>0.9</v>
       </c>
-      <c r="U3" s="5" t="n"/>
-      <c r="V3" s="6" t="n"/>
-      <c r="W3" s="5" t="n"/>
+      <c r="V3" s="5" t="n"/>
+      <c r="W3" s="6" t="n"/>
       <c r="X3" s="5" t="n"/>
-      <c r="Y3" s="2" t="inlineStr">
+      <c r="Y3" s="5" t="n"/>
+      <c r="Z3" s="2" t="inlineStr">
         <is>
           <t>https://betonocentras.lt/</t>
         </is>
       </c>
-      <c r="Z3" s="2" t="inlineStr">
+      <c r="AA3" s="2" t="inlineStr">
         <is>
           <t>https://betonocentras.lt/kontaktai/</t>
         </is>
       </c>
-      <c r="AA3" s="2" t="inlineStr"/>
       <c r="AB3" s="2" t="inlineStr"/>
       <c r="AC3" s="2" t="inlineStr"/>
-      <c r="AD3" s="2" t="inlineStr">
+      <c r="AD3" s="2" t="inlineStr"/>
+      <c r="AE3" s="2" t="inlineStr">
         <is>
           <t>https://betonocentras.lt/kontaktai/</t>
         </is>
       </c>
-      <c r="AE3" s="2" t="inlineStr"/>
-      <c r="AF3" s="2" t="inlineStr">
+      <c r="AF3" s="2" t="inlineStr"/>
+      <c r="AG3" s="2" t="inlineStr">
         <is>
           <t>2026-06-29</t>
         </is>
@@ -1011,42 +1020,43 @@
       </c>
       <c r="Q4" s="2" t="inlineStr"/>
       <c r="R4" s="2" t="inlineStr"/>
-      <c r="S4" s="2" t="inlineStr">
+      <c r="S4" s="2" t="inlineStr"/>
+      <c r="T4" s="2" t="inlineStr">
         <is>
           <t>Viešai skelbiamas Betono centro betono mazgas Klaipėdoje.</t>
         </is>
       </c>
-      <c r="T4" s="4" t="n">
+      <c r="U4" s="4" t="n">
         <v>0.9</v>
       </c>
-      <c r="U4" s="5" t="n"/>
-      <c r="V4" s="6" t="n"/>
-      <c r="W4" s="5" t="n"/>
+      <c r="V4" s="5" t="n"/>
+      <c r="W4" s="6" t="n"/>
       <c r="X4" s="5" t="n"/>
-      <c r="Y4" s="2" t="inlineStr">
+      <c r="Y4" s="5" t="n"/>
+      <c r="Z4" s="2" t="inlineStr">
         <is>
           <t>https://betonocentras.lt/</t>
         </is>
       </c>
-      <c r="Z4" s="2" t="inlineStr">
+      <c r="AA4" s="2" t="inlineStr">
         <is>
           <t>https://betonocentras.lt/kontaktai/</t>
         </is>
       </c>
-      <c r="AA4" s="2" t="inlineStr"/>
       <c r="AB4" s="2" t="inlineStr"/>
       <c r="AC4" s="2" t="inlineStr"/>
-      <c r="AD4" s="2" t="inlineStr">
+      <c r="AD4" s="2" t="inlineStr"/>
+      <c r="AE4" s="2" t="inlineStr">
         <is>
           <t>https://betonocentras.lt/kontaktai/</t>
         </is>
       </c>
-      <c r="AE4" s="2" t="inlineStr">
+      <c r="AF4" s="2" t="inlineStr">
         <is>
           <t>Oficialiame Betono centro kontaktų puslapyje patvirtintas Klaipėdos padalinys.</t>
         </is>
       </c>
-      <c r="AF4" s="2" t="inlineStr">
+      <c r="AG4" s="2" t="inlineStr">
         <is>
           <t>2026-06-30</t>
         </is>
@@ -1131,38 +1141,39 @@
       </c>
       <c r="Q5" s="2" t="inlineStr"/>
       <c r="R5" s="2" t="inlineStr"/>
-      <c r="S5" s="2" t="inlineStr">
+      <c r="S5" s="2" t="inlineStr"/>
+      <c r="T5" s="2" t="inlineStr">
         <is>
           <t>Viešai skelbiamas Betono centro betono mazgas Šiauliuose.</t>
         </is>
       </c>
-      <c r="T5" s="4" t="n">
+      <c r="U5" s="4" t="n">
         <v>0.9</v>
       </c>
-      <c r="U5" s="5" t="n"/>
-      <c r="V5" s="6" t="n"/>
-      <c r="W5" s="5" t="n"/>
+      <c r="V5" s="5" t="n"/>
+      <c r="W5" s="6" t="n"/>
       <c r="X5" s="5" t="n"/>
-      <c r="Y5" s="2" t="inlineStr">
+      <c r="Y5" s="5" t="n"/>
+      <c r="Z5" s="2" t="inlineStr">
         <is>
           <t>https://betonocentras.lt/</t>
         </is>
       </c>
-      <c r="Z5" s="2" t="inlineStr">
+      <c r="AA5" s="2" t="inlineStr">
         <is>
           <t>https://betonocentras.lt/kontaktai/</t>
         </is>
       </c>
-      <c r="AA5" s="2" t="inlineStr"/>
       <c r="AB5" s="2" t="inlineStr"/>
       <c r="AC5" s="2" t="inlineStr"/>
-      <c r="AD5" s="2" t="inlineStr">
+      <c r="AD5" s="2" t="inlineStr"/>
+      <c r="AE5" s="2" t="inlineStr">
         <is>
           <t>https://betonocentras.lt/kontaktai/</t>
         </is>
       </c>
-      <c r="AE5" s="2" t="inlineStr"/>
-      <c r="AF5" s="2" t="inlineStr">
+      <c r="AF5" s="2" t="inlineStr"/>
+      <c r="AG5" s="2" t="inlineStr">
         <is>
           <t>2026-06-29</t>
         </is>
@@ -1247,38 +1258,39 @@
       </c>
       <c r="Q6" s="2" t="inlineStr"/>
       <c r="R6" s="2" t="inlineStr"/>
-      <c r="S6" s="2" t="inlineStr">
+      <c r="S6" s="2" t="inlineStr"/>
+      <c r="T6" s="2" t="inlineStr">
         <is>
           <t>Viešai skelbiamas Betono centro betono mazgas Mažeikiuose.</t>
         </is>
       </c>
-      <c r="T6" s="4" t="n">
+      <c r="U6" s="4" t="n">
         <v>0.9</v>
       </c>
-      <c r="U6" s="5" t="n"/>
-      <c r="V6" s="6" t="n"/>
-      <c r="W6" s="5" t="n"/>
+      <c r="V6" s="5" t="n"/>
+      <c r="W6" s="6" t="n"/>
       <c r="X6" s="5" t="n"/>
-      <c r="Y6" s="2" t="inlineStr">
+      <c r="Y6" s="5" t="n"/>
+      <c r="Z6" s="2" t="inlineStr">
         <is>
           <t>https://betonocentras.lt/</t>
         </is>
       </c>
-      <c r="Z6" s="2" t="inlineStr">
+      <c r="AA6" s="2" t="inlineStr">
         <is>
           <t>https://betonocentras.lt/kontaktai/</t>
         </is>
       </c>
-      <c r="AA6" s="2" t="inlineStr"/>
       <c r="AB6" s="2" t="inlineStr"/>
       <c r="AC6" s="2" t="inlineStr"/>
-      <c r="AD6" s="2" t="inlineStr">
+      <c r="AD6" s="2" t="inlineStr"/>
+      <c r="AE6" s="2" t="inlineStr">
         <is>
           <t>https://betonocentras.lt/kontaktai/</t>
         </is>
       </c>
-      <c r="AE6" s="2" t="inlineStr"/>
-      <c r="AF6" s="2" t="inlineStr">
+      <c r="AF6" s="2" t="inlineStr"/>
+      <c r="AG6" s="2" t="inlineStr">
         <is>
           <t>2026-06-29</t>
         </is>
@@ -1363,38 +1375,39 @@
       </c>
       <c r="Q7" s="2" t="inlineStr"/>
       <c r="R7" s="2" t="inlineStr"/>
-      <c r="S7" s="2" t="inlineStr">
+      <c r="S7" s="2" t="inlineStr"/>
+      <c r="T7" s="2" t="inlineStr">
         <is>
           <t>Viešai skelbiamas Betono centro betono mazgas Panevėžyje.</t>
         </is>
       </c>
-      <c r="T7" s="4" t="n">
+      <c r="U7" s="4" t="n">
         <v>0.9</v>
       </c>
-      <c r="U7" s="5" t="n"/>
-      <c r="V7" s="6" t="n"/>
-      <c r="W7" s="5" t="n"/>
+      <c r="V7" s="5" t="n"/>
+      <c r="W7" s="6" t="n"/>
       <c r="X7" s="5" t="n"/>
-      <c r="Y7" s="2" t="inlineStr">
+      <c r="Y7" s="5" t="n"/>
+      <c r="Z7" s="2" t="inlineStr">
         <is>
           <t>https://betonocentras.lt/</t>
         </is>
       </c>
-      <c r="Z7" s="2" t="inlineStr">
+      <c r="AA7" s="2" t="inlineStr">
         <is>
           <t>https://betonocentras.lt/kontaktai/</t>
         </is>
       </c>
-      <c r="AA7" s="2" t="inlineStr"/>
       <c r="AB7" s="2" t="inlineStr"/>
       <c r="AC7" s="2" t="inlineStr"/>
-      <c r="AD7" s="2" t="inlineStr">
+      <c r="AD7" s="2" t="inlineStr"/>
+      <c r="AE7" s="2" t="inlineStr">
         <is>
           <t>https://betonocentras.lt/kontaktai/</t>
         </is>
       </c>
-      <c r="AE7" s="2" t="inlineStr"/>
-      <c r="AF7" s="2" t="inlineStr">
+      <c r="AF7" s="2" t="inlineStr"/>
+      <c r="AG7" s="2" t="inlineStr">
         <is>
           <t>2026-06-29</t>
         </is>
@@ -1479,42 +1492,43 @@
       </c>
       <c r="Q8" s="2" t="inlineStr"/>
       <c r="R8" s="2" t="inlineStr"/>
-      <c r="S8" s="2" t="inlineStr">
+      <c r="S8" s="2" t="inlineStr"/>
+      <c r="T8" s="2" t="inlineStr">
         <is>
           <t>Viešai skelbiamas Heidelberg Materials betono gamyklų tinklo taškas Vilniuje.</t>
         </is>
       </c>
-      <c r="T8" s="4" t="n">
+      <c r="U8" s="4" t="n">
         <v>0.85</v>
       </c>
-      <c r="U8" s="5" t="n"/>
-      <c r="V8" s="6" t="n"/>
-      <c r="W8" s="5" t="n"/>
+      <c r="V8" s="5" t="n"/>
+      <c r="W8" s="6" t="n"/>
       <c r="X8" s="5" t="n"/>
-      <c r="Y8" s="2" t="inlineStr">
+      <c r="Y8" s="5" t="n"/>
+      <c r="Z8" s="2" t="inlineStr">
         <is>
           <t>https://www.betonas.heidelbergmaterials.lt/lt</t>
         </is>
       </c>
-      <c r="Z8" s="2" t="inlineStr">
+      <c r="AA8" s="2" t="inlineStr">
         <is>
           <t>https://www.betonas.heidelbergmaterials.lt/lt/kontaktine-informacija-0</t>
         </is>
       </c>
-      <c r="AA8" s="2" t="inlineStr"/>
       <c r="AB8" s="2" t="inlineStr"/>
       <c r="AC8" s="2" t="inlineStr"/>
-      <c r="AD8" s="2" t="inlineStr">
+      <c r="AD8" s="2" t="inlineStr"/>
+      <c r="AE8" s="2" t="inlineStr">
         <is>
           <t>https://www.betonas.heidelbergmaterials.lt/lt/kontaktine-informacija-0</t>
         </is>
       </c>
-      <c r="AE8" s="2" t="inlineStr">
+      <c r="AF8" s="2" t="inlineStr">
         <is>
           <t>Oficialus Heidelberg Materials Lietuva Betonas kontaktų puslapis patvirtina betono užsakymų padalinius Lietuvoje.</t>
         </is>
       </c>
-      <c r="AF8" s="2" t="inlineStr">
+      <c r="AG8" s="2" t="inlineStr">
         <is>
           <t>2026-06-29</t>
         </is>
@@ -1599,42 +1613,43 @@
       </c>
       <c r="Q9" s="2" t="inlineStr"/>
       <c r="R9" s="2" t="inlineStr"/>
-      <c r="S9" s="2" t="inlineStr">
+      <c r="S9" s="2" t="inlineStr"/>
+      <c r="T9" s="2" t="inlineStr">
         <is>
           <t>Viešai skelbiamas Heidelberg Materials betono gamyklų tinklo taškas Vilniuje.</t>
         </is>
       </c>
-      <c r="T9" s="4" t="n">
+      <c r="U9" s="4" t="n">
         <v>0.85</v>
       </c>
-      <c r="U9" s="5" t="n"/>
-      <c r="V9" s="6" t="n"/>
-      <c r="W9" s="5" t="n"/>
+      <c r="V9" s="5" t="n"/>
+      <c r="W9" s="6" t="n"/>
       <c r="X9" s="5" t="n"/>
-      <c r="Y9" s="2" t="inlineStr">
+      <c r="Y9" s="5" t="n"/>
+      <c r="Z9" s="2" t="inlineStr">
         <is>
           <t>https://www.betonas.heidelbergmaterials.lt/lt</t>
         </is>
       </c>
-      <c r="Z9" s="2" t="inlineStr">
+      <c r="AA9" s="2" t="inlineStr">
         <is>
           <t>https://www.betonas.heidelbergmaterials.lt/lt/kontaktine-informacija-0</t>
         </is>
       </c>
-      <c r="AA9" s="2" t="inlineStr"/>
       <c r="AB9" s="2" t="inlineStr"/>
       <c r="AC9" s="2" t="inlineStr"/>
-      <c r="AD9" s="2" t="inlineStr">
+      <c r="AD9" s="2" t="inlineStr"/>
+      <c r="AE9" s="2" t="inlineStr">
         <is>
           <t>https://www.betonas.heidelbergmaterials.lt/lt/kontaktine-informacija-0</t>
         </is>
       </c>
-      <c r="AE9" s="2" t="inlineStr">
+      <c r="AF9" s="2" t="inlineStr">
         <is>
           <t>Oficialus Heidelberg Materials Lietuva Betonas kontaktų puslapis patvirtina betono užsakymų padalinius Lietuvoje.</t>
         </is>
       </c>
-      <c r="AF9" s="2" t="inlineStr">
+      <c r="AG9" s="2" t="inlineStr">
         <is>
           <t>2026-06-29</t>
         </is>
@@ -1719,42 +1734,43 @@
       </c>
       <c r="Q10" s="2" t="inlineStr"/>
       <c r="R10" s="2" t="inlineStr"/>
-      <c r="S10" s="2" t="inlineStr">
+      <c r="S10" s="2" t="inlineStr"/>
+      <c r="T10" s="2" t="inlineStr">
         <is>
           <t>Viešai skelbiamas Heidelberg Materials betono gamyklų tinklo taškas Kaune.</t>
         </is>
       </c>
-      <c r="T10" s="4" t="n">
+      <c r="U10" s="4" t="n">
         <v>0.85</v>
       </c>
-      <c r="U10" s="5" t="n"/>
-      <c r="V10" s="6" t="n"/>
-      <c r="W10" s="5" t="n"/>
+      <c r="V10" s="5" t="n"/>
+      <c r="W10" s="6" t="n"/>
       <c r="X10" s="5" t="n"/>
-      <c r="Y10" s="2" t="inlineStr">
+      <c r="Y10" s="5" t="n"/>
+      <c r="Z10" s="2" t="inlineStr">
         <is>
           <t>https://www.betonas.heidelbergmaterials.lt/lt</t>
         </is>
       </c>
-      <c r="Z10" s="2" t="inlineStr">
+      <c r="AA10" s="2" t="inlineStr">
         <is>
           <t>https://www.betonas.heidelbergmaterials.lt/lt/kontaktine-informacija-0</t>
         </is>
       </c>
-      <c r="AA10" s="2" t="inlineStr"/>
       <c r="AB10" s="2" t="inlineStr"/>
       <c r="AC10" s="2" t="inlineStr"/>
-      <c r="AD10" s="2" t="inlineStr">
+      <c r="AD10" s="2" t="inlineStr"/>
+      <c r="AE10" s="2" t="inlineStr">
         <is>
           <t>https://www.betonas.heidelbergmaterials.lt/lt/kontaktine-informacija-0</t>
         </is>
       </c>
-      <c r="AE10" s="2" t="inlineStr">
+      <c r="AF10" s="2" t="inlineStr">
         <is>
           <t>Oficialus Heidelberg Materials Lietuva Betonas kontaktų puslapis patvirtina betono užsakymų padalinius Lietuvoje.</t>
         </is>
       </c>
-      <c r="AF10" s="2" t="inlineStr">
+      <c r="AG10" s="2" t="inlineStr">
         <is>
           <t>2026-06-29</t>
         </is>
@@ -1839,42 +1855,43 @@
       </c>
       <c r="Q11" s="2" t="inlineStr"/>
       <c r="R11" s="2" t="inlineStr"/>
-      <c r="S11" s="2" t="inlineStr">
+      <c r="S11" s="2" t="inlineStr"/>
+      <c r="T11" s="2" t="inlineStr">
         <is>
           <t>Viešai skelbiamas Heidelberg Materials betono gamyklų tinklo taškas Klaipėdoje.</t>
         </is>
       </c>
-      <c r="T11" s="4" t="n">
+      <c r="U11" s="4" t="n">
         <v>0.85</v>
       </c>
-      <c r="U11" s="5" t="n"/>
-      <c r="V11" s="6" t="n"/>
-      <c r="W11" s="5" t="n"/>
+      <c r="V11" s="5" t="n"/>
+      <c r="W11" s="6" t="n"/>
       <c r="X11" s="5" t="n"/>
-      <c r="Y11" s="2" t="inlineStr">
+      <c r="Y11" s="5" t="n"/>
+      <c r="Z11" s="2" t="inlineStr">
         <is>
           <t>https://www.betonas.heidelbergmaterials.lt/lt</t>
         </is>
       </c>
-      <c r="Z11" s="2" t="inlineStr">
+      <c r="AA11" s="2" t="inlineStr">
         <is>
           <t>https://www.betonas.heidelbergmaterials.lt/lt/kontaktine-informacija-0</t>
         </is>
       </c>
-      <c r="AA11" s="2" t="inlineStr"/>
       <c r="AB11" s="2" t="inlineStr"/>
       <c r="AC11" s="2" t="inlineStr"/>
-      <c r="AD11" s="2" t="inlineStr">
+      <c r="AD11" s="2" t="inlineStr"/>
+      <c r="AE11" s="2" t="inlineStr">
         <is>
           <t>https://www.betonas.heidelbergmaterials.lt/lt/kontaktine-informacija-0</t>
         </is>
       </c>
-      <c r="AE11" s="2" t="inlineStr">
+      <c r="AF11" s="2" t="inlineStr">
         <is>
           <t>Oficialus Heidelberg Materials Lietuva Betonas kontaktų puslapis patvirtina betono užsakymų padalinius Lietuvoje.</t>
         </is>
       </c>
-      <c r="AF11" s="2" t="inlineStr">
+      <c r="AG11" s="2" t="inlineStr">
         <is>
           <t>2026-06-29</t>
         </is>
@@ -1959,42 +1976,43 @@
       </c>
       <c r="Q12" s="2" t="inlineStr"/>
       <c r="R12" s="2" t="inlineStr"/>
-      <c r="S12" s="2" t="inlineStr">
+      <c r="S12" s="2" t="inlineStr"/>
+      <c r="T12" s="2" t="inlineStr">
         <is>
           <t>Viešai skelbiamas Heidelberg Materials betono gamyklų tinklo taškas Alytuje.</t>
         </is>
       </c>
-      <c r="T12" s="4" t="n">
+      <c r="U12" s="4" t="n">
         <v>0.85</v>
       </c>
-      <c r="U12" s="5" t="n"/>
-      <c r="V12" s="6" t="n"/>
-      <c r="W12" s="5" t="n"/>
+      <c r="V12" s="5" t="n"/>
+      <c r="W12" s="6" t="n"/>
       <c r="X12" s="5" t="n"/>
-      <c r="Y12" s="2" t="inlineStr">
+      <c r="Y12" s="5" t="n"/>
+      <c r="Z12" s="2" t="inlineStr">
         <is>
           <t>https://www.betonas.heidelbergmaterials.lt/lt</t>
         </is>
       </c>
-      <c r="Z12" s="2" t="inlineStr">
+      <c r="AA12" s="2" t="inlineStr">
         <is>
           <t>https://www.betonas.heidelbergmaterials.lt/lt/kontaktine-informacija-0</t>
         </is>
       </c>
-      <c r="AA12" s="2" t="inlineStr"/>
       <c r="AB12" s="2" t="inlineStr"/>
       <c r="AC12" s="2" t="inlineStr"/>
-      <c r="AD12" s="2" t="inlineStr">
+      <c r="AD12" s="2" t="inlineStr"/>
+      <c r="AE12" s="2" t="inlineStr">
         <is>
           <t>https://www.betonas.heidelbergmaterials.lt/lt/kontaktine-informacija-0</t>
         </is>
       </c>
-      <c r="AE12" s="2" t="inlineStr">
+      <c r="AF12" s="2" t="inlineStr">
         <is>
           <t>Oficialus Heidelberg Materials Lietuva Betonas kontaktų puslapis patvirtina betono užsakymų padalinius Lietuvoje.</t>
         </is>
       </c>
-      <c r="AF12" s="2" t="inlineStr">
+      <c r="AG12" s="2" t="inlineStr">
         <is>
           <t>2026-06-29</t>
         </is>
@@ -2079,42 +2097,43 @@
       </c>
       <c r="Q13" s="2" t="inlineStr"/>
       <c r="R13" s="2" t="inlineStr"/>
-      <c r="S13" s="2" t="inlineStr">
+      <c r="S13" s="2" t="inlineStr"/>
+      <c r="T13" s="2" t="inlineStr">
         <is>
           <t>Viešai skelbiamas Heidelberg Materials betono gamyklų tinklo taškas Pasvalyje.</t>
         </is>
       </c>
-      <c r="T13" s="4" t="n">
+      <c r="U13" s="4" t="n">
         <v>0.8</v>
       </c>
-      <c r="U13" s="5" t="n"/>
-      <c r="V13" s="6" t="n"/>
-      <c r="W13" s="5" t="n"/>
+      <c r="V13" s="5" t="n"/>
+      <c r="W13" s="6" t="n"/>
       <c r="X13" s="5" t="n"/>
-      <c r="Y13" s="2" t="inlineStr">
+      <c r="Y13" s="5" t="n"/>
+      <c r="Z13" s="2" t="inlineStr">
         <is>
           <t>https://www.betonas.heidelbergmaterials.lt/lt</t>
         </is>
       </c>
-      <c r="Z13" s="2" t="inlineStr">
+      <c r="AA13" s="2" t="inlineStr">
         <is>
           <t>https://www.betonas.heidelbergmaterials.lt/lt/kontaktine-informacija-0</t>
         </is>
       </c>
-      <c r="AA13" s="2" t="inlineStr"/>
       <c r="AB13" s="2" t="inlineStr"/>
       <c r="AC13" s="2" t="inlineStr"/>
-      <c r="AD13" s="2" t="inlineStr">
+      <c r="AD13" s="2" t="inlineStr"/>
+      <c r="AE13" s="2" t="inlineStr">
         <is>
           <t>https://www.betonas.heidelbergmaterials.lt/lt/kontaktine-informacija-0</t>
         </is>
       </c>
-      <c r="AE13" s="2" t="inlineStr">
+      <c r="AF13" s="2" t="inlineStr">
         <is>
           <t>Oficialus Heidelberg Materials Lietuva Betonas kontaktų puslapis patvirtina betono užsakymų padalinius Lietuvoje.</t>
         </is>
       </c>
-      <c r="AF13" s="2" t="inlineStr">
+      <c r="AG13" s="2" t="inlineStr">
         <is>
           <t>2026-06-29</t>
         </is>
@@ -2199,38 +2218,39 @@
       </c>
       <c r="Q14" s="2" t="inlineStr"/>
       <c r="R14" s="2" t="inlineStr"/>
-      <c r="S14" s="2" t="inlineStr">
+      <c r="S14" s="2" t="inlineStr"/>
+      <c r="T14" s="2" t="inlineStr">
         <is>
           <t>Viešai skelbiamas betono mišinių tiekėjas Vilniaus regione.</t>
         </is>
       </c>
-      <c r="T14" s="4" t="n">
+      <c r="U14" s="4" t="n">
         <v>0.8</v>
       </c>
-      <c r="U14" s="5" t="n"/>
-      <c r="V14" s="6" t="n"/>
-      <c r="W14" s="5" t="n"/>
+      <c r="V14" s="5" t="n"/>
+      <c r="W14" s="6" t="n"/>
       <c r="X14" s="5" t="n"/>
-      <c r="Y14" s="2" t="inlineStr">
+      <c r="Y14" s="5" t="n"/>
+      <c r="Z14" s="2" t="inlineStr">
         <is>
           <t>https://www.palmusta.lt/</t>
         </is>
       </c>
-      <c r="Z14" s="2" t="inlineStr">
+      <c r="AA14" s="2" t="inlineStr">
         <is>
           <t>https://www.palmusta.lt/</t>
         </is>
       </c>
-      <c r="AA14" s="2" t="inlineStr"/>
       <c r="AB14" s="2" t="inlineStr"/>
       <c r="AC14" s="2" t="inlineStr"/>
-      <c r="AD14" s="2" t="inlineStr">
+      <c r="AD14" s="2" t="inlineStr"/>
+      <c r="AE14" s="2" t="inlineStr">
         <is>
           <t>https://www.palmusta.lt/</t>
         </is>
       </c>
-      <c r="AE14" s="2" t="inlineStr"/>
-      <c r="AF14" s="2" t="inlineStr">
+      <c r="AF14" s="2" t="inlineStr"/>
+      <c r="AG14" s="2" t="inlineStr">
         <is>
           <t>2026-06-29</t>
         </is>
@@ -2311,42 +2331,43 @@
       </c>
       <c r="Q15" s="2" t="inlineStr"/>
       <c r="R15" s="2" t="inlineStr"/>
-      <c r="S15" s="2" t="inlineStr">
+      <c r="S15" s="2" t="inlineStr"/>
+      <c r="T15" s="2" t="inlineStr">
         <is>
           <t>Gelžbetoninių konstrukcijų gamyba Vilniuje.</t>
         </is>
       </c>
-      <c r="T15" s="4" t="n">
+      <c r="U15" s="4" t="n">
         <v>0.9</v>
       </c>
-      <c r="U15" s="5" t="n"/>
-      <c r="V15" s="6" t="n"/>
-      <c r="W15" s="5" t="n"/>
+      <c r="V15" s="5" t="n"/>
+      <c r="W15" s="6" t="n"/>
       <c r="X15" s="5" t="n"/>
-      <c r="Y15" s="2" t="inlineStr">
+      <c r="Y15" s="5" t="n"/>
+      <c r="Z15" s="2" t="inlineStr">
         <is>
           <t>https://www.gkg3.lt/</t>
         </is>
       </c>
-      <c r="Z15" s="2" t="inlineStr">
+      <c r="AA15" s="2" t="inlineStr">
         <is>
           <t>https://gkg3.lt/kontaktai/</t>
         </is>
       </c>
-      <c r="AA15" s="2" t="inlineStr"/>
       <c r="AB15" s="2" t="inlineStr"/>
       <c r="AC15" s="2" t="inlineStr"/>
-      <c r="AD15" s="2" t="inlineStr">
+      <c r="AD15" s="2" t="inlineStr"/>
+      <c r="AE15" s="2" t="inlineStr">
         <is>
           <t>https://gkg3.lt/kontaktai/</t>
         </is>
       </c>
-      <c r="AE15" s="2" t="inlineStr">
+      <c r="AF15" s="2" t="inlineStr">
         <is>
           <t>Koordinatės patikslintos pagal oficialaus GKG3 kontaktų puslapio Google Maps nuorodą.</t>
         </is>
       </c>
-      <c r="AF15" s="2" t="inlineStr">
+      <c r="AG15" s="2" t="inlineStr">
         <is>
           <t>2026-06-29</t>
         </is>
@@ -2425,44 +2446,45 @@
           <t>Perdanga Vilniaus gamykla</t>
         </is>
       </c>
-      <c r="Q16" s="2" t="inlineStr">
+      <c r="Q16" s="2" t="inlineStr"/>
+      <c r="R16" s="2" t="inlineStr">
         <is>
           <t>150 m³/val.</t>
         </is>
       </c>
-      <c r="R16" s="2" t="inlineStr"/>
-      <c r="S16" s="2" t="inlineStr">
+      <c r="S16" s="2" t="inlineStr"/>
+      <c r="T16" s="2" t="inlineStr">
         <is>
           <t>Viešai nurodoma nauja gelžbetonio elementų gamybos linija, kurios našumas 150 m³/val.</t>
         </is>
       </c>
-      <c r="T16" s="4" t="n">
+      <c r="U16" s="4" t="n">
         <v>0.9</v>
       </c>
-      <c r="U16" s="5" t="n"/>
-      <c r="V16" s="6" t="n"/>
-      <c r="W16" s="5" t="n"/>
+      <c r="V16" s="5" t="n"/>
+      <c r="W16" s="6" t="n"/>
       <c r="X16" s="5" t="n"/>
-      <c r="Y16" s="2" t="inlineStr">
+      <c r="Y16" s="5" t="n"/>
+      <c r="Z16" s="2" t="inlineStr">
         <is>
           <t>https://www.perdanga.lt/</t>
         </is>
       </c>
-      <c r="Z16" s="2" t="inlineStr">
+      <c r="AA16" s="2" t="inlineStr">
         <is>
           <t>https://www.perdanga.lt/</t>
         </is>
       </c>
-      <c r="AA16" s="2" t="inlineStr"/>
       <c r="AB16" s="2" t="inlineStr"/>
       <c r="AC16" s="2" t="inlineStr"/>
-      <c r="AD16" s="2" t="inlineStr">
+      <c r="AD16" s="2" t="inlineStr"/>
+      <c r="AE16" s="2" t="inlineStr">
         <is>
           <t>https://www.perdanga.lt/</t>
         </is>
       </c>
-      <c r="AE16" s="2" t="inlineStr"/>
-      <c r="AF16" s="2" t="inlineStr">
+      <c r="AF16" s="2" t="inlineStr"/>
+      <c r="AG16" s="2" t="inlineStr">
         <is>
           <t>2026-06-29</t>
         </is>
@@ -2543,38 +2565,39 @@
       </c>
       <c r="Q17" s="2" t="inlineStr"/>
       <c r="R17" s="2" t="inlineStr"/>
-      <c r="S17" s="2" t="inlineStr">
+      <c r="S17" s="2" t="inlineStr"/>
+      <c r="T17" s="2" t="inlineStr">
         <is>
           <t>Viešai skelbiamas Perdangos padalinys Klaipėdoje.</t>
         </is>
       </c>
-      <c r="T17" s="4" t="n">
+      <c r="U17" s="4" t="n">
         <v>0.85</v>
       </c>
-      <c r="U17" s="5" t="n"/>
-      <c r="V17" s="6" t="n"/>
-      <c r="W17" s="5" t="n"/>
+      <c r="V17" s="5" t="n"/>
+      <c r="W17" s="6" t="n"/>
       <c r="X17" s="5" t="n"/>
-      <c r="Y17" s="2" t="inlineStr">
+      <c r="Y17" s="5" t="n"/>
+      <c r="Z17" s="2" t="inlineStr">
         <is>
           <t>https://www.perdanga.lt/</t>
         </is>
       </c>
-      <c r="Z17" s="2" t="inlineStr">
+      <c r="AA17" s="2" t="inlineStr">
         <is>
           <t>https://www.perdanga.lt/</t>
         </is>
       </c>
-      <c r="AA17" s="2" t="inlineStr"/>
       <c r="AB17" s="2" t="inlineStr"/>
       <c r="AC17" s="2" t="inlineStr"/>
-      <c r="AD17" s="2" t="inlineStr">
+      <c r="AD17" s="2" t="inlineStr"/>
+      <c r="AE17" s="2" t="inlineStr">
         <is>
           <t>https://www.perdanga.lt/</t>
         </is>
       </c>
-      <c r="AE17" s="2" t="inlineStr"/>
-      <c r="AF17" s="2" t="inlineStr">
+      <c r="AF17" s="2" t="inlineStr"/>
+      <c r="AG17" s="2" t="inlineStr">
         <is>
           <t>2026-06-29</t>
         </is>
@@ -2655,42 +2678,43 @@
       </c>
       <c r="Q18" s="2" t="inlineStr"/>
       <c r="R18" s="2" t="inlineStr"/>
-      <c r="S18" s="2" t="inlineStr">
+      <c r="S18" s="2" t="inlineStr"/>
+      <c r="T18" s="2" t="inlineStr">
         <is>
           <t>Viešai skelbiamas gelžbetonio gamintojas Kaune.</t>
         </is>
       </c>
-      <c r="T18" s="4" t="n">
+      <c r="U18" s="4" t="n">
         <v>0.8</v>
       </c>
-      <c r="U18" s="5" t="n"/>
-      <c r="V18" s="6" t="n"/>
-      <c r="W18" s="5" t="n"/>
+      <c r="V18" s="5" t="n"/>
+      <c r="W18" s="6" t="n"/>
       <c r="X18" s="5" t="n"/>
-      <c r="Y18" s="2" t="inlineStr">
+      <c r="Y18" s="5" t="n"/>
+      <c r="Z18" s="2" t="inlineStr">
         <is>
           <t>https://www.kaunogelzbetonis.lt/</t>
         </is>
       </c>
-      <c r="Z18" s="2" t="inlineStr">
+      <c r="AA18" s="2" t="inlineStr">
         <is>
           <t>https://www.kaunogelzbetonis.lt/kontaktai/</t>
         </is>
       </c>
-      <c r="AA18" s="2" t="inlineStr"/>
       <c r="AB18" s="2" t="inlineStr"/>
       <c r="AC18" s="2" t="inlineStr"/>
-      <c r="AD18" s="2" t="inlineStr">
+      <c r="AD18" s="2" t="inlineStr"/>
+      <c r="AE18" s="2" t="inlineStr">
         <is>
           <t>https://www.kaunogelzbetonis.lt/kontaktai/</t>
         </is>
       </c>
-      <c r="AE18" s="2" t="inlineStr">
+      <c r="AF18" s="2" t="inlineStr">
         <is>
           <t>Oficialus Kauno gelžbetonio kontaktų puslapis patvirtina Pramonės pr. 8 adresą.</t>
         </is>
       </c>
-      <c r="AF18" s="2" t="inlineStr">
+      <c r="AG18" s="2" t="inlineStr">
         <is>
           <t>2026-06-29</t>
         </is>
@@ -2771,42 +2795,43 @@
       </c>
       <c r="Q19" s="2" t="inlineStr"/>
       <c r="R19" s="2" t="inlineStr"/>
-      <c r="S19" s="2" t="inlineStr">
+      <c r="S19" s="2" t="inlineStr"/>
+      <c r="T19" s="2" t="inlineStr">
         <is>
           <t>Viešai skelbiamas gelžbetonio gamintojas Ukmergėje.</t>
         </is>
       </c>
-      <c r="T19" s="4" t="n">
+      <c r="U19" s="4" t="n">
         <v>0.8</v>
       </c>
-      <c r="U19" s="5" t="n"/>
-      <c r="V19" s="6" t="n"/>
-      <c r="W19" s="5" t="n"/>
+      <c r="V19" s="5" t="n"/>
+      <c r="W19" s="6" t="n"/>
       <c r="X19" s="5" t="n"/>
-      <c r="Y19" s="2" t="inlineStr">
+      <c r="Y19" s="5" t="n"/>
+      <c r="Z19" s="2" t="inlineStr">
         <is>
           <t>https://ukmergesgelzbetonis.lt/</t>
         </is>
       </c>
-      <c r="Z19" s="2" t="inlineStr">
+      <c r="AA19" s="2" t="inlineStr">
         <is>
           <t>https://ukmergesgelzbetonis.lt/</t>
         </is>
       </c>
-      <c r="AA19" s="2" t="inlineStr"/>
       <c r="AB19" s="2" t="inlineStr"/>
       <c r="AC19" s="2" t="inlineStr"/>
-      <c r="AD19" s="2" t="inlineStr">
+      <c r="AD19" s="2" t="inlineStr"/>
+      <c r="AE19" s="2" t="inlineStr">
         <is>
           <t>https://ukmergesgelzbetonis.lt/</t>
         </is>
       </c>
-      <c r="AE19" s="2" t="inlineStr">
+      <c r="AF19" s="2" t="inlineStr">
         <is>
           <t>Oficiali Ukmergės gelžbetonio svetainė palikta kaip pagrindinis šaltinis; naujų patikimų koordinačių nerasta.</t>
         </is>
       </c>
-      <c r="AF19" s="2" t="inlineStr">
+      <c r="AG19" s="2" t="inlineStr">
         <is>
           <t>2026-06-29</t>
         </is>
@@ -2887,42 +2912,43 @@
       </c>
       <c r="Q20" s="2" t="inlineStr"/>
       <c r="R20" s="2" t="inlineStr"/>
-      <c r="S20" s="2" t="inlineStr">
+      <c r="S20" s="2" t="inlineStr"/>
+      <c r="T20" s="2" t="inlineStr">
         <is>
           <t>Viešai skelbiamas gelžbetonio gamintojas Šiauliuose.</t>
         </is>
       </c>
-      <c r="T20" s="4" t="n">
+      <c r="U20" s="4" t="n">
         <v>0.8</v>
       </c>
-      <c r="U20" s="5" t="n"/>
-      <c r="V20" s="6" t="n"/>
-      <c r="W20" s="5" t="n"/>
+      <c r="V20" s="5" t="n"/>
+      <c r="W20" s="6" t="n"/>
       <c r="X20" s="5" t="n"/>
-      <c r="Y20" s="2" t="inlineStr">
+      <c r="Y20" s="5" t="n"/>
+      <c r="Z20" s="2" t="inlineStr">
         <is>
           <t>https://www.gelzbetonineskonstrukcijos.lt/</t>
         </is>
       </c>
-      <c r="Z20" s="2" t="inlineStr">
+      <c r="AA20" s="2" t="inlineStr">
         <is>
           <t>https://www.gelzbetonineskonstrukcijos.lt/contacts/</t>
         </is>
       </c>
-      <c r="AA20" s="2" t="inlineStr"/>
       <c r="AB20" s="2" t="inlineStr"/>
       <c r="AC20" s="2" t="inlineStr"/>
-      <c r="AD20" s="2" t="inlineStr">
+      <c r="AD20" s="2" t="inlineStr"/>
+      <c r="AE20" s="2" t="inlineStr">
         <is>
           <t>https://www.gelzbetonineskonstrukcijos.lt/contacts/</t>
         </is>
       </c>
-      <c r="AE20" s="2" t="inlineStr">
+      <c r="AF20" s="2" t="inlineStr">
         <is>
           <t>Koordinatės patikslintos pagal oficialaus kontaktų puslapio žemėlapio tašką.</t>
         </is>
       </c>
-      <c r="AF20" s="2" t="inlineStr">
+      <c r="AG20" s="2" t="inlineStr">
         <is>
           <t>2026-06-29</t>
         </is>
@@ -3003,38 +3029,39 @@
       </c>
       <c r="Q21" s="2" t="inlineStr"/>
       <c r="R21" s="2" t="inlineStr"/>
-      <c r="S21" s="2" t="inlineStr">
+      <c r="S21" s="2" t="inlineStr"/>
+      <c r="T21" s="2" t="inlineStr">
         <is>
           <t>Viešai skelbiamas surenkamojo gelžbetonio konstrukcijų gamintojas.</t>
         </is>
       </c>
-      <c r="T21" s="4" t="n">
+      <c r="U21" s="4" t="n">
         <v>0.8</v>
       </c>
-      <c r="U21" s="5" t="n"/>
-      <c r="V21" s="6" t="n"/>
-      <c r="W21" s="5" t="n"/>
+      <c r="V21" s="5" t="n"/>
+      <c r="W21" s="6" t="n"/>
       <c r="X21" s="5" t="n"/>
-      <c r="Y21" s="2" t="inlineStr">
+      <c r="Y21" s="5" t="n"/>
+      <c r="Z21" s="2" t="inlineStr">
         <is>
           <t>https://inhus.eu/</t>
         </is>
       </c>
-      <c r="Z21" s="2" t="inlineStr">
+      <c r="AA21" s="2" t="inlineStr">
         <is>
           <t>https://inhus.eu/</t>
         </is>
       </c>
-      <c r="AA21" s="2" t="inlineStr"/>
       <c r="AB21" s="2" t="inlineStr"/>
       <c r="AC21" s="2" t="inlineStr"/>
-      <c r="AD21" s="2" t="inlineStr">
+      <c r="AD21" s="2" t="inlineStr"/>
+      <c r="AE21" s="2" t="inlineStr">
         <is>
           <t>https://inhus.eu/</t>
         </is>
       </c>
-      <c r="AE21" s="2" t="inlineStr"/>
-      <c r="AF21" s="2" t="inlineStr">
+      <c r="AF21" s="2" t="inlineStr"/>
+      <c r="AG21" s="2" t="inlineStr">
         <is>
           <t>2026-06-29</t>
         </is>
@@ -3115,38 +3142,39 @@
       </c>
       <c r="Q22" s="2" t="inlineStr"/>
       <c r="R22" s="2" t="inlineStr"/>
-      <c r="S22" s="2" t="inlineStr">
+      <c r="S22" s="2" t="inlineStr"/>
+      <c r="T22" s="2" t="inlineStr">
         <is>
           <t>Viešai skelbiamas betono mišinių tiekėjas.</t>
         </is>
       </c>
-      <c r="T22" s="4" t="n">
+      <c r="U22" s="4" t="n">
         <v>0.75</v>
       </c>
-      <c r="U22" s="5" t="n"/>
-      <c r="V22" s="6" t="n"/>
-      <c r="W22" s="5" t="n"/>
+      <c r="V22" s="5" t="n"/>
+      <c r="W22" s="6" t="n"/>
       <c r="X22" s="5" t="n"/>
-      <c r="Y22" s="2" t="inlineStr">
+      <c r="Y22" s="5" t="n"/>
+      <c r="Z22" s="2" t="inlineStr">
         <is>
           <t>https://gelmesta.lt/</t>
         </is>
       </c>
-      <c r="Z22" s="2" t="inlineStr">
+      <c r="AA22" s="2" t="inlineStr">
         <is>
           <t>https://gelmesta.lt/</t>
         </is>
       </c>
-      <c r="AA22" s="2" t="inlineStr"/>
       <c r="AB22" s="2" t="inlineStr"/>
       <c r="AC22" s="2" t="inlineStr"/>
-      <c r="AD22" s="2" t="inlineStr">
+      <c r="AD22" s="2" t="inlineStr"/>
+      <c r="AE22" s="2" t="inlineStr">
         <is>
           <t>https://gelmesta.lt/</t>
         </is>
       </c>
-      <c r="AE22" s="2" t="inlineStr"/>
-      <c r="AF22" s="2" t="inlineStr">
+      <c r="AF22" s="2" t="inlineStr"/>
+      <c r="AG22" s="2" t="inlineStr">
         <is>
           <t>2026-06-29</t>
         </is>
@@ -3225,44 +3253,45 @@
           <t>Sūduvos betono mazgas</t>
         </is>
       </c>
-      <c r="Q23" s="2" t="inlineStr">
+      <c r="Q23" s="2" t="inlineStr"/>
+      <c r="R23" s="2" t="inlineStr">
         <is>
           <t>iki 200 m³ per darbo pamainą</t>
         </is>
       </c>
-      <c r="R23" s="2" t="inlineStr"/>
-      <c r="S23" s="2" t="inlineStr">
+      <c r="S23" s="2" t="inlineStr"/>
+      <c r="T23" s="2" t="inlineStr">
         <is>
           <t>Viešai skelbiamas betono mišinių gamintojas; nurodomas našumas iki 200 m³ per darbo pamainą.</t>
         </is>
       </c>
-      <c r="T23" s="4" t="n">
+      <c r="U23" s="4" t="n">
         <v>0.75</v>
       </c>
-      <c r="U23" s="5" t="n"/>
-      <c r="V23" s="6" t="n"/>
-      <c r="W23" s="5" t="n"/>
+      <c r="V23" s="5" t="n"/>
+      <c r="W23" s="6" t="n"/>
       <c r="X23" s="5" t="n"/>
-      <c r="Y23" s="2" t="inlineStr">
+      <c r="Y23" s="5" t="n"/>
+      <c r="Z23" s="2" t="inlineStr">
         <is>
           <t>https://www.suduvos-betonas.lt/</t>
         </is>
       </c>
-      <c r="Z23" s="2" t="inlineStr">
+      <c r="AA23" s="2" t="inlineStr">
         <is>
           <t>https://www.suduvos-betonas.lt/kontaktai/</t>
         </is>
       </c>
-      <c r="AA23" s="2" t="inlineStr"/>
       <c r="AB23" s="2" t="inlineStr"/>
       <c r="AC23" s="2" t="inlineStr"/>
-      <c r="AD23" s="2" t="inlineStr">
+      <c r="AD23" s="2" t="inlineStr"/>
+      <c r="AE23" s="2" t="inlineStr">
         <is>
           <t>https://www.suduvos-betonas.lt/</t>
         </is>
       </c>
-      <c r="AE23" s="2" t="inlineStr"/>
-      <c r="AF23" s="2" t="inlineStr">
+      <c r="AF23" s="2" t="inlineStr"/>
+      <c r="AG23" s="2" t="inlineStr">
         <is>
           <t>2026-06-29</t>
         </is>
@@ -3345,46 +3374,55 @@
           <t>Statkasta betono mazgas</t>
         </is>
       </c>
-      <c r="Q24" s="2" t="inlineStr"/>
-      <c r="R24" s="2" t="inlineStr"/>
-      <c r="S24" s="2" t="inlineStr">
-        <is>
-          <t>Viešai skelbiamas betono mišinių tiekėjas.</t>
-        </is>
-      </c>
-      <c r="T24" s="4" t="n">
+      <c r="Q24" s="2" t="inlineStr">
+        <is>
+          <t>Ammann Elba CBT60SL, 1 m³</t>
+        </is>
+      </c>
+      <c r="R24" s="2" t="inlineStr">
+        <is>
+          <t>iki 60 m³/h</t>
+        </is>
+      </c>
+      <c r="S24" s="2" t="inlineStr"/>
+      <c r="T24" s="2" t="inlineStr">
+        <is>
+          <t>Betono mazgo gamintojas Ammann Elba; modelis CBT60SL; maišyklė 1 m³; našumas iki 60 m³/h.</t>
+        </is>
+      </c>
+      <c r="U24" s="4" t="n">
         <v>0.75</v>
       </c>
-      <c r="U24" s="5" t="n"/>
-      <c r="V24" s="6" t="n"/>
-      <c r="W24" s="5" t="n"/>
+      <c r="V24" s="5" t="n"/>
+      <c r="W24" s="6" t="n"/>
       <c r="X24" s="5" t="n"/>
-      <c r="Y24" s="2" t="inlineStr">
+      <c r="Y24" s="5" t="n"/>
+      <c r="Z24" s="2" t="inlineStr">
         <is>
           <t>https://statkasta.lt/</t>
         </is>
       </c>
-      <c r="Z24" s="2" t="inlineStr">
+      <c r="AA24" s="2" t="inlineStr">
         <is>
           <t>https://statkasta.lt/kontaktai/</t>
         </is>
       </c>
-      <c r="AA24" s="2" t="inlineStr"/>
       <c r="AB24" s="2" t="inlineStr"/>
       <c r="AC24" s="2" t="inlineStr"/>
-      <c r="AD24" s="2" t="inlineStr">
+      <c r="AD24" s="2" t="inlineStr"/>
+      <c r="AE24" s="2" t="inlineStr">
         <is>
           <t>https://statkasta.lt/kontaktai/</t>
         </is>
       </c>
-      <c r="AE24" s="2" t="inlineStr">
-        <is>
-          <t>Oficialiame Statkasta kontaktų puslapyje nurodytas adresas Gėlių g. 34, Serdokų k.; koordinatės geokoduotos iki vietovės lygio.</t>
-        </is>
-      </c>
       <c r="AF24" s="2" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>Oficialiame Statkasta kontaktų puslapyje nurodytas adresas Gėlių g. 34, Serdokų k.; koordinatės geokoduotos iki vietovės lygio. Rankiniu būdu papildyta techninė informacija: gamintojas Ammann Elba, modelis CBT60SL, maišyklė 1 m³, našumas iki 60 m³/h.</t>
+        </is>
+      </c>
+      <c r="AG24" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
         </is>
       </c>
     </row>
@@ -3459,42 +3497,43 @@
       <c r="P25" s="2" t="inlineStr"/>
       <c r="Q25" s="2" t="inlineStr"/>
       <c r="R25" s="2" t="inlineStr"/>
-      <c r="S25" s="2" t="inlineStr">
+      <c r="S25" s="2" t="inlineStr"/>
+      <c r="T25" s="2" t="inlineStr">
         <is>
           <t>Viešuose šaltiniuose minima betono mišinių veikla; tikslų mazgo pavadinimą reikia patikslinti.</t>
         </is>
       </c>
-      <c r="T25" s="4" t="n">
+      <c r="U25" s="4" t="n">
         <v>0.6</v>
       </c>
-      <c r="U25" s="5" t="n"/>
-      <c r="V25" s="6" t="n"/>
-      <c r="W25" s="5" t="n"/>
+      <c r="V25" s="5" t="n"/>
+      <c r="W25" s="6" t="n"/>
       <c r="X25" s="5" t="n"/>
-      <c r="Y25" s="2" t="inlineStr">
+      <c r="Y25" s="5" t="n"/>
+      <c r="Z25" s="2" t="inlineStr">
         <is>
           <t>https://autokausta.lt/</t>
         </is>
       </c>
-      <c r="Z25" s="2" t="inlineStr">
+      <c r="AA25" s="2" t="inlineStr">
         <is>
           <t>https://www.autokausta.lt/apie-mus/betonas/</t>
         </is>
       </c>
-      <c r="AA25" s="2" t="inlineStr"/>
       <c r="AB25" s="2" t="inlineStr"/>
       <c r="AC25" s="2" t="inlineStr"/>
-      <c r="AD25" s="2" t="inlineStr">
+      <c r="AD25" s="2" t="inlineStr"/>
+      <c r="AE25" s="2" t="inlineStr">
         <is>
           <t>https://www.autokausta.lt/apie-mus/betonas/</t>
         </is>
       </c>
-      <c r="AE25" s="2" t="inlineStr">
+      <c r="AF25" s="2" t="inlineStr">
         <is>
           <t>Oficialus Autokausta betono puslapis patvirtina betono veiklą ir Marvelės g. 199B kontaktą.</t>
         </is>
       </c>
-      <c r="AF25" s="2" t="inlineStr">
+      <c r="AG25" s="2" t="inlineStr">
         <is>
           <t>2026-06-29</t>
         </is>
@@ -3579,42 +3618,43 @@
       </c>
       <c r="Q26" s="2" t="inlineStr"/>
       <c r="R26" s="2" t="inlineStr"/>
-      <c r="S26" s="2" t="inlineStr">
+      <c r="S26" s="2" t="inlineStr"/>
+      <c r="T26" s="2" t="inlineStr">
         <is>
           <t>Viešuose šaltiniuose minima betono mišinių veikla; tikslų mazgo adresą reikia patikslinti.</t>
         </is>
       </c>
-      <c r="T26" s="4" t="n">
+      <c r="U26" s="4" t="n">
         <v>0.65</v>
       </c>
-      <c r="U26" s="5" t="n"/>
-      <c r="V26" s="6" t="n"/>
-      <c r="W26" s="5" t="n"/>
+      <c r="V26" s="5" t="n"/>
+      <c r="W26" s="6" t="n"/>
       <c r="X26" s="5" t="n"/>
-      <c r="Y26" s="2" t="inlineStr">
+      <c r="Y26" s="5" t="n"/>
+      <c r="Z26" s="2" t="inlineStr">
         <is>
           <t>https://www.betonobaze.lt/</t>
         </is>
       </c>
-      <c r="Z26" s="2" t="inlineStr">
+      <c r="AA26" s="2" t="inlineStr">
         <is>
           <t>https://www.betonobaze.lt/kontaktai</t>
         </is>
       </c>
-      <c r="AA26" s="2" t="inlineStr"/>
       <c r="AB26" s="2" t="inlineStr"/>
       <c r="AC26" s="2" t="inlineStr"/>
-      <c r="AD26" s="2" t="inlineStr">
+      <c r="AD26" s="2" t="inlineStr"/>
+      <c r="AE26" s="2" t="inlineStr">
         <is>
           <t>https://www.betonobaze.lt/kontaktai</t>
         </is>
       </c>
-      <c r="AE26" s="2" t="inlineStr">
+      <c r="AF26" s="2" t="inlineStr">
         <is>
           <t>Oficialus kontaktų puslapis patvirtina Elektrinės g. 11 adresą ir betono bazės veiklą.</t>
         </is>
       </c>
-      <c r="AF26" s="2" t="inlineStr">
+      <c r="AG26" s="2" t="inlineStr">
         <is>
           <t>2026-06-29</t>
         </is>
@@ -3695,42 +3735,43 @@
       </c>
       <c r="Q27" s="2" t="inlineStr"/>
       <c r="R27" s="2" t="inlineStr"/>
-      <c r="S27" s="2" t="inlineStr">
+      <c r="S27" s="2" t="inlineStr"/>
+      <c r="T27" s="2" t="inlineStr">
         <is>
           <t>Viešai skelbiamas betono mišinių tiekėjas Druskininkų regione.</t>
         </is>
       </c>
-      <c r="T27" s="4" t="n">
+      <c r="U27" s="4" t="n">
         <v>0.7</v>
       </c>
-      <c r="U27" s="5" t="n"/>
-      <c r="V27" s="6" t="n"/>
-      <c r="W27" s="5" t="n"/>
+      <c r="V27" s="5" t="n"/>
+      <c r="W27" s="6" t="n"/>
       <c r="X27" s="5" t="n"/>
-      <c r="Y27" s="2" t="inlineStr">
+      <c r="Y27" s="5" t="n"/>
+      <c r="Z27" s="2" t="inlineStr">
         <is>
           <t>https://transdosa.lt/</t>
         </is>
       </c>
-      <c r="Z27" s="2" t="inlineStr">
+      <c r="AA27" s="2" t="inlineStr">
         <is>
           <t>https://www.transdosa.lt/kontaktai/</t>
         </is>
       </c>
-      <c r="AA27" s="2" t="inlineStr"/>
       <c r="AB27" s="2" t="inlineStr"/>
       <c r="AC27" s="2" t="inlineStr"/>
-      <c r="AD27" s="2" t="inlineStr">
+      <c r="AD27" s="2" t="inlineStr"/>
+      <c r="AE27" s="2" t="inlineStr">
         <is>
           <t>https://www.transdosa.lt/betonas/</t>
         </is>
       </c>
-      <c r="AE27" s="2" t="inlineStr">
+      <c r="AF27" s="2" t="inlineStr">
         <is>
           <t>Oficialūs Transdosa kontaktų ir betono puslapiai patvirtina Margų karjero betono gamybą adresu Žvyro g. 2A.</t>
         </is>
       </c>
-      <c r="AF27" s="2" t="inlineStr">
+      <c r="AG27" s="2" t="inlineStr">
         <is>
           <t>2026-06-29</t>
         </is>
@@ -3811,42 +3852,43 @@
       </c>
       <c r="Q28" s="2" t="inlineStr"/>
       <c r="R28" s="2" t="inlineStr"/>
-      <c r="S28" s="2" t="inlineStr">
+      <c r="S28" s="2" t="inlineStr"/>
+      <c r="T28" s="2" t="inlineStr">
         <is>
           <t>Viešai skelbiama gelžbetonio ir betono gaminių gamyba Šiauliuose.</t>
         </is>
       </c>
-      <c r="T28" s="4" t="n">
+      <c r="U28" s="4" t="n">
         <v>0.82</v>
       </c>
-      <c r="U28" s="5" t="n"/>
-      <c r="V28" s="6" t="n"/>
-      <c r="W28" s="5" t="n"/>
+      <c r="V28" s="5" t="n"/>
+      <c r="W28" s="6" t="n"/>
       <c r="X28" s="5" t="n"/>
-      <c r="Y28" s="2" t="inlineStr">
+      <c r="Y28" s="5" t="n"/>
+      <c r="Z28" s="2" t="inlineStr">
         <is>
           <t>https://sodbeta.lt/</t>
         </is>
       </c>
-      <c r="Z28" s="2" t="inlineStr">
+      <c r="AA28" s="2" t="inlineStr">
         <is>
           <t>https://sodbeta.lt/</t>
         </is>
       </c>
-      <c r="AA28" s="2" t="inlineStr"/>
       <c r="AB28" s="2" t="inlineStr"/>
       <c r="AC28" s="2" t="inlineStr"/>
-      <c r="AD28" s="2" t="inlineStr">
+      <c r="AD28" s="2" t="inlineStr"/>
+      <c r="AE28" s="2" t="inlineStr">
         <is>
           <t>https://sodbeta.lt/betonas/betono-misiniai/</t>
         </is>
       </c>
-      <c r="AE28" s="2" t="inlineStr">
+      <c r="AF28" s="2" t="inlineStr">
         <is>
           <t>Oficiali Sodbeta svetainė patvirtina Sodo g. 20 adresą ir betono mišinių puslapį.</t>
         </is>
       </c>
-      <c r="AF28" s="2" t="inlineStr">
+      <c r="AG28" s="2" t="inlineStr">
         <is>
           <t>2026-06-30</t>
         </is>
@@ -3931,42 +3973,43 @@
       </c>
       <c r="Q29" s="2" t="inlineStr"/>
       <c r="R29" s="2" t="inlineStr"/>
-      <c r="S29" s="2" t="inlineStr">
+      <c r="S29" s="2" t="inlineStr"/>
+      <c r="T29" s="2" t="inlineStr">
         <is>
           <t>Registrų centro/VDA atviruose duomenyse pagrindinė veikla nurodyta kaip prekinio betono mišinio gamyba (EVRK 23.63).</t>
         </is>
       </c>
-      <c r="T29" s="4" t="n">
+      <c r="U29" s="4" t="n">
         <v>0.85</v>
       </c>
-      <c r="U29" s="5" t="n"/>
-      <c r="V29" s="6" t="n"/>
-      <c r="W29" s="5" t="n"/>
+      <c r="V29" s="5" t="n"/>
+      <c r="W29" s="6" t="n"/>
       <c r="X29" s="5" t="n"/>
-      <c r="Y29" s="2" t="inlineStr">
+      <c r="Y29" s="5" t="n"/>
+      <c r="Z29" s="2" t="inlineStr">
         <is>
           <t>https://alytausgelzbetonis.lt/</t>
         </is>
       </c>
-      <c r="Z29" s="2" t="inlineStr">
+      <c r="AA29" s="2" t="inlineStr">
         <is>
           <t>https://alytausgelzbetonis.lt/kontaktai/</t>
         </is>
       </c>
-      <c r="AA29" s="2" t="inlineStr"/>
       <c r="AB29" s="2" t="inlineStr"/>
       <c r="AC29" s="2" t="inlineStr"/>
-      <c r="AD29" s="2" t="inlineStr">
+      <c r="AD29" s="2" t="inlineStr"/>
+      <c r="AE29" s="2" t="inlineStr">
         <is>
           <t>https://alytausgelzbetonis.lt/kontaktai/</t>
         </is>
       </c>
-      <c r="AE29" s="2" t="inlineStr">
+      <c r="AF29" s="2" t="inlineStr">
         <is>
           <t>Patikslinta pagal oficialų kontaktų puslapį.</t>
         </is>
       </c>
-      <c r="AF29" s="2" t="inlineStr">
+      <c r="AG29" s="2" t="inlineStr">
         <is>
           <t>2026-06-30</t>
         </is>
@@ -4047,42 +4090,43 @@
       </c>
       <c r="Q30" s="2" t="inlineStr"/>
       <c r="R30" s="2" t="inlineStr"/>
-      <c r="S30" s="2" t="inlineStr">
+      <c r="S30" s="2" t="inlineStr"/>
+      <c r="T30" s="2" t="inlineStr">
         <is>
           <t>Viešai skelbiamas betono mišinių tiekėjas Marijampolėje.</t>
         </is>
       </c>
-      <c r="T30" s="4" t="n">
+      <c r="U30" s="4" t="n">
         <v>0.75</v>
       </c>
-      <c r="U30" s="5" t="n"/>
-      <c r="V30" s="6" t="n"/>
-      <c r="W30" s="5" t="n"/>
+      <c r="V30" s="5" t="n"/>
+      <c r="W30" s="6" t="n"/>
       <c r="X30" s="5" t="n"/>
-      <c r="Y30" s="2" t="inlineStr">
+      <c r="Y30" s="5" t="n"/>
+      <c r="Z30" s="2" t="inlineStr">
         <is>
           <t>https://gernora.lt/</t>
         </is>
       </c>
-      <c r="Z30" s="2" t="inlineStr">
+      <c r="AA30" s="2" t="inlineStr">
         <is>
           <t>https://gernora.lt/kontaktai/</t>
         </is>
       </c>
-      <c r="AA30" s="2" t="inlineStr"/>
       <c r="AB30" s="2" t="inlineStr"/>
       <c r="AC30" s="2" t="inlineStr"/>
-      <c r="AD30" s="2" t="inlineStr">
+      <c r="AD30" s="2" t="inlineStr"/>
+      <c r="AE30" s="2" t="inlineStr">
         <is>
           <t>https://gernora.lt/kontaktai/</t>
         </is>
       </c>
-      <c r="AE30" s="2" t="inlineStr">
+      <c r="AF30" s="2" t="inlineStr">
         <is>
           <t>Koordinatės patikslintos pagal oficialaus Gernora kontaktų puslapio Google Maps nuorodą.</t>
         </is>
       </c>
-      <c r="AF30" s="2" t="inlineStr">
+      <c r="AG30" s="2" t="inlineStr">
         <is>
           <t>2026-06-30</t>
         </is>
@@ -4163,38 +4207,39 @@
       </c>
       <c r="Q31" s="2" t="inlineStr"/>
       <c r="R31" s="2" t="inlineStr"/>
-      <c r="S31" s="2" t="inlineStr">
+      <c r="S31" s="2" t="inlineStr"/>
+      <c r="T31" s="2" t="inlineStr">
         <is>
           <t>Viešame kataloge nurodomi betonas, cemento gaminiai, betono siurblys ir pamatų blokai Kretingoje.</t>
         </is>
       </c>
-      <c r="T31" s="4" t="n">
+      <c r="U31" s="4" t="n">
         <v>0.78</v>
       </c>
-      <c r="U31" s="5" t="n"/>
-      <c r="V31" s="6" t="n"/>
-      <c r="W31" s="5" t="n"/>
+      <c r="V31" s="5" t="n"/>
+      <c r="W31" s="6" t="n"/>
       <c r="X31" s="5" t="n"/>
-      <c r="Y31" s="2" t="inlineStr"/>
-      <c r="Z31" s="2" t="inlineStr">
+      <c r="Y31" s="5" t="n"/>
+      <c r="Z31" s="2" t="inlineStr"/>
+      <c r="AA31" s="2" t="inlineStr">
         <is>
           <t>https://www.1551.lt/re-betono-konstrukcijos-uab-betonas-cementas-betono-siurblys-pamatu-blokai-kretingoje-104253/</t>
         </is>
       </c>
-      <c r="AA31" s="2" t="inlineStr"/>
       <c r="AB31" s="2" t="inlineStr"/>
       <c r="AC31" s="2" t="inlineStr"/>
-      <c r="AD31" s="2" t="inlineStr">
+      <c r="AD31" s="2" t="inlineStr"/>
+      <c r="AE31" s="2" t="inlineStr">
         <is>
           <t>https://www.1551.lt/re-betono-konstrukcijos-uab-betonas-cementas-betono-siurblys-pamatu-blokai-kretingoje-104253/</t>
         </is>
       </c>
-      <c r="AE31" s="2" t="inlineStr">
+      <c r="AF31" s="2" t="inlineStr">
         <is>
           <t>Katalogo šaltinis, reikia patikslinti gamybos apimtį.</t>
         </is>
       </c>
-      <c r="AF31" s="2" t="inlineStr">
+      <c r="AG31" s="2" t="inlineStr">
         <is>
           <t>2026-06-30</t>
         </is>
@@ -4275,42 +4320,43 @@
       </c>
       <c r="Q32" s="2" t="inlineStr"/>
       <c r="R32" s="2" t="inlineStr"/>
-      <c r="S32" s="2" t="inlineStr">
+      <c r="S32" s="2" t="inlineStr"/>
+      <c r="T32" s="2" t="inlineStr">
         <is>
           <t>Viešai skelbiama betono gaminių ir statybinių konstrukcijų veikla Šilalės rajone.</t>
         </is>
       </c>
-      <c r="T32" s="4" t="n">
+      <c r="U32" s="4" t="n">
         <v>0.72</v>
       </c>
-      <c r="U32" s="5" t="n"/>
-      <c r="V32" s="6" t="n"/>
-      <c r="W32" s="5" t="n"/>
+      <c r="V32" s="5" t="n"/>
+      <c r="W32" s="6" t="n"/>
       <c r="X32" s="5" t="n"/>
-      <c r="Y32" s="2" t="inlineStr">
+      <c r="Y32" s="5" t="n"/>
+      <c r="Z32" s="2" t="inlineStr">
         <is>
           <t>https://www.silalesstatyba.lt/</t>
         </is>
       </c>
-      <c r="Z32" s="2" t="inlineStr">
+      <c r="AA32" s="2" t="inlineStr">
         <is>
           <t>https://www.silalesstatyba.lt/</t>
         </is>
       </c>
-      <c r="AA32" s="2" t="inlineStr"/>
       <c r="AB32" s="2" t="inlineStr"/>
       <c r="AC32" s="2" t="inlineStr"/>
-      <c r="AD32" s="2" t="inlineStr">
+      <c r="AD32" s="2" t="inlineStr"/>
+      <c r="AE32" s="2" t="inlineStr">
         <is>
           <t>https://www.silalesstatyba.lt/</t>
         </is>
       </c>
-      <c r="AE32" s="2" t="inlineStr">
+      <c r="AF32" s="2" t="inlineStr">
         <is>
           <t>Reikia patikslinti tikslų gaminių asortimentą.</t>
         </is>
       </c>
-      <c r="AF32" s="2" t="inlineStr">
+      <c r="AG32" s="2" t="inlineStr">
         <is>
           <t>2026-06-30</t>
         </is>
@@ -4391,38 +4437,39 @@
       </c>
       <c r="Q33" s="2" t="inlineStr"/>
       <c r="R33" s="2" t="inlineStr"/>
-      <c r="S33" s="2" t="inlineStr">
+      <c r="S33" s="2" t="inlineStr"/>
+      <c r="T33" s="2" t="inlineStr">
         <is>
           <t>Viešame įmonių kataloge nurodomas gelžbetonio gaminių profilis Panevėžyje.</t>
         </is>
       </c>
-      <c r="T33" s="4" t="n">
+      <c r="U33" s="4" t="n">
         <v>0.78</v>
       </c>
-      <c r="U33" s="5" t="n"/>
-      <c r="V33" s="6" t="n"/>
-      <c r="W33" s="5" t="n"/>
+      <c r="V33" s="5" t="n"/>
+      <c r="W33" s="6" t="n"/>
       <c r="X33" s="5" t="n"/>
-      <c r="Y33" s="2" t="inlineStr"/>
-      <c r="Z33" s="2" t="inlineStr">
+      <c r="Y33" s="5" t="n"/>
+      <c r="Z33" s="2" t="inlineStr"/>
+      <c r="AA33" s="2" t="inlineStr">
         <is>
           <t>https://www.spec.lt/imone/panevezio-gelzbetonis-uab</t>
         </is>
       </c>
-      <c r="AA33" s="2" t="inlineStr"/>
       <c r="AB33" s="2" t="inlineStr"/>
       <c r="AC33" s="2" t="inlineStr"/>
-      <c r="AD33" s="2" t="inlineStr">
+      <c r="AD33" s="2" t="inlineStr"/>
+      <c r="AE33" s="2" t="inlineStr">
         <is>
           <t>https://www.spec.lt/imone/panevezio-gelzbetonis-uab</t>
         </is>
       </c>
-      <c r="AE33" s="2" t="inlineStr">
+      <c r="AF33" s="2" t="inlineStr">
         <is>
           <t>Reikia patikrinti veiklos aktyvumą ir produkcijos apimtį.</t>
         </is>
       </c>
-      <c r="AF33" s="2" t="inlineStr">
+      <c r="AG33" s="2" t="inlineStr">
         <is>
           <t>2026-06-30</t>
         </is>
@@ -4503,42 +4550,43 @@
       </c>
       <c r="Q34" s="2" t="inlineStr"/>
       <c r="R34" s="2" t="inlineStr"/>
-      <c r="S34" s="2" t="inlineStr">
+      <c r="S34" s="2" t="inlineStr"/>
+      <c r="T34" s="2" t="inlineStr">
         <is>
           <t>Viešai skelbiami pamatų ir kiti betono gaminiai Telšių rajone.</t>
         </is>
       </c>
-      <c r="T34" s="4" t="n">
+      <c r="U34" s="4" t="n">
         <v>0.72</v>
       </c>
-      <c r="U34" s="5" t="n"/>
-      <c r="V34" s="6" t="n"/>
-      <c r="W34" s="5" t="n"/>
+      <c r="V34" s="5" t="n"/>
+      <c r="W34" s="6" t="n"/>
       <c r="X34" s="5" t="n"/>
-      <c r="Y34" s="2" t="inlineStr">
+      <c r="Y34" s="5" t="n"/>
+      <c r="Z34" s="2" t="inlineStr">
         <is>
           <t>https://pamatas.lt/</t>
         </is>
       </c>
-      <c r="Z34" s="2" t="inlineStr">
+      <c r="AA34" s="2" t="inlineStr">
         <is>
           <t>https://pamatas.lt/</t>
         </is>
       </c>
-      <c r="AA34" s="2" t="inlineStr"/>
       <c r="AB34" s="2" t="inlineStr"/>
       <c r="AC34" s="2" t="inlineStr"/>
-      <c r="AD34" s="2" t="inlineStr">
+      <c r="AD34" s="2" t="inlineStr"/>
+      <c r="AE34" s="2" t="inlineStr">
         <is>
           <t>https://pamatas.lt/</t>
         </is>
       </c>
-      <c r="AE34" s="2" t="inlineStr">
+      <c r="AF34" s="2" t="inlineStr">
         <is>
           <t>Adresas patikslintas pagal lietuvišką įmonės puslapį; koordinatės nustatytos Lietuvos geolokatoriumi.</t>
         </is>
       </c>
-      <c r="AF34" s="2" t="inlineStr">
+      <c r="AG34" s="2" t="inlineStr">
         <is>
           <t>2026-06-30</t>
         </is>
@@ -4619,42 +4667,43 @@
       </c>
       <c r="Q35" s="2" t="inlineStr"/>
       <c r="R35" s="2" t="inlineStr"/>
-      <c r="S35" s="2" t="inlineStr">
+      <c r="S35" s="2" t="inlineStr"/>
+      <c r="T35" s="2" t="inlineStr">
         <is>
           <t>Viešai skelbiamas HAUS blokelių ir betono gaminių gamintojas.</t>
         </is>
       </c>
-      <c r="T35" s="4" t="n">
+      <c r="U35" s="4" t="n">
         <v>0.8</v>
       </c>
-      <c r="U35" s="5" t="n"/>
-      <c r="V35" s="6" t="n"/>
-      <c r="W35" s="5" t="n"/>
+      <c r="V35" s="5" t="n"/>
+      <c r="W35" s="6" t="n"/>
       <c r="X35" s="5" t="n"/>
-      <c r="Y35" s="2" t="inlineStr">
+      <c r="Y35" s="5" t="n"/>
+      <c r="Z35" s="2" t="inlineStr">
         <is>
           <t>https://www.vbg.lt/</t>
         </is>
       </c>
-      <c r="Z35" s="2" t="inlineStr">
+      <c r="AA35" s="2" t="inlineStr">
         <is>
           <t>https://www.vbg.lt/</t>
         </is>
       </c>
-      <c r="AA35" s="2" t="inlineStr"/>
       <c r="AB35" s="2" t="inlineStr"/>
       <c r="AC35" s="2" t="inlineStr"/>
-      <c r="AD35" s="2" t="inlineStr">
+      <c r="AD35" s="2" t="inlineStr"/>
+      <c r="AE35" s="2" t="inlineStr">
         <is>
           <t>https://www.vbg.lt/</t>
         </is>
       </c>
-      <c r="AE35" s="2" t="inlineStr">
+      <c r="AF35" s="2" t="inlineStr">
         <is>
           <t>Žemėlapyje naudotas viešai skelbiamas įmonės adresas; gamybos vietą reikia patikslinti.</t>
         </is>
       </c>
-      <c r="AF35" s="2" t="inlineStr">
+      <c r="AG35" s="2" t="inlineStr">
         <is>
           <t>2026-06-30</t>
         </is>
@@ -4735,42 +4784,43 @@
       </c>
       <c r="Q36" s="2" t="inlineStr"/>
       <c r="R36" s="2" t="inlineStr"/>
-      <c r="S36" s="2" t="inlineStr">
+      <c r="S36" s="2" t="inlineStr"/>
+      <c r="T36" s="2" t="inlineStr">
         <is>
           <t>Viešai skelbiama betono mišinių veikla Klaipėdos rajone.</t>
         </is>
       </c>
-      <c r="T36" s="4" t="n">
+      <c r="U36" s="4" t="n">
         <v>0.75</v>
       </c>
-      <c r="U36" s="5" t="n"/>
-      <c r="V36" s="6" t="n"/>
-      <c r="W36" s="5" t="n"/>
+      <c r="V36" s="5" t="n"/>
+      <c r="W36" s="6" t="n"/>
       <c r="X36" s="5" t="n"/>
-      <c r="Y36" s="2" t="inlineStr">
+      <c r="Y36" s="5" t="n"/>
+      <c r="Z36" s="2" t="inlineStr">
         <is>
           <t>https://pamariogrupe.lt/</t>
         </is>
       </c>
-      <c r="Z36" s="2" t="inlineStr">
+      <c r="AA36" s="2" t="inlineStr">
         <is>
           <t>https://pamariogrupe.lt/</t>
         </is>
       </c>
-      <c r="AA36" s="2" t="inlineStr"/>
       <c r="AB36" s="2" t="inlineStr"/>
       <c r="AC36" s="2" t="inlineStr"/>
-      <c r="AD36" s="2" t="inlineStr">
+      <c r="AD36" s="2" t="inlineStr"/>
+      <c r="AE36" s="2" t="inlineStr">
         <is>
           <t>https://pamariogrupe.lt/</t>
         </is>
       </c>
-      <c r="AE36" s="2" t="inlineStr">
+      <c r="AF36" s="2" t="inlineStr">
         <is>
           <t>Reikia patikslinti našumą ir gamybos režimą.</t>
         </is>
       </c>
-      <c r="AF36" s="2" t="inlineStr">
+      <c r="AG36" s="2" t="inlineStr">
         <is>
           <t>2026-06-30</t>
         </is>
@@ -4851,42 +4901,43 @@
       </c>
       <c r="Q37" s="2" t="inlineStr"/>
       <c r="R37" s="2" t="inlineStr"/>
-      <c r="S37" s="2" t="inlineStr">
+      <c r="S37" s="2" t="inlineStr"/>
+      <c r="T37" s="2" t="inlineStr">
         <is>
           <t>Viešai skelbiama betono gaminių veikla Klaipėdoje.</t>
         </is>
       </c>
-      <c r="T37" s="4" t="n">
+      <c r="U37" s="4" t="n">
         <v>0.65</v>
       </c>
-      <c r="U37" s="5" t="n"/>
-      <c r="V37" s="6" t="n"/>
-      <c r="W37" s="5" t="n"/>
+      <c r="V37" s="5" t="n"/>
+      <c r="W37" s="6" t="n"/>
       <c r="X37" s="5" t="n"/>
-      <c r="Y37" s="2" t="inlineStr">
+      <c r="Y37" s="5" t="n"/>
+      <c r="Z37" s="2" t="inlineStr">
         <is>
           <t>https://betonozona.lt/</t>
         </is>
       </c>
-      <c r="Z37" s="2" t="inlineStr">
+      <c r="AA37" s="2" t="inlineStr">
         <is>
           <t>https://betonozona.lt/</t>
         </is>
       </c>
-      <c r="AA37" s="2" t="inlineStr"/>
       <c r="AB37" s="2" t="inlineStr"/>
       <c r="AC37" s="2" t="inlineStr"/>
-      <c r="AD37" s="2" t="inlineStr">
+      <c r="AD37" s="2" t="inlineStr"/>
+      <c r="AE37" s="2" t="inlineStr">
         <is>
           <t>https://betonozona.lt/</t>
         </is>
       </c>
-      <c r="AE37" s="2" t="inlineStr">
+      <c r="AF37" s="2" t="inlineStr">
         <is>
           <t>Patikrinti, ar įmonė pati gamina, ar tik prekiauja betono gaminiais.</t>
         </is>
       </c>
-      <c r="AF37" s="2" t="inlineStr">
+      <c r="AG37" s="2" t="inlineStr">
         <is>
           <t>2026-06-30</t>
         </is>
@@ -4971,42 +5022,43 @@
       </c>
       <c r="Q38" s="2" t="inlineStr"/>
       <c r="R38" s="2" t="inlineStr"/>
-      <c r="S38" s="2" t="inlineStr">
+      <c r="S38" s="2" t="inlineStr"/>
+      <c r="T38" s="2" t="inlineStr">
         <is>
           <t>Viešai skelbiama betono mišinių gamyba Panevėžyje.</t>
         </is>
       </c>
-      <c r="T38" s="4" t="n">
+      <c r="U38" s="4" t="n">
         <v>0.78</v>
       </c>
-      <c r="U38" s="5" t="n"/>
-      <c r="V38" s="6" t="n"/>
-      <c r="W38" s="5" t="n"/>
+      <c r="V38" s="5" t="n"/>
+      <c r="W38" s="6" t="n"/>
       <c r="X38" s="5" t="n"/>
-      <c r="Y38" s="2" t="inlineStr">
+      <c r="Y38" s="5" t="n"/>
+      <c r="Z38" s="2" t="inlineStr">
         <is>
           <t>https://topbeton.lt/</t>
         </is>
       </c>
-      <c r="Z38" s="2" t="inlineStr">
+      <c r="AA38" s="2" t="inlineStr">
         <is>
           <t>https://www.topbeton.lt/kontaktai/</t>
         </is>
       </c>
-      <c r="AA38" s="2" t="inlineStr"/>
       <c r="AB38" s="2" t="inlineStr"/>
       <c r="AC38" s="2" t="inlineStr"/>
-      <c r="AD38" s="2" t="inlineStr">
+      <c r="AD38" s="2" t="inlineStr"/>
+      <c r="AE38" s="2" t="inlineStr">
         <is>
           <t>https://www.topbeton.lt/kontaktai/</t>
         </is>
       </c>
-      <c r="AE38" s="2" t="inlineStr">
+      <c r="AF38" s="2" t="inlineStr">
         <is>
           <t>Oficialus kontaktų puslapis patvirtina Beržų g. 5C adresą.</t>
         </is>
       </c>
-      <c r="AF38" s="2" t="inlineStr">
+      <c r="AG38" s="2" t="inlineStr">
         <is>
           <t>2026-06-30</t>
         </is>
@@ -5087,42 +5139,43 @@
       </c>
       <c r="Q39" s="2" t="inlineStr"/>
       <c r="R39" s="2" t="inlineStr"/>
-      <c r="S39" s="2" t="inlineStr">
+      <c r="S39" s="2" t="inlineStr"/>
+      <c r="T39" s="2" t="inlineStr">
         <is>
           <t>Viešai skelbiama gelžbetonio gaminių gamyba Panevėžyje.</t>
         </is>
       </c>
-      <c r="T39" s="4" t="n">
+      <c r="U39" s="4" t="n">
         <v>0.72</v>
       </c>
-      <c r="U39" s="5" t="n"/>
-      <c r="V39" s="6" t="n"/>
-      <c r="W39" s="5" t="n"/>
+      <c r="V39" s="5" t="n"/>
+      <c r="W39" s="6" t="n"/>
       <c r="X39" s="5" t="n"/>
-      <c r="Y39" s="2" t="inlineStr">
+      <c r="Y39" s="5" t="n"/>
+      <c r="Z39" s="2" t="inlineStr">
         <is>
           <t>https://gelzbetoniogamyba.lt/</t>
         </is>
       </c>
-      <c r="Z39" s="2" t="inlineStr">
+      <c r="AA39" s="2" t="inlineStr">
         <is>
           <t>https://gelzbetoniogamyba.lt/</t>
         </is>
       </c>
-      <c r="AA39" s="2" t="inlineStr"/>
       <c r="AB39" s="2" t="inlineStr"/>
       <c r="AC39" s="2" t="inlineStr"/>
-      <c r="AD39" s="2" t="inlineStr">
+      <c r="AD39" s="2" t="inlineStr"/>
+      <c r="AE39" s="2" t="inlineStr">
         <is>
           <t>https://gelzbetoniogamyba.lt/</t>
         </is>
       </c>
-      <c r="AE39" s="2" t="inlineStr">
+      <c r="AF39" s="2" t="inlineStr">
         <is>
           <t>Reikia patikslinti ryšį su kitomis S. Kerbedžio g. 52 įmonėmis.</t>
         </is>
       </c>
-      <c r="AF39" s="2" t="inlineStr">
+      <c r="AG39" s="2" t="inlineStr">
         <is>
           <t>2026-06-30</t>
         </is>
@@ -5203,42 +5256,43 @@
       </c>
       <c r="Q40" s="2" t="inlineStr"/>
       <c r="R40" s="2" t="inlineStr"/>
-      <c r="S40" s="2" t="inlineStr">
+      <c r="S40" s="2" t="inlineStr"/>
+      <c r="T40" s="2" t="inlineStr">
         <is>
           <t>Viešai skelbiama betono mišinių veikla Pakruojyje.</t>
         </is>
       </c>
-      <c r="T40" s="4" t="n">
+      <c r="U40" s="4" t="n">
         <v>0.72</v>
       </c>
-      <c r="U40" s="5" t="n"/>
-      <c r="V40" s="6" t="n"/>
-      <c r="W40" s="5" t="n"/>
+      <c r="V40" s="5" t="n"/>
+      <c r="W40" s="6" t="n"/>
       <c r="X40" s="5" t="n"/>
-      <c r="Y40" s="2" t="inlineStr">
+      <c r="Y40" s="5" t="n"/>
+      <c r="Z40" s="2" t="inlineStr">
         <is>
           <t>https://inroma.lt/</t>
         </is>
       </c>
-      <c r="Z40" s="2" t="inlineStr">
+      <c r="AA40" s="2" t="inlineStr">
         <is>
           <t>https://inroma.lt/</t>
         </is>
       </c>
-      <c r="AA40" s="2" t="inlineStr"/>
       <c r="AB40" s="2" t="inlineStr"/>
       <c r="AC40" s="2" t="inlineStr"/>
-      <c r="AD40" s="2" t="inlineStr">
+      <c r="AD40" s="2" t="inlineStr"/>
+      <c r="AE40" s="2" t="inlineStr">
         <is>
           <t>https://inroma.lt/</t>
         </is>
       </c>
-      <c r="AE40" s="2" t="inlineStr">
+      <c r="AF40" s="2" t="inlineStr">
         <is>
           <t>Reikia patikslinti našumą.</t>
         </is>
       </c>
-      <c r="AF40" s="2" t="inlineStr">
+      <c r="AG40" s="2" t="inlineStr">
         <is>
           <t>2026-06-30</t>
         </is>
@@ -5319,38 +5373,39 @@
       </c>
       <c r="Q41" s="2" t="inlineStr"/>
       <c r="R41" s="2" t="inlineStr"/>
-      <c r="S41" s="2" t="inlineStr">
+      <c r="S41" s="2" t="inlineStr"/>
+      <c r="T41" s="2" t="inlineStr">
         <is>
           <t>Viešame kataloge nurodoma prekinio betono gamyba ir prekyba Vilniuje.</t>
         </is>
       </c>
-      <c r="T41" s="4" t="n">
+      <c r="U41" s="4" t="n">
         <v>0.7</v>
       </c>
-      <c r="U41" s="5" t="n"/>
-      <c r="V41" s="6" t="n"/>
-      <c r="W41" s="5" t="n"/>
+      <c r="V41" s="5" t="n"/>
+      <c r="W41" s="6" t="n"/>
       <c r="X41" s="5" t="n"/>
-      <c r="Y41" s="2" t="inlineStr"/>
-      <c r="Z41" s="2" t="inlineStr">
+      <c r="Y41" s="5" t="n"/>
+      <c r="Z41" s="2" t="inlineStr"/>
+      <c r="AA41" s="2" t="inlineStr">
         <is>
           <t>https://www.1551.lt/seldra-uab-prekinio-betono-gamyba-ir-prekyba-vilniuje-219193/</t>
         </is>
       </c>
-      <c r="AA41" s="2" t="inlineStr"/>
       <c r="AB41" s="2" t="inlineStr"/>
       <c r="AC41" s="2" t="inlineStr"/>
-      <c r="AD41" s="2" t="inlineStr">
+      <c r="AD41" s="2" t="inlineStr"/>
+      <c r="AE41" s="2" t="inlineStr">
         <is>
           <t>https://www.1551.lt/seldra-uab-prekinio-betono-gamyba-ir-prekyba-vilniuje-219193/</t>
         </is>
       </c>
-      <c r="AE41" s="2" t="inlineStr">
+      <c r="AF41" s="2" t="inlineStr">
         <is>
           <t>Koordinatė apytikslė pagal adresą; reikia patikslinti gamybos tašką.</t>
         </is>
       </c>
-      <c r="AF41" s="2" t="inlineStr">
+      <c r="AG41" s="2" t="inlineStr">
         <is>
           <t>2026-06-30</t>
         </is>
@@ -5435,42 +5490,43 @@
       </c>
       <c r="Q42" s="2" t="inlineStr"/>
       <c r="R42" s="2" t="inlineStr"/>
-      <c r="S42" s="2" t="inlineStr">
+      <c r="S42" s="2" t="inlineStr"/>
+      <c r="T42" s="2" t="inlineStr">
         <is>
           <t>Viešai skelbiama betono mišinių veikla Utenoje.</t>
         </is>
       </c>
-      <c r="T42" s="4" t="n">
+      <c r="U42" s="4" t="n">
         <v>0.78</v>
       </c>
-      <c r="U42" s="5" t="n"/>
-      <c r="V42" s="6" t="n"/>
-      <c r="W42" s="5" t="n"/>
+      <c r="V42" s="5" t="n"/>
+      <c r="W42" s="6" t="n"/>
       <c r="X42" s="5" t="n"/>
-      <c r="Y42" s="2" t="inlineStr">
+      <c r="Y42" s="5" t="n"/>
+      <c r="Z42" s="2" t="inlineStr">
         <is>
           <t>https://utenosbetonas.lt/</t>
         </is>
       </c>
-      <c r="Z42" s="2" t="inlineStr">
+      <c r="AA42" s="2" t="inlineStr">
         <is>
           <t>https://www.utenosbetonas.lt/kontaktai/</t>
         </is>
       </c>
-      <c r="AA42" s="2" t="inlineStr"/>
       <c r="AB42" s="2" t="inlineStr"/>
       <c r="AC42" s="2" t="inlineStr"/>
-      <c r="AD42" s="2" t="inlineStr">
+      <c r="AD42" s="2" t="inlineStr"/>
+      <c r="AE42" s="2" t="inlineStr">
         <is>
           <t>https://www.utenosbetonas.lt/kontaktai/</t>
         </is>
       </c>
-      <c r="AE42" s="2" t="inlineStr">
+      <c r="AF42" s="2" t="inlineStr">
         <is>
           <t>Oficialus kontaktų puslapis patvirtina Metalo g. 9B adresą.</t>
         </is>
       </c>
-      <c r="AF42" s="2" t="inlineStr">
+      <c r="AG42" s="2" t="inlineStr">
         <is>
           <t>2026-06-30</t>
         </is>
@@ -5555,42 +5611,43 @@
       </c>
       <c r="Q43" s="2" t="inlineStr"/>
       <c r="R43" s="2" t="inlineStr"/>
-      <c r="S43" s="2" t="inlineStr">
+      <c r="S43" s="2" t="inlineStr"/>
+      <c r="T43" s="2" t="inlineStr">
         <is>
           <t>Viešai skelbiama prekinio betono gamyba Jonavoje.</t>
         </is>
       </c>
-      <c r="T43" s="4" t="n">
+      <c r="U43" s="4" t="n">
         <v>0.78</v>
       </c>
-      <c r="U43" s="5" t="n"/>
-      <c r="V43" s="6" t="n"/>
-      <c r="W43" s="5" t="n"/>
+      <c r="V43" s="5" t="n"/>
+      <c r="W43" s="6" t="n"/>
       <c r="X43" s="5" t="n"/>
-      <c r="Y43" s="2" t="inlineStr">
+      <c r="Y43" s="5" t="n"/>
+      <c r="Z43" s="2" t="inlineStr">
         <is>
           <t>https://sbetonas.lt/</t>
         </is>
       </c>
-      <c r="Z43" s="2" t="inlineStr">
+      <c r="AA43" s="2" t="inlineStr">
         <is>
           <t>https://sbetonas.lt/</t>
         </is>
       </c>
-      <c r="AA43" s="2" t="inlineStr"/>
       <c r="AB43" s="2" t="inlineStr"/>
       <c r="AC43" s="2" t="inlineStr"/>
-      <c r="AD43" s="2" t="inlineStr">
+      <c r="AD43" s="2" t="inlineStr"/>
+      <c r="AE43" s="2" t="inlineStr">
         <is>
           <t>https://sbetonas.lt/</t>
         </is>
       </c>
-      <c r="AE43" s="2" t="inlineStr">
+      <c r="AF43" s="2" t="inlineStr">
         <is>
           <t>Papildomai rasta pagal prekinio betono požymį.</t>
         </is>
       </c>
-      <c r="AF43" s="2" t="inlineStr">
+      <c r="AG43" s="2" t="inlineStr">
         <is>
           <t>2026-06-30</t>
         </is>
@@ -5671,38 +5728,39 @@
       </c>
       <c r="Q44" s="2" t="inlineStr"/>
       <c r="R44" s="2" t="inlineStr"/>
-      <c r="S44" s="2" t="inlineStr">
+      <c r="S44" s="2" t="inlineStr"/>
+      <c r="T44" s="2" t="inlineStr">
         <is>
           <t>Viešame kataloge nurodomi betonas, betono mišiniai ir betono gamybos linija Naujojoje Akmenėje.</t>
         </is>
       </c>
-      <c r="T44" s="4" t="n">
+      <c r="U44" s="4" t="n">
         <v>0.78</v>
       </c>
-      <c r="U44" s="5" t="n"/>
-      <c r="V44" s="6" t="n"/>
-      <c r="W44" s="5" t="n"/>
+      <c r="V44" s="5" t="n"/>
+      <c r="W44" s="6" t="n"/>
       <c r="X44" s="5" t="n"/>
-      <c r="Y44" s="2" t="inlineStr"/>
-      <c r="Z44" s="2" t="inlineStr">
+      <c r="Y44" s="5" t="n"/>
+      <c r="Z44" s="2" t="inlineStr"/>
+      <c r="AA44" s="2" t="inlineStr">
         <is>
           <t>https://www.1551.lt/kalcitas-ab-betonas-betono-misiniai-betono-gamybos-linija-technikos-nuoma-naujojoje-akmeneje-59982/</t>
         </is>
       </c>
-      <c r="AA44" s="2" t="inlineStr"/>
       <c r="AB44" s="2" t="inlineStr"/>
       <c r="AC44" s="2" t="inlineStr"/>
-      <c r="AD44" s="2" t="inlineStr">
+      <c r="AD44" s="2" t="inlineStr"/>
+      <c r="AE44" s="2" t="inlineStr">
         <is>
           <t>https://www.1551.lt/kalcitas-ab-betonas-betono-misiniai-betono-gamybos-linija-technikos-nuoma-naujojoje-akmeneje-59982/</t>
         </is>
       </c>
-      <c r="AE44" s="2" t="inlineStr">
+      <c r="AF44" s="2" t="inlineStr">
         <is>
           <t>Reikia patikslinti, ar veikla yra nuolat aktyvi.</t>
         </is>
       </c>
-      <c r="AF44" s="2" t="inlineStr">
+      <c r="AG44" s="2" t="inlineStr">
         <is>
           <t>2026-06-30</t>
         </is>
@@ -5783,48 +5841,49 @@
       </c>
       <c r="Q45" s="2" t="inlineStr"/>
       <c r="R45" s="2" t="inlineStr"/>
-      <c r="S45" s="2" t="inlineStr">
+      <c r="S45" s="2" t="inlineStr"/>
+      <c r="T45" s="2" t="inlineStr">
         <is>
           <t>Įmonė gamina gelžbetonio gaminius, prekinį ir hidrotechninį betoną bei smėlbetonio mišinius.</t>
         </is>
       </c>
-      <c r="T45" s="4" t="n">
+      <c r="U45" s="4" t="n">
         <v>0.9</v>
       </c>
-      <c r="U45" s="5" t="n"/>
-      <c r="V45" s="6" t="n"/>
-      <c r="W45" s="5" t="n">
+      <c r="V45" s="5" t="n"/>
+      <c r="W45" s="6" t="n"/>
+      <c r="X45" s="5" t="n">
         <v>100</v>
       </c>
-      <c r="X45" s="5" t="n"/>
-      <c r="Y45" s="2" t="inlineStr">
+      <c r="Y45" s="5" t="n"/>
+      <c r="Z45" s="2" t="inlineStr">
         <is>
           <t>https://glg.lt/</t>
         </is>
       </c>
-      <c r="Z45" s="2" t="inlineStr">
+      <c r="AA45" s="2" t="inlineStr">
         <is>
           <t>https://glg.lt/kontaktai/</t>
         </is>
       </c>
-      <c r="AA45" s="2" t="inlineStr"/>
-      <c r="AB45" s="2" t="inlineStr">
+      <c r="AB45" s="2" t="inlineStr"/>
+      <c r="AC45" s="2" t="inlineStr">
         <is>
           <t>https://glg.lt/apie-imone/</t>
         </is>
       </c>
-      <c r="AC45" s="2" t="inlineStr"/>
-      <c r="AD45" s="2" t="inlineStr">
+      <c r="AD45" s="2" t="inlineStr"/>
+      <c r="AE45" s="2" t="inlineStr">
         <is>
           <t>https://glg.lt/betonas/betono-misiniai/</t>
         </is>
       </c>
-      <c r="AE45" s="2" t="inlineStr">
+      <c r="AF45" s="2" t="inlineStr">
         <is>
           <t>Patikslinta pagal oficialų glg.lt kontaktų ir įmonės aprašymo puslapius.</t>
         </is>
       </c>
-      <c r="AF45" s="2" t="inlineStr">
+      <c r="AG45" s="2" t="inlineStr">
         <is>
           <t>2026-06-30</t>
         </is>
@@ -5909,38 +5968,39 @@
       </c>
       <c r="Q46" s="2" t="inlineStr"/>
       <c r="R46" s="2" t="inlineStr"/>
-      <c r="S46" s="2" t="inlineStr">
+      <c r="S46" s="2" t="inlineStr"/>
+      <c r="T46" s="2" t="inlineStr">
         <is>
           <t>Viešame kataloge įmonė siejama su betono mišinių veikla.</t>
         </is>
       </c>
-      <c r="T46" s="4" t="n">
+      <c r="U46" s="4" t="n">
         <v>0.62</v>
       </c>
-      <c r="U46" s="5" t="n"/>
-      <c r="V46" s="6" t="n"/>
-      <c r="W46" s="5" t="n"/>
+      <c r="V46" s="5" t="n"/>
+      <c r="W46" s="6" t="n"/>
       <c r="X46" s="5" t="n"/>
-      <c r="Y46" s="2" t="inlineStr"/>
-      <c r="Z46" s="2" t="inlineStr">
+      <c r="Y46" s="5" t="n"/>
+      <c r="Z46" s="2" t="inlineStr"/>
+      <c r="AA46" s="2" t="inlineStr">
         <is>
           <t>https://www.1551.lt/sausta-uab-240915/</t>
         </is>
       </c>
-      <c r="AA46" s="2" t="inlineStr"/>
       <c r="AB46" s="2" t="inlineStr"/>
       <c r="AC46" s="2" t="inlineStr"/>
-      <c r="AD46" s="2" t="inlineStr">
+      <c r="AD46" s="2" t="inlineStr"/>
+      <c r="AE46" s="2" t="inlineStr">
         <is>
           <t>https://www.1551.lt/sausta-uab-240915/</t>
         </is>
       </c>
-      <c r="AE46" s="2" t="inlineStr">
+      <c r="AF46" s="2" t="inlineStr">
         <is>
           <t>Žemos pasitikėjimo įrašas; reikia patikslinti, ar gamyba vykdoma šiame taške.</t>
         </is>
       </c>
-      <c r="AF46" s="2" t="inlineStr">
+      <c r="AG46" s="2" t="inlineStr">
         <is>
           <t>2026-06-30</t>
         </is>
@@ -6025,34 +6085,35 @@
       </c>
       <c r="Q47" s="2" t="inlineStr"/>
       <c r="R47" s="2" t="inlineStr"/>
-      <c r="S47" s="2" t="inlineStr">
+      <c r="S47" s="2" t="inlineStr"/>
+      <c r="T47" s="2" t="inlineStr">
         <is>
           <t>Registrų centro/VDA atviruose duomenyse pagrindinė veikla nurodyta kaip prekinio betono mišinio gamyba (EVRK 23.63).</t>
         </is>
       </c>
-      <c r="T47" s="4" t="n">
+      <c r="U47" s="4" t="n">
         <v>0.82</v>
       </c>
-      <c r="U47" s="5" t="n"/>
-      <c r="V47" s="6" t="n"/>
-      <c r="W47" s="5" t="n"/>
+      <c r="V47" s="5" t="n"/>
+      <c r="W47" s="6" t="n"/>
       <c r="X47" s="5" t="n"/>
-      <c r="Y47" s="2" t="inlineStr"/>
-      <c r="Z47" s="2" t="inlineStr">
+      <c r="Y47" s="5" t="n"/>
+      <c r="Z47" s="2" t="inlineStr"/>
+      <c r="AA47" s="2" t="inlineStr">
         <is>
           <t>https://data.gov.lt/dataset/juridiniu-asmenu-ekonomines-veiklos-rusys-ir-instituciniai-sektoriai/</t>
         </is>
       </c>
-      <c r="AA47" s="2" t="inlineStr"/>
       <c r="AB47" s="2" t="inlineStr"/>
       <c r="AC47" s="2" t="inlineStr"/>
       <c r="AD47" s="2" t="inlineStr"/>
-      <c r="AE47" s="2" t="inlineStr">
+      <c r="AE47" s="2" t="inlineStr"/>
+      <c r="AF47" s="2" t="inlineStr">
         <is>
           <t>Adresas geokoduotas pagal viešai randamą įmonės adresą; betono mazgo vietą verta patikslinti atskiru šaltiniu.</t>
         </is>
       </c>
-      <c r="AF47" s="2" t="inlineStr">
+      <c r="AG47" s="2" t="inlineStr">
         <is>
           <t>2026-06-30</t>
         </is>
@@ -6137,34 +6198,35 @@
       </c>
       <c r="Q48" s="2" t="inlineStr"/>
       <c r="R48" s="2" t="inlineStr"/>
-      <c r="S48" s="2" t="inlineStr">
+      <c r="S48" s="2" t="inlineStr"/>
+      <c r="T48" s="2" t="inlineStr">
         <is>
           <t>Registrų centro/VDA atviruose duomenyse pagrindinė veikla nurodyta kaip prekinio betono mišinio gamyba (EVRK 23.63).</t>
         </is>
       </c>
-      <c r="T48" s="4" t="n">
+      <c r="U48" s="4" t="n">
         <v>0.82</v>
       </c>
-      <c r="U48" s="5" t="n"/>
-      <c r="V48" s="6" t="n"/>
-      <c r="W48" s="5" t="n"/>
+      <c r="V48" s="5" t="n"/>
+      <c r="W48" s="6" t="n"/>
       <c r="X48" s="5" t="n"/>
-      <c r="Y48" s="2" t="inlineStr"/>
-      <c r="Z48" s="2" t="inlineStr">
+      <c r="Y48" s="5" t="n"/>
+      <c r="Z48" s="2" t="inlineStr"/>
+      <c r="AA48" s="2" t="inlineStr">
         <is>
           <t>https://data.gov.lt/dataset/juridiniu-asmenu-ekonomines-veiklos-rusys-ir-instituciniai-sektoriai/</t>
         </is>
       </c>
-      <c r="AA48" s="2" t="inlineStr"/>
       <c r="AB48" s="2" t="inlineStr"/>
       <c r="AC48" s="2" t="inlineStr"/>
       <c r="AD48" s="2" t="inlineStr"/>
-      <c r="AE48" s="2" t="inlineStr">
+      <c r="AE48" s="2" t="inlineStr"/>
+      <c r="AF48" s="2" t="inlineStr">
         <is>
           <t>Adresas geokoduotas pagal viešai randamą įmonės adresą; betono mazgo vietą verta patikslinti atskiru šaltiniu.</t>
         </is>
       </c>
-      <c r="AF48" s="2" t="inlineStr">
+      <c r="AG48" s="2" t="inlineStr">
         <is>
           <t>2026-06-30</t>
         </is>
@@ -6249,34 +6311,35 @@
       </c>
       <c r="Q49" s="2" t="inlineStr"/>
       <c r="R49" s="2" t="inlineStr"/>
-      <c r="S49" s="2" t="inlineStr">
+      <c r="S49" s="2" t="inlineStr"/>
+      <c r="T49" s="2" t="inlineStr">
         <is>
           <t>Registrų centro/VDA atviruose duomenyse pagrindinė veikla nurodyta kaip prekinio betono mišinio gamyba (EVRK 23.63).</t>
         </is>
       </c>
-      <c r="T49" s="4" t="n">
+      <c r="U49" s="4" t="n">
         <v>0.82</v>
       </c>
-      <c r="U49" s="5" t="n"/>
-      <c r="V49" s="6" t="n"/>
-      <c r="W49" s="5" t="n"/>
+      <c r="V49" s="5" t="n"/>
+      <c r="W49" s="6" t="n"/>
       <c r="X49" s="5" t="n"/>
-      <c r="Y49" s="2" t="inlineStr"/>
-      <c r="Z49" s="2" t="inlineStr">
+      <c r="Y49" s="5" t="n"/>
+      <c r="Z49" s="2" t="inlineStr"/>
+      <c r="AA49" s="2" t="inlineStr">
         <is>
           <t>https://data.gov.lt/dataset/juridiniu-asmenu-ekonomines-veiklos-rusys-ir-instituciniai-sektoriai/</t>
         </is>
       </c>
-      <c r="AA49" s="2" t="inlineStr"/>
       <c r="AB49" s="2" t="inlineStr"/>
       <c r="AC49" s="2" t="inlineStr"/>
       <c r="AD49" s="2" t="inlineStr"/>
-      <c r="AE49" s="2" t="inlineStr">
+      <c r="AE49" s="2" t="inlineStr"/>
+      <c r="AF49" s="2" t="inlineStr">
         <is>
           <t>Adresas geokoduotas pagal viešai randamą įmonės adresą; betono mazgo vietą verta patikslinti atskiru šaltiniu.</t>
         </is>
       </c>
-      <c r="AF49" s="2" t="inlineStr">
+      <c r="AG49" s="2" t="inlineStr">
         <is>
           <t>2026-06-30</t>
         </is>
@@ -6361,34 +6424,35 @@
       </c>
       <c r="Q50" s="2" t="inlineStr"/>
       <c r="R50" s="2" t="inlineStr"/>
-      <c r="S50" s="2" t="inlineStr">
+      <c r="S50" s="2" t="inlineStr"/>
+      <c r="T50" s="2" t="inlineStr">
         <is>
           <t>Registrų centro/VDA atviruose duomenyse pagrindinė veikla nurodyta kaip prekinio betono mišinio gamyba (EVRK 23.63).</t>
         </is>
       </c>
-      <c r="T50" s="4" t="n">
+      <c r="U50" s="4" t="n">
         <v>0.82</v>
       </c>
-      <c r="U50" s="5" t="n"/>
-      <c r="V50" s="6" t="n"/>
-      <c r="W50" s="5" t="n"/>
+      <c r="V50" s="5" t="n"/>
+      <c r="W50" s="6" t="n"/>
       <c r="X50" s="5" t="n"/>
-      <c r="Y50" s="2" t="inlineStr"/>
-      <c r="Z50" s="2" t="inlineStr">
+      <c r="Y50" s="5" t="n"/>
+      <c r="Z50" s="2" t="inlineStr"/>
+      <c r="AA50" s="2" t="inlineStr">
         <is>
           <t>https://data.gov.lt/dataset/juridiniu-asmenu-ekonomines-veiklos-rusys-ir-instituciniai-sektoriai/</t>
         </is>
       </c>
-      <c r="AA50" s="2" t="inlineStr"/>
       <c r="AB50" s="2" t="inlineStr"/>
       <c r="AC50" s="2" t="inlineStr"/>
       <c r="AD50" s="2" t="inlineStr"/>
-      <c r="AE50" s="2" t="inlineStr">
+      <c r="AE50" s="2" t="inlineStr"/>
+      <c r="AF50" s="2" t="inlineStr">
         <is>
           <t>Adresas geokoduotas pagal viešai randamą įmonės adresą; betono mazgo vietą verta patikslinti atskiru šaltiniu.</t>
         </is>
       </c>
-      <c r="AF50" s="2" t="inlineStr">
+      <c r="AG50" s="2" t="inlineStr">
         <is>
           <t>2026-06-30</t>
         </is>
@@ -6473,42 +6537,43 @@
       </c>
       <c r="Q51" s="2" t="inlineStr"/>
       <c r="R51" s="2" t="inlineStr"/>
-      <c r="S51" s="2" t="inlineStr">
+      <c r="S51" s="2" t="inlineStr"/>
+      <c r="T51" s="2" t="inlineStr">
         <is>
           <t>Registrų centro/VDA atviruose duomenyse pagrindinė veikla nurodyta kaip prekinio betono mišinio gamyba (EVRK 23.63).</t>
         </is>
       </c>
-      <c r="T51" s="4" t="n">
+      <c r="U51" s="4" t="n">
         <v>0.82</v>
       </c>
-      <c r="U51" s="5" t="n"/>
-      <c r="V51" s="6" t="n"/>
-      <c r="W51" s="5" t="n"/>
+      <c r="V51" s="5" t="n"/>
+      <c r="W51" s="6" t="n"/>
       <c r="X51" s="5" t="n"/>
-      <c r="Y51" s="2" t="inlineStr">
+      <c r="Y51" s="5" t="n"/>
+      <c r="Z51" s="2" t="inlineStr">
         <is>
           <t>https://betonastaurageje.lt/</t>
         </is>
       </c>
-      <c r="Z51" s="2" t="inlineStr">
+      <c r="AA51" s="2" t="inlineStr">
         <is>
           <t>https://betonastaurageje.lt/kontaktai/</t>
         </is>
       </c>
-      <c r="AA51" s="2" t="inlineStr"/>
       <c r="AB51" s="2" t="inlineStr"/>
       <c r="AC51" s="2" t="inlineStr"/>
-      <c r="AD51" s="2" t="inlineStr">
+      <c r="AD51" s="2" t="inlineStr"/>
+      <c r="AE51" s="2" t="inlineStr">
         <is>
           <t>https://betonastaurageje.lt/betonas/</t>
         </is>
       </c>
-      <c r="AE51" s="2" t="inlineStr">
+      <c r="AF51" s="2" t="inlineStr">
         <is>
           <t>Oficiali Vinido svetainė patvirtina Gaurės g. 32 adresą, betono gamybą ir betono mazgą.</t>
         </is>
       </c>
-      <c r="AF51" s="2" t="inlineStr">
+      <c r="AG51" s="2" t="inlineStr">
         <is>
           <t>2026-06-30</t>
         </is>
@@ -6593,42 +6658,43 @@
       </c>
       <c r="Q52" s="2" t="inlineStr"/>
       <c r="R52" s="2" t="inlineStr"/>
-      <c r="S52" s="2" t="inlineStr">
+      <c r="S52" s="2" t="inlineStr"/>
+      <c r="T52" s="2" t="inlineStr">
         <is>
           <t>Registrų centro/VDA atviruose duomenyse pagrindinė veikla nurodyta kaip prekinio betono mišinio gamyba (EVRK 23.63).</t>
         </is>
       </c>
-      <c r="T52" s="4" t="n">
+      <c r="U52" s="4" t="n">
         <v>0.82</v>
       </c>
-      <c r="U52" s="5" t="n"/>
-      <c r="V52" s="6" t="n"/>
-      <c r="W52" s="5" t="n"/>
+      <c r="V52" s="5" t="n"/>
+      <c r="W52" s="6" t="n"/>
       <c r="X52" s="5" t="n"/>
-      <c r="Y52" s="2" t="inlineStr">
+      <c r="Y52" s="5" t="n"/>
+      <c r="Z52" s="2" t="inlineStr">
         <is>
           <t>https://santvara.eu/</t>
         </is>
       </c>
-      <c r="Z52" s="2" t="inlineStr">
+      <c r="AA52" s="2" t="inlineStr">
         <is>
           <t>https://santvara.eu/</t>
         </is>
       </c>
-      <c r="AA52" s="2" t="inlineStr"/>
       <c r="AB52" s="2" t="inlineStr"/>
       <c r="AC52" s="2" t="inlineStr"/>
-      <c r="AD52" s="2" t="inlineStr">
+      <c r="AD52" s="2" t="inlineStr"/>
+      <c r="AE52" s="2" t="inlineStr">
         <is>
           <t>https://santvara.eu/</t>
         </is>
       </c>
-      <c r="AE52" s="2" t="inlineStr">
+      <c r="AF52" s="2" t="inlineStr">
         <is>
           <t>Oficiali Santvara svetainė patvirtina Aruodų g. 34 adresą ir betono bei birių medžiagų veiklą.</t>
         </is>
       </c>
-      <c r="AF52" s="2" t="inlineStr">
+      <c r="AG52" s="2" t="inlineStr">
         <is>
           <t>2026-06-30</t>
         </is>
@@ -6713,34 +6779,35 @@
       </c>
       <c r="Q53" s="2" t="inlineStr"/>
       <c r="R53" s="2" t="inlineStr"/>
-      <c r="S53" s="2" t="inlineStr">
+      <c r="S53" s="2" t="inlineStr"/>
+      <c r="T53" s="2" t="inlineStr">
         <is>
           <t>Registrų centro/VDA atviruose duomenyse pagrindinė veikla nurodyta kaip prekinio betono mišinio gamyba (EVRK 23.63).</t>
         </is>
       </c>
-      <c r="T53" s="4" t="n">
+      <c r="U53" s="4" t="n">
         <v>0.72</v>
       </c>
-      <c r="U53" s="5" t="n"/>
-      <c r="V53" s="6" t="n"/>
-      <c r="W53" s="5" t="n"/>
+      <c r="V53" s="5" t="n"/>
+      <c r="W53" s="6" t="n"/>
       <c r="X53" s="5" t="n"/>
-      <c r="Y53" s="2" t="inlineStr"/>
-      <c r="Z53" s="2" t="inlineStr">
+      <c r="Y53" s="5" t="n"/>
+      <c r="Z53" s="2" t="inlineStr"/>
+      <c r="AA53" s="2" t="inlineStr">
         <is>
           <t>https://data.gov.lt/dataset/juridiniu-asmenu-ekonomines-veiklos-rusys-ir-instituciniai-sektoriai/</t>
         </is>
       </c>
-      <c r="AA53" s="2" t="inlineStr"/>
       <c r="AB53" s="2" t="inlineStr"/>
       <c r="AC53" s="2" t="inlineStr"/>
       <c r="AD53" s="2" t="inlineStr"/>
-      <c r="AE53" s="2" t="inlineStr">
+      <c r="AE53" s="2" t="inlineStr"/>
+      <c r="AF53" s="2" t="inlineStr">
         <is>
           <t>Adresas rastas viešuose kataloguose, bet geokoduotas tik iki Visagino miesto taško; reikia patikslinti tikslų betono mazgo GPS.</t>
         </is>
       </c>
-      <c r="AF53" s="2" t="inlineStr">
+      <c r="AG53" s="2" t="inlineStr">
         <is>
           <t>2026-06-30</t>
         </is>
@@ -6825,34 +6892,35 @@
       </c>
       <c r="Q54" s="2" t="inlineStr"/>
       <c r="R54" s="2" t="inlineStr"/>
-      <c r="S54" s="2" t="inlineStr">
+      <c r="S54" s="2" t="inlineStr"/>
+      <c r="T54" s="2" t="inlineStr">
         <is>
           <t>Registrų centro/VDA atviruose duomenyse pagrindinė veikla nurodyta kaip prekinio betono mišinio gamyba (EVRK 23.63).</t>
         </is>
       </c>
-      <c r="T54" s="4" t="n">
+      <c r="U54" s="4" t="n">
         <v>0.82</v>
       </c>
-      <c r="U54" s="5" t="n"/>
-      <c r="V54" s="6" t="n"/>
-      <c r="W54" s="5" t="n"/>
+      <c r="V54" s="5" t="n"/>
+      <c r="W54" s="6" t="n"/>
       <c r="X54" s="5" t="n"/>
-      <c r="Y54" s="2" t="inlineStr"/>
-      <c r="Z54" s="2" t="inlineStr">
+      <c r="Y54" s="5" t="n"/>
+      <c r="Z54" s="2" t="inlineStr"/>
+      <c r="AA54" s="2" t="inlineStr">
         <is>
           <t>https://data.gov.lt/dataset/juridiniu-asmenu-ekonomines-veiklos-rusys-ir-instituciniai-sektoriai/</t>
         </is>
       </c>
-      <c r="AA54" s="2" t="inlineStr"/>
       <c r="AB54" s="2" t="inlineStr"/>
       <c r="AC54" s="2" t="inlineStr"/>
       <c r="AD54" s="2" t="inlineStr"/>
-      <c r="AE54" s="2" t="inlineStr">
+      <c r="AE54" s="2" t="inlineStr"/>
+      <c r="AF54" s="2" t="inlineStr">
         <is>
           <t>Adresas geokoduotas pagal viešai randamą įmonės adresą; betono mazgo vietą verta patikslinti atskiru šaltiniu.</t>
         </is>
       </c>
-      <c r="AF54" s="2" t="inlineStr">
+      <c r="AG54" s="2" t="inlineStr">
         <is>
           <t>2026-06-30</t>
         </is>
@@ -6937,42 +7005,43 @@
       </c>
       <c r="Q55" s="2" t="inlineStr"/>
       <c r="R55" s="2" t="inlineStr"/>
-      <c r="S55" s="2" t="inlineStr">
+      <c r="S55" s="2" t="inlineStr"/>
+      <c r="T55" s="2" t="inlineStr">
         <is>
           <t>Registrų centro/VDA atviruose duomenyse pagrindinė veikla nurodyta kaip prekinio betono mišinio gamyba (EVRK 23.63).</t>
         </is>
       </c>
-      <c r="T55" s="4" t="n">
+      <c r="U55" s="4" t="n">
         <v>0.82</v>
       </c>
-      <c r="U55" s="5" t="n"/>
-      <c r="V55" s="6" t="n"/>
-      <c r="W55" s="5" t="n"/>
+      <c r="V55" s="5" t="n"/>
+      <c r="W55" s="6" t="n"/>
       <c r="X55" s="5" t="n"/>
-      <c r="Y55" s="2" t="inlineStr">
+      <c r="Y55" s="5" t="n"/>
+      <c r="Z55" s="2" t="inlineStr">
         <is>
           <t>https://ekobetonas.lt/</t>
         </is>
       </c>
-      <c r="Z55" s="2" t="inlineStr">
+      <c r="AA55" s="2" t="inlineStr">
         <is>
           <t>https://ekobetonas.lt/kontaktai-betono-gamyba-armaturinis-plienas/</t>
         </is>
       </c>
-      <c r="AA55" s="2" t="inlineStr"/>
       <c r="AB55" s="2" t="inlineStr"/>
       <c r="AC55" s="2" t="inlineStr"/>
-      <c r="AD55" s="2" t="inlineStr">
+      <c r="AD55" s="2" t="inlineStr"/>
+      <c r="AE55" s="2" t="inlineStr">
         <is>
           <t>https://ekobetonas.lt/kontaktai-betono-gamyba-armaturinis-plienas/</t>
         </is>
       </c>
-      <c r="AE55" s="2" t="inlineStr">
+      <c r="AF55" s="2" t="inlineStr">
         <is>
           <t>Oficialus Ekobetonas kontaktų puslapis patvirtina Gamyklų g. 3 adresą ir betono užsakymų kontaktus.</t>
         </is>
       </c>
-      <c r="AF55" s="2" t="inlineStr">
+      <c r="AG55" s="2" t="inlineStr">
         <is>
           <t>2026-06-30</t>
         </is>
@@ -7057,34 +7126,35 @@
       </c>
       <c r="Q56" s="2" t="inlineStr"/>
       <c r="R56" s="2" t="inlineStr"/>
-      <c r="S56" s="2" t="inlineStr">
+      <c r="S56" s="2" t="inlineStr"/>
+      <c r="T56" s="2" t="inlineStr">
         <is>
           <t>Registrų centro/VDA atviruose duomenyse pagrindinė veikla nurodyta kaip prekinio betono mišinio gamyba (EVRK 23.63).</t>
         </is>
       </c>
-      <c r="T56" s="4" t="n">
+      <c r="U56" s="4" t="n">
         <v>0.72</v>
       </c>
-      <c r="U56" s="5" t="n"/>
-      <c r="V56" s="6" t="n"/>
-      <c r="W56" s="5" t="n"/>
+      <c r="V56" s="5" t="n"/>
+      <c r="W56" s="6" t="n"/>
       <c r="X56" s="5" t="n"/>
-      <c r="Y56" s="2" t="inlineStr"/>
-      <c r="Z56" s="2" t="inlineStr">
+      <c r="Y56" s="5" t="n"/>
+      <c r="Z56" s="2" t="inlineStr"/>
+      <c r="AA56" s="2" t="inlineStr">
         <is>
           <t>https://data.gov.lt/dataset/juridiniu-asmenu-ekonomines-veiklos-rusys-ir-instituciniai-sektoriai/</t>
         </is>
       </c>
-      <c r="AA56" s="2" t="inlineStr"/>
       <c r="AB56" s="2" t="inlineStr"/>
       <c r="AC56" s="2" t="inlineStr"/>
       <c r="AD56" s="2" t="inlineStr"/>
-      <c r="AE56" s="2" t="inlineStr">
+      <c r="AE56" s="2" t="inlineStr"/>
+      <c r="AF56" s="2" t="inlineStr">
         <is>
           <t>Adresas rastas viešuose kataloguose, bet geokoduotas tik iki Rokiškio miesto taško; reikia patikslinti tikslų betono mazgo GPS.</t>
         </is>
       </c>
-      <c r="AF56" s="2" t="inlineStr">
+      <c r="AG56" s="2" t="inlineStr">
         <is>
           <t>2026-06-30</t>
         </is>
@@ -7169,42 +7239,43 @@
       </c>
       <c r="Q57" s="2" t="inlineStr"/>
       <c r="R57" s="2" t="inlineStr"/>
-      <c r="S57" s="2" t="inlineStr">
+      <c r="S57" s="2" t="inlineStr"/>
+      <c r="T57" s="2" t="inlineStr">
         <is>
           <t>Registrų centro/VDA atviruose duomenyse pagrindinė veikla nurodyta kaip prekinio betono mišinio gamyba (EVRK 23.63).</t>
         </is>
       </c>
-      <c r="T57" s="4" t="n">
+      <c r="U57" s="4" t="n">
         <v>0.82</v>
       </c>
-      <c r="U57" s="5" t="n"/>
-      <c r="V57" s="6" t="n"/>
-      <c r="W57" s="5" t="n"/>
+      <c r="V57" s="5" t="n"/>
+      <c r="W57" s="6" t="n"/>
       <c r="X57" s="5" t="n"/>
-      <c r="Y57" s="2" t="inlineStr">
+      <c r="Y57" s="5" t="n"/>
+      <c r="Z57" s="2" t="inlineStr">
         <is>
           <t>https://www.betoneura.lt/</t>
         </is>
       </c>
-      <c r="Z57" s="2" t="inlineStr">
+      <c r="AA57" s="2" t="inlineStr">
         <is>
           <t>https://www.betoneura.lt/kontaktai/</t>
         </is>
       </c>
-      <c r="AA57" s="2" t="inlineStr"/>
       <c r="AB57" s="2" t="inlineStr"/>
       <c r="AC57" s="2" t="inlineStr"/>
-      <c r="AD57" s="2" t="inlineStr">
+      <c r="AD57" s="2" t="inlineStr"/>
+      <c r="AE57" s="2" t="inlineStr">
         <is>
           <t>https://www.betoneura.lt/kontaktai/</t>
         </is>
       </c>
-      <c r="AE57" s="2" t="inlineStr">
+      <c r="AF57" s="2" t="inlineStr">
         <is>
           <t>Oficialus Beton Eura kontaktų puslapis patvirtina Žilvičių g. 2 adresą ir rekvizitus.</t>
         </is>
       </c>
-      <c r="AF57" s="2" t="inlineStr">
+      <c r="AG57" s="2" t="inlineStr">
         <is>
           <t>2026-06-30</t>
         </is>
@@ -7289,38 +7360,39 @@
       </c>
       <c r="Q58" s="2" t="inlineStr"/>
       <c r="R58" s="2" t="inlineStr"/>
-      <c r="S58" s="2" t="inlineStr">
+      <c r="S58" s="2" t="inlineStr"/>
+      <c r="T58" s="2" t="inlineStr">
         <is>
           <t>Registrų centro/VDA atviruose duomenyse pagrindinė veikla nurodyta kaip prekinio betono mišinio gamyba (EVRK 23.63).</t>
         </is>
       </c>
-      <c r="T58" s="4" t="n">
+      <c r="U58" s="4" t="n">
         <v>0.82</v>
       </c>
-      <c r="U58" s="5" t="n"/>
-      <c r="V58" s="6" t="n"/>
-      <c r="W58" s="5" t="n"/>
+      <c r="V58" s="5" t="n"/>
+      <c r="W58" s="6" t="n"/>
       <c r="X58" s="5" t="n"/>
-      <c r="Y58" s="2" t="inlineStr"/>
-      <c r="Z58" s="2" t="inlineStr">
+      <c r="Y58" s="5" t="n"/>
+      <c r="Z58" s="2" t="inlineStr"/>
+      <c r="AA58" s="2" t="inlineStr">
         <is>
           <t>https://data.gov.lt/dataset/juridiniu-asmenu-ekonomines-veiklos-rusys-ir-instituciniai-sektoriai/</t>
         </is>
       </c>
-      <c r="AA58" s="2" t="inlineStr"/>
       <c r="AB58" s="2" t="inlineStr"/>
       <c r="AC58" s="2" t="inlineStr"/>
-      <c r="AD58" s="2" t="inlineStr">
+      <c r="AD58" s="2" t="inlineStr"/>
+      <c r="AE58" s="2" t="inlineStr">
         <is>
           <t>https://fsaskaita.lt/imone/uzdaroji-akcine-bendrove-silutes-betonas-177392928</t>
         </is>
       </c>
-      <c r="AE58" s="2" t="inlineStr">
+      <c r="AF58" s="2" t="inlineStr">
         <is>
           <t>Adresas geokoduotas pagal viešai randamą įmonės adresą; betono mazgo vietą verta patikslinti atskiru šaltiniu.</t>
         </is>
       </c>
-      <c r="AF58" s="2" t="inlineStr">
+      <c r="AG58" s="2" t="inlineStr">
         <is>
           <t>2026-06-30</t>
         </is>
@@ -7405,34 +7477,35 @@
       </c>
       <c r="Q59" s="2" t="inlineStr"/>
       <c r="R59" s="2" t="inlineStr"/>
-      <c r="S59" s="2" t="inlineStr">
+      <c r="S59" s="2" t="inlineStr"/>
+      <c r="T59" s="2" t="inlineStr">
         <is>
           <t>Registrų centro/VDA atviruose duomenyse pagrindinė veikla nurodyta kaip prekinio betono mišinio gamyba (EVRK 23.63).</t>
         </is>
       </c>
-      <c r="T59" s="4" t="n">
+      <c r="U59" s="4" t="n">
         <v>0.82</v>
       </c>
-      <c r="U59" s="5" t="n"/>
-      <c r="V59" s="6" t="n"/>
-      <c r="W59" s="5" t="n"/>
+      <c r="V59" s="5" t="n"/>
+      <c r="W59" s="6" t="n"/>
       <c r="X59" s="5" t="n"/>
-      <c r="Y59" s="2" t="inlineStr"/>
-      <c r="Z59" s="2" t="inlineStr">
+      <c r="Y59" s="5" t="n"/>
+      <c r="Z59" s="2" t="inlineStr"/>
+      <c r="AA59" s="2" t="inlineStr">
         <is>
           <t>https://data.gov.lt/dataset/juridiniu-asmenu-ekonomines-veiklos-rusys-ir-instituciniai-sektoriai/</t>
         </is>
       </c>
-      <c r="AA59" s="2" t="inlineStr"/>
       <c r="AB59" s="2" t="inlineStr"/>
       <c r="AC59" s="2" t="inlineStr"/>
       <c r="AD59" s="2" t="inlineStr"/>
-      <c r="AE59" s="2" t="inlineStr">
+      <c r="AE59" s="2" t="inlineStr"/>
+      <c r="AF59" s="2" t="inlineStr">
         <is>
           <t>Adresas geokoduotas pagal viešai randamą įmonės adresą; betono mazgo vietą verta patikslinti atskiru šaltiniu.</t>
         </is>
       </c>
-      <c r="AF59" s="2" t="inlineStr">
+      <c r="AG59" s="2" t="inlineStr">
         <is>
           <t>2026-06-30</t>
         </is>
@@ -7512,54 +7585,57 @@
       </c>
       <c r="P60" s="2" t="inlineStr">
         <is>
-          <t>Telšių kelių betono mišinių gamyba</t>
+          <t>Elkon</t>
         </is>
       </c>
       <c r="Q60" s="2" t="inlineStr"/>
       <c r="R60" s="2" t="inlineStr"/>
-      <c r="S60" s="2" t="inlineStr">
-        <is>
-          <t>Oficialiame įmonės puslapyje skelbiama betono mišinių gamyba ir prekyba.</t>
-        </is>
-      </c>
-      <c r="T60" s="4" t="n">
+      <c r="S60" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="T60" s="2" t="inlineStr">
+        <is>
+          <t>Oficialiame įmonės puslapyje skelbiama betono mišinių gamyba ir prekyba. Naudotojo duomenimis, betono mazgas vadinasi Elkon, yra 2 silosai.</t>
+        </is>
+      </c>
+      <c r="U60" s="4" t="n">
         <v>0.86</v>
       </c>
-      <c r="U60" s="5" t="n"/>
-      <c r="V60" s="6" t="n"/>
-      <c r="W60" s="5" t="n"/>
+      <c r="V60" s="5" t="n"/>
+      <c r="W60" s="6" t="n"/>
       <c r="X60" s="5" t="n"/>
-      <c r="Y60" s="2" t="inlineStr">
+      <c r="Y60" s="5" t="n"/>
+      <c r="Z60" s="2" t="inlineStr">
         <is>
           <t>https://www.tkeliai.lt/</t>
         </is>
       </c>
-      <c r="Z60" s="2" t="inlineStr">
+      <c r="AA60" s="2" t="inlineStr">
         <is>
           <t>https://www.tkeliai.lt/kitos-paslaugos/</t>
         </is>
       </c>
-      <c r="AA60" s="2" t="inlineStr"/>
       <c r="AB60" s="2" t="inlineStr"/>
       <c r="AC60" s="2" t="inlineStr"/>
-      <c r="AD60" s="2" t="inlineStr">
+      <c r="AD60" s="2" t="inlineStr"/>
+      <c r="AE60" s="2" t="inlineStr">
         <is>
           <t>https://www.tkeliai.lt/kitos-paslaugos/</t>
         </is>
       </c>
-      <c r="AE60" s="2" t="inlineStr">
-        <is>
-          <t>Įtraukta pagal naudotojo informaciją; veikla patvirtinta oficialiame lietuviškame įmonės puslapyje. Koordinatės nustatytos Lietuvos geolokatoriumi pagal Mažeikių g. 18 adresą.</t>
-        </is>
-      </c>
       <c r="AF60" s="2" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>Įtraukta pagal naudotojo informaciją; veikla patvirtinta oficialiame lietuviškame įmonės puslapyje. Naudotojo duomenimis, betono mazgas vadinasi Elkon, yra 2 silosai. Koordinatės nustatytos Lietuvos geolokatoriumi pagal Mažeikių g. 18 adresą.</t>
+        </is>
+      </c>
+      <c r="AG60" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AF60"/>
+  <autoFilter ref="A1:AG60"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -7648,7 +7724,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-07-06T16:45:44.788666+00:00</t>
+          <t>2026-07-06T17:22:34.210438+00:00</t>
         </is>
       </c>
     </row>
@@ -7703,7 +7779,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-07-06T16:45:44.789546+00:00</t>
+          <t>2026-07-06T17:22:34.210438+00:00</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">

</xml_diff>

<commit_message>
Refresh map from Betono centras workbook updates
</commit_message>
<xml_diff>
--- a/data/companies.xlsx
+++ b/data/companies.xlsx
@@ -781,11 +781,19 @@
       </c>
       <c r="P2" s="2" t="inlineStr">
         <is>
-          <t>Vilniaus betono mazgas</t>
-        </is>
-      </c>
-      <c r="Q2" s="2" t="inlineStr"/>
-      <c r="R2" s="2" t="inlineStr"/>
+          <t>Stetter</t>
+        </is>
+      </c>
+      <c r="Q2" s="2" t="inlineStr">
+        <is>
+          <t>2x3,35 m³</t>
+        </is>
+      </c>
+      <c r="R2" s="2" t="inlineStr">
+        <is>
+          <t>100 m³/val.</t>
+        </is>
+      </c>
       <c r="S2" s="2" t="inlineStr"/>
       <c r="T2" s="2" t="inlineStr">
         <is>
@@ -820,7 +828,7 @@
       <c r="AF2" s="2" t="inlineStr"/>
       <c r="AG2" s="2" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-07-06</t>
         </is>
       </c>
     </row>
@@ -7724,7 +7732,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-07-06T17:22:34.210438+00:00</t>
+          <t>2026-07-06T17:40:42.313250+00:00</t>
         </is>
       </c>
     </row>
@@ -7779,7 +7787,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-07-06T17:22:34.210438+00:00</t>
+          <t>2026-07-06T17:40:42.313250+00:00</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">

</xml_diff>

<commit_message>
Simplify competitor map data fields
</commit_message>
<xml_diff>
--- a/data/companies.xlsx
+++ b/data/companies.xlsx
@@ -12,7 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Importo žurnalas" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Įmonės'!$A$1:$AG$60</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Įmonės'!$A$1:$Z$60</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -71,7 +71,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top"/>
@@ -82,13 +82,10 @@
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="3" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -172,9 +169,9 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ImonesTable" displayName="ImonesTable" ref="A1:AG60" headerRowCount="1">
-  <autoFilter ref="A1:AG60"/>
-  <tableColumns count="33">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ImonesTable" displayName="ImonesTable" ref="A1:Z60" headerRowCount="1">
+  <autoFilter ref="A1:Z60"/>
+  <tableColumns count="26">
     <tableColumn id="1" name="Įrašo ID"/>
     <tableColumn id="2" name="Įmonės kodas"/>
     <tableColumn id="3" name="Įmonės pavadinimas"/>
@@ -190,24 +187,17 @@
     <tableColumn id="13" name="Koordinačių šaltinio URL"/>
     <tableColumn id="14" name="Veiklos tipas"/>
     <tableColumn id="15" name="Veikla"/>
-    <tableColumn id="16" name="Betono mazgo / gamyklos pavadinimas"/>
+    <tableColumn id="16" name="Mazgas (gamintojas)"/>
     <tableColumn id="17" name="Maišyklė"/>
     <tableColumn id="18" name="Našumas (realus)"/>
     <tableColumn id="19" name="Silosų skaičius"/>
     <tableColumn id="20" name="Viešas betono mazgo / gamyklos aprašymas"/>
     <tableColumn id="21" name="Klasifikavimo pasitikėjimas"/>
-    <tableColumn id="22" name="Įmonės apyvarta"/>
-    <tableColumn id="23" name="Apyvartos metai"/>
-    <tableColumn id="24" name="Darbuotojų skaičius"/>
-    <tableColumn id="25" name="Automobilių / transporto priemonių skaičius"/>
-    <tableColumn id="26" name="Interneto svetainė"/>
-    <tableColumn id="27" name="Pagrindinis šaltinis"/>
-    <tableColumn id="28" name="Apyvartos šaltinis"/>
-    <tableColumn id="29" name="Darbuotojų šaltinis"/>
-    <tableColumn id="30" name="Transporto šaltinis"/>
-    <tableColumn id="31" name="Betono mazgo / gamyklos šaltinis"/>
-    <tableColumn id="32" name="Pastaba / rankinis papildymas"/>
-    <tableColumn id="33" name="Paskutinio atnaujinimo data"/>
+    <tableColumn id="22" name="Interneto svetainė"/>
+    <tableColumn id="23" name="Pagrindinis šaltinis"/>
+    <tableColumn id="24" name="Betono mazgo / gamyklos šaltinis"/>
+    <tableColumn id="25" name="Pastaba / rankinis papildymas"/>
+    <tableColumn id="26" name="Paskutinio atnaujinimo data"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -502,7 +492,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AG60"/>
+  <dimension ref="A1:Z60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="39" customWidth="1" min="1" max="1"/>
@@ -526,18 +516,11 @@
     <col width="17" customWidth="1" min="19" max="19"/>
     <col width="42" customWidth="1" min="20" max="20"/>
     <col width="29" customWidth="1" min="21" max="21"/>
-    <col width="17" customWidth="1" min="22" max="22"/>
-    <col width="17" customWidth="1" min="23" max="23"/>
-    <col width="21" customWidth="1" min="24" max="24"/>
+    <col width="42" customWidth="1" min="22" max="22"/>
+    <col width="42" customWidth="1" min="23" max="23"/>
+    <col width="42" customWidth="1" min="24" max="24"/>
     <col width="42" customWidth="1" min="25" max="25"/>
-    <col width="42" customWidth="1" min="26" max="26"/>
-    <col width="42" customWidth="1" min="27" max="27"/>
-    <col width="20" customWidth="1" min="28" max="28"/>
-    <col width="28" customWidth="1" min="29" max="29"/>
-    <col width="21" customWidth="1" min="30" max="30"/>
-    <col width="42" customWidth="1" min="31" max="31"/>
-    <col width="42" customWidth="1" min="32" max="32"/>
-    <col width="29" customWidth="1" min="33" max="33"/>
+    <col width="29" customWidth="1" min="26" max="26"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -618,7 +601,7 @@
       </c>
       <c r="P1" s="1" t="inlineStr">
         <is>
-          <t>Betono mazgo / gamyklos pavadinimas</t>
+          <t>Mazgas (gamintojas)</t>
         </is>
       </c>
       <c r="Q1" s="1" t="inlineStr">
@@ -648,60 +631,25 @@
       </c>
       <c r="V1" s="1" t="inlineStr">
         <is>
-          <t>Įmonės apyvarta</t>
+          <t>Interneto svetainė</t>
         </is>
       </c>
       <c r="W1" s="1" t="inlineStr">
         <is>
-          <t>Apyvartos metai</t>
+          <t>Pagrindinis šaltinis</t>
         </is>
       </c>
       <c r="X1" s="1" t="inlineStr">
         <is>
-          <t>Darbuotojų skaičius</t>
+          <t>Betono mazgo / gamyklos šaltinis</t>
         </is>
       </c>
       <c r="Y1" s="1" t="inlineStr">
         <is>
-          <t>Automobilių / transporto priemonių skaičius</t>
+          <t>Pastaba / rankinis papildymas</t>
         </is>
       </c>
       <c r="Z1" s="1" t="inlineStr">
-        <is>
-          <t>Interneto svetainė</t>
-        </is>
-      </c>
-      <c r="AA1" s="1" t="inlineStr">
-        <is>
-          <t>Pagrindinis šaltinis</t>
-        </is>
-      </c>
-      <c r="AB1" s="1" t="inlineStr">
-        <is>
-          <t>Apyvartos šaltinis</t>
-        </is>
-      </c>
-      <c r="AC1" s="1" t="inlineStr">
-        <is>
-          <t>Darbuotojų šaltinis</t>
-        </is>
-      </c>
-      <c r="AD1" s="1" t="inlineStr">
-        <is>
-          <t>Transporto šaltinis</t>
-        </is>
-      </c>
-      <c r="AE1" s="1" t="inlineStr">
-        <is>
-          <t>Betono mazgo / gamyklos šaltinis</t>
-        </is>
-      </c>
-      <c r="AF1" s="1" t="inlineStr">
-        <is>
-          <t>Pastaba / rankinis papildymas</t>
-        </is>
-      </c>
-      <c r="AG1" s="1" t="inlineStr">
         <is>
           <t>Paskutinio atnaujinimo data</t>
         </is>
@@ -794,39 +742,32 @@
           <t>100 m³/val.</t>
         </is>
       </c>
-      <c r="S2" s="2" t="inlineStr"/>
+      <c r="S2" s="4" t="inlineStr"/>
       <c r="T2" s="2" t="inlineStr">
         <is>
           <t>Viešai skelbiamas Betono centro betono mazgas Vilniuje.</t>
         </is>
       </c>
-      <c r="U2" s="4" t="n">
+      <c r="U2" s="5" t="n">
         <v>0.9</v>
       </c>
-      <c r="V2" s="5" t="n"/>
-      <c r="W2" s="6" t="n"/>
-      <c r="X2" s="5" t="n"/>
-      <c r="Y2" s="5" t="n"/>
+      <c r="V2" s="2" t="inlineStr">
+        <is>
+          <t>https://betonocentras.lt/</t>
+        </is>
+      </c>
+      <c r="W2" s="2" t="inlineStr">
+        <is>
+          <t>https://betonocentras.lt/kontaktai/</t>
+        </is>
+      </c>
+      <c r="X2" s="2" t="inlineStr">
+        <is>
+          <t>https://betonocentras.lt/kontaktai/</t>
+        </is>
+      </c>
+      <c r="Y2" s="2" t="inlineStr"/>
       <c r="Z2" s="2" t="inlineStr">
-        <is>
-          <t>https://betonocentras.lt/</t>
-        </is>
-      </c>
-      <c r="AA2" s="2" t="inlineStr">
-        <is>
-          <t>https://betonocentras.lt/kontaktai/</t>
-        </is>
-      </c>
-      <c r="AB2" s="2" t="inlineStr"/>
-      <c r="AC2" s="2" t="inlineStr"/>
-      <c r="AD2" s="2" t="inlineStr"/>
-      <c r="AE2" s="2" t="inlineStr">
-        <is>
-          <t>https://betonocentras.lt/kontaktai/</t>
-        </is>
-      </c>
-      <c r="AF2" s="2" t="inlineStr"/>
-      <c r="AG2" s="2" t="inlineStr">
         <is>
           <t>2026-07-06</t>
         </is>
@@ -911,39 +852,32 @@
       </c>
       <c r="Q3" s="2" t="inlineStr"/>
       <c r="R3" s="2" t="inlineStr"/>
-      <c r="S3" s="2" t="inlineStr"/>
+      <c r="S3" s="4" t="inlineStr"/>
       <c r="T3" s="2" t="inlineStr">
         <is>
           <t>Viešai skelbiamas Betono centro betono mazgas Kaune.</t>
         </is>
       </c>
-      <c r="U3" s="4" t="n">
+      <c r="U3" s="5" t="n">
         <v>0.9</v>
       </c>
-      <c r="V3" s="5" t="n"/>
-      <c r="W3" s="6" t="n"/>
-      <c r="X3" s="5" t="n"/>
-      <c r="Y3" s="5" t="n"/>
+      <c r="V3" s="2" t="inlineStr">
+        <is>
+          <t>https://betonocentras.lt/</t>
+        </is>
+      </c>
+      <c r="W3" s="2" t="inlineStr">
+        <is>
+          <t>https://betonocentras.lt/kontaktai/</t>
+        </is>
+      </c>
+      <c r="X3" s="2" t="inlineStr">
+        <is>
+          <t>https://betonocentras.lt/kontaktai/</t>
+        </is>
+      </c>
+      <c r="Y3" s="2" t="inlineStr"/>
       <c r="Z3" s="2" t="inlineStr">
-        <is>
-          <t>https://betonocentras.lt/</t>
-        </is>
-      </c>
-      <c r="AA3" s="2" t="inlineStr">
-        <is>
-          <t>https://betonocentras.lt/kontaktai/</t>
-        </is>
-      </c>
-      <c r="AB3" s="2" t="inlineStr"/>
-      <c r="AC3" s="2" t="inlineStr"/>
-      <c r="AD3" s="2" t="inlineStr"/>
-      <c r="AE3" s="2" t="inlineStr">
-        <is>
-          <t>https://betonocentras.lt/kontaktai/</t>
-        </is>
-      </c>
-      <c r="AF3" s="2" t="inlineStr"/>
-      <c r="AG3" s="2" t="inlineStr">
         <is>
           <t>2026-06-29</t>
         </is>
@@ -1028,43 +962,36 @@
       </c>
       <c r="Q4" s="2" t="inlineStr"/>
       <c r="R4" s="2" t="inlineStr"/>
-      <c r="S4" s="2" t="inlineStr"/>
+      <c r="S4" s="4" t="inlineStr"/>
       <c r="T4" s="2" t="inlineStr">
         <is>
           <t>Viešai skelbiamas Betono centro betono mazgas Klaipėdoje.</t>
         </is>
       </c>
-      <c r="U4" s="4" t="n">
+      <c r="U4" s="5" t="n">
         <v>0.9</v>
       </c>
-      <c r="V4" s="5" t="n"/>
-      <c r="W4" s="6" t="n"/>
-      <c r="X4" s="5" t="n"/>
-      <c r="Y4" s="5" t="n"/>
+      <c r="V4" s="2" t="inlineStr">
+        <is>
+          <t>https://betonocentras.lt/</t>
+        </is>
+      </c>
+      <c r="W4" s="2" t="inlineStr">
+        <is>
+          <t>https://betonocentras.lt/kontaktai/</t>
+        </is>
+      </c>
+      <c r="X4" s="2" t="inlineStr">
+        <is>
+          <t>https://betonocentras.lt/kontaktai/</t>
+        </is>
+      </c>
+      <c r="Y4" s="2" t="inlineStr">
+        <is>
+          <t>Oficialiame Betono centro kontaktų puslapyje patvirtintas Klaipėdos padalinys.</t>
+        </is>
+      </c>
       <c r="Z4" s="2" t="inlineStr">
-        <is>
-          <t>https://betonocentras.lt/</t>
-        </is>
-      </c>
-      <c r="AA4" s="2" t="inlineStr">
-        <is>
-          <t>https://betonocentras.lt/kontaktai/</t>
-        </is>
-      </c>
-      <c r="AB4" s="2" t="inlineStr"/>
-      <c r="AC4" s="2" t="inlineStr"/>
-      <c r="AD4" s="2" t="inlineStr"/>
-      <c r="AE4" s="2" t="inlineStr">
-        <is>
-          <t>https://betonocentras.lt/kontaktai/</t>
-        </is>
-      </c>
-      <c r="AF4" s="2" t="inlineStr">
-        <is>
-          <t>Oficialiame Betono centro kontaktų puslapyje patvirtintas Klaipėdos padalinys.</t>
-        </is>
-      </c>
-      <c r="AG4" s="2" t="inlineStr">
         <is>
           <t>2026-06-30</t>
         </is>
@@ -1149,39 +1076,32 @@
       </c>
       <c r="Q5" s="2" t="inlineStr"/>
       <c r="R5" s="2" t="inlineStr"/>
-      <c r="S5" s="2" t="inlineStr"/>
+      <c r="S5" s="4" t="inlineStr"/>
       <c r="T5" s="2" t="inlineStr">
         <is>
           <t>Viešai skelbiamas Betono centro betono mazgas Šiauliuose.</t>
         </is>
       </c>
-      <c r="U5" s="4" t="n">
+      <c r="U5" s="5" t="n">
         <v>0.9</v>
       </c>
-      <c r="V5" s="5" t="n"/>
-      <c r="W5" s="6" t="n"/>
-      <c r="X5" s="5" t="n"/>
-      <c r="Y5" s="5" t="n"/>
+      <c r="V5" s="2" t="inlineStr">
+        <is>
+          <t>https://betonocentras.lt/</t>
+        </is>
+      </c>
+      <c r="W5" s="2" t="inlineStr">
+        <is>
+          <t>https://betonocentras.lt/kontaktai/</t>
+        </is>
+      </c>
+      <c r="X5" s="2" t="inlineStr">
+        <is>
+          <t>https://betonocentras.lt/kontaktai/</t>
+        </is>
+      </c>
+      <c r="Y5" s="2" t="inlineStr"/>
       <c r="Z5" s="2" t="inlineStr">
-        <is>
-          <t>https://betonocentras.lt/</t>
-        </is>
-      </c>
-      <c r="AA5" s="2" t="inlineStr">
-        <is>
-          <t>https://betonocentras.lt/kontaktai/</t>
-        </is>
-      </c>
-      <c r="AB5" s="2" t="inlineStr"/>
-      <c r="AC5" s="2" t="inlineStr"/>
-      <c r="AD5" s="2" t="inlineStr"/>
-      <c r="AE5" s="2" t="inlineStr">
-        <is>
-          <t>https://betonocentras.lt/kontaktai/</t>
-        </is>
-      </c>
-      <c r="AF5" s="2" t="inlineStr"/>
-      <c r="AG5" s="2" t="inlineStr">
         <is>
           <t>2026-06-29</t>
         </is>
@@ -1266,39 +1186,32 @@
       </c>
       <c r="Q6" s="2" t="inlineStr"/>
       <c r="R6" s="2" t="inlineStr"/>
-      <c r="S6" s="2" t="inlineStr"/>
+      <c r="S6" s="4" t="inlineStr"/>
       <c r="T6" s="2" t="inlineStr">
         <is>
           <t>Viešai skelbiamas Betono centro betono mazgas Mažeikiuose.</t>
         </is>
       </c>
-      <c r="U6" s="4" t="n">
+      <c r="U6" s="5" t="n">
         <v>0.9</v>
       </c>
-      <c r="V6" s="5" t="n"/>
-      <c r="W6" s="6" t="n"/>
-      <c r="X6" s="5" t="n"/>
-      <c r="Y6" s="5" t="n"/>
+      <c r="V6" s="2" t="inlineStr">
+        <is>
+          <t>https://betonocentras.lt/</t>
+        </is>
+      </c>
+      <c r="W6" s="2" t="inlineStr">
+        <is>
+          <t>https://betonocentras.lt/kontaktai/</t>
+        </is>
+      </c>
+      <c r="X6" s="2" t="inlineStr">
+        <is>
+          <t>https://betonocentras.lt/kontaktai/</t>
+        </is>
+      </c>
+      <c r="Y6" s="2" t="inlineStr"/>
       <c r="Z6" s="2" t="inlineStr">
-        <is>
-          <t>https://betonocentras.lt/</t>
-        </is>
-      </c>
-      <c r="AA6" s="2" t="inlineStr">
-        <is>
-          <t>https://betonocentras.lt/kontaktai/</t>
-        </is>
-      </c>
-      <c r="AB6" s="2" t="inlineStr"/>
-      <c r="AC6" s="2" t="inlineStr"/>
-      <c r="AD6" s="2" t="inlineStr"/>
-      <c r="AE6" s="2" t="inlineStr">
-        <is>
-          <t>https://betonocentras.lt/kontaktai/</t>
-        </is>
-      </c>
-      <c r="AF6" s="2" t="inlineStr"/>
-      <c r="AG6" s="2" t="inlineStr">
         <is>
           <t>2026-06-29</t>
         </is>
@@ -1383,39 +1296,32 @@
       </c>
       <c r="Q7" s="2" t="inlineStr"/>
       <c r="R7" s="2" t="inlineStr"/>
-      <c r="S7" s="2" t="inlineStr"/>
+      <c r="S7" s="4" t="inlineStr"/>
       <c r="T7" s="2" t="inlineStr">
         <is>
           <t>Viešai skelbiamas Betono centro betono mazgas Panevėžyje.</t>
         </is>
       </c>
-      <c r="U7" s="4" t="n">
+      <c r="U7" s="5" t="n">
         <v>0.9</v>
       </c>
-      <c r="V7" s="5" t="n"/>
-      <c r="W7" s="6" t="n"/>
-      <c r="X7" s="5" t="n"/>
-      <c r="Y7" s="5" t="n"/>
+      <c r="V7" s="2" t="inlineStr">
+        <is>
+          <t>https://betonocentras.lt/</t>
+        </is>
+      </c>
+      <c r="W7" s="2" t="inlineStr">
+        <is>
+          <t>https://betonocentras.lt/kontaktai/</t>
+        </is>
+      </c>
+      <c r="X7" s="2" t="inlineStr">
+        <is>
+          <t>https://betonocentras.lt/kontaktai/</t>
+        </is>
+      </c>
+      <c r="Y7" s="2" t="inlineStr"/>
       <c r="Z7" s="2" t="inlineStr">
-        <is>
-          <t>https://betonocentras.lt/</t>
-        </is>
-      </c>
-      <c r="AA7" s="2" t="inlineStr">
-        <is>
-          <t>https://betonocentras.lt/kontaktai/</t>
-        </is>
-      </c>
-      <c r="AB7" s="2" t="inlineStr"/>
-      <c r="AC7" s="2" t="inlineStr"/>
-      <c r="AD7" s="2" t="inlineStr"/>
-      <c r="AE7" s="2" t="inlineStr">
-        <is>
-          <t>https://betonocentras.lt/kontaktai/</t>
-        </is>
-      </c>
-      <c r="AF7" s="2" t="inlineStr"/>
-      <c r="AG7" s="2" t="inlineStr">
         <is>
           <t>2026-06-29</t>
         </is>
@@ -1500,43 +1406,36 @@
       </c>
       <c r="Q8" s="2" t="inlineStr"/>
       <c r="R8" s="2" t="inlineStr"/>
-      <c r="S8" s="2" t="inlineStr"/>
+      <c r="S8" s="4" t="inlineStr"/>
       <c r="T8" s="2" t="inlineStr">
         <is>
           <t>Viešai skelbiamas Heidelberg Materials betono gamyklų tinklo taškas Vilniuje.</t>
         </is>
       </c>
-      <c r="U8" s="4" t="n">
+      <c r="U8" s="5" t="n">
         <v>0.85</v>
       </c>
-      <c r="V8" s="5" t="n"/>
-      <c r="W8" s="6" t="n"/>
-      <c r="X8" s="5" t="n"/>
-      <c r="Y8" s="5" t="n"/>
+      <c r="V8" s="2" t="inlineStr">
+        <is>
+          <t>https://www.betonas.heidelbergmaterials.lt/lt</t>
+        </is>
+      </c>
+      <c r="W8" s="2" t="inlineStr">
+        <is>
+          <t>https://www.betonas.heidelbergmaterials.lt/lt/kontaktine-informacija-0</t>
+        </is>
+      </c>
+      <c r="X8" s="2" t="inlineStr">
+        <is>
+          <t>https://www.betonas.heidelbergmaterials.lt/lt/kontaktine-informacija-0</t>
+        </is>
+      </c>
+      <c r="Y8" s="2" t="inlineStr">
+        <is>
+          <t>Oficialus Heidelberg Materials Lietuva Betonas kontaktų puslapis patvirtina betono užsakymų padalinius Lietuvoje.</t>
+        </is>
+      </c>
       <c r="Z8" s="2" t="inlineStr">
-        <is>
-          <t>https://www.betonas.heidelbergmaterials.lt/lt</t>
-        </is>
-      </c>
-      <c r="AA8" s="2" t="inlineStr">
-        <is>
-          <t>https://www.betonas.heidelbergmaterials.lt/lt/kontaktine-informacija-0</t>
-        </is>
-      </c>
-      <c r="AB8" s="2" t="inlineStr"/>
-      <c r="AC8" s="2" t="inlineStr"/>
-      <c r="AD8" s="2" t="inlineStr"/>
-      <c r="AE8" s="2" t="inlineStr">
-        <is>
-          <t>https://www.betonas.heidelbergmaterials.lt/lt/kontaktine-informacija-0</t>
-        </is>
-      </c>
-      <c r="AF8" s="2" t="inlineStr">
-        <is>
-          <t>Oficialus Heidelberg Materials Lietuva Betonas kontaktų puslapis patvirtina betono užsakymų padalinius Lietuvoje.</t>
-        </is>
-      </c>
-      <c r="AG8" s="2" t="inlineStr">
         <is>
           <t>2026-06-29</t>
         </is>
@@ -1621,43 +1520,36 @@
       </c>
       <c r="Q9" s="2" t="inlineStr"/>
       <c r="R9" s="2" t="inlineStr"/>
-      <c r="S9" s="2" t="inlineStr"/>
+      <c r="S9" s="4" t="inlineStr"/>
       <c r="T9" s="2" t="inlineStr">
         <is>
           <t>Viešai skelbiamas Heidelberg Materials betono gamyklų tinklo taškas Vilniuje.</t>
         </is>
       </c>
-      <c r="U9" s="4" t="n">
+      <c r="U9" s="5" t="n">
         <v>0.85</v>
       </c>
-      <c r="V9" s="5" t="n"/>
-      <c r="W9" s="6" t="n"/>
-      <c r="X9" s="5" t="n"/>
-      <c r="Y9" s="5" t="n"/>
+      <c r="V9" s="2" t="inlineStr">
+        <is>
+          <t>https://www.betonas.heidelbergmaterials.lt/lt</t>
+        </is>
+      </c>
+      <c r="W9" s="2" t="inlineStr">
+        <is>
+          <t>https://www.betonas.heidelbergmaterials.lt/lt/kontaktine-informacija-0</t>
+        </is>
+      </c>
+      <c r="X9" s="2" t="inlineStr">
+        <is>
+          <t>https://www.betonas.heidelbergmaterials.lt/lt/kontaktine-informacija-0</t>
+        </is>
+      </c>
+      <c r="Y9" s="2" t="inlineStr">
+        <is>
+          <t>Oficialus Heidelberg Materials Lietuva Betonas kontaktų puslapis patvirtina betono užsakymų padalinius Lietuvoje.</t>
+        </is>
+      </c>
       <c r="Z9" s="2" t="inlineStr">
-        <is>
-          <t>https://www.betonas.heidelbergmaterials.lt/lt</t>
-        </is>
-      </c>
-      <c r="AA9" s="2" t="inlineStr">
-        <is>
-          <t>https://www.betonas.heidelbergmaterials.lt/lt/kontaktine-informacija-0</t>
-        </is>
-      </c>
-      <c r="AB9" s="2" t="inlineStr"/>
-      <c r="AC9" s="2" t="inlineStr"/>
-      <c r="AD9" s="2" t="inlineStr"/>
-      <c r="AE9" s="2" t="inlineStr">
-        <is>
-          <t>https://www.betonas.heidelbergmaterials.lt/lt/kontaktine-informacija-0</t>
-        </is>
-      </c>
-      <c r="AF9" s="2" t="inlineStr">
-        <is>
-          <t>Oficialus Heidelberg Materials Lietuva Betonas kontaktų puslapis patvirtina betono užsakymų padalinius Lietuvoje.</t>
-        </is>
-      </c>
-      <c r="AG9" s="2" t="inlineStr">
         <is>
           <t>2026-06-29</t>
         </is>
@@ -1742,43 +1634,36 @@
       </c>
       <c r="Q10" s="2" t="inlineStr"/>
       <c r="R10" s="2" t="inlineStr"/>
-      <c r="S10" s="2" t="inlineStr"/>
+      <c r="S10" s="4" t="inlineStr"/>
       <c r="T10" s="2" t="inlineStr">
         <is>
           <t>Viešai skelbiamas Heidelberg Materials betono gamyklų tinklo taškas Kaune.</t>
         </is>
       </c>
-      <c r="U10" s="4" t="n">
+      <c r="U10" s="5" t="n">
         <v>0.85</v>
       </c>
-      <c r="V10" s="5" t="n"/>
-      <c r="W10" s="6" t="n"/>
-      <c r="X10" s="5" t="n"/>
-      <c r="Y10" s="5" t="n"/>
+      <c r="V10" s="2" t="inlineStr">
+        <is>
+          <t>https://www.betonas.heidelbergmaterials.lt/lt</t>
+        </is>
+      </c>
+      <c r="W10" s="2" t="inlineStr">
+        <is>
+          <t>https://www.betonas.heidelbergmaterials.lt/lt/kontaktine-informacija-0</t>
+        </is>
+      </c>
+      <c r="X10" s="2" t="inlineStr">
+        <is>
+          <t>https://www.betonas.heidelbergmaterials.lt/lt/kontaktine-informacija-0</t>
+        </is>
+      </c>
+      <c r="Y10" s="2" t="inlineStr">
+        <is>
+          <t>Oficialus Heidelberg Materials Lietuva Betonas kontaktų puslapis patvirtina betono užsakymų padalinius Lietuvoje.</t>
+        </is>
+      </c>
       <c r="Z10" s="2" t="inlineStr">
-        <is>
-          <t>https://www.betonas.heidelbergmaterials.lt/lt</t>
-        </is>
-      </c>
-      <c r="AA10" s="2" t="inlineStr">
-        <is>
-          <t>https://www.betonas.heidelbergmaterials.lt/lt/kontaktine-informacija-0</t>
-        </is>
-      </c>
-      <c r="AB10" s="2" t="inlineStr"/>
-      <c r="AC10" s="2" t="inlineStr"/>
-      <c r="AD10" s="2" t="inlineStr"/>
-      <c r="AE10" s="2" t="inlineStr">
-        <is>
-          <t>https://www.betonas.heidelbergmaterials.lt/lt/kontaktine-informacija-0</t>
-        </is>
-      </c>
-      <c r="AF10" s="2" t="inlineStr">
-        <is>
-          <t>Oficialus Heidelberg Materials Lietuva Betonas kontaktų puslapis patvirtina betono užsakymų padalinius Lietuvoje.</t>
-        </is>
-      </c>
-      <c r="AG10" s="2" t="inlineStr">
         <is>
           <t>2026-06-29</t>
         </is>
@@ -1863,43 +1748,36 @@
       </c>
       <c r="Q11" s="2" t="inlineStr"/>
       <c r="R11" s="2" t="inlineStr"/>
-      <c r="S11" s="2" t="inlineStr"/>
+      <c r="S11" s="4" t="inlineStr"/>
       <c r="T11" s="2" t="inlineStr">
         <is>
           <t>Viešai skelbiamas Heidelberg Materials betono gamyklų tinklo taškas Klaipėdoje.</t>
         </is>
       </c>
-      <c r="U11" s="4" t="n">
+      <c r="U11" s="5" t="n">
         <v>0.85</v>
       </c>
-      <c r="V11" s="5" t="n"/>
-      <c r="W11" s="6" t="n"/>
-      <c r="X11" s="5" t="n"/>
-      <c r="Y11" s="5" t="n"/>
+      <c r="V11" s="2" t="inlineStr">
+        <is>
+          <t>https://www.betonas.heidelbergmaterials.lt/lt</t>
+        </is>
+      </c>
+      <c r="W11" s="2" t="inlineStr">
+        <is>
+          <t>https://www.betonas.heidelbergmaterials.lt/lt/kontaktine-informacija-0</t>
+        </is>
+      </c>
+      <c r="X11" s="2" t="inlineStr">
+        <is>
+          <t>https://www.betonas.heidelbergmaterials.lt/lt/kontaktine-informacija-0</t>
+        </is>
+      </c>
+      <c r="Y11" s="2" t="inlineStr">
+        <is>
+          <t>Oficialus Heidelberg Materials Lietuva Betonas kontaktų puslapis patvirtina betono užsakymų padalinius Lietuvoje.</t>
+        </is>
+      </c>
       <c r="Z11" s="2" t="inlineStr">
-        <is>
-          <t>https://www.betonas.heidelbergmaterials.lt/lt</t>
-        </is>
-      </c>
-      <c r="AA11" s="2" t="inlineStr">
-        <is>
-          <t>https://www.betonas.heidelbergmaterials.lt/lt/kontaktine-informacija-0</t>
-        </is>
-      </c>
-      <c r="AB11" s="2" t="inlineStr"/>
-      <c r="AC11" s="2" t="inlineStr"/>
-      <c r="AD11" s="2" t="inlineStr"/>
-      <c r="AE11" s="2" t="inlineStr">
-        <is>
-          <t>https://www.betonas.heidelbergmaterials.lt/lt/kontaktine-informacija-0</t>
-        </is>
-      </c>
-      <c r="AF11" s="2" t="inlineStr">
-        <is>
-          <t>Oficialus Heidelberg Materials Lietuva Betonas kontaktų puslapis patvirtina betono užsakymų padalinius Lietuvoje.</t>
-        </is>
-      </c>
-      <c r="AG11" s="2" t="inlineStr">
         <is>
           <t>2026-06-29</t>
         </is>
@@ -1984,43 +1862,36 @@
       </c>
       <c r="Q12" s="2" t="inlineStr"/>
       <c r="R12" s="2" t="inlineStr"/>
-      <c r="S12" s="2" t="inlineStr"/>
+      <c r="S12" s="4" t="inlineStr"/>
       <c r="T12" s="2" t="inlineStr">
         <is>
           <t>Viešai skelbiamas Heidelberg Materials betono gamyklų tinklo taškas Alytuje.</t>
         </is>
       </c>
-      <c r="U12" s="4" t="n">
+      <c r="U12" s="5" t="n">
         <v>0.85</v>
       </c>
-      <c r="V12" s="5" t="n"/>
-      <c r="W12" s="6" t="n"/>
-      <c r="X12" s="5" t="n"/>
-      <c r="Y12" s="5" t="n"/>
+      <c r="V12" s="2" t="inlineStr">
+        <is>
+          <t>https://www.betonas.heidelbergmaterials.lt/lt</t>
+        </is>
+      </c>
+      <c r="W12" s="2" t="inlineStr">
+        <is>
+          <t>https://www.betonas.heidelbergmaterials.lt/lt/kontaktine-informacija-0</t>
+        </is>
+      </c>
+      <c r="X12" s="2" t="inlineStr">
+        <is>
+          <t>https://www.betonas.heidelbergmaterials.lt/lt/kontaktine-informacija-0</t>
+        </is>
+      </c>
+      <c r="Y12" s="2" t="inlineStr">
+        <is>
+          <t>Oficialus Heidelberg Materials Lietuva Betonas kontaktų puslapis patvirtina betono užsakymų padalinius Lietuvoje.</t>
+        </is>
+      </c>
       <c r="Z12" s="2" t="inlineStr">
-        <is>
-          <t>https://www.betonas.heidelbergmaterials.lt/lt</t>
-        </is>
-      </c>
-      <c r="AA12" s="2" t="inlineStr">
-        <is>
-          <t>https://www.betonas.heidelbergmaterials.lt/lt/kontaktine-informacija-0</t>
-        </is>
-      </c>
-      <c r="AB12" s="2" t="inlineStr"/>
-      <c r="AC12" s="2" t="inlineStr"/>
-      <c r="AD12" s="2" t="inlineStr"/>
-      <c r="AE12" s="2" t="inlineStr">
-        <is>
-          <t>https://www.betonas.heidelbergmaterials.lt/lt/kontaktine-informacija-0</t>
-        </is>
-      </c>
-      <c r="AF12" s="2" t="inlineStr">
-        <is>
-          <t>Oficialus Heidelberg Materials Lietuva Betonas kontaktų puslapis patvirtina betono užsakymų padalinius Lietuvoje.</t>
-        </is>
-      </c>
-      <c r="AG12" s="2" t="inlineStr">
         <is>
           <t>2026-06-29</t>
         </is>
@@ -2105,43 +1976,36 @@
       </c>
       <c r="Q13" s="2" t="inlineStr"/>
       <c r="R13" s="2" t="inlineStr"/>
-      <c r="S13" s="2" t="inlineStr"/>
+      <c r="S13" s="4" t="inlineStr"/>
       <c r="T13" s="2" t="inlineStr">
         <is>
           <t>Viešai skelbiamas Heidelberg Materials betono gamyklų tinklo taškas Pasvalyje.</t>
         </is>
       </c>
-      <c r="U13" s="4" t="n">
+      <c r="U13" s="5" t="n">
         <v>0.8</v>
       </c>
-      <c r="V13" s="5" t="n"/>
-      <c r="W13" s="6" t="n"/>
-      <c r="X13" s="5" t="n"/>
-      <c r="Y13" s="5" t="n"/>
+      <c r="V13" s="2" t="inlineStr">
+        <is>
+          <t>https://www.betonas.heidelbergmaterials.lt/lt</t>
+        </is>
+      </c>
+      <c r="W13" s="2" t="inlineStr">
+        <is>
+          <t>https://www.betonas.heidelbergmaterials.lt/lt/kontaktine-informacija-0</t>
+        </is>
+      </c>
+      <c r="X13" s="2" t="inlineStr">
+        <is>
+          <t>https://www.betonas.heidelbergmaterials.lt/lt/kontaktine-informacija-0</t>
+        </is>
+      </c>
+      <c r="Y13" s="2" t="inlineStr">
+        <is>
+          <t>Oficialus Heidelberg Materials Lietuva Betonas kontaktų puslapis patvirtina betono užsakymų padalinius Lietuvoje.</t>
+        </is>
+      </c>
       <c r="Z13" s="2" t="inlineStr">
-        <is>
-          <t>https://www.betonas.heidelbergmaterials.lt/lt</t>
-        </is>
-      </c>
-      <c r="AA13" s="2" t="inlineStr">
-        <is>
-          <t>https://www.betonas.heidelbergmaterials.lt/lt/kontaktine-informacija-0</t>
-        </is>
-      </c>
-      <c r="AB13" s="2" t="inlineStr"/>
-      <c r="AC13" s="2" t="inlineStr"/>
-      <c r="AD13" s="2" t="inlineStr"/>
-      <c r="AE13" s="2" t="inlineStr">
-        <is>
-          <t>https://www.betonas.heidelbergmaterials.lt/lt/kontaktine-informacija-0</t>
-        </is>
-      </c>
-      <c r="AF13" s="2" t="inlineStr">
-        <is>
-          <t>Oficialus Heidelberg Materials Lietuva Betonas kontaktų puslapis patvirtina betono užsakymų padalinius Lietuvoje.</t>
-        </is>
-      </c>
-      <c r="AG13" s="2" t="inlineStr">
         <is>
           <t>2026-06-29</t>
         </is>
@@ -2226,39 +2090,32 @@
       </c>
       <c r="Q14" s="2" t="inlineStr"/>
       <c r="R14" s="2" t="inlineStr"/>
-      <c r="S14" s="2" t="inlineStr"/>
+      <c r="S14" s="4" t="inlineStr"/>
       <c r="T14" s="2" t="inlineStr">
         <is>
           <t>Viešai skelbiamas betono mišinių tiekėjas Vilniaus regione.</t>
         </is>
       </c>
-      <c r="U14" s="4" t="n">
+      <c r="U14" s="5" t="n">
         <v>0.8</v>
       </c>
-      <c r="V14" s="5" t="n"/>
-      <c r="W14" s="6" t="n"/>
-      <c r="X14" s="5" t="n"/>
-      <c r="Y14" s="5" t="n"/>
+      <c r="V14" s="2" t="inlineStr">
+        <is>
+          <t>https://www.palmusta.lt/</t>
+        </is>
+      </c>
+      <c r="W14" s="2" t="inlineStr">
+        <is>
+          <t>https://www.palmusta.lt/</t>
+        </is>
+      </c>
+      <c r="X14" s="2" t="inlineStr">
+        <is>
+          <t>https://www.palmusta.lt/</t>
+        </is>
+      </c>
+      <c r="Y14" s="2" t="inlineStr"/>
       <c r="Z14" s="2" t="inlineStr">
-        <is>
-          <t>https://www.palmusta.lt/</t>
-        </is>
-      </c>
-      <c r="AA14" s="2" t="inlineStr">
-        <is>
-          <t>https://www.palmusta.lt/</t>
-        </is>
-      </c>
-      <c r="AB14" s="2" t="inlineStr"/>
-      <c r="AC14" s="2" t="inlineStr"/>
-      <c r="AD14" s="2" t="inlineStr"/>
-      <c r="AE14" s="2" t="inlineStr">
-        <is>
-          <t>https://www.palmusta.lt/</t>
-        </is>
-      </c>
-      <c r="AF14" s="2" t="inlineStr"/>
-      <c r="AG14" s="2" t="inlineStr">
         <is>
           <t>2026-06-29</t>
         </is>
@@ -2339,43 +2196,36 @@
       </c>
       <c r="Q15" s="2" t="inlineStr"/>
       <c r="R15" s="2" t="inlineStr"/>
-      <c r="S15" s="2" t="inlineStr"/>
+      <c r="S15" s="4" t="inlineStr"/>
       <c r="T15" s="2" t="inlineStr">
         <is>
           <t>Gelžbetoninių konstrukcijų gamyba Vilniuje.</t>
         </is>
       </c>
-      <c r="U15" s="4" t="n">
+      <c r="U15" s="5" t="n">
         <v>0.9</v>
       </c>
-      <c r="V15" s="5" t="n"/>
-      <c r="W15" s="6" t="n"/>
-      <c r="X15" s="5" t="n"/>
-      <c r="Y15" s="5" t="n"/>
+      <c r="V15" s="2" t="inlineStr">
+        <is>
+          <t>https://www.gkg3.lt/</t>
+        </is>
+      </c>
+      <c r="W15" s="2" t="inlineStr">
+        <is>
+          <t>https://gkg3.lt/kontaktai/</t>
+        </is>
+      </c>
+      <c r="X15" s="2" t="inlineStr">
+        <is>
+          <t>https://gkg3.lt/kontaktai/</t>
+        </is>
+      </c>
+      <c r="Y15" s="2" t="inlineStr">
+        <is>
+          <t>Koordinatės patikslintos pagal oficialaus GKG3 kontaktų puslapio Google Maps nuorodą.</t>
+        </is>
+      </c>
       <c r="Z15" s="2" t="inlineStr">
-        <is>
-          <t>https://www.gkg3.lt/</t>
-        </is>
-      </c>
-      <c r="AA15" s="2" t="inlineStr">
-        <is>
-          <t>https://gkg3.lt/kontaktai/</t>
-        </is>
-      </c>
-      <c r="AB15" s="2" t="inlineStr"/>
-      <c r="AC15" s="2" t="inlineStr"/>
-      <c r="AD15" s="2" t="inlineStr"/>
-      <c r="AE15" s="2" t="inlineStr">
-        <is>
-          <t>https://gkg3.lt/kontaktai/</t>
-        </is>
-      </c>
-      <c r="AF15" s="2" t="inlineStr">
-        <is>
-          <t>Koordinatės patikslintos pagal oficialaus GKG3 kontaktų puslapio Google Maps nuorodą.</t>
-        </is>
-      </c>
-      <c r="AG15" s="2" t="inlineStr">
         <is>
           <t>2026-06-29</t>
         </is>
@@ -2460,39 +2310,32 @@
           <t>150 m³/val.</t>
         </is>
       </c>
-      <c r="S16" s="2" t="inlineStr"/>
+      <c r="S16" s="4" t="inlineStr"/>
       <c r="T16" s="2" t="inlineStr">
         <is>
           <t>Viešai nurodoma nauja gelžbetonio elementų gamybos linija, kurios našumas 150 m³/val.</t>
         </is>
       </c>
-      <c r="U16" s="4" t="n">
+      <c r="U16" s="5" t="n">
         <v>0.9</v>
       </c>
-      <c r="V16" s="5" t="n"/>
-      <c r="W16" s="6" t="n"/>
-      <c r="X16" s="5" t="n"/>
-      <c r="Y16" s="5" t="n"/>
+      <c r="V16" s="2" t="inlineStr">
+        <is>
+          <t>https://www.perdanga.lt/</t>
+        </is>
+      </c>
+      <c r="W16" s="2" t="inlineStr">
+        <is>
+          <t>https://www.perdanga.lt/</t>
+        </is>
+      </c>
+      <c r="X16" s="2" t="inlineStr">
+        <is>
+          <t>https://www.perdanga.lt/</t>
+        </is>
+      </c>
+      <c r="Y16" s="2" t="inlineStr"/>
       <c r="Z16" s="2" t="inlineStr">
-        <is>
-          <t>https://www.perdanga.lt/</t>
-        </is>
-      </c>
-      <c r="AA16" s="2" t="inlineStr">
-        <is>
-          <t>https://www.perdanga.lt/</t>
-        </is>
-      </c>
-      <c r="AB16" s="2" t="inlineStr"/>
-      <c r="AC16" s="2" t="inlineStr"/>
-      <c r="AD16" s="2" t="inlineStr"/>
-      <c r="AE16" s="2" t="inlineStr">
-        <is>
-          <t>https://www.perdanga.lt/</t>
-        </is>
-      </c>
-      <c r="AF16" s="2" t="inlineStr"/>
-      <c r="AG16" s="2" t="inlineStr">
         <is>
           <t>2026-06-29</t>
         </is>
@@ -2573,39 +2416,32 @@
       </c>
       <c r="Q17" s="2" t="inlineStr"/>
       <c r="R17" s="2" t="inlineStr"/>
-      <c r="S17" s="2" t="inlineStr"/>
+      <c r="S17" s="4" t="inlineStr"/>
       <c r="T17" s="2" t="inlineStr">
         <is>
           <t>Viešai skelbiamas Perdangos padalinys Klaipėdoje.</t>
         </is>
       </c>
-      <c r="U17" s="4" t="n">
+      <c r="U17" s="5" t="n">
         <v>0.85</v>
       </c>
-      <c r="V17" s="5" t="n"/>
-      <c r="W17" s="6" t="n"/>
-      <c r="X17" s="5" t="n"/>
-      <c r="Y17" s="5" t="n"/>
+      <c r="V17" s="2" t="inlineStr">
+        <is>
+          <t>https://www.perdanga.lt/</t>
+        </is>
+      </c>
+      <c r="W17" s="2" t="inlineStr">
+        <is>
+          <t>https://www.perdanga.lt/</t>
+        </is>
+      </c>
+      <c r="X17" s="2" t="inlineStr">
+        <is>
+          <t>https://www.perdanga.lt/</t>
+        </is>
+      </c>
+      <c r="Y17" s="2" t="inlineStr"/>
       <c r="Z17" s="2" t="inlineStr">
-        <is>
-          <t>https://www.perdanga.lt/</t>
-        </is>
-      </c>
-      <c r="AA17" s="2" t="inlineStr">
-        <is>
-          <t>https://www.perdanga.lt/</t>
-        </is>
-      </c>
-      <c r="AB17" s="2" t="inlineStr"/>
-      <c r="AC17" s="2" t="inlineStr"/>
-      <c r="AD17" s="2" t="inlineStr"/>
-      <c r="AE17" s="2" t="inlineStr">
-        <is>
-          <t>https://www.perdanga.lt/</t>
-        </is>
-      </c>
-      <c r="AF17" s="2" t="inlineStr"/>
-      <c r="AG17" s="2" t="inlineStr">
         <is>
           <t>2026-06-29</t>
         </is>
@@ -2686,43 +2522,36 @@
       </c>
       <c r="Q18" s="2" t="inlineStr"/>
       <c r="R18" s="2" t="inlineStr"/>
-      <c r="S18" s="2" t="inlineStr"/>
+      <c r="S18" s="4" t="inlineStr"/>
       <c r="T18" s="2" t="inlineStr">
         <is>
           <t>Viešai skelbiamas gelžbetonio gamintojas Kaune.</t>
         </is>
       </c>
-      <c r="U18" s="4" t="n">
+      <c r="U18" s="5" t="n">
         <v>0.8</v>
       </c>
-      <c r="V18" s="5" t="n"/>
-      <c r="W18" s="6" t="n"/>
-      <c r="X18" s="5" t="n"/>
-      <c r="Y18" s="5" t="n"/>
+      <c r="V18" s="2" t="inlineStr">
+        <is>
+          <t>https://www.kaunogelzbetonis.lt/</t>
+        </is>
+      </c>
+      <c r="W18" s="2" t="inlineStr">
+        <is>
+          <t>https://www.kaunogelzbetonis.lt/kontaktai/</t>
+        </is>
+      </c>
+      <c r="X18" s="2" t="inlineStr">
+        <is>
+          <t>https://www.kaunogelzbetonis.lt/kontaktai/</t>
+        </is>
+      </c>
+      <c r="Y18" s="2" t="inlineStr">
+        <is>
+          <t>Oficialus Kauno gelžbetonio kontaktų puslapis patvirtina Pramonės pr. 8 adresą.</t>
+        </is>
+      </c>
       <c r="Z18" s="2" t="inlineStr">
-        <is>
-          <t>https://www.kaunogelzbetonis.lt/</t>
-        </is>
-      </c>
-      <c r="AA18" s="2" t="inlineStr">
-        <is>
-          <t>https://www.kaunogelzbetonis.lt/kontaktai/</t>
-        </is>
-      </c>
-      <c r="AB18" s="2" t="inlineStr"/>
-      <c r="AC18" s="2" t="inlineStr"/>
-      <c r="AD18" s="2" t="inlineStr"/>
-      <c r="AE18" s="2" t="inlineStr">
-        <is>
-          <t>https://www.kaunogelzbetonis.lt/kontaktai/</t>
-        </is>
-      </c>
-      <c r="AF18" s="2" t="inlineStr">
-        <is>
-          <t>Oficialus Kauno gelžbetonio kontaktų puslapis patvirtina Pramonės pr. 8 adresą.</t>
-        </is>
-      </c>
-      <c r="AG18" s="2" t="inlineStr">
         <is>
           <t>2026-06-29</t>
         </is>
@@ -2803,43 +2632,36 @@
       </c>
       <c r="Q19" s="2" t="inlineStr"/>
       <c r="R19" s="2" t="inlineStr"/>
-      <c r="S19" s="2" t="inlineStr"/>
+      <c r="S19" s="4" t="inlineStr"/>
       <c r="T19" s="2" t="inlineStr">
         <is>
           <t>Viešai skelbiamas gelžbetonio gamintojas Ukmergėje.</t>
         </is>
       </c>
-      <c r="U19" s="4" t="n">
+      <c r="U19" s="5" t="n">
         <v>0.8</v>
       </c>
-      <c r="V19" s="5" t="n"/>
-      <c r="W19" s="6" t="n"/>
-      <c r="X19" s="5" t="n"/>
-      <c r="Y19" s="5" t="n"/>
+      <c r="V19" s="2" t="inlineStr">
+        <is>
+          <t>https://ukmergesgelzbetonis.lt/</t>
+        </is>
+      </c>
+      <c r="W19" s="2" t="inlineStr">
+        <is>
+          <t>https://ukmergesgelzbetonis.lt/</t>
+        </is>
+      </c>
+      <c r="X19" s="2" t="inlineStr">
+        <is>
+          <t>https://ukmergesgelzbetonis.lt/</t>
+        </is>
+      </c>
+      <c r="Y19" s="2" t="inlineStr">
+        <is>
+          <t>Oficiali Ukmergės gelžbetonio svetainė palikta kaip pagrindinis šaltinis; naujų patikimų koordinačių nerasta.</t>
+        </is>
+      </c>
       <c r="Z19" s="2" t="inlineStr">
-        <is>
-          <t>https://ukmergesgelzbetonis.lt/</t>
-        </is>
-      </c>
-      <c r="AA19" s="2" t="inlineStr">
-        <is>
-          <t>https://ukmergesgelzbetonis.lt/</t>
-        </is>
-      </c>
-      <c r="AB19" s="2" t="inlineStr"/>
-      <c r="AC19" s="2" t="inlineStr"/>
-      <c r="AD19" s="2" t="inlineStr"/>
-      <c r="AE19" s="2" t="inlineStr">
-        <is>
-          <t>https://ukmergesgelzbetonis.lt/</t>
-        </is>
-      </c>
-      <c r="AF19" s="2" t="inlineStr">
-        <is>
-          <t>Oficiali Ukmergės gelžbetonio svetainė palikta kaip pagrindinis šaltinis; naujų patikimų koordinačių nerasta.</t>
-        </is>
-      </c>
-      <c r="AG19" s="2" t="inlineStr">
         <is>
           <t>2026-06-29</t>
         </is>
@@ -2920,43 +2742,36 @@
       </c>
       <c r="Q20" s="2" t="inlineStr"/>
       <c r="R20" s="2" t="inlineStr"/>
-      <c r="S20" s="2" t="inlineStr"/>
+      <c r="S20" s="4" t="inlineStr"/>
       <c r="T20" s="2" t="inlineStr">
         <is>
           <t>Viešai skelbiamas gelžbetonio gamintojas Šiauliuose.</t>
         </is>
       </c>
-      <c r="U20" s="4" t="n">
+      <c r="U20" s="5" t="n">
         <v>0.8</v>
       </c>
-      <c r="V20" s="5" t="n"/>
-      <c r="W20" s="6" t="n"/>
-      <c r="X20" s="5" t="n"/>
-      <c r="Y20" s="5" t="n"/>
+      <c r="V20" s="2" t="inlineStr">
+        <is>
+          <t>https://www.gelzbetonineskonstrukcijos.lt/</t>
+        </is>
+      </c>
+      <c r="W20" s="2" t="inlineStr">
+        <is>
+          <t>https://www.gelzbetonineskonstrukcijos.lt/contacts/</t>
+        </is>
+      </c>
+      <c r="X20" s="2" t="inlineStr">
+        <is>
+          <t>https://www.gelzbetonineskonstrukcijos.lt/contacts/</t>
+        </is>
+      </c>
+      <c r="Y20" s="2" t="inlineStr">
+        <is>
+          <t>Koordinatės patikslintos pagal oficialaus kontaktų puslapio žemėlapio tašką.</t>
+        </is>
+      </c>
       <c r="Z20" s="2" t="inlineStr">
-        <is>
-          <t>https://www.gelzbetonineskonstrukcijos.lt/</t>
-        </is>
-      </c>
-      <c r="AA20" s="2" t="inlineStr">
-        <is>
-          <t>https://www.gelzbetonineskonstrukcijos.lt/contacts/</t>
-        </is>
-      </c>
-      <c r="AB20" s="2" t="inlineStr"/>
-      <c r="AC20" s="2" t="inlineStr"/>
-      <c r="AD20" s="2" t="inlineStr"/>
-      <c r="AE20" s="2" t="inlineStr">
-        <is>
-          <t>https://www.gelzbetonineskonstrukcijos.lt/contacts/</t>
-        </is>
-      </c>
-      <c r="AF20" s="2" t="inlineStr">
-        <is>
-          <t>Koordinatės patikslintos pagal oficialaus kontaktų puslapio žemėlapio tašką.</t>
-        </is>
-      </c>
-      <c r="AG20" s="2" t="inlineStr">
         <is>
           <t>2026-06-29</t>
         </is>
@@ -3037,39 +2852,32 @@
       </c>
       <c r="Q21" s="2" t="inlineStr"/>
       <c r="R21" s="2" t="inlineStr"/>
-      <c r="S21" s="2" t="inlineStr"/>
+      <c r="S21" s="4" t="inlineStr"/>
       <c r="T21" s="2" t="inlineStr">
         <is>
           <t>Viešai skelbiamas surenkamojo gelžbetonio konstrukcijų gamintojas.</t>
         </is>
       </c>
-      <c r="U21" s="4" t="n">
+      <c r="U21" s="5" t="n">
         <v>0.8</v>
       </c>
-      <c r="V21" s="5" t="n"/>
-      <c r="W21" s="6" t="n"/>
-      <c r="X21" s="5" t="n"/>
-      <c r="Y21" s="5" t="n"/>
+      <c r="V21" s="2" t="inlineStr">
+        <is>
+          <t>https://inhus.eu/</t>
+        </is>
+      </c>
+      <c r="W21" s="2" t="inlineStr">
+        <is>
+          <t>https://inhus.eu/</t>
+        </is>
+      </c>
+      <c r="X21" s="2" t="inlineStr">
+        <is>
+          <t>https://inhus.eu/</t>
+        </is>
+      </c>
+      <c r="Y21" s="2" t="inlineStr"/>
       <c r="Z21" s="2" t="inlineStr">
-        <is>
-          <t>https://inhus.eu/</t>
-        </is>
-      </c>
-      <c r="AA21" s="2" t="inlineStr">
-        <is>
-          <t>https://inhus.eu/</t>
-        </is>
-      </c>
-      <c r="AB21" s="2" t="inlineStr"/>
-      <c r="AC21" s="2" t="inlineStr"/>
-      <c r="AD21" s="2" t="inlineStr"/>
-      <c r="AE21" s="2" t="inlineStr">
-        <is>
-          <t>https://inhus.eu/</t>
-        </is>
-      </c>
-      <c r="AF21" s="2" t="inlineStr"/>
-      <c r="AG21" s="2" t="inlineStr">
         <is>
           <t>2026-06-29</t>
         </is>
@@ -3150,39 +2958,32 @@
       </c>
       <c r="Q22" s="2" t="inlineStr"/>
       <c r="R22" s="2" t="inlineStr"/>
-      <c r="S22" s="2" t="inlineStr"/>
+      <c r="S22" s="4" t="inlineStr"/>
       <c r="T22" s="2" t="inlineStr">
         <is>
           <t>Viešai skelbiamas betono mišinių tiekėjas.</t>
         </is>
       </c>
-      <c r="U22" s="4" t="n">
+      <c r="U22" s="5" t="n">
         <v>0.75</v>
       </c>
-      <c r="V22" s="5" t="n"/>
-      <c r="W22" s="6" t="n"/>
-      <c r="X22" s="5" t="n"/>
-      <c r="Y22" s="5" t="n"/>
+      <c r="V22" s="2" t="inlineStr">
+        <is>
+          <t>https://gelmesta.lt/</t>
+        </is>
+      </c>
+      <c r="W22" s="2" t="inlineStr">
+        <is>
+          <t>https://gelmesta.lt/</t>
+        </is>
+      </c>
+      <c r="X22" s="2" t="inlineStr">
+        <is>
+          <t>https://gelmesta.lt/</t>
+        </is>
+      </c>
+      <c r="Y22" s="2" t="inlineStr"/>
       <c r="Z22" s="2" t="inlineStr">
-        <is>
-          <t>https://gelmesta.lt/</t>
-        </is>
-      </c>
-      <c r="AA22" s="2" t="inlineStr">
-        <is>
-          <t>https://gelmesta.lt/</t>
-        </is>
-      </c>
-      <c r="AB22" s="2" t="inlineStr"/>
-      <c r="AC22" s="2" t="inlineStr"/>
-      <c r="AD22" s="2" t="inlineStr"/>
-      <c r="AE22" s="2" t="inlineStr">
-        <is>
-          <t>https://gelmesta.lt/</t>
-        </is>
-      </c>
-      <c r="AF22" s="2" t="inlineStr"/>
-      <c r="AG22" s="2" t="inlineStr">
         <is>
           <t>2026-06-29</t>
         </is>
@@ -3267,39 +3068,32 @@
           <t>iki 200 m³ per darbo pamainą</t>
         </is>
       </c>
-      <c r="S23" s="2" t="inlineStr"/>
+      <c r="S23" s="4" t="inlineStr"/>
       <c r="T23" s="2" t="inlineStr">
         <is>
           <t>Viešai skelbiamas betono mišinių gamintojas; nurodomas našumas iki 200 m³ per darbo pamainą.</t>
         </is>
       </c>
-      <c r="U23" s="4" t="n">
+      <c r="U23" s="5" t="n">
         <v>0.75</v>
       </c>
-      <c r="V23" s="5" t="n"/>
-      <c r="W23" s="6" t="n"/>
-      <c r="X23" s="5" t="n"/>
-      <c r="Y23" s="5" t="n"/>
+      <c r="V23" s="2" t="inlineStr">
+        <is>
+          <t>https://www.suduvos-betonas.lt/</t>
+        </is>
+      </c>
+      <c r="W23" s="2" t="inlineStr">
+        <is>
+          <t>https://www.suduvos-betonas.lt/kontaktai/</t>
+        </is>
+      </c>
+      <c r="X23" s="2" t="inlineStr">
+        <is>
+          <t>https://www.suduvos-betonas.lt/</t>
+        </is>
+      </c>
+      <c r="Y23" s="2" t="inlineStr"/>
       <c r="Z23" s="2" t="inlineStr">
-        <is>
-          <t>https://www.suduvos-betonas.lt/</t>
-        </is>
-      </c>
-      <c r="AA23" s="2" t="inlineStr">
-        <is>
-          <t>https://www.suduvos-betonas.lt/kontaktai/</t>
-        </is>
-      </c>
-      <c r="AB23" s="2" t="inlineStr"/>
-      <c r="AC23" s="2" t="inlineStr"/>
-      <c r="AD23" s="2" t="inlineStr"/>
-      <c r="AE23" s="2" t="inlineStr">
-        <is>
-          <t>https://www.suduvos-betonas.lt/</t>
-        </is>
-      </c>
-      <c r="AF23" s="2" t="inlineStr"/>
-      <c r="AG23" s="2" t="inlineStr">
         <is>
           <t>2026-06-29</t>
         </is>
@@ -3392,43 +3186,36 @@
           <t>iki 60 m³/h</t>
         </is>
       </c>
-      <c r="S24" s="2" t="inlineStr"/>
+      <c r="S24" s="4" t="inlineStr"/>
       <c r="T24" s="2" t="inlineStr">
         <is>
           <t>Betono mazgo gamintojas Ammann Elba; modelis CBT60SL; maišyklė 1 m³; našumas iki 60 m³/h.</t>
         </is>
       </c>
-      <c r="U24" s="4" t="n">
+      <c r="U24" s="5" t="n">
         <v>0.75</v>
       </c>
-      <c r="V24" s="5" t="n"/>
-      <c r="W24" s="6" t="n"/>
-      <c r="X24" s="5" t="n"/>
-      <c r="Y24" s="5" t="n"/>
+      <c r="V24" s="2" t="inlineStr">
+        <is>
+          <t>https://statkasta.lt/</t>
+        </is>
+      </c>
+      <c r="W24" s="2" t="inlineStr">
+        <is>
+          <t>https://statkasta.lt/kontaktai/</t>
+        </is>
+      </c>
+      <c r="X24" s="2" t="inlineStr">
+        <is>
+          <t>https://statkasta.lt/kontaktai/</t>
+        </is>
+      </c>
+      <c r="Y24" s="2" t="inlineStr">
+        <is>
+          <t>Oficialiame Statkasta kontaktų puslapyje nurodytas adresas Gėlių g. 34, Serdokų k.; koordinatės geokoduotos iki vietovės lygio. Rankiniu būdu papildyta techninė informacija: gamintojas Ammann Elba, modelis CBT60SL, maišyklė 1 m³, našumas iki 60 m³/h.</t>
+        </is>
+      </c>
       <c r="Z24" s="2" t="inlineStr">
-        <is>
-          <t>https://statkasta.lt/</t>
-        </is>
-      </c>
-      <c r="AA24" s="2" t="inlineStr">
-        <is>
-          <t>https://statkasta.lt/kontaktai/</t>
-        </is>
-      </c>
-      <c r="AB24" s="2" t="inlineStr"/>
-      <c r="AC24" s="2" t="inlineStr"/>
-      <c r="AD24" s="2" t="inlineStr"/>
-      <c r="AE24" s="2" t="inlineStr">
-        <is>
-          <t>https://statkasta.lt/kontaktai/</t>
-        </is>
-      </c>
-      <c r="AF24" s="2" t="inlineStr">
-        <is>
-          <t>Oficialiame Statkasta kontaktų puslapyje nurodytas adresas Gėlių g. 34, Serdokų k.; koordinatės geokoduotos iki vietovės lygio. Rankiniu būdu papildyta techninė informacija: gamintojas Ammann Elba, modelis CBT60SL, maišyklė 1 m³, našumas iki 60 m³/h.</t>
-        </is>
-      </c>
-      <c r="AG24" s="2" t="inlineStr">
         <is>
           <t>2026-07-06</t>
         </is>
@@ -3505,43 +3292,36 @@
       <c r="P25" s="2" t="inlineStr"/>
       <c r="Q25" s="2" t="inlineStr"/>
       <c r="R25" s="2" t="inlineStr"/>
-      <c r="S25" s="2" t="inlineStr"/>
+      <c r="S25" s="4" t="inlineStr"/>
       <c r="T25" s="2" t="inlineStr">
         <is>
           <t>Viešuose šaltiniuose minima betono mišinių veikla; tikslų mazgo pavadinimą reikia patikslinti.</t>
         </is>
       </c>
-      <c r="U25" s="4" t="n">
+      <c r="U25" s="5" t="n">
         <v>0.6</v>
       </c>
-      <c r="V25" s="5" t="n"/>
-      <c r="W25" s="6" t="n"/>
-      <c r="X25" s="5" t="n"/>
-      <c r="Y25" s="5" t="n"/>
+      <c r="V25" s="2" t="inlineStr">
+        <is>
+          <t>https://autokausta.lt/</t>
+        </is>
+      </c>
+      <c r="W25" s="2" t="inlineStr">
+        <is>
+          <t>https://www.autokausta.lt/apie-mus/betonas/</t>
+        </is>
+      </c>
+      <c r="X25" s="2" t="inlineStr">
+        <is>
+          <t>https://www.autokausta.lt/apie-mus/betonas/</t>
+        </is>
+      </c>
+      <c r="Y25" s="2" t="inlineStr">
+        <is>
+          <t>Oficialus Autokausta betono puslapis patvirtina betono veiklą ir Marvelės g. 199B kontaktą.</t>
+        </is>
+      </c>
       <c r="Z25" s="2" t="inlineStr">
-        <is>
-          <t>https://autokausta.lt/</t>
-        </is>
-      </c>
-      <c r="AA25" s="2" t="inlineStr">
-        <is>
-          <t>https://www.autokausta.lt/apie-mus/betonas/</t>
-        </is>
-      </c>
-      <c r="AB25" s="2" t="inlineStr"/>
-      <c r="AC25" s="2" t="inlineStr"/>
-      <c r="AD25" s="2" t="inlineStr"/>
-      <c r="AE25" s="2" t="inlineStr">
-        <is>
-          <t>https://www.autokausta.lt/apie-mus/betonas/</t>
-        </is>
-      </c>
-      <c r="AF25" s="2" t="inlineStr">
-        <is>
-          <t>Oficialus Autokausta betono puslapis patvirtina betono veiklą ir Marvelės g. 199B kontaktą.</t>
-        </is>
-      </c>
-      <c r="AG25" s="2" t="inlineStr">
         <is>
           <t>2026-06-29</t>
         </is>
@@ -3626,43 +3406,36 @@
       </c>
       <c r="Q26" s="2" t="inlineStr"/>
       <c r="R26" s="2" t="inlineStr"/>
-      <c r="S26" s="2" t="inlineStr"/>
+      <c r="S26" s="4" t="inlineStr"/>
       <c r="T26" s="2" t="inlineStr">
         <is>
           <t>Viešuose šaltiniuose minima betono mišinių veikla; tikslų mazgo adresą reikia patikslinti.</t>
         </is>
       </c>
-      <c r="U26" s="4" t="n">
+      <c r="U26" s="5" t="n">
         <v>0.65</v>
       </c>
-      <c r="V26" s="5" t="n"/>
-      <c r="W26" s="6" t="n"/>
-      <c r="X26" s="5" t="n"/>
-      <c r="Y26" s="5" t="n"/>
+      <c r="V26" s="2" t="inlineStr">
+        <is>
+          <t>https://www.betonobaze.lt/</t>
+        </is>
+      </c>
+      <c r="W26" s="2" t="inlineStr">
+        <is>
+          <t>https://www.betonobaze.lt/kontaktai</t>
+        </is>
+      </c>
+      <c r="X26" s="2" t="inlineStr">
+        <is>
+          <t>https://www.betonobaze.lt/kontaktai</t>
+        </is>
+      </c>
+      <c r="Y26" s="2" t="inlineStr">
+        <is>
+          <t>Oficialus kontaktų puslapis patvirtina Elektrinės g. 11 adresą ir betono bazės veiklą.</t>
+        </is>
+      </c>
       <c r="Z26" s="2" t="inlineStr">
-        <is>
-          <t>https://www.betonobaze.lt/</t>
-        </is>
-      </c>
-      <c r="AA26" s="2" t="inlineStr">
-        <is>
-          <t>https://www.betonobaze.lt/kontaktai</t>
-        </is>
-      </c>
-      <c r="AB26" s="2" t="inlineStr"/>
-      <c r="AC26" s="2" t="inlineStr"/>
-      <c r="AD26" s="2" t="inlineStr"/>
-      <c r="AE26" s="2" t="inlineStr">
-        <is>
-          <t>https://www.betonobaze.lt/kontaktai</t>
-        </is>
-      </c>
-      <c r="AF26" s="2" t="inlineStr">
-        <is>
-          <t>Oficialus kontaktų puslapis patvirtina Elektrinės g. 11 adresą ir betono bazės veiklą.</t>
-        </is>
-      </c>
-      <c r="AG26" s="2" t="inlineStr">
         <is>
           <t>2026-06-29</t>
         </is>
@@ -3743,43 +3516,36 @@
       </c>
       <c r="Q27" s="2" t="inlineStr"/>
       <c r="R27" s="2" t="inlineStr"/>
-      <c r="S27" s="2" t="inlineStr"/>
+      <c r="S27" s="4" t="inlineStr"/>
       <c r="T27" s="2" t="inlineStr">
         <is>
           <t>Viešai skelbiamas betono mišinių tiekėjas Druskininkų regione.</t>
         </is>
       </c>
-      <c r="U27" s="4" t="n">
+      <c r="U27" s="5" t="n">
         <v>0.7</v>
       </c>
-      <c r="V27" s="5" t="n"/>
-      <c r="W27" s="6" t="n"/>
-      <c r="X27" s="5" t="n"/>
-      <c r="Y27" s="5" t="n"/>
+      <c r="V27" s="2" t="inlineStr">
+        <is>
+          <t>https://transdosa.lt/</t>
+        </is>
+      </c>
+      <c r="W27" s="2" t="inlineStr">
+        <is>
+          <t>https://www.transdosa.lt/kontaktai/</t>
+        </is>
+      </c>
+      <c r="X27" s="2" t="inlineStr">
+        <is>
+          <t>https://www.transdosa.lt/betonas/</t>
+        </is>
+      </c>
+      <c r="Y27" s="2" t="inlineStr">
+        <is>
+          <t>Oficialūs Transdosa kontaktų ir betono puslapiai patvirtina Margų karjero betono gamybą adresu Žvyro g. 2A.</t>
+        </is>
+      </c>
       <c r="Z27" s="2" t="inlineStr">
-        <is>
-          <t>https://transdosa.lt/</t>
-        </is>
-      </c>
-      <c r="AA27" s="2" t="inlineStr">
-        <is>
-          <t>https://www.transdosa.lt/kontaktai/</t>
-        </is>
-      </c>
-      <c r="AB27" s="2" t="inlineStr"/>
-      <c r="AC27" s="2" t="inlineStr"/>
-      <c r="AD27" s="2" t="inlineStr"/>
-      <c r="AE27" s="2" t="inlineStr">
-        <is>
-          <t>https://www.transdosa.lt/betonas/</t>
-        </is>
-      </c>
-      <c r="AF27" s="2" t="inlineStr">
-        <is>
-          <t>Oficialūs Transdosa kontaktų ir betono puslapiai patvirtina Margų karjero betono gamybą adresu Žvyro g. 2A.</t>
-        </is>
-      </c>
-      <c r="AG27" s="2" t="inlineStr">
         <is>
           <t>2026-06-29</t>
         </is>
@@ -3860,43 +3626,36 @@
       </c>
       <c r="Q28" s="2" t="inlineStr"/>
       <c r="R28" s="2" t="inlineStr"/>
-      <c r="S28" s="2" t="inlineStr"/>
+      <c r="S28" s="4" t="inlineStr"/>
       <c r="T28" s="2" t="inlineStr">
         <is>
           <t>Viešai skelbiama gelžbetonio ir betono gaminių gamyba Šiauliuose.</t>
         </is>
       </c>
-      <c r="U28" s="4" t="n">
+      <c r="U28" s="5" t="n">
         <v>0.82</v>
       </c>
-      <c r="V28" s="5" t="n"/>
-      <c r="W28" s="6" t="n"/>
-      <c r="X28" s="5" t="n"/>
-      <c r="Y28" s="5" t="n"/>
+      <c r="V28" s="2" t="inlineStr">
+        <is>
+          <t>https://sodbeta.lt/</t>
+        </is>
+      </c>
+      <c r="W28" s="2" t="inlineStr">
+        <is>
+          <t>https://sodbeta.lt/</t>
+        </is>
+      </c>
+      <c r="X28" s="2" t="inlineStr">
+        <is>
+          <t>https://sodbeta.lt/betonas/betono-misiniai/</t>
+        </is>
+      </c>
+      <c r="Y28" s="2" t="inlineStr">
+        <is>
+          <t>Oficiali Sodbeta svetainė patvirtina Sodo g. 20 adresą ir betono mišinių puslapį.</t>
+        </is>
+      </c>
       <c r="Z28" s="2" t="inlineStr">
-        <is>
-          <t>https://sodbeta.lt/</t>
-        </is>
-      </c>
-      <c r="AA28" s="2" t="inlineStr">
-        <is>
-          <t>https://sodbeta.lt/</t>
-        </is>
-      </c>
-      <c r="AB28" s="2" t="inlineStr"/>
-      <c r="AC28" s="2" t="inlineStr"/>
-      <c r="AD28" s="2" t="inlineStr"/>
-      <c r="AE28" s="2" t="inlineStr">
-        <is>
-          <t>https://sodbeta.lt/betonas/betono-misiniai/</t>
-        </is>
-      </c>
-      <c r="AF28" s="2" t="inlineStr">
-        <is>
-          <t>Oficiali Sodbeta svetainė patvirtina Sodo g. 20 adresą ir betono mišinių puslapį.</t>
-        </is>
-      </c>
-      <c r="AG28" s="2" t="inlineStr">
         <is>
           <t>2026-06-30</t>
         </is>
@@ -3981,43 +3740,36 @@
       </c>
       <c r="Q29" s="2" t="inlineStr"/>
       <c r="R29" s="2" t="inlineStr"/>
-      <c r="S29" s="2" t="inlineStr"/>
+      <c r="S29" s="4" t="inlineStr"/>
       <c r="T29" s="2" t="inlineStr">
         <is>
           <t>Registrų centro/VDA atviruose duomenyse pagrindinė veikla nurodyta kaip prekinio betono mišinio gamyba (EVRK 23.63).</t>
         </is>
       </c>
-      <c r="U29" s="4" t="n">
+      <c r="U29" s="5" t="n">
         <v>0.85</v>
       </c>
-      <c r="V29" s="5" t="n"/>
-      <c r="W29" s="6" t="n"/>
-      <c r="X29" s="5" t="n"/>
-      <c r="Y29" s="5" t="n"/>
+      <c r="V29" s="2" t="inlineStr">
+        <is>
+          <t>https://alytausgelzbetonis.lt/</t>
+        </is>
+      </c>
+      <c r="W29" s="2" t="inlineStr">
+        <is>
+          <t>https://alytausgelzbetonis.lt/kontaktai/</t>
+        </is>
+      </c>
+      <c r="X29" s="2" t="inlineStr">
+        <is>
+          <t>https://alytausgelzbetonis.lt/kontaktai/</t>
+        </is>
+      </c>
+      <c r="Y29" s="2" t="inlineStr">
+        <is>
+          <t>Patikslinta pagal oficialų kontaktų puslapį.</t>
+        </is>
+      </c>
       <c r="Z29" s="2" t="inlineStr">
-        <is>
-          <t>https://alytausgelzbetonis.lt/</t>
-        </is>
-      </c>
-      <c r="AA29" s="2" t="inlineStr">
-        <is>
-          <t>https://alytausgelzbetonis.lt/kontaktai/</t>
-        </is>
-      </c>
-      <c r="AB29" s="2" t="inlineStr"/>
-      <c r="AC29" s="2" t="inlineStr"/>
-      <c r="AD29" s="2" t="inlineStr"/>
-      <c r="AE29" s="2" t="inlineStr">
-        <is>
-          <t>https://alytausgelzbetonis.lt/kontaktai/</t>
-        </is>
-      </c>
-      <c r="AF29" s="2" t="inlineStr">
-        <is>
-          <t>Patikslinta pagal oficialų kontaktų puslapį.</t>
-        </is>
-      </c>
-      <c r="AG29" s="2" t="inlineStr">
         <is>
           <t>2026-06-30</t>
         </is>
@@ -4098,43 +3850,36 @@
       </c>
       <c r="Q30" s="2" t="inlineStr"/>
       <c r="R30" s="2" t="inlineStr"/>
-      <c r="S30" s="2" t="inlineStr"/>
+      <c r="S30" s="4" t="inlineStr"/>
       <c r="T30" s="2" t="inlineStr">
         <is>
           <t>Viešai skelbiamas betono mišinių tiekėjas Marijampolėje.</t>
         </is>
       </c>
-      <c r="U30" s="4" t="n">
+      <c r="U30" s="5" t="n">
         <v>0.75</v>
       </c>
-      <c r="V30" s="5" t="n"/>
-      <c r="W30" s="6" t="n"/>
-      <c r="X30" s="5" t="n"/>
-      <c r="Y30" s="5" t="n"/>
+      <c r="V30" s="2" t="inlineStr">
+        <is>
+          <t>https://gernora.lt/</t>
+        </is>
+      </c>
+      <c r="W30" s="2" t="inlineStr">
+        <is>
+          <t>https://gernora.lt/kontaktai/</t>
+        </is>
+      </c>
+      <c r="X30" s="2" t="inlineStr">
+        <is>
+          <t>https://gernora.lt/kontaktai/</t>
+        </is>
+      </c>
+      <c r="Y30" s="2" t="inlineStr">
+        <is>
+          <t>Koordinatės patikslintos pagal oficialaus Gernora kontaktų puslapio Google Maps nuorodą.</t>
+        </is>
+      </c>
       <c r="Z30" s="2" t="inlineStr">
-        <is>
-          <t>https://gernora.lt/</t>
-        </is>
-      </c>
-      <c r="AA30" s="2" t="inlineStr">
-        <is>
-          <t>https://gernora.lt/kontaktai/</t>
-        </is>
-      </c>
-      <c r="AB30" s="2" t="inlineStr"/>
-      <c r="AC30" s="2" t="inlineStr"/>
-      <c r="AD30" s="2" t="inlineStr"/>
-      <c r="AE30" s="2" t="inlineStr">
-        <is>
-          <t>https://gernora.lt/kontaktai/</t>
-        </is>
-      </c>
-      <c r="AF30" s="2" t="inlineStr">
-        <is>
-          <t>Koordinatės patikslintos pagal oficialaus Gernora kontaktų puslapio Google Maps nuorodą.</t>
-        </is>
-      </c>
-      <c r="AG30" s="2" t="inlineStr">
         <is>
           <t>2026-06-30</t>
         </is>
@@ -4215,39 +3960,32 @@
       </c>
       <c r="Q31" s="2" t="inlineStr"/>
       <c r="R31" s="2" t="inlineStr"/>
-      <c r="S31" s="2" t="inlineStr"/>
+      <c r="S31" s="4" t="inlineStr"/>
       <c r="T31" s="2" t="inlineStr">
         <is>
           <t>Viešame kataloge nurodomi betonas, cemento gaminiai, betono siurblys ir pamatų blokai Kretingoje.</t>
         </is>
       </c>
-      <c r="U31" s="4" t="n">
+      <c r="U31" s="5" t="n">
         <v>0.78</v>
       </c>
-      <c r="V31" s="5" t="n"/>
-      <c r="W31" s="6" t="n"/>
-      <c r="X31" s="5" t="n"/>
-      <c r="Y31" s="5" t="n"/>
-      <c r="Z31" s="2" t="inlineStr"/>
-      <c r="AA31" s="2" t="inlineStr">
+      <c r="V31" s="2" t="inlineStr"/>
+      <c r="W31" s="2" t="inlineStr">
         <is>
           <t>https://www.1551.lt/re-betono-konstrukcijos-uab-betonas-cementas-betono-siurblys-pamatu-blokai-kretingoje-104253/</t>
         </is>
       </c>
-      <c r="AB31" s="2" t="inlineStr"/>
-      <c r="AC31" s="2" t="inlineStr"/>
-      <c r="AD31" s="2" t="inlineStr"/>
-      <c r="AE31" s="2" t="inlineStr">
+      <c r="X31" s="2" t="inlineStr">
         <is>
           <t>https://www.1551.lt/re-betono-konstrukcijos-uab-betonas-cementas-betono-siurblys-pamatu-blokai-kretingoje-104253/</t>
         </is>
       </c>
-      <c r="AF31" s="2" t="inlineStr">
+      <c r="Y31" s="2" t="inlineStr">
         <is>
           <t>Katalogo šaltinis, reikia patikslinti gamybos apimtį.</t>
         </is>
       </c>
-      <c r="AG31" s="2" t="inlineStr">
+      <c r="Z31" s="2" t="inlineStr">
         <is>
           <t>2026-06-30</t>
         </is>
@@ -4328,43 +4066,36 @@
       </c>
       <c r="Q32" s="2" t="inlineStr"/>
       <c r="R32" s="2" t="inlineStr"/>
-      <c r="S32" s="2" t="inlineStr"/>
+      <c r="S32" s="4" t="inlineStr"/>
       <c r="T32" s="2" t="inlineStr">
         <is>
           <t>Viešai skelbiama betono gaminių ir statybinių konstrukcijų veikla Šilalės rajone.</t>
         </is>
       </c>
-      <c r="U32" s="4" t="n">
+      <c r="U32" s="5" t="n">
         <v>0.72</v>
       </c>
-      <c r="V32" s="5" t="n"/>
-      <c r="W32" s="6" t="n"/>
-      <c r="X32" s="5" t="n"/>
-      <c r="Y32" s="5" t="n"/>
+      <c r="V32" s="2" t="inlineStr">
+        <is>
+          <t>https://www.silalesstatyba.lt/</t>
+        </is>
+      </c>
+      <c r="W32" s="2" t="inlineStr">
+        <is>
+          <t>https://www.silalesstatyba.lt/</t>
+        </is>
+      </c>
+      <c r="X32" s="2" t="inlineStr">
+        <is>
+          <t>https://www.silalesstatyba.lt/</t>
+        </is>
+      </c>
+      <c r="Y32" s="2" t="inlineStr">
+        <is>
+          <t>Reikia patikslinti tikslų gaminių asortimentą.</t>
+        </is>
+      </c>
       <c r="Z32" s="2" t="inlineStr">
-        <is>
-          <t>https://www.silalesstatyba.lt/</t>
-        </is>
-      </c>
-      <c r="AA32" s="2" t="inlineStr">
-        <is>
-          <t>https://www.silalesstatyba.lt/</t>
-        </is>
-      </c>
-      <c r="AB32" s="2" t="inlineStr"/>
-      <c r="AC32" s="2" t="inlineStr"/>
-      <c r="AD32" s="2" t="inlineStr"/>
-      <c r="AE32" s="2" t="inlineStr">
-        <is>
-          <t>https://www.silalesstatyba.lt/</t>
-        </is>
-      </c>
-      <c r="AF32" s="2" t="inlineStr">
-        <is>
-          <t>Reikia patikslinti tikslų gaminių asortimentą.</t>
-        </is>
-      </c>
-      <c r="AG32" s="2" t="inlineStr">
         <is>
           <t>2026-06-30</t>
         </is>
@@ -4445,39 +4176,32 @@
       </c>
       <c r="Q33" s="2" t="inlineStr"/>
       <c r="R33" s="2" t="inlineStr"/>
-      <c r="S33" s="2" t="inlineStr"/>
+      <c r="S33" s="4" t="inlineStr"/>
       <c r="T33" s="2" t="inlineStr">
         <is>
           <t>Viešame įmonių kataloge nurodomas gelžbetonio gaminių profilis Panevėžyje.</t>
         </is>
       </c>
-      <c r="U33" s="4" t="n">
+      <c r="U33" s="5" t="n">
         <v>0.78</v>
       </c>
-      <c r="V33" s="5" t="n"/>
-      <c r="W33" s="6" t="n"/>
-      <c r="X33" s="5" t="n"/>
-      <c r="Y33" s="5" t="n"/>
-      <c r="Z33" s="2" t="inlineStr"/>
-      <c r="AA33" s="2" t="inlineStr">
+      <c r="V33" s="2" t="inlineStr"/>
+      <c r="W33" s="2" t="inlineStr">
         <is>
           <t>https://www.spec.lt/imone/panevezio-gelzbetonis-uab</t>
         </is>
       </c>
-      <c r="AB33" s="2" t="inlineStr"/>
-      <c r="AC33" s="2" t="inlineStr"/>
-      <c r="AD33" s="2" t="inlineStr"/>
-      <c r="AE33" s="2" t="inlineStr">
+      <c r="X33" s="2" t="inlineStr">
         <is>
           <t>https://www.spec.lt/imone/panevezio-gelzbetonis-uab</t>
         </is>
       </c>
-      <c r="AF33" s="2" t="inlineStr">
+      <c r="Y33" s="2" t="inlineStr">
         <is>
           <t>Reikia patikrinti veiklos aktyvumą ir produkcijos apimtį.</t>
         </is>
       </c>
-      <c r="AG33" s="2" t="inlineStr">
+      <c r="Z33" s="2" t="inlineStr">
         <is>
           <t>2026-06-30</t>
         </is>
@@ -4558,43 +4282,36 @@
       </c>
       <c r="Q34" s="2" t="inlineStr"/>
       <c r="R34" s="2" t="inlineStr"/>
-      <c r="S34" s="2" t="inlineStr"/>
+      <c r="S34" s="4" t="inlineStr"/>
       <c r="T34" s="2" t="inlineStr">
         <is>
           <t>Viešai skelbiami pamatų ir kiti betono gaminiai Telšių rajone.</t>
         </is>
       </c>
-      <c r="U34" s="4" t="n">
+      <c r="U34" s="5" t="n">
         <v>0.72</v>
       </c>
-      <c r="V34" s="5" t="n"/>
-      <c r="W34" s="6" t="n"/>
-      <c r="X34" s="5" t="n"/>
-      <c r="Y34" s="5" t="n"/>
+      <c r="V34" s="2" t="inlineStr">
+        <is>
+          <t>https://pamatas.lt/</t>
+        </is>
+      </c>
+      <c r="W34" s="2" t="inlineStr">
+        <is>
+          <t>https://pamatas.lt/</t>
+        </is>
+      </c>
+      <c r="X34" s="2" t="inlineStr">
+        <is>
+          <t>https://pamatas.lt/</t>
+        </is>
+      </c>
+      <c r="Y34" s="2" t="inlineStr">
+        <is>
+          <t>Adresas patikslintas pagal lietuvišką įmonės puslapį; koordinatės nustatytos Lietuvos geolokatoriumi.</t>
+        </is>
+      </c>
       <c r="Z34" s="2" t="inlineStr">
-        <is>
-          <t>https://pamatas.lt/</t>
-        </is>
-      </c>
-      <c r="AA34" s="2" t="inlineStr">
-        <is>
-          <t>https://pamatas.lt/</t>
-        </is>
-      </c>
-      <c r="AB34" s="2" t="inlineStr"/>
-      <c r="AC34" s="2" t="inlineStr"/>
-      <c r="AD34" s="2" t="inlineStr"/>
-      <c r="AE34" s="2" t="inlineStr">
-        <is>
-          <t>https://pamatas.lt/</t>
-        </is>
-      </c>
-      <c r="AF34" s="2" t="inlineStr">
-        <is>
-          <t>Adresas patikslintas pagal lietuvišką įmonės puslapį; koordinatės nustatytos Lietuvos geolokatoriumi.</t>
-        </is>
-      </c>
-      <c r="AG34" s="2" t="inlineStr">
         <is>
           <t>2026-06-30</t>
         </is>
@@ -4675,43 +4392,36 @@
       </c>
       <c r="Q35" s="2" t="inlineStr"/>
       <c r="R35" s="2" t="inlineStr"/>
-      <c r="S35" s="2" t="inlineStr"/>
+      <c r="S35" s="4" t="inlineStr"/>
       <c r="T35" s="2" t="inlineStr">
         <is>
           <t>Viešai skelbiamas HAUS blokelių ir betono gaminių gamintojas.</t>
         </is>
       </c>
-      <c r="U35" s="4" t="n">
+      <c r="U35" s="5" t="n">
         <v>0.8</v>
       </c>
-      <c r="V35" s="5" t="n"/>
-      <c r="W35" s="6" t="n"/>
-      <c r="X35" s="5" t="n"/>
-      <c r="Y35" s="5" t="n"/>
+      <c r="V35" s="2" t="inlineStr">
+        <is>
+          <t>https://www.vbg.lt/</t>
+        </is>
+      </c>
+      <c r="W35" s="2" t="inlineStr">
+        <is>
+          <t>https://www.vbg.lt/</t>
+        </is>
+      </c>
+      <c r="X35" s="2" t="inlineStr">
+        <is>
+          <t>https://www.vbg.lt/</t>
+        </is>
+      </c>
+      <c r="Y35" s="2" t="inlineStr">
+        <is>
+          <t>Žemėlapyje naudotas viešai skelbiamas įmonės adresas; gamybos vietą reikia patikslinti.</t>
+        </is>
+      </c>
       <c r="Z35" s="2" t="inlineStr">
-        <is>
-          <t>https://www.vbg.lt/</t>
-        </is>
-      </c>
-      <c r="AA35" s="2" t="inlineStr">
-        <is>
-          <t>https://www.vbg.lt/</t>
-        </is>
-      </c>
-      <c r="AB35" s="2" t="inlineStr"/>
-      <c r="AC35" s="2" t="inlineStr"/>
-      <c r="AD35" s="2" t="inlineStr"/>
-      <c r="AE35" s="2" t="inlineStr">
-        <is>
-          <t>https://www.vbg.lt/</t>
-        </is>
-      </c>
-      <c r="AF35" s="2" t="inlineStr">
-        <is>
-          <t>Žemėlapyje naudotas viešai skelbiamas įmonės adresas; gamybos vietą reikia patikslinti.</t>
-        </is>
-      </c>
-      <c r="AG35" s="2" t="inlineStr">
         <is>
           <t>2026-06-30</t>
         </is>
@@ -4792,43 +4502,36 @@
       </c>
       <c r="Q36" s="2" t="inlineStr"/>
       <c r="R36" s="2" t="inlineStr"/>
-      <c r="S36" s="2" t="inlineStr"/>
+      <c r="S36" s="4" t="inlineStr"/>
       <c r="T36" s="2" t="inlineStr">
         <is>
           <t>Viešai skelbiama betono mišinių veikla Klaipėdos rajone.</t>
         </is>
       </c>
-      <c r="U36" s="4" t="n">
+      <c r="U36" s="5" t="n">
         <v>0.75</v>
       </c>
-      <c r="V36" s="5" t="n"/>
-      <c r="W36" s="6" t="n"/>
-      <c r="X36" s="5" t="n"/>
-      <c r="Y36" s="5" t="n"/>
+      <c r="V36" s="2" t="inlineStr">
+        <is>
+          <t>https://pamariogrupe.lt/</t>
+        </is>
+      </c>
+      <c r="W36" s="2" t="inlineStr">
+        <is>
+          <t>https://pamariogrupe.lt/</t>
+        </is>
+      </c>
+      <c r="X36" s="2" t="inlineStr">
+        <is>
+          <t>https://pamariogrupe.lt/</t>
+        </is>
+      </c>
+      <c r="Y36" s="2" t="inlineStr">
+        <is>
+          <t>Reikia patikslinti našumą ir gamybos režimą.</t>
+        </is>
+      </c>
       <c r="Z36" s="2" t="inlineStr">
-        <is>
-          <t>https://pamariogrupe.lt/</t>
-        </is>
-      </c>
-      <c r="AA36" s="2" t="inlineStr">
-        <is>
-          <t>https://pamariogrupe.lt/</t>
-        </is>
-      </c>
-      <c r="AB36" s="2" t="inlineStr"/>
-      <c r="AC36" s="2" t="inlineStr"/>
-      <c r="AD36" s="2" t="inlineStr"/>
-      <c r="AE36" s="2" t="inlineStr">
-        <is>
-          <t>https://pamariogrupe.lt/</t>
-        </is>
-      </c>
-      <c r="AF36" s="2" t="inlineStr">
-        <is>
-          <t>Reikia patikslinti našumą ir gamybos režimą.</t>
-        </is>
-      </c>
-      <c r="AG36" s="2" t="inlineStr">
         <is>
           <t>2026-06-30</t>
         </is>
@@ -4909,43 +4612,36 @@
       </c>
       <c r="Q37" s="2" t="inlineStr"/>
       <c r="R37" s="2" t="inlineStr"/>
-      <c r="S37" s="2" t="inlineStr"/>
+      <c r="S37" s="4" t="inlineStr"/>
       <c r="T37" s="2" t="inlineStr">
         <is>
           <t>Viešai skelbiama betono gaminių veikla Klaipėdoje.</t>
         </is>
       </c>
-      <c r="U37" s="4" t="n">
+      <c r="U37" s="5" t="n">
         <v>0.65</v>
       </c>
-      <c r="V37" s="5" t="n"/>
-      <c r="W37" s="6" t="n"/>
-      <c r="X37" s="5" t="n"/>
-      <c r="Y37" s="5" t="n"/>
+      <c r="V37" s="2" t="inlineStr">
+        <is>
+          <t>https://betonozona.lt/</t>
+        </is>
+      </c>
+      <c r="W37" s="2" t="inlineStr">
+        <is>
+          <t>https://betonozona.lt/</t>
+        </is>
+      </c>
+      <c r="X37" s="2" t="inlineStr">
+        <is>
+          <t>https://betonozona.lt/</t>
+        </is>
+      </c>
+      <c r="Y37" s="2" t="inlineStr">
+        <is>
+          <t>Patikrinti, ar įmonė pati gamina, ar tik prekiauja betono gaminiais.</t>
+        </is>
+      </c>
       <c r="Z37" s="2" t="inlineStr">
-        <is>
-          <t>https://betonozona.lt/</t>
-        </is>
-      </c>
-      <c r="AA37" s="2" t="inlineStr">
-        <is>
-          <t>https://betonozona.lt/</t>
-        </is>
-      </c>
-      <c r="AB37" s="2" t="inlineStr"/>
-      <c r="AC37" s="2" t="inlineStr"/>
-      <c r="AD37" s="2" t="inlineStr"/>
-      <c r="AE37" s="2" t="inlineStr">
-        <is>
-          <t>https://betonozona.lt/</t>
-        </is>
-      </c>
-      <c r="AF37" s="2" t="inlineStr">
-        <is>
-          <t>Patikrinti, ar įmonė pati gamina, ar tik prekiauja betono gaminiais.</t>
-        </is>
-      </c>
-      <c r="AG37" s="2" t="inlineStr">
         <is>
           <t>2026-06-30</t>
         </is>
@@ -5030,43 +4726,36 @@
       </c>
       <c r="Q38" s="2" t="inlineStr"/>
       <c r="R38" s="2" t="inlineStr"/>
-      <c r="S38" s="2" t="inlineStr"/>
+      <c r="S38" s="4" t="inlineStr"/>
       <c r="T38" s="2" t="inlineStr">
         <is>
           <t>Viešai skelbiama betono mišinių gamyba Panevėžyje.</t>
         </is>
       </c>
-      <c r="U38" s="4" t="n">
+      <c r="U38" s="5" t="n">
         <v>0.78</v>
       </c>
-      <c r="V38" s="5" t="n"/>
-      <c r="W38" s="6" t="n"/>
-      <c r="X38" s="5" t="n"/>
-      <c r="Y38" s="5" t="n"/>
+      <c r="V38" s="2" t="inlineStr">
+        <is>
+          <t>https://topbeton.lt/</t>
+        </is>
+      </c>
+      <c r="W38" s="2" t="inlineStr">
+        <is>
+          <t>https://www.topbeton.lt/kontaktai/</t>
+        </is>
+      </c>
+      <c r="X38" s="2" t="inlineStr">
+        <is>
+          <t>https://www.topbeton.lt/kontaktai/</t>
+        </is>
+      </c>
+      <c r="Y38" s="2" t="inlineStr">
+        <is>
+          <t>Oficialus kontaktų puslapis patvirtina Beržų g. 5C adresą.</t>
+        </is>
+      </c>
       <c r="Z38" s="2" t="inlineStr">
-        <is>
-          <t>https://topbeton.lt/</t>
-        </is>
-      </c>
-      <c r="AA38" s="2" t="inlineStr">
-        <is>
-          <t>https://www.topbeton.lt/kontaktai/</t>
-        </is>
-      </c>
-      <c r="AB38" s="2" t="inlineStr"/>
-      <c r="AC38" s="2" t="inlineStr"/>
-      <c r="AD38" s="2" t="inlineStr"/>
-      <c r="AE38" s="2" t="inlineStr">
-        <is>
-          <t>https://www.topbeton.lt/kontaktai/</t>
-        </is>
-      </c>
-      <c r="AF38" s="2" t="inlineStr">
-        <is>
-          <t>Oficialus kontaktų puslapis patvirtina Beržų g. 5C adresą.</t>
-        </is>
-      </c>
-      <c r="AG38" s="2" t="inlineStr">
         <is>
           <t>2026-06-30</t>
         </is>
@@ -5147,43 +4836,36 @@
       </c>
       <c r="Q39" s="2" t="inlineStr"/>
       <c r="R39" s="2" t="inlineStr"/>
-      <c r="S39" s="2" t="inlineStr"/>
+      <c r="S39" s="4" t="inlineStr"/>
       <c r="T39" s="2" t="inlineStr">
         <is>
           <t>Viešai skelbiama gelžbetonio gaminių gamyba Panevėžyje.</t>
         </is>
       </c>
-      <c r="U39" s="4" t="n">
+      <c r="U39" s="5" t="n">
         <v>0.72</v>
       </c>
-      <c r="V39" s="5" t="n"/>
-      <c r="W39" s="6" t="n"/>
-      <c r="X39" s="5" t="n"/>
-      <c r="Y39" s="5" t="n"/>
+      <c r="V39" s="2" t="inlineStr">
+        <is>
+          <t>https://gelzbetoniogamyba.lt/</t>
+        </is>
+      </c>
+      <c r="W39" s="2" t="inlineStr">
+        <is>
+          <t>https://gelzbetoniogamyba.lt/</t>
+        </is>
+      </c>
+      <c r="X39" s="2" t="inlineStr">
+        <is>
+          <t>https://gelzbetoniogamyba.lt/</t>
+        </is>
+      </c>
+      <c r="Y39" s="2" t="inlineStr">
+        <is>
+          <t>Reikia patikslinti ryšį su kitomis S. Kerbedžio g. 52 įmonėmis.</t>
+        </is>
+      </c>
       <c r="Z39" s="2" t="inlineStr">
-        <is>
-          <t>https://gelzbetoniogamyba.lt/</t>
-        </is>
-      </c>
-      <c r="AA39" s="2" t="inlineStr">
-        <is>
-          <t>https://gelzbetoniogamyba.lt/</t>
-        </is>
-      </c>
-      <c r="AB39" s="2" t="inlineStr"/>
-      <c r="AC39" s="2" t="inlineStr"/>
-      <c r="AD39" s="2" t="inlineStr"/>
-      <c r="AE39" s="2" t="inlineStr">
-        <is>
-          <t>https://gelzbetoniogamyba.lt/</t>
-        </is>
-      </c>
-      <c r="AF39" s="2" t="inlineStr">
-        <is>
-          <t>Reikia patikslinti ryšį su kitomis S. Kerbedžio g. 52 įmonėmis.</t>
-        </is>
-      </c>
-      <c r="AG39" s="2" t="inlineStr">
         <is>
           <t>2026-06-30</t>
         </is>
@@ -5264,43 +4946,36 @@
       </c>
       <c r="Q40" s="2" t="inlineStr"/>
       <c r="R40" s="2" t="inlineStr"/>
-      <c r="S40" s="2" t="inlineStr"/>
+      <c r="S40" s="4" t="inlineStr"/>
       <c r="T40" s="2" t="inlineStr">
         <is>
           <t>Viešai skelbiama betono mišinių veikla Pakruojyje.</t>
         </is>
       </c>
-      <c r="U40" s="4" t="n">
+      <c r="U40" s="5" t="n">
         <v>0.72</v>
       </c>
-      <c r="V40" s="5" t="n"/>
-      <c r="W40" s="6" t="n"/>
-      <c r="X40" s="5" t="n"/>
-      <c r="Y40" s="5" t="n"/>
+      <c r="V40" s="2" t="inlineStr">
+        <is>
+          <t>https://inroma.lt/</t>
+        </is>
+      </c>
+      <c r="W40" s="2" t="inlineStr">
+        <is>
+          <t>https://inroma.lt/</t>
+        </is>
+      </c>
+      <c r="X40" s="2" t="inlineStr">
+        <is>
+          <t>https://inroma.lt/</t>
+        </is>
+      </c>
+      <c r="Y40" s="2" t="inlineStr">
+        <is>
+          <t>Reikia patikslinti našumą.</t>
+        </is>
+      </c>
       <c r="Z40" s="2" t="inlineStr">
-        <is>
-          <t>https://inroma.lt/</t>
-        </is>
-      </c>
-      <c r="AA40" s="2" t="inlineStr">
-        <is>
-          <t>https://inroma.lt/</t>
-        </is>
-      </c>
-      <c r="AB40" s="2" t="inlineStr"/>
-      <c r="AC40" s="2" t="inlineStr"/>
-      <c r="AD40" s="2" t="inlineStr"/>
-      <c r="AE40" s="2" t="inlineStr">
-        <is>
-          <t>https://inroma.lt/</t>
-        </is>
-      </c>
-      <c r="AF40" s="2" t="inlineStr">
-        <is>
-          <t>Reikia patikslinti našumą.</t>
-        </is>
-      </c>
-      <c r="AG40" s="2" t="inlineStr">
         <is>
           <t>2026-06-30</t>
         </is>
@@ -5381,39 +5056,32 @@
       </c>
       <c r="Q41" s="2" t="inlineStr"/>
       <c r="R41" s="2" t="inlineStr"/>
-      <c r="S41" s="2" t="inlineStr"/>
+      <c r="S41" s="4" t="inlineStr"/>
       <c r="T41" s="2" t="inlineStr">
         <is>
           <t>Viešame kataloge nurodoma prekinio betono gamyba ir prekyba Vilniuje.</t>
         </is>
       </c>
-      <c r="U41" s="4" t="n">
+      <c r="U41" s="5" t="n">
         <v>0.7</v>
       </c>
-      <c r="V41" s="5" t="n"/>
-      <c r="W41" s="6" t="n"/>
-      <c r="X41" s="5" t="n"/>
-      <c r="Y41" s="5" t="n"/>
-      <c r="Z41" s="2" t="inlineStr"/>
-      <c r="AA41" s="2" t="inlineStr">
+      <c r="V41" s="2" t="inlineStr"/>
+      <c r="W41" s="2" t="inlineStr">
         <is>
           <t>https://www.1551.lt/seldra-uab-prekinio-betono-gamyba-ir-prekyba-vilniuje-219193/</t>
         </is>
       </c>
-      <c r="AB41" s="2" t="inlineStr"/>
-      <c r="AC41" s="2" t="inlineStr"/>
-      <c r="AD41" s="2" t="inlineStr"/>
-      <c r="AE41" s="2" t="inlineStr">
+      <c r="X41" s="2" t="inlineStr">
         <is>
           <t>https://www.1551.lt/seldra-uab-prekinio-betono-gamyba-ir-prekyba-vilniuje-219193/</t>
         </is>
       </c>
-      <c r="AF41" s="2" t="inlineStr">
+      <c r="Y41" s="2" t="inlineStr">
         <is>
           <t>Koordinatė apytikslė pagal adresą; reikia patikslinti gamybos tašką.</t>
         </is>
       </c>
-      <c r="AG41" s="2" t="inlineStr">
+      <c r="Z41" s="2" t="inlineStr">
         <is>
           <t>2026-06-30</t>
         </is>
@@ -5498,43 +5166,36 @@
       </c>
       <c r="Q42" s="2" t="inlineStr"/>
       <c r="R42" s="2" t="inlineStr"/>
-      <c r="S42" s="2" t="inlineStr"/>
+      <c r="S42" s="4" t="inlineStr"/>
       <c r="T42" s="2" t="inlineStr">
         <is>
           <t>Viešai skelbiama betono mišinių veikla Utenoje.</t>
         </is>
       </c>
-      <c r="U42" s="4" t="n">
+      <c r="U42" s="5" t="n">
         <v>0.78</v>
       </c>
-      <c r="V42" s="5" t="n"/>
-      <c r="W42" s="6" t="n"/>
-      <c r="X42" s="5" t="n"/>
-      <c r="Y42" s="5" t="n"/>
+      <c r="V42" s="2" t="inlineStr">
+        <is>
+          <t>https://utenosbetonas.lt/</t>
+        </is>
+      </c>
+      <c r="W42" s="2" t="inlineStr">
+        <is>
+          <t>https://www.utenosbetonas.lt/kontaktai/</t>
+        </is>
+      </c>
+      <c r="X42" s="2" t="inlineStr">
+        <is>
+          <t>https://www.utenosbetonas.lt/kontaktai/</t>
+        </is>
+      </c>
+      <c r="Y42" s="2" t="inlineStr">
+        <is>
+          <t>Oficialus kontaktų puslapis patvirtina Metalo g. 9B adresą.</t>
+        </is>
+      </c>
       <c r="Z42" s="2" t="inlineStr">
-        <is>
-          <t>https://utenosbetonas.lt/</t>
-        </is>
-      </c>
-      <c r="AA42" s="2" t="inlineStr">
-        <is>
-          <t>https://www.utenosbetonas.lt/kontaktai/</t>
-        </is>
-      </c>
-      <c r="AB42" s="2" t="inlineStr"/>
-      <c r="AC42" s="2" t="inlineStr"/>
-      <c r="AD42" s="2" t="inlineStr"/>
-      <c r="AE42" s="2" t="inlineStr">
-        <is>
-          <t>https://www.utenosbetonas.lt/kontaktai/</t>
-        </is>
-      </c>
-      <c r="AF42" s="2" t="inlineStr">
-        <is>
-          <t>Oficialus kontaktų puslapis patvirtina Metalo g. 9B adresą.</t>
-        </is>
-      </c>
-      <c r="AG42" s="2" t="inlineStr">
         <is>
           <t>2026-06-30</t>
         </is>
@@ -5619,43 +5280,36 @@
       </c>
       <c r="Q43" s="2" t="inlineStr"/>
       <c r="R43" s="2" t="inlineStr"/>
-      <c r="S43" s="2" t="inlineStr"/>
+      <c r="S43" s="4" t="inlineStr"/>
       <c r="T43" s="2" t="inlineStr">
         <is>
           <t>Viešai skelbiama prekinio betono gamyba Jonavoje.</t>
         </is>
       </c>
-      <c r="U43" s="4" t="n">
+      <c r="U43" s="5" t="n">
         <v>0.78</v>
       </c>
-      <c r="V43" s="5" t="n"/>
-      <c r="W43" s="6" t="n"/>
-      <c r="X43" s="5" t="n"/>
-      <c r="Y43" s="5" t="n"/>
+      <c r="V43" s="2" t="inlineStr">
+        <is>
+          <t>https://sbetonas.lt/</t>
+        </is>
+      </c>
+      <c r="W43" s="2" t="inlineStr">
+        <is>
+          <t>https://sbetonas.lt/</t>
+        </is>
+      </c>
+      <c r="X43" s="2" t="inlineStr">
+        <is>
+          <t>https://sbetonas.lt/</t>
+        </is>
+      </c>
+      <c r="Y43" s="2" t="inlineStr">
+        <is>
+          <t>Papildomai rasta pagal prekinio betono požymį.</t>
+        </is>
+      </c>
       <c r="Z43" s="2" t="inlineStr">
-        <is>
-          <t>https://sbetonas.lt/</t>
-        </is>
-      </c>
-      <c r="AA43" s="2" t="inlineStr">
-        <is>
-          <t>https://sbetonas.lt/</t>
-        </is>
-      </c>
-      <c r="AB43" s="2" t="inlineStr"/>
-      <c r="AC43" s="2" t="inlineStr"/>
-      <c r="AD43" s="2" t="inlineStr"/>
-      <c r="AE43" s="2" t="inlineStr">
-        <is>
-          <t>https://sbetonas.lt/</t>
-        </is>
-      </c>
-      <c r="AF43" s="2" t="inlineStr">
-        <is>
-          <t>Papildomai rasta pagal prekinio betono požymį.</t>
-        </is>
-      </c>
-      <c r="AG43" s="2" t="inlineStr">
         <is>
           <t>2026-06-30</t>
         </is>
@@ -5736,39 +5390,32 @@
       </c>
       <c r="Q44" s="2" t="inlineStr"/>
       <c r="R44" s="2" t="inlineStr"/>
-      <c r="S44" s="2" t="inlineStr"/>
+      <c r="S44" s="4" t="inlineStr"/>
       <c r="T44" s="2" t="inlineStr">
         <is>
           <t>Viešame kataloge nurodomi betonas, betono mišiniai ir betono gamybos linija Naujojoje Akmenėje.</t>
         </is>
       </c>
-      <c r="U44" s="4" t="n">
+      <c r="U44" s="5" t="n">
         <v>0.78</v>
       </c>
-      <c r="V44" s="5" t="n"/>
-      <c r="W44" s="6" t="n"/>
-      <c r="X44" s="5" t="n"/>
-      <c r="Y44" s="5" t="n"/>
-      <c r="Z44" s="2" t="inlineStr"/>
-      <c r="AA44" s="2" t="inlineStr">
+      <c r="V44" s="2" t="inlineStr"/>
+      <c r="W44" s="2" t="inlineStr">
         <is>
           <t>https://www.1551.lt/kalcitas-ab-betonas-betono-misiniai-betono-gamybos-linija-technikos-nuoma-naujojoje-akmeneje-59982/</t>
         </is>
       </c>
-      <c r="AB44" s="2" t="inlineStr"/>
-      <c r="AC44" s="2" t="inlineStr"/>
-      <c r="AD44" s="2" t="inlineStr"/>
-      <c r="AE44" s="2" t="inlineStr">
+      <c r="X44" s="2" t="inlineStr">
         <is>
           <t>https://www.1551.lt/kalcitas-ab-betonas-betono-misiniai-betono-gamybos-linija-technikos-nuoma-naujojoje-akmeneje-59982/</t>
         </is>
       </c>
-      <c r="AF44" s="2" t="inlineStr">
+      <c r="Y44" s="2" t="inlineStr">
         <is>
           <t>Reikia patikslinti, ar veikla yra nuolat aktyvi.</t>
         </is>
       </c>
-      <c r="AG44" s="2" t="inlineStr">
+      <c r="Z44" s="2" t="inlineStr">
         <is>
           <t>2026-06-30</t>
         </is>
@@ -5849,49 +5496,36 @@
       </c>
       <c r="Q45" s="2" t="inlineStr"/>
       <c r="R45" s="2" t="inlineStr"/>
-      <c r="S45" s="2" t="inlineStr"/>
+      <c r="S45" s="4" t="inlineStr"/>
       <c r="T45" s="2" t="inlineStr">
         <is>
           <t>Įmonė gamina gelžbetonio gaminius, prekinį ir hidrotechninį betoną bei smėlbetonio mišinius.</t>
         </is>
       </c>
-      <c r="U45" s="4" t="n">
+      <c r="U45" s="5" t="n">
         <v>0.9</v>
       </c>
-      <c r="V45" s="5" t="n"/>
-      <c r="W45" s="6" t="n"/>
-      <c r="X45" s="5" t="n">
-        <v>100</v>
-      </c>
-      <c r="Y45" s="5" t="n"/>
+      <c r="V45" s="2" t="inlineStr">
+        <is>
+          <t>https://glg.lt/</t>
+        </is>
+      </c>
+      <c r="W45" s="2" t="inlineStr">
+        <is>
+          <t>https://glg.lt/kontaktai/</t>
+        </is>
+      </c>
+      <c r="X45" s="2" t="inlineStr">
+        <is>
+          <t>https://glg.lt/betonas/betono-misiniai/</t>
+        </is>
+      </c>
+      <c r="Y45" s="2" t="inlineStr">
+        <is>
+          <t>Patikslinta pagal oficialų glg.lt kontaktų ir įmonės aprašymo puslapius.</t>
+        </is>
+      </c>
       <c r="Z45" s="2" t="inlineStr">
-        <is>
-          <t>https://glg.lt/</t>
-        </is>
-      </c>
-      <c r="AA45" s="2" t="inlineStr">
-        <is>
-          <t>https://glg.lt/kontaktai/</t>
-        </is>
-      </c>
-      <c r="AB45" s="2" t="inlineStr"/>
-      <c r="AC45" s="2" t="inlineStr">
-        <is>
-          <t>https://glg.lt/apie-imone/</t>
-        </is>
-      </c>
-      <c r="AD45" s="2" t="inlineStr"/>
-      <c r="AE45" s="2" t="inlineStr">
-        <is>
-          <t>https://glg.lt/betonas/betono-misiniai/</t>
-        </is>
-      </c>
-      <c r="AF45" s="2" t="inlineStr">
-        <is>
-          <t>Patikslinta pagal oficialų glg.lt kontaktų ir įmonės aprašymo puslapius.</t>
-        </is>
-      </c>
-      <c r="AG45" s="2" t="inlineStr">
         <is>
           <t>2026-06-30</t>
         </is>
@@ -5976,39 +5610,32 @@
       </c>
       <c r="Q46" s="2" t="inlineStr"/>
       <c r="R46" s="2" t="inlineStr"/>
-      <c r="S46" s="2" t="inlineStr"/>
+      <c r="S46" s="4" t="inlineStr"/>
       <c r="T46" s="2" t="inlineStr">
         <is>
           <t>Viešame kataloge įmonė siejama su betono mišinių veikla.</t>
         </is>
       </c>
-      <c r="U46" s="4" t="n">
+      <c r="U46" s="5" t="n">
         <v>0.62</v>
       </c>
-      <c r="V46" s="5" t="n"/>
-      <c r="W46" s="6" t="n"/>
-      <c r="X46" s="5" t="n"/>
-      <c r="Y46" s="5" t="n"/>
-      <c r="Z46" s="2" t="inlineStr"/>
-      <c r="AA46" s="2" t="inlineStr">
+      <c r="V46" s="2" t="inlineStr"/>
+      <c r="W46" s="2" t="inlineStr">
         <is>
           <t>https://www.1551.lt/sausta-uab-240915/</t>
         </is>
       </c>
-      <c r="AB46" s="2" t="inlineStr"/>
-      <c r="AC46" s="2" t="inlineStr"/>
-      <c r="AD46" s="2" t="inlineStr"/>
-      <c r="AE46" s="2" t="inlineStr">
+      <c r="X46" s="2" t="inlineStr">
         <is>
           <t>https://www.1551.lt/sausta-uab-240915/</t>
         </is>
       </c>
-      <c r="AF46" s="2" t="inlineStr">
+      <c r="Y46" s="2" t="inlineStr">
         <is>
           <t>Žemos pasitikėjimo įrašas; reikia patikslinti, ar gamyba vykdoma šiame taške.</t>
         </is>
       </c>
-      <c r="AG46" s="2" t="inlineStr">
+      <c r="Z46" s="2" t="inlineStr">
         <is>
           <t>2026-06-30</t>
         </is>
@@ -6093,35 +5720,28 @@
       </c>
       <c r="Q47" s="2" t="inlineStr"/>
       <c r="R47" s="2" t="inlineStr"/>
-      <c r="S47" s="2" t="inlineStr"/>
+      <c r="S47" s="4" t="inlineStr"/>
       <c r="T47" s="2" t="inlineStr">
         <is>
           <t>Registrų centro/VDA atviruose duomenyse pagrindinė veikla nurodyta kaip prekinio betono mišinio gamyba (EVRK 23.63).</t>
         </is>
       </c>
-      <c r="U47" s="4" t="n">
+      <c r="U47" s="5" t="n">
         <v>0.82</v>
       </c>
-      <c r="V47" s="5" t="n"/>
-      <c r="W47" s="6" t="n"/>
-      <c r="X47" s="5" t="n"/>
-      <c r="Y47" s="5" t="n"/>
-      <c r="Z47" s="2" t="inlineStr"/>
-      <c r="AA47" s="2" t="inlineStr">
+      <c r="V47" s="2" t="inlineStr"/>
+      <c r="W47" s="2" t="inlineStr">
         <is>
           <t>https://data.gov.lt/dataset/juridiniu-asmenu-ekonomines-veiklos-rusys-ir-instituciniai-sektoriai/</t>
         </is>
       </c>
-      <c r="AB47" s="2" t="inlineStr"/>
-      <c r="AC47" s="2" t="inlineStr"/>
-      <c r="AD47" s="2" t="inlineStr"/>
-      <c r="AE47" s="2" t="inlineStr"/>
-      <c r="AF47" s="2" t="inlineStr">
+      <c r="X47" s="2" t="inlineStr"/>
+      <c r="Y47" s="2" t="inlineStr">
         <is>
           <t>Adresas geokoduotas pagal viešai randamą įmonės adresą; betono mazgo vietą verta patikslinti atskiru šaltiniu.</t>
         </is>
       </c>
-      <c r="AG47" s="2" t="inlineStr">
+      <c r="Z47" s="2" t="inlineStr">
         <is>
           <t>2026-06-30</t>
         </is>
@@ -6206,35 +5826,28 @@
       </c>
       <c r="Q48" s="2" t="inlineStr"/>
       <c r="R48" s="2" t="inlineStr"/>
-      <c r="S48" s="2" t="inlineStr"/>
+      <c r="S48" s="4" t="inlineStr"/>
       <c r="T48" s="2" t="inlineStr">
         <is>
           <t>Registrų centro/VDA atviruose duomenyse pagrindinė veikla nurodyta kaip prekinio betono mišinio gamyba (EVRK 23.63).</t>
         </is>
       </c>
-      <c r="U48" s="4" t="n">
+      <c r="U48" s="5" t="n">
         <v>0.82</v>
       </c>
-      <c r="V48" s="5" t="n"/>
-      <c r="W48" s="6" t="n"/>
-      <c r="X48" s="5" t="n"/>
-      <c r="Y48" s="5" t="n"/>
-      <c r="Z48" s="2" t="inlineStr"/>
-      <c r="AA48" s="2" t="inlineStr">
+      <c r="V48" s="2" t="inlineStr"/>
+      <c r="W48" s="2" t="inlineStr">
         <is>
           <t>https://data.gov.lt/dataset/juridiniu-asmenu-ekonomines-veiklos-rusys-ir-instituciniai-sektoriai/</t>
         </is>
       </c>
-      <c r="AB48" s="2" t="inlineStr"/>
-      <c r="AC48" s="2" t="inlineStr"/>
-      <c r="AD48" s="2" t="inlineStr"/>
-      <c r="AE48" s="2" t="inlineStr"/>
-      <c r="AF48" s="2" t="inlineStr">
+      <c r="X48" s="2" t="inlineStr"/>
+      <c r="Y48" s="2" t="inlineStr">
         <is>
           <t>Adresas geokoduotas pagal viešai randamą įmonės adresą; betono mazgo vietą verta patikslinti atskiru šaltiniu.</t>
         </is>
       </c>
-      <c r="AG48" s="2" t="inlineStr">
+      <c r="Z48" s="2" t="inlineStr">
         <is>
           <t>2026-06-30</t>
         </is>
@@ -6319,35 +5932,28 @@
       </c>
       <c r="Q49" s="2" t="inlineStr"/>
       <c r="R49" s="2" t="inlineStr"/>
-      <c r="S49" s="2" t="inlineStr"/>
+      <c r="S49" s="4" t="inlineStr"/>
       <c r="T49" s="2" t="inlineStr">
         <is>
           <t>Registrų centro/VDA atviruose duomenyse pagrindinė veikla nurodyta kaip prekinio betono mišinio gamyba (EVRK 23.63).</t>
         </is>
       </c>
-      <c r="U49" s="4" t="n">
+      <c r="U49" s="5" t="n">
         <v>0.82</v>
       </c>
-      <c r="V49" s="5" t="n"/>
-      <c r="W49" s="6" t="n"/>
-      <c r="X49" s="5" t="n"/>
-      <c r="Y49" s="5" t="n"/>
-      <c r="Z49" s="2" t="inlineStr"/>
-      <c r="AA49" s="2" t="inlineStr">
+      <c r="V49" s="2" t="inlineStr"/>
+      <c r="W49" s="2" t="inlineStr">
         <is>
           <t>https://data.gov.lt/dataset/juridiniu-asmenu-ekonomines-veiklos-rusys-ir-instituciniai-sektoriai/</t>
         </is>
       </c>
-      <c r="AB49" s="2" t="inlineStr"/>
-      <c r="AC49" s="2" t="inlineStr"/>
-      <c r="AD49" s="2" t="inlineStr"/>
-      <c r="AE49" s="2" t="inlineStr"/>
-      <c r="AF49" s="2" t="inlineStr">
+      <c r="X49" s="2" t="inlineStr"/>
+      <c r="Y49" s="2" t="inlineStr">
         <is>
           <t>Adresas geokoduotas pagal viešai randamą įmonės adresą; betono mazgo vietą verta patikslinti atskiru šaltiniu.</t>
         </is>
       </c>
-      <c r="AG49" s="2" t="inlineStr">
+      <c r="Z49" s="2" t="inlineStr">
         <is>
           <t>2026-06-30</t>
         </is>
@@ -6432,35 +6038,28 @@
       </c>
       <c r="Q50" s="2" t="inlineStr"/>
       <c r="R50" s="2" t="inlineStr"/>
-      <c r="S50" s="2" t="inlineStr"/>
+      <c r="S50" s="4" t="inlineStr"/>
       <c r="T50" s="2" t="inlineStr">
         <is>
           <t>Registrų centro/VDA atviruose duomenyse pagrindinė veikla nurodyta kaip prekinio betono mišinio gamyba (EVRK 23.63).</t>
         </is>
       </c>
-      <c r="U50" s="4" t="n">
+      <c r="U50" s="5" t="n">
         <v>0.82</v>
       </c>
-      <c r="V50" s="5" t="n"/>
-      <c r="W50" s="6" t="n"/>
-      <c r="X50" s="5" t="n"/>
-      <c r="Y50" s="5" t="n"/>
-      <c r="Z50" s="2" t="inlineStr"/>
-      <c r="AA50" s="2" t="inlineStr">
+      <c r="V50" s="2" t="inlineStr"/>
+      <c r="W50" s="2" t="inlineStr">
         <is>
           <t>https://data.gov.lt/dataset/juridiniu-asmenu-ekonomines-veiklos-rusys-ir-instituciniai-sektoriai/</t>
         </is>
       </c>
-      <c r="AB50" s="2" t="inlineStr"/>
-      <c r="AC50" s="2" t="inlineStr"/>
-      <c r="AD50" s="2" t="inlineStr"/>
-      <c r="AE50" s="2" t="inlineStr"/>
-      <c r="AF50" s="2" t="inlineStr">
+      <c r="X50" s="2" t="inlineStr"/>
+      <c r="Y50" s="2" t="inlineStr">
         <is>
           <t>Adresas geokoduotas pagal viešai randamą įmonės adresą; betono mazgo vietą verta patikslinti atskiru šaltiniu.</t>
         </is>
       </c>
-      <c r="AG50" s="2" t="inlineStr">
+      <c r="Z50" s="2" t="inlineStr">
         <is>
           <t>2026-06-30</t>
         </is>
@@ -6545,43 +6144,36 @@
       </c>
       <c r="Q51" s="2" t="inlineStr"/>
       <c r="R51" s="2" t="inlineStr"/>
-      <c r="S51" s="2" t="inlineStr"/>
+      <c r="S51" s="4" t="inlineStr"/>
       <c r="T51" s="2" t="inlineStr">
         <is>
           <t>Registrų centro/VDA atviruose duomenyse pagrindinė veikla nurodyta kaip prekinio betono mišinio gamyba (EVRK 23.63).</t>
         </is>
       </c>
-      <c r="U51" s="4" t="n">
+      <c r="U51" s="5" t="n">
         <v>0.82</v>
       </c>
-      <c r="V51" s="5" t="n"/>
-      <c r="W51" s="6" t="n"/>
-      <c r="X51" s="5" t="n"/>
-      <c r="Y51" s="5" t="n"/>
+      <c r="V51" s="2" t="inlineStr">
+        <is>
+          <t>https://betonastaurageje.lt/</t>
+        </is>
+      </c>
+      <c r="W51" s="2" t="inlineStr">
+        <is>
+          <t>https://betonastaurageje.lt/kontaktai/</t>
+        </is>
+      </c>
+      <c r="X51" s="2" t="inlineStr">
+        <is>
+          <t>https://betonastaurageje.lt/betonas/</t>
+        </is>
+      </c>
+      <c r="Y51" s="2" t="inlineStr">
+        <is>
+          <t>Oficiali Vinido svetainė patvirtina Gaurės g. 32 adresą, betono gamybą ir betono mazgą.</t>
+        </is>
+      </c>
       <c r="Z51" s="2" t="inlineStr">
-        <is>
-          <t>https://betonastaurageje.lt/</t>
-        </is>
-      </c>
-      <c r="AA51" s="2" t="inlineStr">
-        <is>
-          <t>https://betonastaurageje.lt/kontaktai/</t>
-        </is>
-      </c>
-      <c r="AB51" s="2" t="inlineStr"/>
-      <c r="AC51" s="2" t="inlineStr"/>
-      <c r="AD51" s="2" t="inlineStr"/>
-      <c r="AE51" s="2" t="inlineStr">
-        <is>
-          <t>https://betonastaurageje.lt/betonas/</t>
-        </is>
-      </c>
-      <c r="AF51" s="2" t="inlineStr">
-        <is>
-          <t>Oficiali Vinido svetainė patvirtina Gaurės g. 32 adresą, betono gamybą ir betono mazgą.</t>
-        </is>
-      </c>
-      <c r="AG51" s="2" t="inlineStr">
         <is>
           <t>2026-06-30</t>
         </is>
@@ -6666,43 +6258,36 @@
       </c>
       <c r="Q52" s="2" t="inlineStr"/>
       <c r="R52" s="2" t="inlineStr"/>
-      <c r="S52" s="2" t="inlineStr"/>
+      <c r="S52" s="4" t="inlineStr"/>
       <c r="T52" s="2" t="inlineStr">
         <is>
           <t>Registrų centro/VDA atviruose duomenyse pagrindinė veikla nurodyta kaip prekinio betono mišinio gamyba (EVRK 23.63).</t>
         </is>
       </c>
-      <c r="U52" s="4" t="n">
+      <c r="U52" s="5" t="n">
         <v>0.82</v>
       </c>
-      <c r="V52" s="5" t="n"/>
-      <c r="W52" s="6" t="n"/>
-      <c r="X52" s="5" t="n"/>
-      <c r="Y52" s="5" t="n"/>
+      <c r="V52" s="2" t="inlineStr">
+        <is>
+          <t>https://santvara.eu/</t>
+        </is>
+      </c>
+      <c r="W52" s="2" t="inlineStr">
+        <is>
+          <t>https://santvara.eu/</t>
+        </is>
+      </c>
+      <c r="X52" s="2" t="inlineStr">
+        <is>
+          <t>https://santvara.eu/</t>
+        </is>
+      </c>
+      <c r="Y52" s="2" t="inlineStr">
+        <is>
+          <t>Oficiali Santvara svetainė patvirtina Aruodų g. 34 adresą ir betono bei birių medžiagų veiklą.</t>
+        </is>
+      </c>
       <c r="Z52" s="2" t="inlineStr">
-        <is>
-          <t>https://santvara.eu/</t>
-        </is>
-      </c>
-      <c r="AA52" s="2" t="inlineStr">
-        <is>
-          <t>https://santvara.eu/</t>
-        </is>
-      </c>
-      <c r="AB52" s="2" t="inlineStr"/>
-      <c r="AC52" s="2" t="inlineStr"/>
-      <c r="AD52" s="2" t="inlineStr"/>
-      <c r="AE52" s="2" t="inlineStr">
-        <is>
-          <t>https://santvara.eu/</t>
-        </is>
-      </c>
-      <c r="AF52" s="2" t="inlineStr">
-        <is>
-          <t>Oficiali Santvara svetainė patvirtina Aruodų g. 34 adresą ir betono bei birių medžiagų veiklą.</t>
-        </is>
-      </c>
-      <c r="AG52" s="2" t="inlineStr">
         <is>
           <t>2026-06-30</t>
         </is>
@@ -6787,35 +6372,28 @@
       </c>
       <c r="Q53" s="2" t="inlineStr"/>
       <c r="R53" s="2" t="inlineStr"/>
-      <c r="S53" s="2" t="inlineStr"/>
+      <c r="S53" s="4" t="inlineStr"/>
       <c r="T53" s="2" t="inlineStr">
         <is>
           <t>Registrų centro/VDA atviruose duomenyse pagrindinė veikla nurodyta kaip prekinio betono mišinio gamyba (EVRK 23.63).</t>
         </is>
       </c>
-      <c r="U53" s="4" t="n">
+      <c r="U53" s="5" t="n">
         <v>0.72</v>
       </c>
-      <c r="V53" s="5" t="n"/>
-      <c r="W53" s="6" t="n"/>
-      <c r="X53" s="5" t="n"/>
-      <c r="Y53" s="5" t="n"/>
-      <c r="Z53" s="2" t="inlineStr"/>
-      <c r="AA53" s="2" t="inlineStr">
+      <c r="V53" s="2" t="inlineStr"/>
+      <c r="W53" s="2" t="inlineStr">
         <is>
           <t>https://data.gov.lt/dataset/juridiniu-asmenu-ekonomines-veiklos-rusys-ir-instituciniai-sektoriai/</t>
         </is>
       </c>
-      <c r="AB53" s="2" t="inlineStr"/>
-      <c r="AC53" s="2" t="inlineStr"/>
-      <c r="AD53" s="2" t="inlineStr"/>
-      <c r="AE53" s="2" t="inlineStr"/>
-      <c r="AF53" s="2" t="inlineStr">
+      <c r="X53" s="2" t="inlineStr"/>
+      <c r="Y53" s="2" t="inlineStr">
         <is>
           <t>Adresas rastas viešuose kataloguose, bet geokoduotas tik iki Visagino miesto taško; reikia patikslinti tikslų betono mazgo GPS.</t>
         </is>
       </c>
-      <c r="AG53" s="2" t="inlineStr">
+      <c r="Z53" s="2" t="inlineStr">
         <is>
           <t>2026-06-30</t>
         </is>
@@ -6900,35 +6478,28 @@
       </c>
       <c r="Q54" s="2" t="inlineStr"/>
       <c r="R54" s="2" t="inlineStr"/>
-      <c r="S54" s="2" t="inlineStr"/>
+      <c r="S54" s="4" t="inlineStr"/>
       <c r="T54" s="2" t="inlineStr">
         <is>
           <t>Registrų centro/VDA atviruose duomenyse pagrindinė veikla nurodyta kaip prekinio betono mišinio gamyba (EVRK 23.63).</t>
         </is>
       </c>
-      <c r="U54" s="4" t="n">
+      <c r="U54" s="5" t="n">
         <v>0.82</v>
       </c>
-      <c r="V54" s="5" t="n"/>
-      <c r="W54" s="6" t="n"/>
-      <c r="X54" s="5" t="n"/>
-      <c r="Y54" s="5" t="n"/>
-      <c r="Z54" s="2" t="inlineStr"/>
-      <c r="AA54" s="2" t="inlineStr">
+      <c r="V54" s="2" t="inlineStr"/>
+      <c r="W54" s="2" t="inlineStr">
         <is>
           <t>https://data.gov.lt/dataset/juridiniu-asmenu-ekonomines-veiklos-rusys-ir-instituciniai-sektoriai/</t>
         </is>
       </c>
-      <c r="AB54" s="2" t="inlineStr"/>
-      <c r="AC54" s="2" t="inlineStr"/>
-      <c r="AD54" s="2" t="inlineStr"/>
-      <c r="AE54" s="2" t="inlineStr"/>
-      <c r="AF54" s="2" t="inlineStr">
+      <c r="X54" s="2" t="inlineStr"/>
+      <c r="Y54" s="2" t="inlineStr">
         <is>
           <t>Adresas geokoduotas pagal viešai randamą įmonės adresą; betono mazgo vietą verta patikslinti atskiru šaltiniu.</t>
         </is>
       </c>
-      <c r="AG54" s="2" t="inlineStr">
+      <c r="Z54" s="2" t="inlineStr">
         <is>
           <t>2026-06-30</t>
         </is>
@@ -7013,43 +6584,36 @@
       </c>
       <c r="Q55" s="2" t="inlineStr"/>
       <c r="R55" s="2" t="inlineStr"/>
-      <c r="S55" s="2" t="inlineStr"/>
+      <c r="S55" s="4" t="inlineStr"/>
       <c r="T55" s="2" t="inlineStr">
         <is>
           <t>Registrų centro/VDA atviruose duomenyse pagrindinė veikla nurodyta kaip prekinio betono mišinio gamyba (EVRK 23.63).</t>
         </is>
       </c>
-      <c r="U55" s="4" t="n">
+      <c r="U55" s="5" t="n">
         <v>0.82</v>
       </c>
-      <c r="V55" s="5" t="n"/>
-      <c r="W55" s="6" t="n"/>
-      <c r="X55" s="5" t="n"/>
-      <c r="Y55" s="5" t="n"/>
+      <c r="V55" s="2" t="inlineStr">
+        <is>
+          <t>https://ekobetonas.lt/</t>
+        </is>
+      </c>
+      <c r="W55" s="2" t="inlineStr">
+        <is>
+          <t>https://ekobetonas.lt/kontaktai-betono-gamyba-armaturinis-plienas/</t>
+        </is>
+      </c>
+      <c r="X55" s="2" t="inlineStr">
+        <is>
+          <t>https://ekobetonas.lt/kontaktai-betono-gamyba-armaturinis-plienas/</t>
+        </is>
+      </c>
+      <c r="Y55" s="2" t="inlineStr">
+        <is>
+          <t>Oficialus Ekobetonas kontaktų puslapis patvirtina Gamyklų g. 3 adresą ir betono užsakymų kontaktus.</t>
+        </is>
+      </c>
       <c r="Z55" s="2" t="inlineStr">
-        <is>
-          <t>https://ekobetonas.lt/</t>
-        </is>
-      </c>
-      <c r="AA55" s="2" t="inlineStr">
-        <is>
-          <t>https://ekobetonas.lt/kontaktai-betono-gamyba-armaturinis-plienas/</t>
-        </is>
-      </c>
-      <c r="AB55" s="2" t="inlineStr"/>
-      <c r="AC55" s="2" t="inlineStr"/>
-      <c r="AD55" s="2" t="inlineStr"/>
-      <c r="AE55" s="2" t="inlineStr">
-        <is>
-          <t>https://ekobetonas.lt/kontaktai-betono-gamyba-armaturinis-plienas/</t>
-        </is>
-      </c>
-      <c r="AF55" s="2" t="inlineStr">
-        <is>
-          <t>Oficialus Ekobetonas kontaktų puslapis patvirtina Gamyklų g. 3 adresą ir betono užsakymų kontaktus.</t>
-        </is>
-      </c>
-      <c r="AG55" s="2" t="inlineStr">
         <is>
           <t>2026-06-30</t>
         </is>
@@ -7134,35 +6698,28 @@
       </c>
       <c r="Q56" s="2" t="inlineStr"/>
       <c r="R56" s="2" t="inlineStr"/>
-      <c r="S56" s="2" t="inlineStr"/>
+      <c r="S56" s="4" t="inlineStr"/>
       <c r="T56" s="2" t="inlineStr">
         <is>
           <t>Registrų centro/VDA atviruose duomenyse pagrindinė veikla nurodyta kaip prekinio betono mišinio gamyba (EVRK 23.63).</t>
         </is>
       </c>
-      <c r="U56" s="4" t="n">
+      <c r="U56" s="5" t="n">
         <v>0.72</v>
       </c>
-      <c r="V56" s="5" t="n"/>
-      <c r="W56" s="6" t="n"/>
-      <c r="X56" s="5" t="n"/>
-      <c r="Y56" s="5" t="n"/>
-      <c r="Z56" s="2" t="inlineStr"/>
-      <c r="AA56" s="2" t="inlineStr">
+      <c r="V56" s="2" t="inlineStr"/>
+      <c r="W56" s="2" t="inlineStr">
         <is>
           <t>https://data.gov.lt/dataset/juridiniu-asmenu-ekonomines-veiklos-rusys-ir-instituciniai-sektoriai/</t>
         </is>
       </c>
-      <c r="AB56" s="2" t="inlineStr"/>
-      <c r="AC56" s="2" t="inlineStr"/>
-      <c r="AD56" s="2" t="inlineStr"/>
-      <c r="AE56" s="2" t="inlineStr"/>
-      <c r="AF56" s="2" t="inlineStr">
+      <c r="X56" s="2" t="inlineStr"/>
+      <c r="Y56" s="2" t="inlineStr">
         <is>
           <t>Adresas rastas viešuose kataloguose, bet geokoduotas tik iki Rokiškio miesto taško; reikia patikslinti tikslų betono mazgo GPS.</t>
         </is>
       </c>
-      <c r="AG56" s="2" t="inlineStr">
+      <c r="Z56" s="2" t="inlineStr">
         <is>
           <t>2026-06-30</t>
         </is>
@@ -7247,43 +6804,36 @@
       </c>
       <c r="Q57" s="2" t="inlineStr"/>
       <c r="R57" s="2" t="inlineStr"/>
-      <c r="S57" s="2" t="inlineStr"/>
+      <c r="S57" s="4" t="inlineStr"/>
       <c r="T57" s="2" t="inlineStr">
         <is>
           <t>Registrų centro/VDA atviruose duomenyse pagrindinė veikla nurodyta kaip prekinio betono mišinio gamyba (EVRK 23.63).</t>
         </is>
       </c>
-      <c r="U57" s="4" t="n">
+      <c r="U57" s="5" t="n">
         <v>0.82</v>
       </c>
-      <c r="V57" s="5" t="n"/>
-      <c r="W57" s="6" t="n"/>
-      <c r="X57" s="5" t="n"/>
-      <c r="Y57" s="5" t="n"/>
+      <c r="V57" s="2" t="inlineStr">
+        <is>
+          <t>https://www.betoneura.lt/</t>
+        </is>
+      </c>
+      <c r="W57" s="2" t="inlineStr">
+        <is>
+          <t>https://www.betoneura.lt/kontaktai/</t>
+        </is>
+      </c>
+      <c r="X57" s="2" t="inlineStr">
+        <is>
+          <t>https://www.betoneura.lt/kontaktai/</t>
+        </is>
+      </c>
+      <c r="Y57" s="2" t="inlineStr">
+        <is>
+          <t>Oficialus Beton Eura kontaktų puslapis patvirtina Žilvičių g. 2 adresą ir rekvizitus.</t>
+        </is>
+      </c>
       <c r="Z57" s="2" t="inlineStr">
-        <is>
-          <t>https://www.betoneura.lt/</t>
-        </is>
-      </c>
-      <c r="AA57" s="2" t="inlineStr">
-        <is>
-          <t>https://www.betoneura.lt/kontaktai/</t>
-        </is>
-      </c>
-      <c r="AB57" s="2" t="inlineStr"/>
-      <c r="AC57" s="2" t="inlineStr"/>
-      <c r="AD57" s="2" t="inlineStr"/>
-      <c r="AE57" s="2" t="inlineStr">
-        <is>
-          <t>https://www.betoneura.lt/kontaktai/</t>
-        </is>
-      </c>
-      <c r="AF57" s="2" t="inlineStr">
-        <is>
-          <t>Oficialus Beton Eura kontaktų puslapis patvirtina Žilvičių g. 2 adresą ir rekvizitus.</t>
-        </is>
-      </c>
-      <c r="AG57" s="2" t="inlineStr">
         <is>
           <t>2026-06-30</t>
         </is>
@@ -7368,39 +6918,32 @@
       </c>
       <c r="Q58" s="2" t="inlineStr"/>
       <c r="R58" s="2" t="inlineStr"/>
-      <c r="S58" s="2" t="inlineStr"/>
+      <c r="S58" s="4" t="inlineStr"/>
       <c r="T58" s="2" t="inlineStr">
         <is>
           <t>Registrų centro/VDA atviruose duomenyse pagrindinė veikla nurodyta kaip prekinio betono mišinio gamyba (EVRK 23.63).</t>
         </is>
       </c>
-      <c r="U58" s="4" t="n">
+      <c r="U58" s="5" t="n">
         <v>0.82</v>
       </c>
-      <c r="V58" s="5" t="n"/>
-      <c r="W58" s="6" t="n"/>
-      <c r="X58" s="5" t="n"/>
-      <c r="Y58" s="5" t="n"/>
-      <c r="Z58" s="2" t="inlineStr"/>
-      <c r="AA58" s="2" t="inlineStr">
+      <c r="V58" s="2" t="inlineStr"/>
+      <c r="W58" s="2" t="inlineStr">
         <is>
           <t>https://data.gov.lt/dataset/juridiniu-asmenu-ekonomines-veiklos-rusys-ir-instituciniai-sektoriai/</t>
         </is>
       </c>
-      <c r="AB58" s="2" t="inlineStr"/>
-      <c r="AC58" s="2" t="inlineStr"/>
-      <c r="AD58" s="2" t="inlineStr"/>
-      <c r="AE58" s="2" t="inlineStr">
+      <c r="X58" s="2" t="inlineStr">
         <is>
           <t>https://fsaskaita.lt/imone/uzdaroji-akcine-bendrove-silutes-betonas-177392928</t>
         </is>
       </c>
-      <c r="AF58" s="2" t="inlineStr">
+      <c r="Y58" s="2" t="inlineStr">
         <is>
           <t>Adresas geokoduotas pagal viešai randamą įmonės adresą; betono mazgo vietą verta patikslinti atskiru šaltiniu.</t>
         </is>
       </c>
-      <c r="AG58" s="2" t="inlineStr">
+      <c r="Z58" s="2" t="inlineStr">
         <is>
           <t>2026-06-30</t>
         </is>
@@ -7485,35 +7028,28 @@
       </c>
       <c r="Q59" s="2" t="inlineStr"/>
       <c r="R59" s="2" t="inlineStr"/>
-      <c r="S59" s="2" t="inlineStr"/>
+      <c r="S59" s="4" t="inlineStr"/>
       <c r="T59" s="2" t="inlineStr">
         <is>
           <t>Registrų centro/VDA atviruose duomenyse pagrindinė veikla nurodyta kaip prekinio betono mišinio gamyba (EVRK 23.63).</t>
         </is>
       </c>
-      <c r="U59" s="4" t="n">
+      <c r="U59" s="5" t="n">
         <v>0.82</v>
       </c>
-      <c r="V59" s="5" t="n"/>
-      <c r="W59" s="6" t="n"/>
-      <c r="X59" s="5" t="n"/>
-      <c r="Y59" s="5" t="n"/>
-      <c r="Z59" s="2" t="inlineStr"/>
-      <c r="AA59" s="2" t="inlineStr">
+      <c r="V59" s="2" t="inlineStr"/>
+      <c r="W59" s="2" t="inlineStr">
         <is>
           <t>https://data.gov.lt/dataset/juridiniu-asmenu-ekonomines-veiklos-rusys-ir-instituciniai-sektoriai/</t>
         </is>
       </c>
-      <c r="AB59" s="2" t="inlineStr"/>
-      <c r="AC59" s="2" t="inlineStr"/>
-      <c r="AD59" s="2" t="inlineStr"/>
-      <c r="AE59" s="2" t="inlineStr"/>
-      <c r="AF59" s="2" t="inlineStr">
+      <c r="X59" s="2" t="inlineStr"/>
+      <c r="Y59" s="2" t="inlineStr">
         <is>
           <t>Adresas geokoduotas pagal viešai randamą įmonės adresą; betono mazgo vietą verta patikslinti atskiru šaltiniu.</t>
         </is>
       </c>
-      <c r="AG59" s="2" t="inlineStr">
+      <c r="Z59" s="2" t="inlineStr">
         <is>
           <t>2026-06-30</t>
         </is>
@@ -7598,7 +7134,7 @@
       </c>
       <c r="Q60" s="2" t="inlineStr"/>
       <c r="R60" s="2" t="inlineStr"/>
-      <c r="S60" s="2" t="n">
+      <c r="S60" s="4" t="n">
         <v>2</v>
       </c>
       <c r="T60" s="2" t="inlineStr">
@@ -7606,44 +7142,37 @@
           <t>Oficialiame įmonės puslapyje skelbiama betono mišinių gamyba ir prekyba. Naudotojo duomenimis, betono mazgas vadinasi Elkon, yra 2 silosai.</t>
         </is>
       </c>
-      <c r="U60" s="4" t="n">
+      <c r="U60" s="5" t="n">
         <v>0.86</v>
       </c>
-      <c r="V60" s="5" t="n"/>
-      <c r="W60" s="6" t="n"/>
-      <c r="X60" s="5" t="n"/>
-      <c r="Y60" s="5" t="n"/>
+      <c r="V60" s="2" t="inlineStr">
+        <is>
+          <t>https://www.tkeliai.lt/</t>
+        </is>
+      </c>
+      <c r="W60" s="2" t="inlineStr">
+        <is>
+          <t>https://www.tkeliai.lt/kitos-paslaugos/</t>
+        </is>
+      </c>
+      <c r="X60" s="2" t="inlineStr">
+        <is>
+          <t>https://www.tkeliai.lt/kitos-paslaugos/</t>
+        </is>
+      </c>
+      <c r="Y60" s="2" t="inlineStr">
+        <is>
+          <t>Įtraukta pagal naudotojo informaciją; veikla patvirtinta oficialiame lietuviškame įmonės puslapyje. Naudotojo duomenimis, betono mazgas vadinasi Elkon, yra 2 silosai. Koordinatės nustatytos Lietuvos geolokatoriumi pagal Mažeikių g. 18 adresą.</t>
+        </is>
+      </c>
       <c r="Z60" s="2" t="inlineStr">
-        <is>
-          <t>https://www.tkeliai.lt/</t>
-        </is>
-      </c>
-      <c r="AA60" s="2" t="inlineStr">
-        <is>
-          <t>https://www.tkeliai.lt/kitos-paslaugos/</t>
-        </is>
-      </c>
-      <c r="AB60" s="2" t="inlineStr"/>
-      <c r="AC60" s="2" t="inlineStr"/>
-      <c r="AD60" s="2" t="inlineStr"/>
-      <c r="AE60" s="2" t="inlineStr">
-        <is>
-          <t>https://www.tkeliai.lt/kitos-paslaugos/</t>
-        </is>
-      </c>
-      <c r="AF60" s="2" t="inlineStr">
-        <is>
-          <t>Įtraukta pagal naudotojo informaciją; veikla patvirtinta oficialiame lietuviškame įmonės puslapyje. Naudotojo duomenimis, betono mazgas vadinasi Elkon, yra 2 silosai. Koordinatės nustatytos Lietuvos geolokatoriumi pagal Mažeikių g. 18 adresą.</t>
-        </is>
-      </c>
-      <c r="AG60" s="2" t="inlineStr">
         <is>
           <t>2026-07-06</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AG60"/>
+  <autoFilter ref="A1:Z60"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -7665,7 +7194,7 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="7" t="inlineStr">
+      <c r="A1" s="6" t="inlineStr">
         <is>
           <t>Projektas</t>
         </is>
@@ -7677,7 +7206,7 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="7" t="inlineStr">
+      <c r="A2" s="6" t="inlineStr">
         <is>
           <t>Apimtis</t>
         </is>
@@ -7689,7 +7218,7 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="7" t="inlineStr">
+      <c r="A3" s="6" t="inlineStr">
         <is>
           <t>Įtraukta</t>
         </is>
@@ -7701,7 +7230,7 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="7" t="inlineStr">
+      <c r="A4" s="6" t="inlineStr">
         <is>
           <t>Neįtraukta</t>
         </is>
@@ -7713,7 +7242,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="7" t="inlineStr">
+      <c r="A5" s="6" t="inlineStr">
         <is>
           <t>Duomenų modelis</t>
         </is>
@@ -7725,14 +7254,14 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="7" t="inlineStr">
+      <c r="A6" s="6" t="inlineStr">
         <is>
           <t>Sugeneruota</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-07-06T17:40:42.313250+00:00</t>
+          <t>2026-07-07T09:56:51.153981+00:00</t>
         </is>
       </c>
     </row>
@@ -7758,27 +7287,27 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="8" t="inlineStr">
+      <c r="A1" s="7" t="inlineStr">
         <is>
           <t>Paleidimo laikas</t>
         </is>
       </c>
-      <c r="B1" s="8" t="inlineStr">
+      <c r="B1" s="7" t="inlineStr">
         <is>
           <t>Būsena</t>
         </is>
       </c>
-      <c r="C1" s="8" t="inlineStr">
+      <c r="C1" s="7" t="inlineStr">
         <is>
           <t>Šaltinis</t>
         </is>
       </c>
-      <c r="D1" s="8" t="inlineStr">
+      <c r="D1" s="7" t="inlineStr">
         <is>
           <t>Eilučių skaičius</t>
         </is>
       </c>
-      <c r="E1" s="8" t="inlineStr">
+      <c r="E1" s="7" t="inlineStr">
         <is>
           <t>Pastabos</t>
         </is>
@@ -7787,7 +7316,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-07-06T17:40:42.313250+00:00</t>
+          <t>2026-07-07T09:56:51.155693+00:00</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">

</xml_diff>

<commit_message>
Update Transdosa plant technical data
</commit_message>
<xml_diff>
--- a/data/companies.xlsx
+++ b/data/companies.xlsx
@@ -3511,15 +3511,25 @@
       </c>
       <c r="P27" s="2" t="inlineStr">
         <is>
-          <t>Transdosa betono mazgas</t>
-        </is>
-      </c>
-      <c r="Q27" s="2" t="inlineStr"/>
-      <c r="R27" s="2" t="inlineStr"/>
-      <c r="S27" s="4" t="inlineStr"/>
+          <t>Elkomix-90 quick master</t>
+        </is>
+      </c>
+      <c r="Q27" s="2" t="inlineStr">
+        <is>
+          <t>1,5 m³</t>
+        </is>
+      </c>
+      <c r="R27" s="2" t="inlineStr">
+        <is>
+          <t>40 m³/h</t>
+        </is>
+      </c>
+      <c r="S27" s="4" t="n">
+        <v>2</v>
+      </c>
       <c r="T27" s="2" t="inlineStr">
         <is>
-          <t>Viešai skelbiamas betono mišinių tiekėjas Druskininkų regione.</t>
+          <t>Viešai skelbiamas betono mišinių tiekėjas Druskininkų regione. Naudotojo duomenimis, mazgas (gamintojas) yra Elkomix-90 quick master, maišyklė 1,5 m³, realus našumas 40 m³/h, 2 silosai.</t>
         </is>
       </c>
       <c r="U27" s="5" t="n">
@@ -3542,12 +3552,12 @@
       </c>
       <c r="Y27" s="2" t="inlineStr">
         <is>
-          <t>Oficialūs Transdosa kontaktų ir betono puslapiai patvirtina Margų karjero betono gamybą adresu Žvyro g. 2A.</t>
+          <t>Oficialūs Transdosa kontaktų ir betono puslapiai patvirtina Margų karjero betono gamybą adresu Žvyro g. 2A. Techniniai mazgo duomenys įrašyti pagal naudotojo pateiktą informaciją.</t>
         </is>
       </c>
       <c r="Z27" s="2" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-07-07</t>
         </is>
       </c>
     </row>
@@ -7261,7 +7271,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-07-07T09:56:51.153981+00:00</t>
+          <t>2026-07-07T10:10:08.467905+00:00</t>
         </is>
       </c>
     </row>
@@ -7316,7 +7326,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-07-07T09:56:51.155693+00:00</t>
+          <t>2026-07-07T10:10:08.467905+00:00</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">

</xml_diff>

<commit_message>
Clean Transdosa public description
</commit_message>
<xml_diff>
--- a/data/companies.xlsx
+++ b/data/companies.xlsx
@@ -3529,7 +3529,7 @@
       </c>
       <c r="T27" s="2" t="inlineStr">
         <is>
-          <t>Viešai skelbiamas betono mišinių tiekėjas Druskininkų regione. Naudotojo duomenimis, mazgas (gamintojas) yra Elkomix-90 quick master, maišyklė 1,5 m³, realus našumas 40 m³/h, 2 silosai.</t>
+          <t>Viešai skelbiamas betono mišinių tiekėjas Druskininkų regione.</t>
         </is>
       </c>
       <c r="U27" s="5" t="n">
@@ -7271,7 +7271,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-07-07T10:10:08.467905+00:00</t>
+          <t>2026-07-07T10:16:56.320843+00:00</t>
         </is>
       </c>
     </row>
@@ -7326,7 +7326,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-07-07T10:10:08.467905+00:00</t>
+          <t>2026-07-07T10:16:56.323168+00:00</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">

</xml_diff>

<commit_message>
Update Klaipeda plant data and add VPA
</commit_message>
<xml_diff>
--- a/data/companies.xlsx
+++ b/data/companies.xlsx
@@ -12,7 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Importo žurnalas" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Įmonės'!$A$1:$Z$60</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Įmonės'!$A$1:$Z$61</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -169,8 +169,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ImonesTable" displayName="ImonesTable" ref="A1:Z60" headerRowCount="1">
-  <autoFilter ref="A1:Z60"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ImonesTable" displayName="ImonesTable" ref="A1:Z61" headerRowCount="1">
+  <autoFilter ref="A1:Z61"/>
   <tableColumns count="26">
     <tableColumn id="1" name="Įrašo ID"/>
     <tableColumn id="2" name="Įmonės kodas"/>
@@ -492,7 +492,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z60"/>
+  <dimension ref="A1:Z61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="39" customWidth="1" min="1" max="1"/>
@@ -1743,12 +1743,22 @@
       </c>
       <c r="P11" s="2" t="inlineStr">
         <is>
-          <t>Klaipėdos betono gamykla</t>
-        </is>
-      </c>
-      <c r="Q11" s="2" t="inlineStr"/>
-      <c r="R11" s="2" t="inlineStr"/>
-      <c r="S11" s="4" t="inlineStr"/>
+          <t>Wiggert</t>
+        </is>
+      </c>
+      <c r="Q11" s="2" t="inlineStr">
+        <is>
+          <t>3 m³</t>
+        </is>
+      </c>
+      <c r="R11" s="2" t="inlineStr">
+        <is>
+          <t>60-80 m³/h</t>
+        </is>
+      </c>
+      <c r="S11" s="4" t="n">
+        <v>2</v>
+      </c>
       <c r="T11" s="2" t="inlineStr">
         <is>
           <t>Viešai skelbiamas Heidelberg Materials betono gamyklų tinklo taškas Klaipėdoje.</t>
@@ -1774,12 +1784,12 @@
       </c>
       <c r="Y11" s="2" t="inlineStr">
         <is>
-          <t>Oficialus Heidelberg Materials Lietuva Betonas kontaktų puslapis patvirtina betono užsakymų padalinius Lietuvoje.</t>
+          <t>Oficialus Heidelberg Materials Lietuva Betonas kontaktų puslapis patvirtina betono užsakymų padalinius Lietuvoje. Klaipėdos mazgo techniniai duomenys įrašyti pagal naudotojo pateiktą informaciją.</t>
         </is>
       </c>
       <c r="Z11" s="2" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-07-07</t>
         </is>
       </c>
     </row>
@@ -2411,11 +2421,19 @@
       </c>
       <c r="P17" s="2" t="inlineStr">
         <is>
-          <t>Perdanga Klaipėdos padalinys</t>
-        </is>
-      </c>
-      <c r="Q17" s="2" t="inlineStr"/>
-      <c r="R17" s="2" t="inlineStr"/>
+          <t>Stetter</t>
+        </is>
+      </c>
+      <c r="Q17" s="2" t="inlineStr">
+        <is>
+          <t>2x3 m³</t>
+        </is>
+      </c>
+      <c r="R17" s="2" t="inlineStr">
+        <is>
+          <t>80-100 m³/h</t>
+        </is>
+      </c>
       <c r="S17" s="4" t="inlineStr"/>
       <c r="T17" s="2" t="inlineStr">
         <is>
@@ -2437,13 +2455,17 @@
       </c>
       <c r="X17" s="2" t="inlineStr">
         <is>
-          <t>https://www.perdanga.lt/</t>
-        </is>
-      </c>
-      <c r="Y17" s="2" t="inlineStr"/>
+          <t>https://www.perdanga.lt/lt/produkcija/betono-misiniai/gamyba-transportavimas</t>
+        </is>
+      </c>
+      <c r="Y17" s="2" t="inlineStr">
+        <is>
+          <t>Oficialus Perdangos puslapis nurodo, kad Klaipėdoje betono mišiniai gaminami STETTER technologinėmis linijomis. Maišyklės ir našumo duomenys įrašyti pagal naudotojo pateiktą informaciją.</t>
+        </is>
+      </c>
       <c r="Z17" s="2" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-07-07</t>
         </is>
       </c>
     </row>
@@ -7181,8 +7203,132 @@
         </is>
       </c>
     </row>
+    <row r="61">
+      <c r="A61" s="2" t="inlineStr">
+        <is>
+          <t>vpa-laistai</t>
+        </is>
+      </c>
+      <c r="B61" s="2" t="inlineStr">
+        <is>
+          <t>110185819</t>
+        </is>
+      </c>
+      <c r="C61" s="2" t="inlineStr">
+        <is>
+          <t>UAB V. Paulius &amp; Associates</t>
+        </is>
+      </c>
+      <c r="D61" s="2" t="inlineStr">
+        <is>
+          <t>VPA</t>
+        </is>
+      </c>
+      <c r="E61" s="2" t="inlineStr">
+        <is>
+          <t>Papildomai įtraukta pagal naudotojo informaciją</t>
+        </is>
+      </c>
+      <c r="F61" s="2" t="inlineStr">
+        <is>
+          <t>Laistai</t>
+        </is>
+      </c>
+      <c r="G61" s="2" t="inlineStr">
+        <is>
+          <t>Klaipėdos r. sav.</t>
+        </is>
+      </c>
+      <c r="H61" s="2" t="inlineStr">
+        <is>
+          <t>Stariškės g. 9, Laistų k., Dovilų sen., Klaipėdos r. sav.</t>
+        </is>
+      </c>
+      <c r="I61" s="3" t="n">
+        <v>55.636908</v>
+      </c>
+      <c r="J61" s="3" t="n">
+        <v>21.209254</v>
+      </c>
+      <c r="K61" s="2" t="inlineStr">
+        <is>
+          <t>Naudotojo pateiktos Google Maps nuorodos taškas</t>
+        </is>
+      </c>
+      <c r="L61" s="2" t="inlineStr">
+        <is>
+          <t>Google Maps nuoroda</t>
+        </is>
+      </c>
+      <c r="M61" s="2" t="inlineStr">
+        <is>
+          <t>https://maps.app.goo.gl/2geTBr4zmdrmPY548</t>
+        </is>
+      </c>
+      <c r="N61" s="2" t="inlineStr">
+        <is>
+          <t>ready_mix_concrete</t>
+        </is>
+      </c>
+      <c r="O61" s="2" t="inlineStr">
+        <is>
+          <t>Betono mišiniai</t>
+        </is>
+      </c>
+      <c r="P61" s="2" t="inlineStr">
+        <is>
+          <t>Liebherr</t>
+        </is>
+      </c>
+      <c r="Q61" s="2" t="inlineStr">
+        <is>
+          <t>3 m³</t>
+        </is>
+      </c>
+      <c r="R61" s="2" t="inlineStr">
+        <is>
+          <t>60-80 m³/h</t>
+        </is>
+      </c>
+      <c r="S61" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="T61" s="2" t="inlineStr">
+        <is>
+          <t>VPA betono mazgas Klaipėdos rajone.</t>
+        </is>
+      </c>
+      <c r="U61" s="5" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="V61" s="2" t="inlineStr">
+        <is>
+          <t>https://www.vpa.lt/</t>
+        </is>
+      </c>
+      <c r="W61" s="2" t="inlineStr">
+        <is>
+          <t>https://www.vpa.lt/?Kontaktai=</t>
+        </is>
+      </c>
+      <c r="X61" s="2" t="inlineStr">
+        <is>
+          <t>https://maps.app.goo.gl/2geTBr4zmdrmPY548</t>
+        </is>
+      </c>
+      <c r="Y61" s="2" t="inlineStr">
+        <is>
+          <t>Vieta nustatyta pagal naudotojo pateiktą Google Maps nuorodą. VPA kontaktų puslapis nurodo Stariškės g. 9, Laistų k. adresą. Techniniai mazgo duomenys įrašyti pagal naudotojo pateiktą informaciją.</t>
+        </is>
+      </c>
+      <c r="Z61" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:Z60"/>
+  <autoFilter ref="A1:Z61"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -7271,7 +7417,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-07-07T10:16:56.320843+00:00</t>
+          <t>2026-07-07T15:42:45.790008+00:00</t>
         </is>
       </c>
     </row>
@@ -7326,7 +7472,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-07-07T10:16:56.323168+00:00</t>
+          <t>2026-07-07T15:42:45.790008+00:00</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -7340,7 +7486,7 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Fix coordinate source for Rudninkai plants
</commit_message>
<xml_diff>
--- a/data/companies.xlsx
+++ b/data/companies.xlsx
@@ -956,7 +956,11 @@
           <t>Naudotojo pateiktos koordinatės</t>
         </is>
       </c>
-      <c r="M4" s="2" t="inlineStr"/>
+      <c r="M4" s="2" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps?q=54.43883333333333,25.081</t>
+        </is>
+      </c>
       <c r="N4" s="2" t="inlineStr">
         <is>
           <t>ready_mix_concrete</t>
@@ -1005,7 +1009,11 @@
           <t>https://betonocentras.lt/kontaktai/</t>
         </is>
       </c>
-      <c r="X4" s="2" t="inlineStr"/>
+      <c r="X4" s="2" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps?q=54.43883333333333,25.081</t>
+        </is>
+      </c>
       <c r="Y4" s="2" t="inlineStr">
         <is>
           <t>Papildomas Betono centro mazgas įtrauktas pagal naudotojo pateiktą informaciją. Koordinatės pateiktos DMS formatu: 54°26'19.8"N 25°04'51.6"E.</t>
@@ -1013,7 +1021,7 @@
       </c>
       <c r="Z4" s="2" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
     </row>
@@ -1074,7 +1082,11 @@
           <t>Naudotojo pateiktos koordinatės</t>
         </is>
       </c>
-      <c r="M5" s="2" t="inlineStr"/>
+      <c r="M5" s="2" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps?q=54.439245484061935,25.080984271007022</t>
+        </is>
+      </c>
       <c r="N5" s="2" t="inlineStr">
         <is>
           <t>ready_mix_concrete</t>
@@ -1123,7 +1135,11 @@
           <t>https://betonocentras.lt/kontaktai/</t>
         </is>
       </c>
-      <c r="X5" s="2" t="inlineStr"/>
+      <c r="X5" s="2" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps?q=54.439245484061935,25.080984271007022</t>
+        </is>
+      </c>
       <c r="Y5" s="2" t="inlineStr">
         <is>
           <t>Papildomas Betono centro mazgas įtrauktas pagal naudotojo pateiktą informaciją. Koordinatės pateiktos dešimtainiu formatu.</t>
@@ -1131,7 +1147,7 @@
       </c>
       <c r="Z5" s="2" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
     </row>
@@ -7823,7 +7839,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-07-09T13:04:48.352757+00:00</t>
+          <t>2026-07-10T03:25:32.948243+00:00</t>
         </is>
       </c>
     </row>
@@ -7878,7 +7894,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-07-09T13:04:48.353564+00:00</t>
+          <t>2026-07-10T03:25:32.948243+00:00</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">

</xml_diff>

<commit_message>
Update Suduvos betonas company data
</commit_message>
<xml_diff>
--- a/data/companies.xlsx
+++ b/data/companies.xlsx
@@ -513,7 +513,7 @@
     <col width="40" customWidth="1" min="16" max="16"/>
     <col width="27" customWidth="1" min="17" max="17"/>
     <col width="30" customWidth="1" min="18" max="18"/>
-    <col width="17" customWidth="1" min="19" max="19"/>
+    <col width="19" customWidth="1" min="19" max="19"/>
     <col width="42" customWidth="1" min="20" max="20"/>
     <col width="29" customWidth="1" min="21" max="21"/>
     <col width="42" customWidth="1" min="22" max="22"/>
@@ -3439,10 +3439,14 @@
           <t>suduvos-betonas-marijampole</t>
         </is>
       </c>
-      <c r="B26" s="2" t="inlineStr"/>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>302330957</t>
+        </is>
+      </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>UAB Sūduvos betonas</t>
+          <t>UAB Surenkamos statybos konstrukcijos</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
@@ -3467,7 +3471,7 @@
       </c>
       <c r="H26" s="2" t="inlineStr">
         <is>
-          <t>Sporto g. 9H, Marijampolė</t>
+          <t>Sporto g. 9H, LT-68108 Marijampolė</t>
         </is>
       </c>
       <c r="I26" s="3" t="n">
@@ -3506,20 +3510,28 @@
           <t>Sūduvos betono mazgas</t>
         </is>
       </c>
-      <c r="Q26" s="2" t="inlineStr"/>
+      <c r="Q26" s="2" t="inlineStr">
+        <is>
+          <t>Nenurodyta viešai</t>
+        </is>
+      </c>
       <c r="R26" s="2" t="inlineStr">
         <is>
           <t>iki 200 m³ per darbo pamainą</t>
         </is>
       </c>
-      <c r="S26" s="4" t="inlineStr"/>
+      <c r="S26" s="4" t="inlineStr">
+        <is>
+          <t>Nenurodyta viešai</t>
+        </is>
+      </c>
       <c r="T26" s="2" t="inlineStr">
         <is>
-          <t>Viešai skelbiamas betono mišinių gamintojas; nurodomas našumas iki 200 m³ per darbo pamainą.</t>
+          <t>Oficialiame puslapyje nurodoma betono mišinių gamyba ir pristatymas; Marijampolėje esantis 130 arų betono mazgas gali pagaminti iki 200 m³ betono per darbo pamainą.</t>
         </is>
       </c>
       <c r="U26" s="5" t="n">
-        <v>0.75</v>
+        <v>0.9</v>
       </c>
       <c r="V26" s="2" t="inlineStr">
         <is>
@@ -3533,13 +3545,17 @@
       </c>
       <c r="X26" s="2" t="inlineStr">
         <is>
-          <t>https://www.suduvos-betonas.lt/</t>
-        </is>
-      </c>
-      <c r="Y26" s="2" t="inlineStr"/>
+          <t>https://www.suduvos-betonas.lt/betono-misiniai/</t>
+        </is>
+      </c>
+      <c r="Y26" s="2" t="inlineStr">
+        <is>
+          <t>Atnaujinta pagal oficialų suduvos-betonas.lt kontaktų, pradinį ir betono mišinių puslapius: juridinis pavadinimas, įmonės kodas, adresas, betono mišinių veikla ir viešas mazgo aprašymas.</t>
+        </is>
+      </c>
       <c r="Z26" s="2" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-07-13</t>
         </is>
       </c>
     </row>
@@ -7839,7 +7855,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-07-10T03:25:32.948243+00:00</t>
+          <t>2026-07-13T04:27:42.668209+00:00</t>
         </is>
       </c>
     </row>
@@ -7894,7 +7910,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-07-10T03:25:32.948243+00:00</t>
+          <t>2026-07-13T04:27:42.670874+00:00</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">

</xml_diff>

<commit_message>
Add C3 Beton plant locations
</commit_message>
<xml_diff>
--- a/data/companies.xlsx
+++ b/data/companies.xlsx
@@ -1,18 +1,18 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Įmonės" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Metaduomenys" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Importo žurnalas" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Įmonės" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Metaduomenys" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Importo žurnalas" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Įmonės'!$A$1:$Z$64</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Įmonės'!$A$1:$Z$68</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -169,8 +169,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ImonesTable" displayName="ImonesTable" ref="A1:Z64" headerRowCount="1">
-  <autoFilter ref="A1:Z64"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ImonesTable" displayName="ImonesTable" ref="A1:Z68" headerRowCount="1">
+  <autoFilter ref="A1:Z68"/>
   <tableColumns count="26">
     <tableColumn id="1" name="Įrašo ID"/>
     <tableColumn id="2" name="Įmonės kodas"/>
@@ -492,11 +492,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z64"/>
+  <dimension ref="A1:Z68"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="39" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="19" customWidth="1" min="2" max="2"/>
     <col width="42" customWidth="1" min="3" max="3"/>
     <col width="33" customWidth="1" min="4" max="4"/>
     <col width="42" customWidth="1" min="5" max="5"/>
@@ -7765,8 +7765,512 @@
         </is>
       </c>
     </row>
+    <row r="65">
+      <c r="A65" s="2" t="inlineStr">
+        <is>
+          <t>c3-beton-baisogala</t>
+        </is>
+      </c>
+      <c r="B65" s="2" t="inlineStr">
+        <is>
+          <t>Nenurodyta viešai</t>
+        </is>
+      </c>
+      <c r="C65" s="2" t="inlineStr">
+        <is>
+          <t>C3 Betonas</t>
+        </is>
+      </c>
+      <c r="D65" s="2" t="inlineStr">
+        <is>
+          <t>C3 Betonas</t>
+        </is>
+      </c>
+      <c r="E65" s="2" t="inlineStr">
+        <is>
+          <t>Konkurentas</t>
+        </is>
+      </c>
+      <c r="F65" s="2" t="inlineStr">
+        <is>
+          <t>Baisogala</t>
+        </is>
+      </c>
+      <c r="G65" s="2" t="inlineStr">
+        <is>
+          <t>Radviliškio r. sav.</t>
+        </is>
+      </c>
+      <c r="H65" s="2" t="inlineStr">
+        <is>
+          <t>Dvaro g., Baisogala, Radviliškio r. sav.</t>
+        </is>
+      </c>
+      <c r="I65" s="3" t="n">
+        <v>55.6372</v>
+      </c>
+      <c r="J65" s="3" t="n">
+        <v>23.7183</v>
+      </c>
+      <c r="K65" s="2" t="inlineStr">
+        <is>
+          <t>Oficialiame puslapyje pateiktas gamyklos taškas</t>
+        </is>
+      </c>
+      <c r="L65" s="2" t="inlineStr">
+        <is>
+          <t>C3 Betonas oficialus puslapis</t>
+        </is>
+      </c>
+      <c r="M65" s="2" t="inlineStr">
+        <is>
+          <t>https://c3beton.com/lt/betonas</t>
+        </is>
+      </c>
+      <c r="N65" s="2" t="inlineStr">
+        <is>
+          <t>ready_mix_concrete</t>
+        </is>
+      </c>
+      <c r="O65" s="2" t="inlineStr">
+        <is>
+          <t>Betono mišiniai</t>
+        </is>
+      </c>
+      <c r="P65" s="2" t="inlineStr">
+        <is>
+          <t>Baisiogala Plant</t>
+        </is>
+      </c>
+      <c r="Q65" s="2" t="inlineStr">
+        <is>
+          <t>Nenurodyta viešai</t>
+        </is>
+      </c>
+      <c r="R65" s="2" t="inlineStr">
+        <is>
+          <t>Nenurodyta viešai</t>
+        </is>
+      </c>
+      <c r="S65" s="4" t="inlineStr">
+        <is>
+          <t>Nenurodyta viešai</t>
+        </is>
+      </c>
+      <c r="T65" s="2" t="inlineStr">
+        <is>
+          <t>Oficialiame C3 Betonas puslapyje ši vieta rodoma kaip C3 betono gamykla Lietuvos tinkle. C3 nurodo, kad aplink gamyklas taikomas 50 km pristatymo spindulys.</t>
+        </is>
+      </c>
+      <c r="U65" s="5" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="V65" s="2" t="inlineStr">
+        <is>
+          <t>https://c3beton.com/</t>
+        </is>
+      </c>
+      <c r="W65" s="2" t="inlineStr">
+        <is>
+          <t>https://c3beton.com/lt/betonas</t>
+        </is>
+      </c>
+      <c r="X65" s="2" t="inlineStr">
+        <is>
+          <t>https://c3beton.com/lt/betonas</t>
+        </is>
+      </c>
+      <c r="Y65" s="2" t="inlineStr">
+        <is>
+          <t>Įtraukta pagal oficialaus C3 Betonas puslapio žemėlapį. Koordinatės paimtos iš oficialaus puslapio programinio kodo; adresas patikslintas pagal koordinates. Įmonės kodas ir techniniai mazgo duomenys viešai nenurodyti.</t>
+        </is>
+      </c>
+      <c r="Z65" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="2" t="inlineStr">
+        <is>
+          <t>c3-beton-martiniskis</t>
+        </is>
+      </c>
+      <c r="B66" s="2" t="inlineStr">
+        <is>
+          <t>Nenurodyta viešai</t>
+        </is>
+      </c>
+      <c r="C66" s="2" t="inlineStr">
+        <is>
+          <t>C3 Betonas</t>
+        </is>
+      </c>
+      <c r="D66" s="2" t="inlineStr">
+        <is>
+          <t>C3 Betonas</t>
+        </is>
+      </c>
+      <c r="E66" s="2" t="inlineStr">
+        <is>
+          <t>Konkurentas</t>
+        </is>
+      </c>
+      <c r="F66" s="2" t="inlineStr">
+        <is>
+          <t>Martiniškis</t>
+        </is>
+      </c>
+      <c r="G66" s="2" t="inlineStr">
+        <is>
+          <t>Jonavos r. sav.</t>
+        </is>
+      </c>
+      <c r="H66" s="2" t="inlineStr">
+        <is>
+          <t>Vanagiškiai, Kulvos sen., Jonavos r. sav.</t>
+        </is>
+      </c>
+      <c r="I66" s="3" t="n">
+        <v>55.1441659</v>
+      </c>
+      <c r="J66" s="3" t="n">
+        <v>24.1869636</v>
+      </c>
+      <c r="K66" s="2" t="inlineStr">
+        <is>
+          <t>Oficialiame puslapyje pateiktas gamyklos taškas</t>
+        </is>
+      </c>
+      <c r="L66" s="2" t="inlineStr">
+        <is>
+          <t>C3 Betonas oficialus puslapis</t>
+        </is>
+      </c>
+      <c r="M66" s="2" t="inlineStr">
+        <is>
+          <t>https://c3beton.com/lt/betonas</t>
+        </is>
+      </c>
+      <c r="N66" s="2" t="inlineStr">
+        <is>
+          <t>ready_mix_concrete</t>
+        </is>
+      </c>
+      <c r="O66" s="2" t="inlineStr">
+        <is>
+          <t>Betono mišiniai</t>
+        </is>
+      </c>
+      <c r="P66" s="2" t="inlineStr">
+        <is>
+          <t>Martiniškis Plant</t>
+        </is>
+      </c>
+      <c r="Q66" s="2" t="inlineStr">
+        <is>
+          <t>Nenurodyta viešai</t>
+        </is>
+      </c>
+      <c r="R66" s="2" t="inlineStr">
+        <is>
+          <t>Nenurodyta viešai</t>
+        </is>
+      </c>
+      <c r="S66" s="4" t="inlineStr">
+        <is>
+          <t>Nenurodyta viešai</t>
+        </is>
+      </c>
+      <c r="T66" s="2" t="inlineStr">
+        <is>
+          <t>Oficialiame C3 Betonas puslapyje ši vieta rodoma kaip C3 betono gamykla Lietuvos tinkle. C3 nurodo, kad aplink gamyklas taikomas 50 km pristatymo spindulys.</t>
+        </is>
+      </c>
+      <c r="U66" s="5" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="V66" s="2" t="inlineStr">
+        <is>
+          <t>https://c3beton.com/</t>
+        </is>
+      </c>
+      <c r="W66" s="2" t="inlineStr">
+        <is>
+          <t>https://c3beton.com/lt/betonas</t>
+        </is>
+      </c>
+      <c r="X66" s="2" t="inlineStr">
+        <is>
+          <t>https://c3beton.com/lt/betonas</t>
+        </is>
+      </c>
+      <c r="Y66" s="2" t="inlineStr">
+        <is>
+          <t>Įtraukta pagal oficialaus C3 Betonas puslapio žemėlapį. Koordinatės paimtos iš oficialaus puslapio programinio kodo; adresas patikslintas pagal koordinates. Įmonės kodas ir techniniai mazgo duomenys viešai nenurodyti.</t>
+        </is>
+      </c>
+      <c r="Z66" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="2" t="inlineStr">
+        <is>
+          <t>c3-beton-stasenai</t>
+        </is>
+      </c>
+      <c r="B67" s="2" t="inlineStr">
+        <is>
+          <t>Nenurodyta viešai</t>
+        </is>
+      </c>
+      <c r="C67" s="2" t="inlineStr">
+        <is>
+          <t>C3 Betonas</t>
+        </is>
+      </c>
+      <c r="D67" s="2" t="inlineStr">
+        <is>
+          <t>C3 Betonas</t>
+        </is>
+      </c>
+      <c r="E67" s="2" t="inlineStr">
+        <is>
+          <t>Konkurentas</t>
+        </is>
+      </c>
+      <c r="F67" s="2" t="inlineStr">
+        <is>
+          <t>Stašėnai</t>
+        </is>
+      </c>
+      <c r="G67" s="2" t="inlineStr">
+        <is>
+          <t>Jonavos r. sav.</t>
+        </is>
+      </c>
+      <c r="H67" s="2" t="inlineStr">
+        <is>
+          <t>Dirvaliai, Šveicarijos sen., Jonavos r. sav.</t>
+        </is>
+      </c>
+      <c r="I67" s="3" t="n">
+        <v>55.033</v>
+      </c>
+      <c r="J67" s="3" t="n">
+        <v>24.183</v>
+      </c>
+      <c r="K67" s="2" t="inlineStr">
+        <is>
+          <t>Oficialiame puslapyje pateiktas gamyklos taškas</t>
+        </is>
+      </c>
+      <c r="L67" s="2" t="inlineStr">
+        <is>
+          <t>C3 Betonas oficialus puslapis</t>
+        </is>
+      </c>
+      <c r="M67" s="2" t="inlineStr">
+        <is>
+          <t>https://c3beton.com/lt/betonas</t>
+        </is>
+      </c>
+      <c r="N67" s="2" t="inlineStr">
+        <is>
+          <t>ready_mix_concrete</t>
+        </is>
+      </c>
+      <c r="O67" s="2" t="inlineStr">
+        <is>
+          <t>Betono mišiniai</t>
+        </is>
+      </c>
+      <c r="P67" s="2" t="inlineStr">
+        <is>
+          <t>Stašėnai Plant</t>
+        </is>
+      </c>
+      <c r="Q67" s="2" t="inlineStr">
+        <is>
+          <t>Nenurodyta viešai</t>
+        </is>
+      </c>
+      <c r="R67" s="2" t="inlineStr">
+        <is>
+          <t>Nenurodyta viešai</t>
+        </is>
+      </c>
+      <c r="S67" s="4" t="inlineStr">
+        <is>
+          <t>Nenurodyta viešai</t>
+        </is>
+      </c>
+      <c r="T67" s="2" t="inlineStr">
+        <is>
+          <t>Oficialiame C3 Betonas puslapyje ši vieta rodoma kaip C3 betono gamykla Lietuvos tinkle. C3 nurodo, kad aplink gamyklas taikomas 50 km pristatymo spindulys.</t>
+        </is>
+      </c>
+      <c r="U67" s="5" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="V67" s="2" t="inlineStr">
+        <is>
+          <t>https://c3beton.com/</t>
+        </is>
+      </c>
+      <c r="W67" s="2" t="inlineStr">
+        <is>
+          <t>https://c3beton.com/lt/betonas</t>
+        </is>
+      </c>
+      <c r="X67" s="2" t="inlineStr">
+        <is>
+          <t>https://c3beton.com/lt/betonas</t>
+        </is>
+      </c>
+      <c r="Y67" s="2" t="inlineStr">
+        <is>
+          <t>Įtraukta pagal oficialaus C3 Betonas puslapio žemėlapį. Koordinatės paimtos iš oficialaus puslapio programinio kodo; adresas patikslintas pagal koordinates. Įmonės kodas ir techniniai mazgo duomenys viešai nenurodyti.</t>
+        </is>
+      </c>
+      <c r="Z67" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="2" t="inlineStr">
+        <is>
+          <t>c3-beton-runeikiai</t>
+        </is>
+      </c>
+      <c r="B68" s="2" t="inlineStr">
+        <is>
+          <t>Nenurodyta viešai</t>
+        </is>
+      </c>
+      <c r="C68" s="2" t="inlineStr">
+        <is>
+          <t>C3 Betonas</t>
+        </is>
+      </c>
+      <c r="D68" s="2" t="inlineStr">
+        <is>
+          <t>C3 Betonas</t>
+        </is>
+      </c>
+      <c r="E68" s="2" t="inlineStr">
+        <is>
+          <t>Konkurentas</t>
+        </is>
+      </c>
+      <c r="F68" s="2" t="inlineStr">
+        <is>
+          <t>Runeikiai</t>
+        </is>
+      </c>
+      <c r="G68" s="2" t="inlineStr">
+        <is>
+          <t>Kėdainių r. sav.</t>
+        </is>
+      </c>
+      <c r="H68" s="2" t="inlineStr">
+        <is>
+          <t>Paguiriai, Šėtos sen., Kėdainių r. sav.</t>
+        </is>
+      </c>
+      <c r="I68" s="3" t="n">
+        <v>55.3327393</v>
+      </c>
+      <c r="J68" s="3" t="n">
+        <v>24.3501308</v>
+      </c>
+      <c r="K68" s="2" t="inlineStr">
+        <is>
+          <t>Oficialiame puslapyje pateiktas gamyklos taškas</t>
+        </is>
+      </c>
+      <c r="L68" s="2" t="inlineStr">
+        <is>
+          <t>C3 Betonas oficialus puslapis</t>
+        </is>
+      </c>
+      <c r="M68" s="2" t="inlineStr">
+        <is>
+          <t>https://c3beton.com/lt/betonas</t>
+        </is>
+      </c>
+      <c r="N68" s="2" t="inlineStr">
+        <is>
+          <t>ready_mix_concrete</t>
+        </is>
+      </c>
+      <c r="O68" s="2" t="inlineStr">
+        <is>
+          <t>Betono mišiniai</t>
+        </is>
+      </c>
+      <c r="P68" s="2" t="inlineStr">
+        <is>
+          <t>Runeikiai Plant</t>
+        </is>
+      </c>
+      <c r="Q68" s="2" t="inlineStr">
+        <is>
+          <t>Nenurodyta viešai</t>
+        </is>
+      </c>
+      <c r="R68" s="2" t="inlineStr">
+        <is>
+          <t>Nenurodyta viešai</t>
+        </is>
+      </c>
+      <c r="S68" s="4" t="inlineStr">
+        <is>
+          <t>Nenurodyta viešai</t>
+        </is>
+      </c>
+      <c r="T68" s="2" t="inlineStr">
+        <is>
+          <t>Oficialiame C3 Betonas puslapyje ši vieta rodoma kaip C3 betono gamykla Lietuvos tinkle. C3 nurodo, kad aplink gamyklas taikomas 50 km pristatymo spindulys.</t>
+        </is>
+      </c>
+      <c r="U68" s="5" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="V68" s="2" t="inlineStr">
+        <is>
+          <t>https://c3beton.com/</t>
+        </is>
+      </c>
+      <c r="W68" s="2" t="inlineStr">
+        <is>
+          <t>https://c3beton.com/lt/betonas</t>
+        </is>
+      </c>
+      <c r="X68" s="2" t="inlineStr">
+        <is>
+          <t>https://c3beton.com/lt/betonas</t>
+        </is>
+      </c>
+      <c r="Y68" s="2" t="inlineStr">
+        <is>
+          <t>Įtraukta pagal oficialaus C3 Betonas puslapio žemėlapį. Koordinatės paimtos iš oficialaus puslapio programinio kodo; adresas patikslintas pagal koordinates. Įmonės kodas ir techniniai mazgo duomenys viešai nenurodyti.</t>
+        </is>
+      </c>
+      <c r="Z68" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:Z64"/>
+  <autoFilter ref="A1:Z68"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -7855,7 +8359,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-07-13T13:32:47.759862+00:00</t>
+          <t>2026-07-14T04:45:36.169029+00:00</t>
         </is>
       </c>
     </row>
@@ -7910,7 +8414,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-07-13T13:32:47.760623+00:00</t>
+          <t>2026-07-14T04:45:36.169029+00:00</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -7924,7 +8428,7 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Update C3 Beton Martiniskis plant details
</commit_message>
<xml_diff>
--- a/data/companies.xlsx
+++ b/data/companies.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Įmonės" sheetId="1" r:id="R10e4d03a89544b35"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Metaduomenys" sheetId="2" r:id="R7cfe2c7e8f56454e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Importo žurnalas" sheetId="3" r:id="Re5662bdcfc4f4608"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Įmonės" sheetId="1" r:id="R4b332577e3944bc0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Metaduomenys" sheetId="2" r:id="R421057b3ef7b495c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Importo žurnalas" sheetId="3" r:id="R0b410843a08f4230"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -8698,25 +8698,17 @@
           <x:t xml:space="preserve">Martiniškis Plant</x:t>
         </x:is>
       </x:c>
-      <x:c r="Q66" s="2" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Nenurodyta viešai</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="R66" s="2" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Nenurodyta viešai</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="S66" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Nenurodyta viešai</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="T66" s="2" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Oficialiame C3 Betonas puslapyje ši vieta rodoma kaip C3 betono gamykla Lietuvos tinkle. C3 nurodo, kad aplink gamyklas taikomas 50 km pristatymo spindulys.</x:t>
-        </x:is>
+      <x:c r="Q66" s="2" t="str">
+        <x:v>Ammann Elba Euromix C120, 3 m³</x:v>
+      </x:c>
+      <x:c r="R66" s="2" t="str">
+        <x:v>60–80 m³/val.</x:v>
+      </x:c>
+      <x:c r="S66" s="4" t="str">
+        <x:v>2x85 t</x:v>
+      </x:c>
+      <x:c r="T66" s="2" t="str">
+        <x:v>Betono mazgas Ammann Elba Euromix C120; maišyklė 3 m³; našumas 60–80 m³/val.; silosai 2x85 t.</x:v>
       </x:c>
       <x:c r="U66" s="5" t="n">
         <x:v>0.9</x:v>
@@ -8736,15 +8728,11 @@
           <x:t xml:space="preserve">https://c3beton.com/lt/betonas</x:t>
         </x:is>
       </x:c>
-      <x:c r="Y66" s="2" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Įtraukta pagal oficialaus C3 Betonas puslapio žemėlapį. Koordinatės paimtos iš oficialaus puslapio programinio kodo; adresas patikslintas pagal koordinates. Įmonės kodas ir techniniai mazgo duomenys viešai nenurodyti.</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="Z66" s="2" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">2026-07-14</x:t>
-        </x:is>
+      <x:c r="Y66" s="2" t="str">
+        <x:v>Įtraukta pagal oficialaus C3 Betonas puslapio žemėlapį. Koordinatės paimtos iš oficialaus puslapio programinio kodo; adresas patikslintas pagal koordinates. Techniniai duomenys papildyti pagal naudotojo pateiktą informaciją.</x:v>
+      </x:c>
+      <x:c r="Z66" s="2" t="str">
+        <x:v>2026-07-14</x:v>
       </x:c>
     </x:row>
     <x:row r="67">
@@ -8990,7 +8978,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R284d885e4e6d4b60"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R51fe119d5ed448aa"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
Update C3 Beton Runeikiai plant details
</commit_message>
<xml_diff>
--- a/data/companies.xlsx
+++ b/data/companies.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Įmonės" sheetId="1" r:id="R4b332577e3944bc0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Metaduomenys" sheetId="2" r:id="R421057b3ef7b495c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Importo žurnalas" sheetId="3" r:id="R0b410843a08f4230"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Įmonės" sheetId="1" r:id="R4a589dff238840d2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Metaduomenys" sheetId="2" r:id="R56454f474c474d59"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Importo žurnalas" sheetId="3" r:id="R5a8ff13d88a94e10"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -8926,25 +8926,17 @@
           <x:t xml:space="preserve">Runeikiai Plant</x:t>
         </x:is>
       </x:c>
-      <x:c r="Q68" s="2" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Nenurodyta viešai</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="R68" s="2" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Nenurodyta viešai</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="S68" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Nenurodyta viešai</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="T68" s="2" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Oficialiame C3 Betonas puslapyje ši vieta rodoma kaip C3 betono gamykla Lietuvos tinkle. C3 nurodo, kad aplink gamyklas taikomas 50 km pristatymo spindulys.</x:t>
-        </x:is>
+      <x:c r="Q68" s="2" t="str">
+        <x:v>Ammann Elba Euromix C120, 3 m³</x:v>
+      </x:c>
+      <x:c r="R68" s="2" t="str">
+        <x:v>60–80 m³/val.</x:v>
+      </x:c>
+      <x:c r="S68" s="4" t="str">
+        <x:v>2x85 t</x:v>
+      </x:c>
+      <x:c r="T68" s="2" t="str">
+        <x:v>Betono mazgas Ammann Elba Euromix C120; maišyklė 3 m³; našumas 60–80 m³/val.; silosai 2x85 t.</x:v>
       </x:c>
       <x:c r="U68" s="5" t="n">
         <x:v>0.9</x:v>
@@ -8964,21 +8956,17 @@
           <x:t xml:space="preserve">https://c3beton.com/lt/betonas</x:t>
         </x:is>
       </x:c>
-      <x:c r="Y68" s="2" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Įtraukta pagal oficialaus C3 Betonas puslapio žemėlapį. Koordinatės paimtos iš oficialaus puslapio programinio kodo; adresas patikslintas pagal koordinates. Įmonės kodas ir techniniai mazgo duomenys viešai nenurodyti.</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="Z68" s="2" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">2026-07-14</x:t>
-        </x:is>
+      <x:c r="Y68" s="2" t="str">
+        <x:v>Įtraukta pagal oficialaus C3 Betonas puslapio žemėlapį. Koordinatės paimtos iš oficialaus puslapio programinio kodo; adresas patikslintas pagal koordinates. Techniniai duomenys papildyti pagal naudotojo pateiktą informaciją.</x:v>
+      </x:c>
+      <x:c r="Z68" s="2" t="str">
+        <x:v>2026-07-14</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R51fe119d5ed448aa"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf69e06476c314939"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
Add Reljef Rukla concrete plant
</commit_message>
<xml_diff>
--- a/data/companies.xlsx
+++ b/data/companies.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Įmonės" sheetId="1" r:id="R4a589dff238840d2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Metaduomenys" sheetId="2" r:id="R56454f474c474d59"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Importo žurnalas" sheetId="3" r:id="R5a8ff13d88a94e10"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Įmonės" sheetId="1" r:id="Ra1c1d3add2f147c7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Metaduomenys" sheetId="2" r:id="Rf216069d720a499d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Importo žurnalas" sheetId="3" r:id="R7716828eabb84aa6"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -15,8 +15,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:numFmts count="1">
+  <x:numFmts count="2">
     <x:numFmt numFmtId="164" formatCode="0.000000"/>
+    <x:numFmt numFmtId="200" formatCode="yyyy-mm-dd hh:mm:ss"/>
   </x:numFmts>
   <x:fonts count="2">
     <x:font>
@@ -58,7 +59,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="8">
+  <x:cellXfs count="9">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyAlignment="1">
       <x:alignment vertical="top"/>
@@ -79,6 +80,7 @@
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyAlignment="1">
       <x:alignment vertical="center"/>
     </x:xf>
+    <x:xf numFmtId="200" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -155,8 +157,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ImonesTable" displayName="ImonesTable" ref="A1:Z68" headerRowCount="1">
-  <x:autoFilter ref="A1:Z68"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ImonesTable" displayName="ImonesTable" ref="A1:Z69" headerRowCount="1" totalsRowCount="0">
+  <x:autoFilter ref="A1:Z69"/>
   <x:tableColumns count="26">
     <x:tableColumn id="1" name="Įrašo ID"/>
     <x:tableColumn id="2" name="Įmonės kodas"/>
@@ -8963,10 +8965,90 @@
         <x:v>2026-07-14</x:v>
       </x:c>
     </x:row>
+    <x:row r="69">
+      <x:c r="A69" t="str">
+        <x:v>reljef-rukla</x:v>
+      </x:c>
+      <x:c r="B69" t="str">
+        <x:v>301731961</x:v>
+      </x:c>
+      <x:c r="C69" t="str">
+        <x:v>UAB Reljef</x:v>
+      </x:c>
+      <x:c r="D69" t="str">
+        <x:v>Reljef</x:v>
+      </x:c>
+      <x:c r="E69" t="str">
+        <x:v>Konkurentas</x:v>
+      </x:c>
+      <x:c r="F69" t="str">
+        <x:v>Rukla</x:v>
+      </x:c>
+      <x:c r="G69" t="str">
+        <x:v>Jonavos r. sav.</x:v>
+      </x:c>
+      <x:c r="H69" t="str">
+        <x:v>Rukla, Jonavos r. sav.</x:v>
+      </x:c>
+      <x:c r="I69" t="n">
+        <x:v>55.05225</x:v>
+      </x:c>
+      <x:c r="J69" t="n">
+        <x:v>24.4064167</x:v>
+      </x:c>
+      <x:c r="K69" t="str">
+        <x:v>Tikslus naudotojo pateiktas taškas; adresas artimiausias pagal OpenStreetMap</x:v>
+      </x:c>
+      <x:c r="L69" t="str">
+        <x:v>Naudotojo pateiktos koordinatės</x:v>
+      </x:c>
+      <x:c r="M69" t="str">
+        <x:v>https://www.openstreetmap.org/?mlat=55.05225&amp;mlon=24.4064167#map=18/55.05225/24.4064167</x:v>
+      </x:c>
+      <x:c r="N69" t="str">
+        <x:v>ready_mix_concrete</x:v>
+      </x:c>
+      <x:c r="O69" t="str">
+        <x:v>Betono mišiniai</x:v>
+      </x:c>
+      <x:c r="P69" t="str">
+        <x:v>Ammann Elba</x:v>
+      </x:c>
+      <x:c r="Q69" t="str">
+        <x:v>Nenustatyta</x:v>
+      </x:c>
+      <x:c r="R69" t="str">
+        <x:v>Nenustatytas</x:v>
+      </x:c>
+      <x:c r="S69" t="str">
+        <x:v>2x65 t</x:v>
+      </x:c>
+      <x:c r="T69" t="str">
+        <x:v>Rukloje veikiantis UAB Reljef betono mazgas: Ammann Elba, 2x65 t silosai. Maišyklė ir našumas nenustatyti.</x:v>
+      </x:c>
+      <x:c r="U69" t="n">
+        <x:v>0.82</x:v>
+      </x:c>
+      <x:c r="V69" t="str">
+        <x:v>https://www.reljef.lt/</x:v>
+      </x:c>
+      <x:c r="W69" t="str">
+        <x:v>https://www.reljef.lt/</x:v>
+      </x:c>
+      <x:c r="X69" t="str">
+        <x:v>https://www.openstreetmap.org/?mlat=55.05225&amp;mlon=24.4064167#map=18/55.05225/24.4064167</x:v>
+      </x:c>
+      <x:c r="Y69" t="str">
+        <x:v>Įmonės rekvizitai paimti iš oficialaus UAB Reljef puslapio. Betono mazgo gamintojas, silosai ir lokacija įrašyti pagal naudotojo pateiktą informaciją. Artimiausias viešai geokoduotas adresas nustatytas pagal OpenStreetMap.</x:v>
+      </x:c>
+      <x:c r="Z69" t="str">
+        <x:v>2026-07-17</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf69e06476c314939"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra5df30accd144ba2"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9045,10 +9127,8 @@
           <x:t xml:space="preserve">Sugeneruota</x:t>
         </x:is>
       </x:c>
-      <x:c r="B6" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">2026-07-14T04:45:36.169029+00:00</x:t>
-        </x:is>
+      <x:c r="B6" s="8" t="n">
+        <x:v>46220.44885988426</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -9095,10 +9175,8 @@
       </x:c>
     </x:row>
     <x:row r="2">
-      <x:c r="A2" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">2026-07-14T04:45:36.169029+00:00</x:t>
-        </x:is>
+      <x:c r="A2" s="8" t="n">
+        <x:v>46220.44885988426</x:v>
       </x:c>
       <x:c r="B2" t="inlineStr">
         <x:is>
@@ -9111,7 +9189,7 @@
         </x:is>
       </x:c>
       <x:c r="D2" t="n">
-        <x:v>67</x:v>
+        <x:v>68</x:v>
       </x:c>
       <x:c r="E2" t="inlineStr">
         <x:is>

</xml_diff>